<commit_message>
docs: add capture-first rule (T051) — log every discussion point before replying
CLAUDE.md now mandates that any point needing a fix or discussion (any size)
is logged as a Pending task in docs/TASK_PIPELINE.xlsx BEFORE answering, with
its T### stated in the reply. Stays Pending until done/decided.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2971,6 +2971,53 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>T051</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Capture-first workflow rule</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Infra/Docs</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Locked 2026-06-03 at the user's request: every time the user raises ANY point that needs fixing or discussion — big or small (bug, design tweak, decision, idea, 'look into X') — the FIRST action BEFORE replying is to log it here as a new Pending task with the next T### id, then answer (and tell the user the id). It stays Pending until actually done/decided, then flips to Done/Deferred/Parked/Reverted. Encoded as the CAPTURE-FIRST mandate in CLAUDE.md so it persists across sessions.</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Ongoing discipline — applies to every future turn. Nothing to build.</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>CLAUDE.md (CAPTURE-FIRST bullet); scripts/build_task_pipeline_xlsx.py</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -2986,7 +3033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3022,102 +3069,119 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
+          <t>CAPTURE-FIRST RULE (locked 2026-06-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Every time a point comes up that needs fixing or discussion — ANY size — it gets logged here as a Pending task with a new T### id BEFORE the assistant replies, then it's answered. It stays Pending until the work is actually done/decided, then flips to Done (or Deferred/Parked/Reverted). Small items are exactly what gets lost, so nothing is too small to capture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="8" customHeight="1">
+      <c r="A8" s="14" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
           <t>STATUS VALUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Done — shipped (and usually deployed/committed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>In progress — actively being iterated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Pending — agreed/known but not started.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Deferred — intentionally postponed (waiting on something or a user decision).</t>
+          <t>Done — shipped (and usually deployed/committed).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Parked — discussed then set aside; needs a user decision to re-open.</t>
+          <t>In progress — actively being iterated.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
+          <t>Pending — agreed/known but not started.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Deferred — intentionally postponed (waiting on something or a user decision).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Parked — discussed then set aside; needs a user decision to re-open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
           <t>Reverted — was tried, then undone.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="8" customHeight="1">
-      <c r="A13" s="14" t="inlineStr"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
+    <row r="16" ht="8" customHeight="1">
+      <c r="A16" s="14" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>HOW TO UPDATE (the .xlsx is GENERATED, do not hand-edit)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>1. Edit the TASKS list in scripts/build_task_pipeline_xlsx.py (add a row / flip a status / update the 'where we left off' + 'next' text).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>New tasks get the next free T### id. Never reuse or renumber an id.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="8" customHeight="1">
-      <c r="A19" s="14" t="inlineStr"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="22" ht="8" customHeight="1">
+      <c r="A22" s="14" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>SCOPE NOTE</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Seeded 2026-06-03 from the current CLAUDE.md + recent sessions. Older sessions weren't fully transcribed, so the 'prior' rows are best-effort reconstructions of completed features. Treat this as the authoritative living record from here forward — keep it current.</t>
         </is>

</xml_diff>

<commit_message>
docs: log T052 (hydration — count non-water fluids toward goal)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3013,6 +3013,53 @@
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>T052</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Hydration: count non-water fluids toward goal</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>User wants the hydration goal to feel realistic — almost nobody drinks the full plain-water target every day. Asked whether science supports counting non-water fluids. Answer = yes: National Academies (IOM 2004) frames the daily target as TOTAL water from all sources (~80% from beverages of every kind, ~20% from food); Maughan et al. 2016 Beverage Hydration Index shows milk / juice / oral-rehydration hydrate AS WELL AS or better than water, and coffee / tea / soda ~= water (the 'caffeine dehydrates you' idea is a myth at normal intake, Killer 2014); alcohol is the real diuretic exception. Presented a decision on how granular to count fluids. Sub-task of T016 (hydration page redesign).</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>User to pick the counting model: (1) all non-alcoholic beverages count 1:1, (2) science-weighted per-drink multipliers (BHI), or (3) hybrid — 1:1 for non-alcoholic, alcohol discounted/excluded. Then reframe goal as 'total fluid' + add a fluid-type logging UI on the hydration page.</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
docs: hydration BHI decided (T052) + log T053-T056 (picker, eligibility, log, progress)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3039,27 +3039,215 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>User wants the hydration goal to feel realistic — almost nobody drinks the full plain-water target every day. Asked whether science supports counting non-water fluids. Answer = yes: National Academies (IOM 2004) frames the daily target as TOTAL water from all sources (~80% from beverages of every kind, ~20% from food); Maughan et al. 2016 Beverage Hydration Index shows milk / juice / oral-rehydration hydrate AS WELL AS or better than water, and coffee / tea / soda ~= water (the 'caffeine dehydrates you' idea is a myth at normal intake, Killer 2014); alcohol is the real diuretic exception. Presented a decision on how granular to count fluids. Sub-task of T016 (hydration page redesign).</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-06-03 = option 2 (science-weighted Beverage Hydration Index multipliers). Curated eligible drinks + multipliers: water / sparkling water / coffee / tea / diet-or-zero soda = 1.0, milk = 1.5 (the one allowed calorie drink, and the best-hydrating). Effective hydration = sum(ml x multiplier) vs the 35 ml/kg goal. Umbrella for build sub-tasks T053 (fast picker), T054 (eligibility messaging), T055 (log shows the drink), T056 (non-intimidating progress display).</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>T053</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Hydration: fast drink picker (no dropdowns)</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>User wants the hydration goal to feel realistic — almost nobody drinks the full plain-water target every day. Asked whether science supports counting non-water fluids. Answer = yes: National Academies (IOM 2004) frames the daily target as TOTAL water from all sources (~80% from beverages of every kind, ~20% from food); Maughan et al. 2016 Beverage Hydration Index shows milk / juice / oral-rehydration hydrate AS WELL AS or better than water, and coffee / tea / soda ~= water (the 'caffeine dehydrates you' idea is a myth at normal intake, Killer 2014); alcohol is the real diuretic exception. Presented a decision on how granular to count fluids. Sub-task of T016 (hydration page redesign).</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>User to pick the counting model: (1) all non-alcoholic beverages count 1:1, (2) science-weighted per-drink multipliers (BHI), or (3) hybrid — 1:1 for non-alcoholic, alcohol discounted/excluded. Then reframe goal as 'total fluid' + add a fluid-type logging UI on the hydration page.</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>User: need a clever picker for drink TYPE + SIZE that's fast to tap — explicitly NO dropdowns (a dropdown puts selection effort on the user and won't go well). Proposed two-tap design on one sheet: row of drink-type tiles (icon + tiny label: Water / Sparkling / Coffee / Tea / Diet soda / Milk) + a row of VESSEL-icon size chips (glass / cup / mug / bottle / large bottle mapped to common ml) instead of numbers; optional 'custom' chip opens the existing PhantomWheel for an exact amount.</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Build after the progress-display direction (T056) is locked. Confirm the eligible type list + the vessel-size presets with the user.</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx; PhantomWheel for custom path</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>T054</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Hydration: eligibility messaging</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>User: make it explicit that only zero-calorie, low-calorie, milk, and non-alcoholic drinks count. Plan: the picker only ever offers eligible drink types (no alcohol, no full-sugar drinks) — that curation is itself the clearest signal — plus a short static info-pill explainer (intent-only per the info-pill rule, no formulas): roughly 'Only no/low-calorie, non-alcoholic drinks count toward hydration — plus milk. Sugary and alcoholic drinks don't.'</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Write the final copy + wire the info pill. Confirm whether borderline drinks (juice, sports drinks) are excluded (current read: yes — they're calorie drinks; milk is the sole calorie exception).</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>mobile/app/(app)/hydration.tsx</t>
         </is>
       </c>
-      <c r="I55" s="5" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>T055</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Hydration: log shows what was drunk</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>User: the log should show what was drunk, not just a fluid total. Plan: each entry row shows drink icon + type + size + time (e.g. 'Milk · 250 ml · 9:14a'), optionally its hydration contribution.</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Build the per-entry log row; decide whether to surface the per-drink multiplier contribution.</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>T056</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Hydration: non-intimidating progress display</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>User: raw fluid value (e.g. '2547 ml') is too intimidating as the headline — wants something friendlier. Options proposed: (A) percent + mascot mood, (B) 'cups' metaphor (effective hydration / ~250 ml -&gt; N cups; milk visibly fills 1.5, making the science tangible), (C) rising water level in the existing PixelScene tied to the mascot (pure visual, most on-brand). Recommended C as the headline with a quiet 'cups' readout, raw ml only on tap.</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>User to pick A / B / C (recommended C + cups readout). Then build into the hydration page over the existing HydrationPet + PixelScene.</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx; HydrationPet.tsx; PixelScene.tsx</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
fix(hydration): attribution matches detail-page footer style (T057); lock T056 progress display
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>User to pick A / B / C (recommended C + cups readout). Then build into the hydration page over the existing HydrationPet + PixelScene.</t>
+          <t>DECIDED 2026-06-03 = option C (rising water level in the PixelScene as the headline) + a quiet 'cups' readout; raw ml only on tap. Build pending as part of the T052 feature.</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -3248,6 +3248,53 @@
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>T057</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Hydration: attribution styling to match other pages</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>User: the hydration attribution should look like the credit line on other detail pages — the small dimmed dot-separated footer (strength 'Epley · Brzycki · Lombardi averaged', cardio 'Riegel · Daniels' · Seiler ...'). FIXED 2026-06-03: hydration's s.attribution now matches the house tinyText style (muted, 11px, lineHeight 16, left-aligned) and was moved to the BOTTOM of the progress card as a footer credit — same placement as strength/cardio (it used to be centered between the readout and the quick-add chips).</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
feat(hydration): weight drinks by Beverage Hydration Index (T052-T056)
- Migration: water_logs.drink_type (default water, CHECK to 6 eligible types).
- Drink picker (no dropdowns): 6 type tiles -> size chips 250/350/500 + Custom wheel.
- Eligibility note: only no/low-cal, non-alcoholic drinks + milk count.
- Effective hydration = sum(amount_ml * BHI multiplier); milk = 1.5x.
- Progress = rising water "pond" in PixelScene + friendly "cups" readout
  (tap -> exact mL); 7-day chart now plots effective mL.
- Log rows show the drink (icon + label + size) with a x1.5 badge on milk.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -3039,9 +3039,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E55" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>DECIDED 2026-06-03 = option 2 (science-weighted Beverage Hydration Index multipliers). Curated eligible drinks + multipliers: water / sparkling water / coffee / tea / diet-or-zero soda = 1.0, milk = 1.5 (the one allowed calorie drink, and the best-hydrating). Effective hydration = sum(ml x multiplier) vs the 35 ml/kg goal. Umbrella for build sub-tasks T053 (fast picker), T054 (eligibility messaging), T055 (log shows the drink), T056 (non-intimidating progress display).</t>
+          <t>BUILT 2026-06-03 (option 2, BHI multipliers). DB: migration add_drink_type_to_water_logs (water_logs.drink_type, default 'water', CHECK to the 6 eligible types). App (hydration.tsx): drink registry water/sparkling/coffee/tea/soda=1.0 + milk=1.5; effective hydration = sum(amount_ml x multiplier) drives the pet/water-level, the cups readout, AND the 7-day chart; 35 mL/kg goal unchanged. Sub-parts T053-T056 all Done. tsc clean. Possible polish later: wavy water top, save-confirm flash.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -3086,9 +3086,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>REFINED 2026-06-03 (user): size presets must be REALISTIC PER DRINK TYPE, not one shared size row — a 750 ml 'large bottle' of soda or milk isn't a real choice. Proposed per-type vessels: Water = Glass 250 / Bottle 500 / Large 1 L; Sparkling = Glass 250 / Can 330 / Bottle 500; Coffee = Espresso 60 / Cup 250 / Large 350; Tea = Cup 250 / Mug 350 / Large 450; Diet soda = Glass 250 / Can 330 / Bottle 500; Milk = Small 150 / Glass 250 / Large 350. Plus a Custom chip (PhantomWheel). Awaiting user confirm, then build.</t>
+          <t>BUILT 2026-06-03: 6 drink-type tiles (lucide GlassWater/Droplets/Coffee/Leaf/CupSoda/Milk) -&gt; tap reveals a size row (250/350/500 mL or 8/12/16 oz) + a Custom chip that opens the PhantomWheel in a modal. Two taps, no dropdowns. Inline FadeInUp expansion (Pattern 5).</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -3133,9 +3133,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Write the final copy + wire the info pill. Confirm whether borderline drinks (juice, sports drinks) are excluded (current read: yes — they're calorie drinks; milk is the sole calorie exception).</t>
+          <t>BUILT 2026-06-03: the picker only offers eligible types (no alcohol, no full-sugar drinks) + a static note under it: 'Only no- and low-calorie, non-alcoholic drinks count toward hydration — milk included.' Juice / sports drinks excluded as calorie drinks; milk is the sole calorie exception.</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -3180,9 +3180,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Build the per-entry log row; decide whether to surface the per-drink multiplier contribution.</t>
+          <t>BUILT 2026-06-03: each log row shows the drink's icon + label + size + time; milk rows carry a small 'x1.5' badge so the BHI bonus is visible.</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
@@ -3227,9 +3227,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>DECIDED 2026-06-03 = option C (rising water level in the PixelScene as the headline) + a quiet 'cups' readout; raw ml only on tap. Build pending as part of the T052 feature.</t>
+          <t>BUILT 2026-06-03: PixelScene gained a fillFrac prop that draws a translucent rising 'pond' (up to ~66% of the scene) from progress; HydrationPet passes the effective fill. Headline readout is a friendly 'X of Y cups' (a cup ~ 250 mL effective); tap it to flip to exact effective-vs-target mL.</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(hydration): remove water pond + replace-not-expand picker (T058,T061)
- Remove the rising-water Skia render from PixelScene + fillFrac wiring (T058).
- Picker now swaps the type grid for the chosen drink's sizes with a
  "Change drink" back button — no inline expansion / Animated.View (T061).
- Drop the FadeInUp animation that likely caused the page-wide dead-touch
  regression (T059/T060); unit + delete logic were already correct.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3295,6 +3295,194 @@
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>T058</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Hydration: remove the rising-water pond</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>User doesn't want the 'water flowing' effect in the pixel art. Revert the T056 PixelScene water Rects + the fillFrac prop wiring on HydrationPet/PixelScene. Keep the cups readout (that part stays) — only the in-scene water is removed.</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-03: removed the water Group from PixelScene + the fillFrac prop on PixelScene &amp; HydrationPet. Scene is back to the original day/night art; the cups readout stays as the progress indicator.</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>mobile/src/components/PixelScene.tsx; HydrationPet.tsx</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>T059</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Hydration BUG: fl-oz unit not applied + picker dead</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>After switching Settings fluid unit to fl oz, the hydration page stayed in mL AND the picker buttons stopped responding. Regression from the T052-T056 build. Diagnose: (a) does Settings write fluid_unit='oz' and does the profile propagate to the page; (b) why the picker Pressables stopped firing (suspect the FadeInUp Animated.View / Modal / half-loaded bundle).</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>Settings writes fluid_unit='oz'/'mL' (confirmed); the page derives fluidUnit + sizes reactively from profile, so a correct profile shows oz. The dead-touch triad (picker + delete + unit all frozen at once) most likely a half-applied Fast Refresh — no clean reload was possible (adb couldn't reach the phone). Rewrote the picker, removing the Animated.View expansion (the likely real culprit). CONFIRM after a FULL app restart; if oz still doesn't show, investigate whether a Settings save propagates the profile context to the other tabs.</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx; settings.tsx; AuthContext</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>T060</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Hydration BUG: log entries won't delete</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Deleting today's log rows did nothing. deleteEntry itself was unchanged, so the regression is likely the new log-row layout (lucide Icon intercepting touches inside DeleteAction) or the same page-wide dead-touch issue as T059.</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>DeleteAction + deleteEntry are unchanged &amp; correct (two-tap: tap trash -&gt; red check -&gt; deletes). The dead delete was part of the same page-wide frozen-touch symptom as T059, not delete-specific. Should clear with the rewrite + a clean reload. CONFIRM after restart (tap the trash icon on a row, then the red check).</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx; DeleteAction.tsx</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>T061</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Hydration: picker REPLACES, not expands</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>User rejects the expanding picker. Wanted behaviour: tapping a drink type REPLACES the type-tile row with the size buttons for that drink (with a back / change-drink affordance), instead of revealing an extra row below. Removes the FadeInUp inline expansion entirely.</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-03: picker is now a two-state swap — the 6-type grid is REPLACED by the chosen drink's size buttons (250/350/500 + Custom) with a 'Change drink' back button (ChevronLeft); logging a size returns to the grid. No FadeInUp expansion. tsc clean.</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
fix(hydration): attribution unit-free + source-names-first to match other pages (T062)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Settings writes fluid_unit='oz'/'mL' (confirmed); the page derives fluidUnit + sizes reactively from profile, so a correct profile shows oz. The dead-touch triad (picker + delete + unit all frozen at once) most likely a half-applied Fast Refresh — no clean reload was possible (adb couldn't reach the phone). Rewrote the picker, removing the Animated.View expansion (the likely real culprit). CONFIRM after a FULL app restart; if oz still doesn't show, investigate whether a Settings save propagates the profile context to the other tabs.</t>
+          <t>UPDATE 2026-06-03: the 'unit stayed mL' part was the ATTRIBUTION line (hardcoded '35 mL/kg ...') — fixed in T062. The size buttons DO switch with the unit (they derive from profile). The dead picker/delete touches were the page-wide frozen-touch symptom (half-applied Fast Refresh + the Animated.View expansion, now removed). Picker/delete still to CONFIRM after a clean restart; if they remain dead, dig into that specific surface with the app reachable.</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -3483,6 +3483,53 @@
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>T062</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Hydration attribution: drop mL + source-names-first</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>User: the attribution still read '35 mL/kg bodyweight ...' — so it showed mL even with oz selected, and its FORMAT didn't match other pages (which lead with source NAMES: strength 'Epley · Brzycki · Lombardi ...', cardio 'Riegel · Daniels' ...'). This is what the earlier 'unit stayed in mL' (T059) actually referred to — the hardcoded mL in this line, not the size buttons. FIXED 2026-06-03: targetAttribution is now unit-free + source-names-first — hasWeight 'National Academies · Mayo Clinic · EFSA · by bodyweight'; no-weight 'National Academies · EFSA · sex-based estimate'. (Dropped the 'log your weight to personalize' prose for format parity; the 35 mL/kg science stays in the code comment.)</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
docs: close T059/T060 (hydration page confirmed working)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -3368,9 +3368,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E62" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>UPDATE 2026-06-03: the 'unit stayed mL' part was the ATTRIBUTION line (hardcoded '35 mL/kg ...') — fixed in T062. The size buttons DO switch with the unit (they derive from profile). The dead picker/delete touches were the page-wide frozen-touch symptom (half-applied Fast Refresh + the Animated.View expansion, now removed). Picker/delete still to CONFIRM after a clean restart; if they remain dead, dig into that specific surface with the app reachable.</t>
+          <t>RESOLVED 2026-06-03: the 'unit stayed mL' part was the ATTRIBUTION line (fixed in T062); the size buttons derive from profile and switch with the unit. The dead picker/delete touches were the page-wide frozen-touch symptom (half-applied Fast Refresh + the now-removed Animated.View expansion). Closed per user 'this is done' — they've been interacting with the live picker through every follow-up tweak, so touches work.</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -3415,9 +3415,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E63" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>DeleteAction + deleteEntry are unchanged &amp; correct (two-tap: tap trash -&gt; red check -&gt; deletes). The dead delete was part of the same page-wide frozen-touch symptom as T059, not delete-specific. Should clear with the rewrite + a clean reload. CONFIRM after restart (tap the trash icon on a row, then the red check).</t>
+          <t>RESOLVED 2026-06-03: DeleteAction + deleteEntry were unchanged &amp; correct (two-tap: trash -&gt; red check). The dead delete was the same page-wide frozen-touch symptom as T059, now cleared. Closed per user 'this is done'.</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">

</xml_diff>

<commit_message>
chore: close T013/T040, drop rom_records (T049), scrub mobility from legal (T050)
- Ledger: closed radial-nav redesign (T013) + direct integrations (T040).
- T049: migration drops rom_records; patched anonymize_account_now() to stop
  deleting from it; removed it from delete-user edge fn's table list.
- T050: removed mobility/ROM wording from Privacy Policy, DPA, Coach Agreement.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -81,7 +81,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
     <fill>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Reverted</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Radial-nav design rework is still wanted by the user but the green direction is rejected. Re-open when the user picks a new direction.</t>
+          <t>CLOSED 2026-06-03 per user. Green direction rejected + already reverted; not pursuing a radial-nav redesign for now. Reopen if the user picks a new direction.</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -2475,9 +2475,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Not started. First three (Strava/Fitbit/HealthKit) have no approval delay; the rest are gated on developer-program approvals (apply in parallel). See docs/integrations/developer-program-applications.md.</t>
+          <t>CLOSED 2026-06-03 per user — not pursuing direct per-platform wearable integrations for now. Health Connect Phase 1 (T036) remains in the app as the Android path. Reopen if revisited; the build order + infra notes above are preserved.</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -2898,19 +2898,19 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>After T012 removed the Mobility UI, the rom_records table is orphaned (no UI reads it; delete-user/export functions still clean it). Dropping it is destructive (deletes historical ROM data) so it was intentionally left for the user to decide.</t>
+          <t>After T012 removed the Mobility UI, the rom_records table was orphaned (no UI reads it). Dropping it is destructive (deletes historical ROM data) so it waited for user OK.</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>User decision: keep (historical) or drop. If drop, also remove the table refs in the delete-user/export edge functions.</t>
+          <t>DONE 2026-06-03 per user 'run 8'. Migration 20260603d_drop_rom_records: patched anonymize_account_now() to drop its 'DELETE FROM rom_records' line, then DROP TABLE rom_records CASCADE (RLS policies + activity-log trigger went with it). Verified gone; only trg_log_data_activity keeps a harmless dead 'rom_records' CASE-string branch. delete-user edge-fn source had its rom_records entry removed (per-table try/catch made it non-fatal anyway) — needs a routine `supabase functions deploy delete-user` (non-urgent, admin-only path).</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -2945,19 +2945,19 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E53" s="12" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Privacy Policy / DPA / Coach Agreement still list 'mobility / range-of-motion assessments' as a collected data category. Left untouched in T012 because legal copy is sensitive (and historical rom_records data still exists).</t>
+          <t>Privacy Policy / DPA / Coach Agreement listed 'mobility / range-of-motion' as a collected data category. Left until T012's owner OK'd it.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>User/legal decision on whether to remove the ROM data-category language.</t>
+          <t>DONE 2026-06-03 per user 'run 9'. Removed the mobility/ROM wording: PrivacyPolicy (workout-entries list + 'mobility / range-of-motion assessments' + 'ROM records' in the deletion paragraph), DataProcessingAgreement ('mobility ROM'), CoachAgreement ('Mobility' in the training-logs line). Ships with the next web deploy.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -3550,7 +3550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3649,56 +3649,63 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="8" customHeight="1">
-      <c r="A16" s="14" t="inlineStr"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Closed — dropped / won't do for now (can be reopened).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1">
+      <c r="A17" s="14" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>HOW TO UPDATE (the .xlsx is GENERATED, do not hand-edit)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>1. Edit the TASKS list in scripts/build_task_pipeline_xlsx.py (add a row / flip a status / update the 'where we left off' + 'next' text).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
+          <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
+          <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
           <t>New tasks get the next free T### id. Never reuse or renumber an id.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="8" customHeight="1">
-      <c r="A22" s="14" t="inlineStr"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="23" ht="8" customHeight="1">
+      <c r="A23" s="14" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>SCOPE NOTE</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Seeded 2026-06-03 from the current CLAUDE.md + recent sessions. Older sessions weren't fully transcribed, so the 'prior' rows are best-effort reconstructions of completed features. Treat this as the authoritative living record from here forward — keep it current.</t>
         </is>

</xml_diff>

<commit_message>
feat(dashboard): add Sleep + Hydration stat chips, mirrored to admin + coach (T014)
- Mobile dashboard: 😴 avg sleep (7 nights, from sleep_sessions) + 💧 days
  hit water goal (last 7, effective mL vs 35 mL/kg) chips.
- Mirrored to admin AdminUserDetail + coach CoachClientDetail snapshot badges
  (SnapshotBadge gained indigo/cyan). Each chip hides when there's no data.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -86,12 +86,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -1253,19 +1253,19 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Current pills: Strength PRs, Cardio PRs, Food streak, Lowest HR, Weekly weight. Gap pages were Sleep, Hydration, Mobility. PROPOSED + recommended: add Sleep ('avg Xh / 7 nights', indigo) and Hydration ('X days hit water goal / 14', cyan). Mobility pill DROPPED (feature removed, T012). Data confirmed available (sleep_sessions, water_logs). Whatever lands MUST mirror to admin + coach client dashboards.</t>
+          <t>Gap pages were Sleep + Hydration (Mobility pill dropped — feature removed in T012). Added two chips on ALL three surfaces: 'Nh avg sleep . 7 nights' (indigo, from sleep_sessions.duration_s) + 'N days hit water goal . 7d' (cyan: days in the last 7 where sum(amount_ml x BHI multiplier) &gt;= 35 mL/kg of latest bodyweight). Each chip hides when there's no data, like the existing chips.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Awaiting user go-ahead on the two pills (Sleep avg + Hydration streak). Then implement on mobile dashboard + admin AdminUserDetail + coach CoachClientDetail.</t>
+          <t>DONE 2026-06-03 (awaiting user device test). Surfaces: mobile dashboard.tsx; web AdminUserDetail.jsx + CoachClientDetail.jsx (their SnapshotBadge gained indigo/cyan colors). mobile tsc clean + web build clean. Sleep/Hydration coaching-surface promotions (T043/T044) are separate roadmap items.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1300,7 +1300,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -1347,7 +1347,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2522,7 +2522,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E44" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2616,7 +2616,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2663,7 +2663,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2710,7 +2710,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E48" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2757,7 +2757,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E49" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2851,7 +2851,7 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
docs: log T063-T065 (stat pills uniform layout, weight=change, 30-day windows)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3530,6 +3530,147 @@
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>T063</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard stat pills: uniform size + grid layout</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E66" s="10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>User wants all stat pills EXACTLY the same size, laid out with '3 on each side' and the last pill centered under them (reads as a 2-column grid: 3 left + 3 right + 7th centered; could also mean 3-per-row — to confirm). Today the 7 pills wrap with text-driven variable widths. Needs fixed-width pills + terse uniform wording so they fit. Mobile dashboard + admin + coach (mirror).</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Confirm layout (2-col vs 3-per-row) + the terse label set + a single 'Last 30 days' caption above the group so each pill stays short. Then build fixed-width equal pills on all 3 surfaces (last-if-odd centers via centered flex-wrap).</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>T064</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Weight pill: show change only, not current weight</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>User: the weight pill must always show weight CHANGE, never the current weight. Today it falls back to current weight when there's only one weigh-in. Remove that fallback; show change only and hide the pill when there's nothing to compare.</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>Compute change over the last 30 days (latest − earliest weigh-in in the window) per T065; hide if &lt;2 logs in the window. All 3 surfaces.</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>T065</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Standardize stat windows to rolling 'last 30 days'</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E68" s="10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>User: replace 'this month' (calendar) with 'in last 30 days' (rolling) on the PR pills, and unify the other stats to the same 30-day window for consistency + simpler math. Proposed mapping: Strength/Cardio PRs = best-ever within last 30d; Food = days logged in last 30d (today it's a 14-day STREAK — would become a count); Lowest HR = min bpm last 30d; Weight = change over last 30d (T064); Sleep = avg hrs last 30d; Hydration = days hit goal last 30d. Nuance to confirm: lowest-HR over 30d is more anomaly-prone than 7d (more samples).</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Confirm the per-metric mapping (esp. food streak-&gt;count + HR 30d), then update logic + wording on all 3 surfaces.</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
chore: redeploy delete-user (T066 done); harden capture rule (flagged work = own item); confirm pills layout A
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>Confirm layout (2-col vs 3-per-row) + the terse label set + a single 'Last 30 days' caption above the group so each pill stays short. Then build fixed-width equal pills on all 3 surfaces (last-if-odd centers via centered flex-wrap).</t>
+          <t>CONFIRMED 2026-06-03: layout A — two columns (3 pills left / 3 right / 7th centered under them). Labels accepted: 'N Strength', 'N Cardio', 'N Food', 'N HR low', '+/-N kg', 'Nh Sleep', 'N Water' (with emoji), under one 'Last 30 days' caption so each pill stays short + equal-width. Build on all 3 surfaces (centered flex-wrap so a lone last pill centers).</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
@@ -3671,6 +3671,53 @@
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>T066</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Redeploy delete-user edge function (rom_records removal)</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>Flagged during T049 (rom_records drop): the delete-user edge function's SOURCE had its rom_records table-list entry removed, but the LIVE function still needed a deploy. Tracked as its own row (not buried in the closed T049) after the user's process callout.</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-03: deployed via MCP deploy_edge_function (CLI had no access token). delete-user is now version 12 (was 11), verify_jwt on; live USER_DATA_TABLES no longer includes rom_records. Source was already committed in 6a58fc3 — this was the runtime push.</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>supabase/functions/delete-user/index.ts</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
docs: correct T065 scope (PR pills only -> last 30 days; other windows unchanged)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -3568,7 +3568,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>CONFIRMED 2026-06-03: layout A — two columns (3 pills left / 3 right / 7th centered under them). Labels accepted: 'N Strength', 'N Cardio', 'N Food', 'N HR low', '+/-N kg', 'Nh Sleep', 'N Water' (with emoji), under one 'Last 30 days' caption so each pill stays short + equal-width. Build on all 3 surfaces (centered flex-wrap so a lone last pill centers).</t>
+          <t>CONFIRMED 2026-06-03: layout A — two columns (3 pills left / 3 right / 7th centered under them), all pills EXACTLY equal size (fixed width + min-height; centered flex-wrap so a lone last pill centers). NO shared 'Last 30 days' caption — windows differ per pill (PRs 'last 30 days', Food 'last 14 days', HR '7d', Sleep '7 nights', Hydration '7d'), so each keeps its own window text; the equal SIZE comes from the fixed box (text wraps inside). Build on all 3 surfaces.</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Standardize stat windows to rolling 'last 30 days'</t>
+          <t>PR pills: 'this month' -&gt; rolling 'last 30 days'</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -3657,12 +3657,12 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>User: replace 'this month' (calendar) with 'in last 30 days' (rolling) on the PR pills, and unify the other stats to the same 30-day window for consistency + simpler math. Proposed mapping: Strength/Cardio PRs = best-ever within last 30d; Food = days logged in last 30d (today it's a 14-day STREAK — would become a count); Lowest HR = min bpm last 30d; Weight = change over last 30d (T064); Sleep = avg hrs last 30d; Hydration = days hit goal last 30d. Nuance to confirm: lowest-HR over 30d is more anomaly-prone than 7d (more samples).</t>
+          <t>CORRECTED 2026-06-03 (user): ONLY the PR pills change — 'this month' (calendar) becomes 'last 30 days' (rolling 30-day window); the count logic switches from monthStart to a 30-day cutoff (a PR counts if the best-ever for that exercise/activity was hit within the last 30 days). Every OTHER pill KEEPS its existing window + wording: Food stays 'last 14 days' (still a STREAK, not a count), Lowest HR stays 'last 7 days', Sleep stays '7 nights', Hydration stays '7d', Weight stays 'since last weigh-in'. My earlier 'unify everything to 30d' reading was wrong.</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>Confirm the per-metric mapping (esp. food streak-&gt;count + HR 30d), then update logic + wording on all 3 surfaces.</t>
+          <t>Change Strength + Cardio PR counts from calendar-month to a rolling 30-day cutoff + reword to 'last 30 days', on mobile + admin + coach. Leave every other pill's window untouched.</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(dashboard): pills -> layout A (equal-size 2-col), PRs last 30 days, weight change-only (T063/T064/T065)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -3556,9 +3556,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E66" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>CONFIRMED 2026-06-03: layout A — two columns (3 pills left / 3 right / 7th centered under them), all pills EXACTLY equal size (fixed width + min-height; centered flex-wrap so a lone last pill centers). NO shared 'Last 30 days' caption — windows differ per pill (PRs 'last 30 days', Food 'last 14 days', HR '7d', Sleep '7 nights', Hydration '7d'), so each keeps its own window text; the equal SIZE comes from the fixed box (text wraps inside). Build on all 3 surfaces.</t>
+          <t>DONE 2026-06-03: built + deployed on all 3 surfaces. Mobile: statChip width 48% + minHeight 44 + radius 12, statsRow justify-center, statChipText flex:1. Web (admin + coach): SnapshotBadge -&gt; flex w-[48%] min-h-[2.75rem] rounded-xl text-center (was an inline-flex whitespace-nowrap pill), container flex-wrap + justify-center. 6 chips form 3 rows of 2 + lone 7th centered; each pill keeps its own window wording.</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
@@ -3603,9 +3603,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E67" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Compute change over the last 30 days (latest − earliest weigh-in in the window) per T065; hide if &lt;2 logs in the window. All 3 surfaces.</t>
+          <t>DONE 2026-06-03: weight chip is change-only on all 3 surfaces — removed the '· latest' current-weight fallback (mobile + admin + coach). Shows the signed change since the last weigh-in (latest − previous); the chip hides entirely when there's only one weigh-in to compare.</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
@@ -3650,9 +3650,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E68" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>Change Strength + Cardio PR counts from calendar-month to a rolling 30-day cutoff + reword to 'last 30 days', on mobile + admin + coach. Leave every other pill's window untouched.</t>
+          <t>DONE 2026-06-03: PR pills use a rolling 30-day cutoff + read 'last 30 days' on all 3 surfaces (mobile: isThisMonth -&gt; isWithinLast30Days; web admin + coach: monthStartISO -&gt; thirtyAgoISO). Every other pill's window left untouched (Food 14d, HR 7d, Sleep 7 nights, Hydration 7d, Weight since last weigh-in).</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(dashboard): strip pill labels + drop emojis (T067); weight pill uses 2 most-recent weigh-ins (T068)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3718,6 +3718,100 @@
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>T067</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard pills: strip labels + remove emojis</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Screenshot review after T063 shipped: the pills look awful — labels are too verbose ('strength PRs last 30 days', 'days logged in last 14 days', 'days hit water goal · 7d') and wrap to 2-3 lines inside the 48% chips, stranding the number on its own line. User: strip the text 'just enough to be understandable' AND remove ALL emojis (the 🏆 🍴 ❤️ 😴 💧 ⚖️ prefixes). Mobile + admin + coach.</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-03: removed ALL emoji prefixes + stripped labels to single-line forms on all 3 surfaces — 'N strength PRs · 30d', 'N cardio PR(s) · 30d', 'N food days · 14d', 'N low bpm · 7d', '±N lb change', 'N.Nh sleep · 7d', 'N water days · 7d'. Mobile: chips single-line + centered (minHeight 34, removed flex:1 wrap on the label). Web: SnapshotBadge -&gt; min-h-[2.25rem] + leading-tight, content centered. Built + deployed.</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>T068</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard weight pill missing (change-only edge)</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>After T064 made the weight pill change-only (no current-weight fallback), it vanished from the user's dashboard. Cause: the change needs 2 weigh-ins inside the dashboard's fetch window, and the user has &lt;2 in range (their previous weigh-in is older than the window). User flagged the missing pill.</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-03: change now computes from the 2 most-recent weigh-ins regardless of date — mobile reuses the latest-5 `bw` fetch; web admin + coach dropped the 14-day gte on their bodyweight query. Still change-only (hides only when there's genuinely one weigh-in ever). Built + deployed.</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
feat(dashboard,mobile): pills compute over fixed windows + 'no recent' when empty; weight = 30d change (T069)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3773,45 +3773,92 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
+          <t>T069</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard pills: window-based compute + 'no recent data' (don't hide)</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>User rejected T068's 'latest-N-logs' weight computation — wants every pill computed STRICTLY over its designated rolling window (PRs 30d, food 14d, HR/sleep/hydration 7d, weight = its own designated window). And instead of HIDING a pill when its window has no data, ALWAYS show the pill with a 'no recent data' placeholder (also keeps the fixed 3+3+1 / 7-pill layout stable). Weight window was not specified — assistant designating 30 days (shown as '· 30d'), easily changed.</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>MOBILE DONE + reloaded 2026-06-03: weight = change over rolling 30d (latest − earliest weigh-in in the 30d window; reverted the latest-5-logs hack), shown '±N lb · 30d' or 'no recent weight'; all pills always render — count pills (strength/cardio/food) show 0, measurement pills (HR/weight/sleep/water) show 'no recent &lt;metric&gt;' when empty. WEB (admin + coach) MIRROR PENDING the user's confirmation of the mobile look + the 30d weight window.</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; (then) web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
           <t>T068</t>
         </is>
       </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="B72" s="5" t="inlineStr">
         <is>
           <t>Dashboard weight pill missing (change-only edge)</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>Cross</t>
         </is>
       </c>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F71" s="7" t="inlineStr">
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
         <is>
           <t>After T064 made the weight pill change-only (no current-weight fallback), it vanished from the user's dashboard. Cause: the change needs 2 weigh-ins inside the dashboard's fetch window, and the user has &lt;2 in range (their previous weigh-in is older than the window). User flagged the missing pill.</t>
         </is>
       </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="G72" s="5" t="inlineStr">
         <is>
           <t>DONE 2026-06-03: change now computes from the 2 most-recent weigh-ins regardless of date — mobile reuses the latest-5 `bw` fetch; web admin + coach dropped the 14-day gte on their bodyweight query. Still change-only (hides only when there's genuinely one weigh-in ever). Built + deployed.</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H72" s="5" t="inlineStr">
         <is>
           <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
         </is>
       </c>
-      <c r="I71" s="5" t="inlineStr">
+      <c r="I72" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
feat(dashboard,mobile): page icons on each pill + teal highlight on weight pill (T070)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3773,12 +3773,12 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>T069</t>
+          <t>T070</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Dashboard pills: window-based compute + 'no recent data' (don't hide)</t>
+          <t>Dashboard pills: page icons + highlight weight pill</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -3798,12 +3798,12 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>User rejected T068's 'latest-N-logs' weight computation — wants every pill computed STRICTLY over its designated rolling window (PRs 30d, food 14d, HR/sleep/hydration 7d, weight = its own designated window). And instead of HIDING a pill when its window has no data, ALWAYS show the pill with a 'no recent data' placeholder (also keeps the fixed 3+3+1 / 7-pill layout stable). Weight window was not specified — assistant designating 30 days (shown as '· 30d'), easily changed.</t>
+          <t>User (after seeing the emoji-free pills): use each PAGE's lucide icon on its pill instead of no icon — Strength=Dumbbell, Cardio=Activity, Food=Flame, HR=Heart, Weight=Weight/Scale, Sleep=Moon, Hydration=Droplet (confirm exact icons + accents from the nav/RadialNav). Also the weight pill's slate tint blends into the card background — give it a more visible highlight (a distinct colored border/bg, not clashing with the other 6).</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>MOBILE DONE + reloaded 2026-06-03: weight = change over rolling 30d (latest − earliest weigh-in in the 30d window; reverted the latest-5-logs hack), shown '±N lb · 30d' or 'no recent weight'; all pills always render — count pills (strength/cardio/food) show 0, measurement pills (HR/weight/sleep/water) show 'no recent &lt;metric&gt;' when empty. WEB (admin + coach) MIRROR PENDING the user's confirmation of the mobile look + the 30d weight window.</t>
+          <t>MOBILE DONE + reloaded 2026-06-03: each pill now leads with its page's lucide icon (Dumbbell / Activity / Flame / Heart / Weight / Moon / Droplet) in the page accent; weight chip switched from the near-invisible slate to a teal tint (border 0.34 / bg 0.12) so it stands out. WEB (admin + coach) mirror still PENDING the user's confirmation, to be bundled with the T069 changes.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -3820,45 +3820,92 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
+          <t>T069</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard pills: window-based compute + 'no recent data' (don't hide)</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>User rejected T068's 'latest-N-logs' weight computation — wants every pill computed STRICTLY over its designated rolling window (PRs 30d, food 14d, HR/sleep/hydration 7d, weight = its own designated window). And instead of HIDING a pill when its window has no data, ALWAYS show the pill with a 'no recent data' placeholder (also keeps the fixed 3+3+1 / 7-pill layout stable). Weight window was not specified — assistant designating 30 days (shown as '· 30d'), easily changed.</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>MOBILE DONE + reloaded 2026-06-03: weight = change over rolling 30d (latest − earliest weigh-in in the 30d window; reverted the latest-5-logs hack), shown '±N lb · 30d' or 'no recent weight'; all pills always render — count pills (strength/cardio/food) show 0, measurement pills (HR/weight/sleep/water) show 'no recent &lt;metric&gt;' when empty. WEB (admin + coach) MIRROR PENDING the user's confirmation of the mobile look + the 30d weight window.</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; (then) web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
           <t>T068</t>
         </is>
       </c>
-      <c r="B72" s="5" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>Dashboard weight pill missing (change-only edge)</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>Cross</t>
         </is>
       </c>
-      <c r="E72" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
         <is>
           <t>After T064 made the weight pill change-only (no current-weight fallback), it vanished from the user's dashboard. Cause: the change needs 2 weigh-ins inside the dashboard's fetch window, and the user has &lt;2 in range (their previous weigh-in is older than the window). User flagged the missing pill.</t>
         </is>
       </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="G73" s="7" t="inlineStr">
         <is>
           <t>DONE 2026-06-03: change now computes from the 2 most-recent weigh-ins regardless of date — mobile reuses the latest-5 `bw` fetch; web admin + coach dropped the 14-day gte on their bodyweight query. Still change-only (hides only when there's genuinely one weigh-in ever). Built + deployed.</t>
         </is>
       </c>
-      <c r="H72" s="5" t="inlineStr">
+      <c r="H73" s="7" t="inlineStr">
         <is>
           <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
         </is>
       </c>
-      <c r="I72" s="5" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
fix(dashboard,mobile): weight pill emerald (bodyweight-page green), heart pill fuchsia — distinct (T071)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3906,6 +3906,53 @@
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>T071</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard weight pill color — distinct from heart</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>User: the weight pill (teal, from T070) and the heart pill (emerald) read as almost the same color. REVISED direction: give the weight pill the SAME green the Bodyweight page uses (so the pill matches its page), and recolor the HEART pill to something else (off green) so the two are clearly distinguishable.</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-03: weight pill now uses EMERALD (the Bodyweight page's accent green — reuses statChipEmerald); heart pill moved to FUCHSIA (new statChipFuchsia). Clearly distinguishable now. Mobile only; web admin+coach inherits both colours when the T069/T070 mirror lands.</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
feat(dashboard,mobile): pills sorted by tier + gated per user tier (free=2/corerx=5/fullrx=7) (T072)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3953,6 +3953,53 @@
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>T072</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard pills — sort by tier + gate by user's tier</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>User: re-sort the stat pills by app tier and only show the pills for the user's tier (and below). Free = 2 pills (Strength, Cardio); CoreRX adds Weight + Heart + Food; FullRX adds Sleep + Hydration. Tier-&gt;pill mapping mirrors RadialNav's NAV_BY_HREF: strength/cardio = free; bodyweight(weight)/heart/calories(food) = corerx; sleep/hydration = fullrx. Uneven count -&gt; last pill centers (already handled by statsRow justify-center + 48% fixed width).</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>MOBILE DONE 2026-06-03: replicated RadialNav's resolveTier + TIER_RANK in dashboard.tsx; pills reordered to tier/nav order (Strength, Cardio = free; Weight, Heart, Food = corerx; Sleep, Hydration = fullrx) and each gated on `tierRank &gt;= TIER_RANK[pillTier]`. Free user sees 2 pills, corerx 5, fullrx 7; uneven count centers the lone last pill (statsRow justify-center + 48% width). WEB (admin+coach) mirror still PENDING — bundle with T069/T070/T071.</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; (then) web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>

</xml_diff>

<commit_message>
feat(dashboard,web): mirror pills to admin+coach — tier sort/gate, page icons, emerald/fuchsia, no-recent, 30d weight (T069-T072)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -570,7 +570,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-03 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
+          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-04 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
         </is>
       </c>
     </row>
@@ -3791,9 +3791,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E71" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>MOBILE DONE + reloaded 2026-06-03: each pill now leads with its page's lucide icon (Dumbbell / Activity / Flame / Heart / Weight / Moon / Droplet) in the page accent; weight chip switched from the near-invisible slate to a teal tint (border 0.34 / bg 0.12) so it stands out. WEB (admin + coach) mirror still PENDING the user's confirmation, to be bundled with the T069 changes.</t>
+          <t>MOBILE DONE + reloaded 2026-06-03: each pill now leads with its page's lucide icon (Dumbbell / Activity / Flame / Heart / Weight / Moon / Droplet) in the page accent; weight chip switched from the near-invisible slate to a teal tint (border 0.34 / bg 0.12) so it stands out. WEB (admin + coach) MIRRORED 2026-06-04 — page icons added, built + deployed.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -3838,9 +3838,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E72" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>MOBILE DONE + reloaded 2026-06-03: weight = change over rolling 30d (latest − earliest weigh-in in the 30d window; reverted the latest-5-logs hack), shown '±N lb · 30d' or 'no recent weight'; all pills always render — count pills (strength/cardio/food) show 0, measurement pills (HR/weight/sleep/water) show 'no recent &lt;metric&gt;' when empty. WEB (admin + coach) MIRROR PENDING the user's confirmation of the mobile look + the 30d weight window.</t>
+          <t>MOBILE DONE + reloaded 2026-06-03: weight = change over rolling 30d (latest − earliest weigh-in in the 30d window; reverted the latest-5-logs hack), shown '±N lb · 30d' or 'no recent weight'; all pills always render — count pills (strength/cardio/food) show 0, measurement pills (HR/weight/sleep/water) show 'no recent &lt;metric&gt;' when empty. WEB (admin + coach) MIRRORED 2026-06-04 — built + deployed.</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>DONE 2026-06-03: weight pill now uses EMERALD (the Bodyweight page's accent green — reuses statChipEmerald); heart pill moved to FUCHSIA (new statChipFuchsia). Clearly distinguishable now. Mobile only; web admin+coach inherits both colours when the T069/T070 mirror lands.</t>
+          <t>DONE 2026-06-03: weight pill now uses EMERALD (the Bodyweight page's accent green — reuses statChipEmerald); heart pill moved to FUCHSIA (new statChipFuchsia). Clearly distinguishable now. WEB (admin + coach) mirrored 2026-06-04 (weight = emerald, heart = fuchsia).</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -3979,9 +3979,9 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E75" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>MOBILE DONE 2026-06-03: replicated RadialNav's resolveTier + TIER_RANK in dashboard.tsx; pills reordered to tier/nav order (Strength, Cardio = free; Weight, Heart, Food = corerx; Sleep, Hydration = fullrx) and each gated on `tierRank &gt;= TIER_RANK[pillTier]`. Free user sees 2 pills, corerx 5, fullrx 7; uneven count centers the lone last pill (statsRow justify-center + 48% width). WEB (admin+coach) mirror still PENDING — bundle with T069/T070/T071.</t>
+          <t>MOBILE DONE 2026-06-03: replicated RadialNav's resolveTier + TIER_RANK in dashboard.tsx; pills reordered to tier/nav order (Strength, Cardio = free; Weight, Heart, Food = corerx; Sleep, Hydration = fullrx) and each gated on `tierRank &gt;= TIER_RANK[pillTier]`. Free user sees 2 pills, corerx 5, fullrx 7; uneven count centers the lone last pill (statsRow justify-center + 48% width). WEB (admin + coach) MIRRORED 2026-06-04 — replicated resolveTier on both files (client tier comes from the admin get_user_for_admin RPC + the coach profiles select('*'), both already return b2c_subscription_tier); reorder + tier-gate + icons + colors + no-recent states + 30d weight; built + deployed. So a coach-attached client (fullrx) shows all 7; a free B2C client shows 2.</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(dashboard,web): empty pills keep accent color + muted text (T073); log T074 water-logs = test taps
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4002,6 +4002,100 @@
       <c r="I75" s="5" t="inlineStr">
         <is>
           <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>T073</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Web empty-state pills lost their accent color (all grey)</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Screenshot (admin client view): the empty 'no recent weight / HR / sleep / water' pills all render grey (zinc) instead of keeping their accent tint, so weight (emerald) and heart (fuchsia) are indistinguishable when empty AND it doesn't match mobile — where an empty pill keeps its accent chip border/bg with muted icon + muted text. The T069-T072 web-mirror agent used color='zinc' for all empty states.</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-04 (background agent + assistant deploy): added a `muted` prop to SnapshotBadge — keeps the accent border/bg from `color` but forces text to `!text-muted-foreground`; the 4 empty pills now pass their accent color + muted (weight=green, heart=fuchsia, sleep=indigo, hydration=cyan) with muted icon+text, matching mobile. Both web files; built + deployed.</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>T074</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Phantom water_logs appearing for users who never logged water</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>User: water_logs rows exist for accounts that never logged water. rasp_86 (Test Client, id 3d41a692-7c59-4636-bfee-96b76d1bcf3e) shows 2 days logged with NO visible log entries; motaz.jarrah shows 1 day, no log history. The mobile hydration pill reads '0 days' (NOT 'no recent') — so the count path SEES water_logs rows but counts 0 days hitting goal, i.e. rows exist but don't surface in the page's log list and the user doesn't know what's inserting them.</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-04 — NOT a phantom inserter, it's real test taps. The rows' amounts are EXACTLY 236.588 / 354.882 / 473.176 ml = 8 / 12 / 16 oz (the hydration page's oz quick-add/picker presets run through ozToMl()); logged_at = created_at, clustered in bursts seconds apart on 2026-05-29 + 05-30 (rasp_86, ~18 rows) and 06-03 22:53 (motaz, 1 row) — i.e. manual button-mashing during the hydration-page dev/test sessions. The ONLY water_logs INSERT in the whole codebase is hydration.tsx addDrink (tap-triggered; grep confirmed nothing auto-inserts — sync/HC/Samsung/migrations don't write water_logs, they only DELETE in delete-user). 'No log showing' = the page's log list shows TODAY only (these are past days); 'pill says 0' = computeHydrationDaysHit counts days HITTING the daily goal in 7d (=0, each day was under goal) but rows exist so it reads 0 not 'no recent'. Offered to delete the junk test rows; awaiting user.</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>mobile hydration.tsx; src/lib/healthConnect.ts, integrations/*; supabase functions/migrations</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(dashboard): 0-count pills read 'no recent <metric>' not '0' — consistent across all 7 (T075)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4094,6 +4094,53 @@
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>T075</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Stat pills: a 0 count should read 'no recent', not '0'</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>User (admin screenshot): count pills show '0 cardio PRs · 30d' and '0 food days · 14d' while measurement pills show 'no recent weight/HR/sleep/water' — inconsistent. The count-vs-measurement split I built shows the number even at 0 for PRs/food. Make the count pills read the muted 'no recent ...' empty state (accent-tinted, like the measurement empties) when the count is 0, and show the number only when &gt; 0. (0 PRs = no PR set in the window — the client may still have trained — so 'no recent strength/cardio PRs' is accurate.)</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-04: count pills now show muted 'no recent strength PRs / no recent cardio PRs / no recent food' (accent-tinted, like the measurement empties) when the count is 0, and the number+label only when &gt; 0. Mobile + admin + coach; built + deployed. All 7 pills now read consistently — a value when there's something recent, 'no recent &lt;metric&gt;' otherwise.</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx; web AdminUserDetail.jsx, CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
fix: coach first-name-only on mobile dash + simplify sign-in heading
- Dashboard "Coached by" badge now strips to the first word at render
  time, so it shows first name only even when a stale cached coachInfo
  holds the full name (T076).
- Mobile sign-in collapses the redundant "Sign in" eyebrow + "Sign in
  to MyRX" title into a single "Sign in" heading (T077). Web Auth.jsx
  differs ("Welcome back"), so no mirror needed.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4141,6 +4141,100 @@
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>T076</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Mobile 'Coached by' shows full name, should be first only</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>On the client's mobile dashboard the 'Coached by …' badge showed the coach's FULL name (e.g. 'Coached by Taz Jarrah'); should show first name only ('Coached by Taz'). The coachInfo handler already stripped to split(' ')[0], but a stale cached coachInfo (hydrated from dataCache before the stripping shipped) rendered the full name.</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>Fixed: the badge now strips to the first word at RENDER time — (coachInfo.full_name ?? '').trim().split(' ')[0] — so it shows first name only regardless of what's cached. (Athlete dashboard is mobile-only, no web mirror.)</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>T077</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Mobile sign-in heading 'Sign in to MyRX' -&gt; 'Sign in'</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Mobile sign-in page had an eyebrow 'Sign in' + a title 'Sign in to MyRX' (redundant); user wants just 'Sign in'.</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>Fixed: removed the redundant eyebrow and set the title to 'Sign in' (single clean heading). Web Auth.jsx differs — heading is 'Welcome back' + subtitle 'Sign in to continue to MyRX', not the same string — so left as-is (mobile-only fix).</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(auth)/sign-in.tsx; web Auth.jsx</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
docs: reconcile task ledger + domain status per user dispositions
- Close T041/T042 (Bodyweight/Calories coaching promotions — stay
  tracking/logging surfaces by design).
- Mark Done: T016, T043, T044, T045 (Hydration redesign + Sleep,
  Hydration, Sleep/Water tracking already built with coaching).
- Defer T046 (iOS launch — triggered only when Android-complete).
- T048 -> In progress (investigating the ~19 filter/dedup rules wired
  into the SYNC scripts).
- T015 -> In progress (admin/coach parity, resuming next).
- Reframe T047: "Health Connect Phase 2" -> "Finalize Connect page and
  logic", kept open.
- Sync CLAUDE.md domain-status + roadmap to match (Cardio/Sleep/
  Hydration done; Bodyweight/Calories coaching closed; Mobility removed).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -57,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -86,22 +86,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -164,9 +159,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1302,17 +1294,17 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>User noted the admin and coach portals don't present the client 'preview' identically. Both render the same MacroPlanEditor (identical), so the difference is in the surrounding wrappers (admin has Food Log/Manual Logs/Macro Plan sub-tabs; coach shows just the editor behind a 'Manage macros' gate) + different tab sets/profile cards. User dismissed the clarifying question and parked it.</t>
+          <t>User noted the admin and coach portals don't present the client 'preview' identically. Both render the same MacroPlanEditor (identical), so the difference is in the surrounding wrappers (admin has Food Log/Manual Logs/Macro Plan sub-tabs; coach shows just the editor behind a 'Manage macros' gate) + different tab sets/profile cards.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Re-open when the user decides which surface to match and how (whole client page vs just the macro/preview area).</t>
+          <t>Resuming 2026-06-04: user wants to work on this right after the task-pipeline update. Next: scope which surface is the reference and align the other.</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -1322,7 +1314,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -1347,19 +1339,19 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>User wants to rework the Hydration page (beyond the mascot, T001). They said they'll give the specific direction next. This is the NEXT active task after the task-ledger work.</t>
+          <t>Confirmed done by user 2026-06-04: the Hydration page redesign landed via the T052-T062 batch (fluid counting, fast picker, non-intimidating progress, attribution, pond removal, bug fixes).</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Get the specific direction from the user, then implement on mobile hydration.tsx.</t>
+          <t>Shipped via T052-T062.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -1369,7 +1361,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2522,29 +2514,29 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Roadmap: promote Bodyweight from a tracking surface to a coaching surface (a 'what's my next step' experience like Strength).</t>
+          <t>Closed by user 2026-06-04 (same call as T042): the Bodyweight page stays a tracking surface — weight + chart + goal, no separate coaching layer.</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Not started. Mission/roadmap item.</t>
+          <t>Won't do — bodyweight remains a tracking surface by design.</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>(planned) mobile bodyweight.tsx</t>
+          <t>mobile bodyweight.tsx</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2569,29 +2561,29 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Roadmap: Calories is being promoted to a coaching surface. The self-coached plan wizard (PlanWizardSheet) + the timeline work (T009) are part of this. Per CLAUDE.md the wizard is in active iteration (mobile-only until locked).</t>
+          <t>Closed by user 2026-06-04: the Calories page intentionally stays a food-logging surface — no coaching layer. The plan wizard + timeline (T009) cover the planning side; there is no separate 'next step' coaching ambition for calories.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Continue iterating the plan wizard / next-step coaching; lock when the user signs off.</t>
+          <t>Won't do — calories remains a logging surface by design.</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>mobile PlanWizardSheet.tsx, calories.tsx</t>
+          <t>mobile calories.tsx</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>ongoing</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2616,29 +2608,29 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Roadmap: promote Sleep to a coaching surface. Data exists (sleep_sessions, sleep_stages).</t>
+          <t>Confirmed done by user 2026-06-04: the Sleep page is already built and already does coaching (next-step guidance), not just tracking.</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Not started.</t>
+          <t>Shipped. Sleep is a coaching surface.</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>(planned) mobile sleep.tsx</t>
+          <t>mobile sleep.tsx</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2663,29 +2655,29 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E47" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Roadmap: promote Hydration to a coaching surface. Data exists (water_logs) + daily target computed. Related to the mascot (T001) and the upcoming page redesign (T016).</t>
+          <t>Confirmed done by user 2026-06-04: the Hydration coaching surface is already finalized (target + guidance), on top of the recent redesign (T052-T062).</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Not started as a 'coaching' promotion; the page redesign (T016) may feed into this.</t>
+          <t>Shipped. Hydration is a coaching surface.</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>(planned) mobile hydration.tsx</t>
+          <t>mobile hydration.tsx</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2710,29 +2702,29 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E48" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Roadmap (segment table-stakes for the coach arm): build Sleep / Water / Habits tracking surfaces, likely via Apple Health / Google Fit integrations rather than first-party logging.</t>
+          <t>Confirmed done by user 2026-06-04: Sleep and Water (Hydration) tracking surfaces are built. (Sleep/Hydration also do coaching — see T043/T044.)</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Not started. Decide first-party vs integration per surface.</t>
+          <t>Shipped.</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>(planned)</t>
+          <t>mobile sleep.tsx, hydration.tsx</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2759,17 +2751,17 @@
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Pre-iOS-launch work documented in CLAUDE.md: HealthKit entitlements + Info.plist usage strings, IAP/receipt validation, Sign in with Apple (if social login), SMS autofill, edge-swipe parity, EAS iOS build profile, etc.</t>
+          <t>Pre-iOS-launch work: HealthKit entitlements + Info.plist usage strings, IAP/receipt validation, Sign in with Apple, SMS autofill, edge-swipe parity, EAS iOS build profile, etc.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Not started. Gated on iOS build + App Store account setup.</t>
+          <t>Deferred by user 2026-06-04: only triggered once the app is Android-complete. Revisit after Android ships.</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -2779,7 +2771,7 @@
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2783,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Health Connect Phase 2</t>
+          <t>Finalize Connect page and logic</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -2804,29 +2796,29 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Background sync (WorkManager/BackgroundTasks), write-back to HC, app-launch auto-sync. HR-series storage schema is an open question (hr_samples vs extended column).</t>
+          <t>Reframed by user 2026-06-04 (was 'Health Connect Phase 2'): finalize the Connect page (Settings -&gt; Connect) and its sync logic. Covers wiring the integration rows to real connect/sync/disconnect behaviour + the last-sync display. (Background sync / HC write-back from the old Phase-2 scope can fold in here as sub-items.)</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Deferred until at least one direct integration (T040) is live.</t>
+          <t>Open — finalize the Connect page UI + connect/sync logic.</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>(planned)</t>
+          <t>mobile profile.tsx (ConnectTab), src/lib/healthConnect.ts, src/lib/lastSyncStorage.ts</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2851,29 +2843,29 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E51" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Known gap: the incremental sync scripts (sync_usda / sync_on) predate filters.mjs and use a legacy shouldSkip; bulk import already applies the full filter + dedup pipeline. Sync needs enrichFood + shouldKeepFood + dedup wired in.</t>
+          <t>User 2026-06-04: this is supposed to be done — investigate and make sure all ~19 filter+dedup rules (Tier 1-4 rules 1-14 in filters.mjs + Tier 5 dedup rules 15-19) are wired into BOTH sync paths (orchestrator scripts/sync/run.mjs and legacy scripts/d1_migrate/sync_usda.mjs / sync_on.mjs). Bulk import already applies the full pipeline; verify sync matches.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Not started.</t>
+          <t>Investigating: audit run.mjs + sync_usda.mjs + sync_on.mjs vs filters.mjs + dedup; wire in any missing rules.</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>scripts/d1_migrate/sync_usda.mjs, sync_on.mjs</t>
+          <t>scripts/sync/run.mjs, scripts/d1_migrate/sync_usda.mjs, sync_on.mjs, scripts/d1_migrate/lib/filters.mjs</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>prior</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -4262,155 +4254,155 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>MyRX — Task Pipeline · how to use</t>
         </is>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1">
-      <c r="A2" s="14" t="inlineStr"/>
+      <c r="A2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>WHY THIS EXISTS</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>We fork across many sessions and lose track of what's open / where we stopped. This is the single remembered list. Every task has a stable numeric ID (T001, T002, ...). Refer to one with "pick up T021" and this sheet says exactly where we left off and what's next.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1">
-      <c r="A5" s="14" t="inlineStr"/>
+      <c r="A5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>CAPTURE-FIRST RULE (locked 2026-06-03)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Every time a point comes up that needs fixing or discussion — ANY size — it gets logged here as a Pending task with a new T### id BEFORE the assistant replies, then it's answered. It stays Pending until the work is actually done/decided, then flips to Done (or Deferred/Parked/Reverted). Small items are exactly what gets lost, so nothing is too small to capture.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="14" t="inlineStr"/>
+      <c r="A8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>STATUS VALUES</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Done — shipped (and usually deployed/committed).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>In progress — actively being iterated.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Pending — agreed/known but not started.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Deferred — intentionally postponed (waiting on something or a user decision).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Parked — discussed then set aside; needs a user decision to re-open.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Reverted — was tried, then undone.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Closed — dropped / won't do for now (can be reopened).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="14" t="inlineStr"/>
+      <c r="A17" s="13" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>HOW TO UPDATE (the .xlsx is GENERATED, do not hand-edit)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>1. Edit the TASKS list in scripts/build_task_pipeline_xlsx.py (add a row / flip a status / update the 'where we left off' + 'next' text).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>New tasks get the next free T### id. Never reuse or renumber an id.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="8" customHeight="1">
-      <c r="A23" s="14" t="inlineStr"/>
+      <c r="A23" s="13" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>SCOPE NOTE</t>
         </is>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Seeded 2026-06-03 from the current CLAUDE.md + recent sessions. Older sessions weren't fully transcribed, so the 'prior' rows are best-effort reconstructions of completed features. Treat this as the authoritative living record from here forward — keep it current.</t>
         </is>

</xml_diff>

<commit_message>
docs: T048 done — sync already applies the full 19-rule pipeline
Audit confirmed the production sync orchestrator (scripts/sync/run.mjs)
reuses the bulk-import loaders (enrichFood + shouldKeepFood, rules 1-14)
and applyDedup (rules 15-19), so every sync filters/dedups identically
to a full rebuild. Legacy sync_usda/sync_on are dead and themselves
already migrated to the filter lib.

- T048 -> Done in the ledger.
- Fixed two stale CLAUDE.md bullets that claimed sync skips filters
  ("known-pending revamp" / "remaining gap").
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -2843,24 +2843,24 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>User 2026-06-04: this is supposed to be done — investigate and make sure all ~19 filter+dedup rules (Tier 1-4 rules 1-14 in filters.mjs + Tier 5 dedup rules 15-19) are wired into BOTH sync paths (orchestrator scripts/sync/run.mjs and legacy scripts/d1_migrate/sync_usda.mjs / sync_on.mjs). Bulk import already applies the full pipeline; verify sync matches.</t>
+          <t>Audited 2026-06-04: ALREADY DONE. The production sync orchestrator (scripts/sync/run.mjs) reuses the bulk-import loaders (loadUsda/loadOn -&gt; enrichFood + shouldKeepFood = Rules 1-14) and applyDedup (dedup_in_memory.mjs = Rules 15-19), so all 19 rules run on every sync and produce a byte-identical filtered/deduped result to a full rebuild. The 'Sync now' button dispatches sync-food-library.yml -&gt; node scripts/sync/run.mjs (plus monthly cron 0 3 1 * *).</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Investigating: audit run.mjs + sync_usda.mjs + sync_on.mjs vs filters.mjs + dedup; wire in any missing rules.</t>
+          <t>No code change needed. Legacy scripts/d1_migrate/sync_usda.mjs + sync_on.mjs are dead/superseded (no workflow/package.json refs) and have themselves been migrated to enrichFood + getFilterReason anyway. Also fixed the two stale CLAUDE.md bullets that wrongly claimed sync skips the filter pipeline.</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>scripts/sync/run.mjs, scripts/d1_migrate/sync_usda.mjs, sync_on.mjs, scripts/d1_migrate/lib/filters.mjs</t>
+          <t>scripts/sync/run.mjs, scripts/bulk_import/lib/{usda_loader,on_loader,dedup_in_memory}.mjs, scripts/d1_migrate/lib/filters.mjs</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: park T015 with scoping question queued for resume
User paused the admin/coach parity work; will resume later with
questions asked one at a time. Captured the audited diff + the ready
Q1 (which surface is the reference) in the ledger so the next session
picks up cleanly.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -86,7 +86,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -1294,22 +1294,22 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Parked</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>User noted the admin and coach portals don't present the client 'preview' identically. Both render the same MacroPlanEditor (identical), so the difference is in the surrounding wrappers (admin has Food Log/Manual Logs/Macro Plan sub-tabs; coach shows just the editor behind a 'Manage macros' gate) + different tab sets/profile cards.</t>
+          <t>Audited 2026-06-04: the two client pages are already mostly identical (same Dashboard/Efforts/Bodyweight/Calories tabs + same Age/Gender/Phone/Weight/Height profile card). Real diffs: (a) Admin has 2 extra tabs (Billing, Activity Feed) — admin-only by nature; (b) the Calories tab differs — Admin renders the rich AdminUserCalories.jsx (Food Log / Manual Logs / Macro Plan sub-tabs), Coach renders just the inline Macro Plan editor gated behind 'Manage macros'.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Resuming 2026-06-04: user wants to work on this right after the task-pipeline update. Next: scope which surface is the reference and align the other.</t>
+          <t>PAUSED by user 2026-06-04 — resume later, asking scoping questions ONE AT A TIME. Q1 (ready): which is the reference? [A] Coach matches Admin (richer Calories tab; recommended, lowest risk) / [B] Admin matches Coach (simpler) / [C] unify to one shared role-gated component. Confirm assumption: Billing + Activity Feed stay admin-only.</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>web admin/tabs/AdminUserCalories.jsx; coach/CoachClientDetail.jsx</t>
+          <t>web admin/tabs/AdminUserCalories.jsx; web admin/AdminUserDetail.jsx; coach/CoachClientDetail.jsx</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: re-scope parity into T078 (finalize admin view) + T015 (mirror)
User re-scoped: finalize the admin client-detail view first, then
mirror to coach once we fully understand it.
- New T078: Finalize the Admin client-detail view (in progress).
- T015 reframed to phase-2 "mirror finalized admin -> coach", blocked
  on T078.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -57,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +99,11 @@
         <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -126,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -159,6 +164,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -538,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1279,7 +1287,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Admin vs Coach client-view design parity</t>
+          <t>Mirror finalized admin client-view to coach</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1299,17 +1307,17 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Audited 2026-06-04: the two client pages are already mostly identical (same Dashboard/Efforts/Bodyweight/Calories tabs + same Age/Gender/Phone/Weight/Height profile card). Real diffs: (a) Admin has 2 extra tabs (Billing, Activity Feed) — admin-only by nature; (b) the Calories tab differs — Admin renders the rich AdminUserCalories.jsx (Food Log / Manual Logs / Macro Plan sub-tabs), Coach renders just the inline Macro Plan editor gated behind 'Manage macros'.</t>
+          <t>Phase 2 of the admin/coach parity work. User re-scoped 2026-06-04: finalize the ADMIN client-detail view first (T078), THEN mirror the finalized result to the coach client view. Audited diffs so far: Admin has 2 extra tabs (Billing, Activity Feed, admin-only by nature) + a richer Calories tab (Food Log / Manual Logs / Macro Plan) vs the coach's inline Macro Plan editor behind 'Manage macros'. Exact mirror scope is TBD until T078 lands.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>PAUSED by user 2026-06-04 — resume later, asking scoping questions ONE AT A TIME. Q1 (ready): which is the reference? [A] Coach matches Admin (richer Calories tab; recommended, lowest risk) / [B] Admin matches Coach (simpler) / [C] unify to one shared role-gated component. Confirm assumption: Billing + Activity Feed stay admin-only.</t>
+          <t>BLOCKED on T078 (finalize admin client view). Resume after admin is final: decide per-area what mirrors to coach and what stays admin-only.</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>web admin/tabs/AdminUserCalories.jsx; web admin/AdminUserDetail.jsx; coach/CoachClientDetail.jsx</t>
+          <t>web admin/AdminUserDetail.jsx + tabs/*; coach/CoachClientDetail.jsx</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -4227,6 +4235,53 @@
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>T078</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Finalize the Admin client-detail view</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-04 re-scoped the parity task: before mirroring admin-&gt;coach (T015), finalize the ADMIN client-detail view first so we have a full understanding of what exists + what needs mirroring. Admin client page = web/src/pages/admin/AdminUserDetail.jsx (shell) with 6 tabs: Dashboard, Efforts (AdminUserActivity), Bodyweight (AdminUserBody), Calories (AdminUserCalories - Food Log/Manual Logs/Macro Plan sub-tabs), Billing, Activity Feed (timeline).</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>In progress: inventory each admin client-view tab, then finalize tab-by-tab via one-question-at-a-time Q&amp;A. Mirror to coach (T015) comes after.</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/admin/tabs/*.jsx</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
@@ -4254,155 +4309,155 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>MyRX — Task Pipeline · how to use</t>
         </is>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1">
-      <c r="A2" s="13" t="inlineStr"/>
+      <c r="A2" s="14" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>WHY THIS EXISTS</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>We fork across many sessions and lose track of what's open / where we stopped. This is the single remembered list. Every task has a stable numeric ID (T001, T002, ...). Refer to one with "pick up T021" and this sheet says exactly where we left off and what's next.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1">
-      <c r="A5" s="13" t="inlineStr"/>
+      <c r="A5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>CAPTURE-FIRST RULE (locked 2026-06-03)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Every time a point comes up that needs fixing or discussion — ANY size — it gets logged here as a Pending task with a new T### id BEFORE the assistant replies, then it's answered. It stays Pending until the work is actually done/decided, then flips to Done (or Deferred/Parked/Reverted). Small items are exactly what gets lost, so nothing is too small to capture.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="13" t="inlineStr"/>
+      <c r="A8" s="14" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>STATUS VALUES</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Done — shipped (and usually deployed/committed).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>In progress — actively being iterated.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Pending — agreed/known but not started.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Deferred — intentionally postponed (waiting on something or a user decision).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Parked — discussed then set aside; needs a user decision to re-open.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Reverted — was tried, then undone.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Closed — dropped / won't do for now (can be reopened).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="13" t="inlineStr"/>
+      <c r="A17" s="14" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>HOW TO UPDATE (the .xlsx is GENERATED, do not hand-edit)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>1. Edit the TASKS list in scripts/build_task_pipeline_xlsx.py (add a row / flip a status / update the 'where we left off' + 'next' text).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>New tasks get the next free T### id. Never reuse or renumber an id.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="8" customHeight="1">
-      <c r="A23" s="13" t="inlineStr"/>
+      <c r="A23" s="14" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>SCOPE NOTE</t>
         </is>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Seeded 2026-06-03 from the current CLAUDE.md + recent sessions. Older sessions weren't fully transcribed, so the 'prior' rows are best-effort reconstructions of completed features. Treat this as the authoritative living record from here forward — keep it current.</t>
         </is>

</xml_diff>

<commit_message>
docs: capture admin client-view inventory findings under T078
7 finalize items recorded (Dashboard placeholder + Food Log add =
decisions; weigh-in crash, dead AdminUserProfile.jsx, billing deep-link,
cardio best-stat parser, cosmetic save-button styles = clear fixes).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4273,12 +4273,12 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>In progress: inventory each admin client-view tab, then finalize tab-by-tab via one-question-at-a-time Q&amp;A. Mirror to coach (T015) comes after.</t>
+          <t>Inventory done 2026-06-04. Finalize items: (1) Dashboard tab is an empty 'Snapshot coming soon' placeholder AND it's the DEFAULT landing tab [DECISION]. (2) BUG: AdminUserBody.jsx save-weigh-in button crashes — Loader2 used (l.197) but not imported (l.3) [FIX]. (3) Dead code: tabs/AdminUserProfile.jsx (530 lines) imported (AdminUserDetail l.10) but never rendered; settings drawer uses AccountSettings [FIX]. (4) ?tab=billing deep-link broken — 'billing' missing from validTabs (l.492) [FIX]. (5) Efforts 'Best' cardio stat only parses /km pace; speed/cal-min/floors/mi/500m/100m show nothing — extend to shell's parseCardioBest [FIX]. (6) Calories Food Log: admin can view+delete client food but not add on their behalf [DECISION]. (7) Cosmetic: stale ClientSettingsDrawer docstring + inconsistent save-button feedback styles [FIX]. Clear fixes (2,3,4,5,7) can batch; decisions (1,6) need user. One at a time.</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/admin/tabs/*.jsx</t>
+          <t>web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/admin/tabs/*.jsx; components/{BillingView,MacroPlanEditor,AccountSettings,ClientSettingsDrawer}.jsx</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(admin): Efforts tab -> read-only Strength/Cardio mirror (T080)
Per-page pass, Efforts (list view):
- Keep one combined Efforts tab; replace the All/Strength/Cardio filter
  pills with a clean Strength | Cardio segmented toggle (default
  Strength, "All" dropped) so a coach switches between the two the way
  the athlete has two separate pages.
- Make it read-only: removed the Add-effort form, the backdate picker,
  the "Add effort" button, and the insert path (coach input is a
  separate track). Movement list + drill-into-detail unchanged.

Next for Efforts: coaching add-ons on the list + a detail-screen
rebuild to match the athlete coaching surfaces.

Deployed to myrxfit.com.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4329,6 +4329,53 @@
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>T080</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Efforts page — align coach view to athlete + coaching add-ons</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Per-page pass (Phase 2 of T079), starting with Efforts at user request 2026-06-04. Goal: make the admin Efforts tab's FIRST view show what the athlete sees on their Strength + Cardio pages (read-only, no inputs — coach input is a separate track), then propose coaching add-ons. Open structural question: athlete has SEPARATE Strength + Cardio pages; admin combines them into one 'Efforts' tab (AdminUserActivity.jsx: filter pills + per-movement cards -&gt; detail route). Decide split-vs-combined + remove the Add-effort input.</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>STRUCTURE DECIDED 2026-06-04: keep ONE combined Efforts tab with an internal Strength|Cardio segmented toggle (dropped 'All', default Strength). LIST-VIEW read-only mirror DONE + deployed 2026-06-04 — removed the Add-effort form + backdate + button; AdminUserActivity is now read-only (207-&gt;193 lines). NEXT: (a) coaching add-ons for the list (candidates: last-trained recency, stalled-lift flag, training frequency/volume trend, PR timeline, strength/cardio balance, adherence/consistency) — suggest, user picks; (b) DETAIL-SCREEN rebuild — admin detail routes (AdminEffortDetail = bare 10-tile grid; AdminCardioDetail = old pace model w/ banned 'lower=faster') don't mirror the athlete coaching surfaces; also remove swipe-delete there for read-only.</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/tabs/AdminUserActivity.jsx; web AdminEffortDetail/AdminCardioDetail; mirror mobile/app/(app)/{strength,cardio}.tsx + effort detail pages</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
docs: T081 — roll out Efforts detail mirrors to all variants
Wave 1 (strength variants) spawning via parallel agents; then cardio,
then list variant-collapsing. Read-only + per-effort delete, mirroring
the athlete coaching surfaces, same pattern as AdminStrengthWeightedDetail.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4376,6 +4376,53 @@
         </is>
       </c>
       <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>T081</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Roll out Efforts detail mirrors — all strength + cardio variants + list collapsing</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E84" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>User approved the Weighted Standard pattern (T080) 2026-06-04 and said 'proceed with all' (multiple agents OK if no issues). Roll the AdminStrengthWeightedDetail read-only+delete pattern out to every remaining Efforts detail variant. Strength dispatch (in StrengthDetail, by movement looked up by BASE name after stripping ' [Band + Knee]'/' [Band]'/' [Knee]'): isSledWorkConsolidated (exercise==='Sled Work'), isIsometric (strength_type==='isometric'), isAssistedMachine (equipment==='assisted'), isCarry (equipment==='carry'), band/knee suffix &amp;&amp; base equipment!=='bodyweight' -&gt; RepsOnly, isBodyweightExercise (equipment==='bodyweight') -&gt; bodyweight consolidated, else weighted (done). Cardio route is SEPARATE: /admin/user/:id/effort/cardio/:slug -&gt; AdminCardioDetail (variants: pace/Group-A incl Concept2 ergs, air bike, swimming consolidated, rucking, stairmill, duration, beat-your-best).</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>WAVES (verify each): W1 strength variants (AdminStrength{Bodyweight,Assisted,Carry,Isometric,RepsOnly}Detail) -&gt; wire AdminEffortDetail base-name dispatch -&gt; build/deploy/QA; W2 cardio variants -&gt; wire AdminCardioDetail; W3 list variant-collapsing in AdminUserActivity (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge). W1 spawned 2026-06-04 via 5 parallel agents.</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/detail/AdminStrength*.jsx + AdminCardio*.jsx; AdminEffortDetail.jsx; AdminCardioDetail.jsx; AdminUserActivity.jsx; mirror mobile [exercise].tsx + [activity].tsx</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
feat(admin): collapse variant families in Efforts list (T081 Wave 3)
The read-only Efforts list now mirrors the athlete index: bodyweight
assist tiers collapse to one base row + tier badge (FULL RX/BAND/KNEE/
B+K via useMovements), the 4 swim strokes collapse to one Swimming row +
stroke badge, and Sled Work [Push]/[Drag] collapse to one Sled Work row
+ PUSH/DRAG badge. Collapsed rows navigate to the consolidated detail
mirror. Best-stat aggregates across the family.

Completes T081 — the entire Efforts page (list + every strength & cardio
detail variant) now mirrors the athlete read-only with delete kept.
Deployed to myrxfit.com (index-EfS3aeG1).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4402,9 +4402,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E84" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>WAVES (verify each): W1 strength variants (AdminStrength{Bodyweight,Assisted,Carry,Isometric,RepsOnly}Detail) -&gt; wire AdminEffortDetail base-name dispatch -&gt; build/deploy/QA; W2 cardio variants -&gt; wire AdminCardioDetail; W3 list variant-collapsing in AdminUserActivity (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge). W1 DONE + deployed 2026-06-04: 5 strength variants (bodyweight/assisted/carry+sled/isometric/repsonly) built via parallel agents + wired into AdminEffortDetail base-name dispatch (Sled Work handled by exercise name; isometric via strength_type; band/knee suffix + non-bodyweight -&gt; repsonly); build clean. W2 (cardio) DONE + deployed 2026-06-04: 6 variants (pace incl Concept2 Row/Ski erg; air bike; swimming consolidated; rucking; stairmill; beat-your-best) built via parallel agents; AdminCardioDetail rewritten as a slim dispatcher mirroring the athlete categorizeActivity (Bike Erg -&gt; stationary_bike -&gt; BeatYourBest; Row/Ski Erg -&gt; Pace); build clean. W3 (list variant-collapsing in AdminUserActivity) NEXT.</t>
+          <t>WAVES (verify each): W1 strength variants (AdminStrength{Bodyweight,Assisted,Carry,Isometric,RepsOnly}Detail) -&gt; wire AdminEffortDetail base-name dispatch -&gt; build/deploy/QA; W2 cardio variants -&gt; wire AdminCardioDetail; W3 list variant-collapsing in AdminUserActivity (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge). W1 DONE + deployed 2026-06-04: 5 strength variants (bodyweight/assisted/carry+sled/isometric/repsonly) built via parallel agents + wired into AdminEffortDetail base-name dispatch (Sled Work handled by exercise name; isometric via strength_type; band/knee suffix + non-bodyweight -&gt; repsonly); build clean. W2 (cardio) DONE + deployed 2026-06-04: 6 variants (pace incl Concept2 Row/Ski erg; air bike; swimming consolidated; rucking; stairmill; beat-your-best) built via parallel agents; AdminCardioDetail rewritten as a slim dispatcher mirroring the athlete categorizeActivity (Bike Erg -&gt; stationary_bike -&gt; BeatYourBest; Row/Ski Erg -&gt; Pace); build clean. W3 DONE + deployed 2026-06-04: AdminUserActivity collapses bodyweight tiers (base + tier badge FULL RX/BAND/KNEE/B+K via useMovements) / swim strokes (Swimming + FREE/BACK/BREAST/FLY badge) / sled push-drag (Sled Work + PUSH/DRAG badge) into one row each, navigating to the consolidated detail. ALL WAVES COMPLETE — the entire Efforts page (read-only list + every strength &amp; cardio detail variant) now mirrors the athlete with per-effort delete kept. Next for Efforts: the deferred coaching add-ons (recency, stalled flag, frequency, PR timeline, balance, adherence).</t>
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: T082 (cross-check mirrors vs actual mobile render) + T083 (dashboard pill refresh)
Root cause of StairMill mismatch: mirrors were built from stale CLAUDE.md
specs; the mobile code is the source of truth. Verify+fix sweep across all
detail surfaces. Plus T083: mobile dashboard pills stale after on-dashboard
effort delete.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4423,6 +4423,100 @@
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>T082</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Cross-check ALL Efforts detail mirrors vs ACTUAL mobile render + fix</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>ROOT CAUSE (user 2026-06-04): the detail mirrors were built partly from the CLAUDE.md 'locked design spec' sections, which LAG the actual mobile code. StairMill was built to the stale zone-pill spec instead of the current mobile tile/plan-queue render, so it doesn't look like mobile. The mobile COMPONENT CODE is the sole source of truth for the visual — CLAUDE.md is context/intent only, not the render spec. Likely affects other variants too.</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>Verify+fix agent per surface (6 strength + 6 cardio): read the ACTUAL mobile render for the variant, diff vs the web mirror, fix the web to match the mobile render (Recharts/click-pills substitutions OK; read-only + delete kept). StairMill = full rebuild to the current mobile model. Then build/deploy + user QAs every move. Wave A = strength, Wave B = cardio.</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/detail/AdminStrength*.jsx + AdminCardio*.jsx; mirror mobile [exercise].tsx + [activity].tsx</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>T083</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Mobile dashboard pills don't refresh on effort delete</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E86" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-04: on the mobile dashboard, deleting an effort does NOT update the stat pills in real time — the user must navigate away and back (which remounts + refetches) to see the corrected pill values. The pills derive from efforts data that isn't refetched/recomputed after an on-dashboard delete.</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>Agent: read mobile/app/(app)/dashboard.tsx, find the pill computation + the on-dashboard effort delete, and refresh the pill data immediately after a successful delete (update in-memory state or refetch via the existing pattern). tsc-clean.</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/dashboard.tsx</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
fix(mobile): refresh dashboard pills after on-dashboard effort delete (T083)
handleDelete optimistically removed the item from the recent-activity
list but never re-ran fetchDashboard, which computes the pill aggregates
(PRs / streak / HR / weight / hydration / sleep / food) from separate
queries. So the pills stayed stale until the tab re-gained focus. Now
call fetchDashboard() right after the delete (no setLoading(true), so no
skeleton flash).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4496,9 +4496,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E86" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Agent: read mobile/app/(app)/dashboard.tsx, find the pill computation + the on-dashboard effort delete, and refresh the pill data immediately after a successful delete (update in-memory state or refetch via the existing pattern). tsc-clean.</t>
+          <t>FIXED 2026-06-04 (done directly — agent quota was rate-limited): handleDelete optimistically updated the recent-activity list but never re-ran fetchDashboard, which computes the pill aggregates (PRs/streak/HR/weight/hydration/sleep/food) from their own queries. Added fetchDashboard() right after the delete; it never sets loading=true so there's no skeleton flash. tsc clean.</t>
         </is>
       </c>
       <c r="H86" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(admin): cross-check all cardio detail mirrors vs actual mobile render (T082 complete)
Mobile code = source of truth (not the stale CLAUDE.md specs):
- Pace: FIX section-order inversion — mobile is tiles->hero, not
  hero->queue; remove invented "COMING UP" heading + tile rest line +
  fade-edges; fix help text.
- StairMill: same inversion fix (it had mirrored the pre-fix Pace).
- Air Bike: confirmed pill model is correct; copy/caption fixes.
- Swimming: near-clean; coach-voice help text.
- Rucking: chart heading weight; remove invented caption.
- Beat-Your-Best: add "All entries" log header; caption + hint copy.

Completes T082 — all 12 Efforts detail surfaces (6 strength + 6 cardio)
now verified against the live mobile render. Deployed (index-CwEUcOHi).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4449,9 +4449,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E85" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Verify+fix agent per surface (6 strength + 6 cardio): read the ACTUAL mobile render for the variant, diff vs the web mirror, fix the web to match the mobile render (Recharts/click-pills substitutions OK; read-only + delete kept). StairMill = full rebuild to the current mobile model. Then build/deploy + user QAs every move. PROGRESS 2026-06-04: agent BURST limit when spawning 7 at once (single agents work) — running the sweep in small batches of ~3. StairMill REBUILT to the plan-queue tile model (matching actual mobile: 8-step queue tile row + selected-step hero, not the stale zone-pill) + deployed. Remaining 11 surfaces (6 strength + 5 cardio) being cross-checked in batches.</t>
+          <t>Verify+fix agent per surface (6 strength + 6 cardio): read the ACTUAL mobile render for the variant, diff vs the web mirror, fix the web to match the mobile render (Recharts/click-pills substitutions OK; read-only + delete kept). StairMill = full rebuild to the current mobile model. Then build/deploy + user QAs every move. PROGRESS 2026-06-04: agent BURST limit when spawning 7 at once (single agents work) — running the sweep in small batches of ~3. StairMill REBUILT to the plan-queue tile model (matching actual mobile: 8-step queue tile row + selected-step hero, not the stale zone-pill) + deployed. ALL 12 surfaces cross-checked + fixed 2026-06-04 (batches of 3, mobile code = truth). Real stale-spec divergences corrected: weighted (restored hero title spec said removed), bodyweight (removed phantom band-progression strip), assisted (removed invented fade-edge gradients), isometric (removed phantom in-card phase-pill + info-panel; restored hero title + min-height), repsonly (removed invented STRENGTH pill + chart placeholder; added log header), pace + stairmill (FIXED hero/tiles ORDER inversion — mobile is tiles-&gt;hero, not hero-&gt;queue; removed invented 'COMING UP' heading + tile rest line + fade-edges), rucking + beatyourbest (chart headings, removed/added captions + log header). AirBike + Swimming were near-clean (copy only). All eslint+esbuild clean, deployed.</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(cardio): interval terminology, not reps, in coaching copy (T084)
Cardio prescriptions are intervals, not reps. Fixed the user-facing copy
on StairMill, Air Bike, and Swimming (mobile + the web admin mirrors):
- hero row descriptors "per rep" / "est. per rep" -> "per interval"
- cues "Each rep should take" -> "Each interval", "between reps" ->
  "between intervals"
- zone whyText "Sustained hard reps" -> "intervals", "Longer reps than
  sprint" -> "Longer intervals"

Pace/Duration already used interval wording. Internal field names
(reps/repKm/repSecs) + code comments left untouched. Mobile tsc clean;
web deployed (mobile applies via Fast Refresh).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4517,6 +4517,53 @@
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>T084</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Cardio copy: 'per rep' -&gt; 'per interval' (StairMill + sweep)</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Cardio</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Mobile+Web</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-04: StairMill (and other cardio) display copy says 'per rep' / 'between reps' / 'Each rep' — cardio prescriptions are INTERVALS, not reps. Fix the user-facing copy to interval terminology where it makes sense (hero row descriptors + cue lines + zone whyText). Internal code identifiers (reps, repKm, repSecs fields) stay. Pace already uses 'per interval' for its descriptors.</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>Mobile [activity].tsx: StairMill hero rows (4455/4461) + cues (4155/4158) + VO2 whyText (4090), Air Bike hero (3609) + cues (3327/3330) + threshold whyText (3259), Swimming cue (693) -&gt; interval wording. Mirror to web AdminCardio{StairMill,AirBike,Swimming}Detail.jsx. tsc + build/deploy + reload. DONE 2026-06-04: hero descriptors 'per rep'-&gt;'per interval' + 'est. per rep'-&gt;'est. per interval'; cues 'Each rep'-&gt;'Each interval', 'between reps'-&gt;'between intervals'; whyText 'Sustained hard reps'-&gt;'intervals' + 'Longer reps than sprint'-&gt;'Longer intervals'. Pace/Duration already used interval wording. Internal field names (reps/repKm/repSecs) + code comments left as-is. tsc clean; web deployed; mobile Fast-Refresh.</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/effort/cardio/[activity].tsx; web AdminCardio*Detail.jsx</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
fix(hydration): credit the Beverage Hydration Index in the attribution (T085)
The BHI weighting was already wired correctly into the cups (effective mL
= sum(amount_ml × multiplier), milk 1.5x; cups = round(effectiveMl/250)),
but the attribution line only credited the daily-target formula (35 mL/kg
bodyweight) and never the drink-hydration science that powers the cups.
Added "Maughan 2016 · … hydration-weighted" to the attribution on mobile
hydration.tsx + the web AdminUserHydration coach mirror. tsc clean,
web deployed.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4564,6 +4564,53 @@
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>T085</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Hydration: verify BHI weighting wired into cups + attribution states the science</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Hydration</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-04: (1) we researched the Beverage-Hydration-Index weighting for how much hydration each drink gives (milk ~1.5x, water/coffee/tea/diet-soda ~1.0x). Is it ACTUALLY wired into the CUPS number displayed, or are cups computed from raw mL? (2) The attribution/science line on the hydration page doesn't state the science the way other pages do (strength 'Epley · Brzycki · Lombardi'; cardio 'Riegel · Daniels'...'). Verify both + fix.</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>Read mobile/app/(app)/hydration.tsx: confirm cups = round(effectiveBhiMl/250) of round(targetMl/250) using the BHI multiplier (not raw mL); check the attribution line content + styling. Fix the cups wiring if wrong + add/correct the BHI attribution line to match other pages. VERIFIED+FIXED 2026-06-04: (1) BHI IS wired correctly — DRINKS registry sets multipliers (milk 1.5, rest 1.0, Maughan 2016), todayEffectiveMl = sum(amount_ml × multiplierFor(drink_type)), cupsDone = round(todayEffectiveMl/250); milk even shows a ×1.5 badge. No cups fix needed. (2) Attribution credited ONLY the target formula (35 mL/kg, National Academies/Mayo/EFSA), not the BHI — added 'Maughan 2016 · ... hydration-weighted' to mobile hydration.tsx + mirrored to web AdminUserHydration.jsx. tsc clean, deployed.</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/hydration.tsx</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
refactor(admin): strip athlete-only copy from coach mirrors — hydration + batch 1 (T086)
Coach view = client data + prescription, not athlete education. Removed
always-visible athlete-facing prose (kept all data, the prescription/cue
lines, and the opt-in "why this zone" info pills):
- Hydration: motivational helper line, eligibility note, attribution footer.
- Sleep: attribution citations, per-dimension "why this matters" science,
  feature help-text; neutralized "wear your watch" instructions + empty states.
- Heart: chart help-text, resting-HR coaching-tip advice.
- Weighted strength: "Epley · Brzycki · Lombardi" attribution + the
  "Pick an adaptation zone, then tap a rep target" help-text.

This intentionally diverges the coach mirrors from mobile (which keeps the
copy for the athlete). Deployed.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4611,6 +4611,53 @@
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>T086</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Strip athlete-only explanatory copy from web coach mirrors</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E89" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-04 (viewing web AdminUserHydration): athlete-facing explanatory text has no value to a coach + clutters the coach view. Flagged examples: motivational 'Steady sips beat chugging it all at once.', eligibility note 'Only no- and low-calorie... milk included.', and the attribution 'National Academies · ... Maughan 2016 ...'. Sweep ALL web coach-mirror pages, judge coach-meaningful vs athlete-only, REMOVE the unnecessary explanations. Coach view = client DATA + actionable prescription; strip athlete motivation, how/what-to-log instructions, eligibility notes, feature help-text, science attributions. These STAY on the MOBILE athlete pages — only the WEB coach mirrors get stripped (so this intentionally DIVERGES the mirrors from mobile; the T082 cross-check no longer applies to these prose blocks).</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>REMOVE (always-visible athlete prose): attribution footers, motivational/encouragement lines, eligibility/instruction notes, feature help-text subtitles. KEEP: data (charts/logs/best/PR/current), prescription numbers + the cue line, headers/badges/tiles, and the opt-in 'why this zone' info pills (collapsed, not clutter — flag if user wants those gone too). Surfaces: tabs AdminUser{Sleep,Hydration,Heart}; detail AdminStrength* + AdminCardio*. Hydration done as exemplar, then agent-sweep the rest in batches of 3; build/deploy.</t>
+        </is>
+      </c>
+      <c r="H89" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/tabs/AdminUser{Sleep,Hydration,Heart}.jsx; web/src/pages/admin/detail/AdminStrength*.jsx + AdminCardio*.jsx</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
refactor(admin): strip athlete-only copy from all detail coach mirrors (T086 complete)
Workflow sweep of the remaining 11 detail surfaces (5 strength + 6 cardio),
same criteria as the hydration/Sleep/Heart/Weighted exemplars. Removed
always-visible athlete-facing prose — attribution/citation footers, feature
help-text subtitles ("Pick an adaptation zone…", "Pick a training focus…"),
tier-criteria methodology subtitles, motivational/eligibility lines — and
neutralized athlete-instruction empty states ("Log your first…" → "No X
logged yet").

KEPT: all client data (charts, tiles, logs, PRs, hero numbers), the
prescription cue lines, section titles, badges, and the opt-in "why this
zone" info pills (per user). Coach mirrors now intentionally diverge from
mobile on these prose blocks (mobile keeps them for the athlete). All
eslint+esbuild clean; deployed to myrxfit.com.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4637,9 +4637,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E89" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>REMOVE (always-visible athlete prose): attribution footers, motivational/encouragement lines, eligibility/instruction notes, feature help-text subtitles. KEEP: data (charts/logs/best/PR/current), prescription numbers + the cue line, headers/badges/tiles, and the opt-in 'why this zone' info pills (collapsed, not clutter — flag if user wants those gone too). Surfaces: tabs AdminUser{Sleep,Hydration,Heart}; detail AdminStrength* + AdminCardio*. Hydration done as exemplar, then agent-sweep the rest in batches of 3; build/deploy.</t>
+          <t>REMOVE (always-visible athlete prose): attribution footers, motivational/encouragement lines, eligibility/instruction notes, feature help-text subtitles. KEEP: data (charts/logs/best/PR/current), prescription numbers + the cue line, headers/badges/tiles, and the opt-in 'why this zone' info pills (collapsed, not clutter — flag if user wants those gone too). Surfaces: tabs AdminUser{Sleep,Hydration,Heart}; detail AdminStrength* + AdminCardio*. Hydration done as exemplar, then agent-sweep the rest in batches of 3; build/deploy. DONE 2026-06-04: Hydration (me) + Batch 1 (Sleep/Heart/Weighted-strength) + a background Workflow over the remaining 11 detail surfaces (5 strength + 6 cardio) in chunks of 3. Removed: attribution/citation footers, feature help-text subtitles ('Pick an adaptation zone...', 'Pick a training focus...'), tier-criteria methodology subtitles, motivational/eligibility prose; neutralized athlete-instruction empty states ('Log your first...' -&gt; 'No X logged yet') + removed PartyPopper/emoji decoration. KEPT: all data (charts/tiles/logs/PRs/hero numbers), the prescription cue lines, section titles, badges, and the opt-in 'why this zone' info pills. User confirmed keeping the info pills. All eslint+esbuild clean (agents self-verified); web build clean; deployed. Coach mirrors now intentionally diverge from mobile on these prose blocks (mobile athlete pages keep them).</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: capture T087 — strength cue needs build-up/progression science
User flagged that "Do 4-5 sets of 5 reps at 140" (the next 5RM target) is
self-contradictory — you cannot do multiple sets at your 5RM, and you
build to a new PR over sessions. Brainstorm stage; design pending.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4658,6 +4658,53 @@
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>T087</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Strength cue: build-up/progression science to reach a new rep-max PR</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Strength</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Mobile+Web</t>
+        </is>
+      </c>
+      <c r="E90" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-04 (thinking out loud, viewing Bench Press 5RM): the weighted-standard coaching cue 'Do 4-5 sets of 5 reps at 140 lb' is off. 140 is the NEXT 5RM target (current 5RM=135). Two problems: (1) a 5RM means 5 reps is your 1-set MAX, so you physically can't do 4-5 SETS of 5 at your 5RM — multi-set work must be submaximal (reps in reserve); (2) you don't hit a new PR cold — you build up over sessions. User senses there should be progression science (progressive overload / RIR / double-progression) + a separate PR-attempt, not one impossible cue. Asked 'am I right?' -&gt; YES.</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>BRAINSTORM stage — do NOT implement until the model is agreed. Design a progression-aware strength cue that separates (a) the WORKING prescription (submaximal, RIR-based, day-to-day), (b) the PROGRESSION rule (when to bump load — e.g. double progression: add reps to top of range across all sets, then +smallest jump), (c) the PR ATTEMPT (one top set at the target, periodically). Affects the locked Weighted Standard next-target card + ADP_ZONE defaults (sets/RIR/rest). Plain-English, one decision at a time.</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/effort/strength/[exercise].tsx (Weighted Standard cue + ADP_ZONE_CONFIG); web AdminStrengthWeightedDetail.jsx; CLAUDE.md Weighted Standard spec</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>

</xml_diff>

<commit_message>
docs: T088 — full science audit of all 11 progression models (strength + cardio)
11 evidence audits (WebSearch/WebFetch). Tier-A correctness/safety issues:
Olympic lifts on rep-max math, rucking no-BW-cap, plyometrics-as-max-reps,
StairMill FPM anchor + units error. Tier-B anchor fixes across bodyweight,
isometric, pace, swim, air-bike. Tier-C copy. Consolidated citeable sources
per domain recorded. Awaiting user triage on implementation.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -570,7 +570,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-04 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
+          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-05 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
         </is>
       </c>
     </row>
@@ -4707,6 +4707,53 @@
       <c r="I90" s="5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>T088</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Science-audit EVERY progression model (strength + cardio) for next-target correctness</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Strength+Cardio</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (+Web mirror)</t>
+        </is>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-04/05 (after T087): asked to cross-check every movement category, not just barbell lifts — read all moves per category for strength AND all cardio, and research the science so each category's NEXT PROGRESSION is actually correct. Pulled the live movements table: 11 distinct progression models (6 strength, 5 cardio). Ran 11 parallel evidence audits via WebSearch/WebFetch.</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>VERDICTS by severity. TIER A (correctness/safety): (A1) Olympic &amp; ballistic lifts (snatch, C&amp;J, power clean, KB swing/snatch) must NOT use rep-max math — a 20RM snatch is meaningless + suggests a dangerous practice; route to low-rep %1RM/velocity model. (A2) Rucking has NO bodyweight cap + mislabeled tiers (Tough=35lb is actually GoRuck HEAVY dry; true Tough=20/30lb by BW); 80lb ladder top = 53% BW for a 150lb user, past the ~1/3 BW safe limit — make tiers BW-relative + add ~1/3 BW hard cap. (A3) Plyometrics/jumps/jump-rope treated as max-reps — wrong; progress on OUTPUT (jump height/distance, box height) + contact budget + rest. (A4) StairMill: FPM is a machine SETTING not earned capacity (+ floor=16 vs 22 steps across models, peak-of-any-effort inflates); anchor on sustained held SPM / vertical m-per-min over a continuous block. TIER B (anchors mis-set): (B5) Bodyweight graduation 10 reps -&gt; ~5-8 (10 reps = endurance, ~70-75% 1RM). (B6) Isometric: tag axis time|load|leverage — time holds keep 2-min cap, loadable holds add load after ~30-60s, skill-leverage holds (planche/levers/flag/L-sit) drop the 120s grid -&gt; variant ladder. (B7) Pace cardio: anchor on Critical Speed (2-3 efforts) not single best pace; zones as %threshold per modality (power for ergs/bike, HR/RPE elliptical) not fixed running s/km offsets. (B8) Swim: replace Riegel single-point CSS with 2-point linear slope per stroke (1.06 is a running exponent, worse for fly/breast); kill 'fastest projection' (biased high); deepen VO2 to CSS-8..-10. (B9) Air bike: watts=cal/min*17.4 is arithmetically ok at 25% GE but 25% is optimistic AND doesn't match the console (~24.75 W/cal-min on Assault) so 'hold &gt;=X W' is unreadable — drop overlay or calibrate to console + name brand. (B10) Weighted 15/20RM tiles are guesses (cap grid ~10-12RM); + the T087 cue fix (submaximal + RIR + double progression). TIER C (copy/labels): hypertrophy '6-12' too strict (growth 5-30+ near failure); carry 'load+distance same session' (zones already do one-axis); assisted 'BW-assist-&gt;1RM' is a relative index not a true 1RM (counterweight is constant through ROM, pull-up hardest at bottom) — relabel + add reps/negatives; soften 'polarized 80/20 is best' (pyramidal = for recreational); CLAUDE.md air-bike '17.4 standard Assault/Echo conversion' claim is FALSE; StairMill cites Honda 2014 (a GLUCOSE study, drop it), Allison was 20s not 60s, Boreham was accumulated bouts not 20-min continuous; StairMill gender baseline 12 FPM ~= 192 SPM EXCEEDS the machine max (units error, real ~4-5 FPM). SOUND AS-IS: loaded carry (one copy tweak), the swim/pace 3-zone + easy-floor STRUCTURE. CONSOLIDATED CITEABLE SOURCES: strength = Epley/Brzycki/Lombardi + Reynolds-Robergs 2006 + Schoenfeld rep-continuum 2021 + NSCA Haff&amp;Triplett + Prilepin + Helms/Zourdos RIR + ACSM; bodyweight = Ebben 2012 + Nuzzo 2023 (ECC:CON 1.41) + Steven Low; plyo/skill = NSCA plyo + Markovic&amp;Mikulic 2010 + Ramirez-Campillo + McGill + GMB; iso = Oranchuk 2019 + Schott 1995 + Kitai&amp;Sale 1989 + McGill; carry = McGill strongman EMG + Winwood/Keogh/Cronin + NSCA + Dan John; pace = Daniels VDOT + Seiler 80/20 + Critical Power (Jones/Vanhatalo) + Coggan FTP + ACSM; swim = Wakayoshi 1992 + Maglischo + Costill + Gonjo 2024; air bike = Peronnet&amp;Massicotte 1991 + Concept2 formula + Gibala SIT + Seiler; ruck = Knapik + US Army ATP 3-21.18 + GoRuck + EIB/Ranger 12mi; stairmill = Allison 2017 + Boreham 2000 + ACSM + Ainsworth Compendium + Seiler. STATUS: research complete, awaiting user TRIAGE on what to implement — most surfaces are locked, but math/bug fixes (StairMill baseline, air-bike watts, ruck BW cap, Olympic-lift rep-max) are allowed on locked surfaces per the finalized-surfaces rule; design changes need explicit unlock.</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/effort/strength/[exercise].tsx; mobile/app/(app)/effort/cardio/[activity].tsx; mobile/src/lib/formulas.ts + movements.ts; web admin detail mirrors; CLAUDE.md locked specs; how-we-compute copy</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark T089 (swipe-acceptance rule) done - user-confirmed on device
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4778,9 +4778,9 @@
           <t>Mobile (+Web later)</t>
         </is>
       </c>
-      <c r="E92" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E92" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>Mobile shipped + tsc clean. Web coach mirrors NOT yet aligned (lighter swipe impl) -- separate pass if wanted. Verify on device: swipe BW chart -&gt; tier changes + hero follows; swipe Weighted hero -&gt; zone changes; BW log + Weighted/Carry/AirBike/Ruck charts+logs do NOT swipe.</t>
+          <t>DONE + user-confirmed on device 2026-06-05: swipeable elements run the slide animation (BW chart slides + flips tiers with the hero pager following; Weighted hero slides the pill identically to a pill swipe). ONLY remaining sub-item = web coach-mirror swipe parity (lighter impl) -- deferred unless requested.</t>
         </is>
       </c>
       <c r="H92" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(strength-log): exclude Olympic/ballistic from the "Estimated 1RM" chip (T090)
Verify-first (Explore-agent map of strength.tsx): the live summary chip is ALREADY
move-type-aware -- the liveOneRM guard nulls it for isometric, carry, band/knee, and
rep-only bodyweight, each of which shows its own type-appropriate chip. The only gap
was the Olympic/ballistic lifts tagged this session: with no isOlympic/isBallistic
flag in the log form they fell through to the weighted branch and showed a
meaningless "Estimated 1RM" (audit A1: a 20RM snatch implies bad practice).

Added isOlympic/isBallistic (movementRecord.lift_type), excluded both from the
liveOneRM guard, and show a neutral "Working set -- W unit x reps" chip instead.
Logged as T090 (Done) in the pipeline. Web end-user log form is frozen.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I92"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4799,6 +4799,53 @@
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>T090</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Strength log: move-type-aware live summary chip ('Estimated 1RM' banner)</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Strength</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-05 (mid Model-4): the live 'Estimated 1RM' chip under the strength log form 'doesn't make sense for most moves now'; asked to fix it to show something relevant + register a task so we don't forget. VERIFY-FIRST (read strength.tsx via an Explore agent before changing anything): the chip is ALREADY move-type-aware -- the liveOneRM guard (strength.tsx ~L424) nulls it for isometric, carry, band/knee-assisted, and rep-only bodyweight, and each of those types renders its OWN chip instead (load-hold: 'W unit x duration'; carry: 'W . dist of work'; band/knee: 'band . reps'; assisted: 'BW - assist = effective' breakdown; plain iso: hold time). So the user's 'shows 1RM for most moves' was the pre-Olympic mental model -- 4th audit/assumption this session that our code already handled (band/knee, BW-in-1RM, now this).</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>THE ONE REAL GAP + FIX: Olympic + ballistic lifts (lift_type tagged THIS session in Model 1) had no isOlympic/isBallistic flag in the LOG form, so they fell through to the generic weighted branch and showed 'Estimated 1RM' -- exactly the meaningless/dangerous readout audit A1 flagged (a 20RM snatch). Mobile strength.tsx: added isOlympic/isBallistic flags (read movementRecord.lift_type), excluded both from the liveOneRM guard, added a neutral 'Working set -- W unit x reps' chip for them instead (echoes the load being logged, matching the other non-1RM chips' input-echo pattern, no 1RM claim). Web end-user log form FROZEN (2026-05-12) -&gt; no web mirror. OPTIONAL DEFERRED: the assisted-machine log chip shows a bare effective-1RM value at its right edge with no label (agent suggested 'Effective 1RM') -- minor clarity nit, not a misnomer, left as-is.</t>
+        </is>
+      </c>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/strength.tsx (isOlympic/isBallistic flags, liveOneRM guard, Working-set chip)</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>

</xml_diff>

<commit_message>
docs(T088): mark complete — all 11 progression models audited + corrected
All 5 cardio models done in one run (Rucking soft cap, StairMill citations, Air Bike
watts drop, Swim 2-point CSS, Pace Critical Speed). T088 status -> Done. Verify-first
scorecard + deferred (Phase 2) items recorded.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4731,9 +4731,9 @@
           <t>Mobile (+Web mirror)</t>
         </is>
       </c>
-      <c r="E91" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>VERDICTS by severity. TIER A (correctness/safety): (A1) Olympic &amp; ballistic lifts (snatch, C&amp;J, power clean, KB swing/snatch) must NOT use rep-max math — a 20RM snatch is meaningless + suggests a dangerous practice; route to low-rep %1RM/velocity model. (A2) Rucking has NO bodyweight cap + mislabeled tiers (Tough=35lb is actually GoRuck HEAVY dry; true Tough=20/30lb by BW); 80lb ladder top = 53% BW for a 150lb user, past the ~1/3 BW safe limit — make tiers BW-relative + add ~1/3 BW hard cap. (A3) Plyometrics/jumps/jump-rope treated as max-reps — wrong; progress on OUTPUT (jump height/distance, box height) + contact budget + rest. (A4) StairMill: FPM is a machine SETTING not earned capacity (+ floor=16 vs 22 steps across models, peak-of-any-effort inflates); anchor on sustained held SPM / vertical m-per-min over a continuous block. TIER B (anchors mis-set): (B5) Bodyweight graduation 10 reps -&gt; ~5-8 (10 reps = endurance, ~70-75% 1RM). (B6) Isometric: tag axis time|load|leverage — time holds keep 2-min cap, loadable holds add load after ~30-60s, skill-leverage holds (planche/levers/flag/L-sit) drop the 120s grid -&gt; variant ladder. (B7) Pace cardio: anchor on Critical Speed (2-3 efforts) not single best pace; zones as %threshold per modality (power for ergs/bike, HR/RPE elliptical) not fixed running s/km offsets. (B8) Swim: replace Riegel single-point CSS with 2-point linear slope per stroke (1.06 is a running exponent, worse for fly/breast); kill 'fastest projection' (biased high); deepen VO2 to CSS-8..-10. (B9) Air bike: watts=cal/min*17.4 is arithmetically ok at 25% GE but 25% is optimistic AND doesn't match the console (~24.75 W/cal-min on Assault) so 'hold &gt;=X W' is unreadable — drop overlay or calibrate to console + name brand. (B10) Weighted 15/20RM tiles are guesses (cap grid ~10-12RM); + the T087 cue fix (submaximal + RIR + double progression). TIER C (copy/labels): hypertrophy '6-12' too strict (growth 5-30+ near failure); carry 'load+distance same session' (zones already do one-axis); assisted 'BW-assist-&gt;1RM' is a relative index not a true 1RM (counterweight is constant through ROM, pull-up hardest at bottom) — relabel + add reps/negatives; soften 'polarized 80/20 is best' (pyramidal = for recreational); CLAUDE.md air-bike '17.4 standard Assault/Echo conversion' claim is FALSE; StairMill cites Honda 2014 (a GLUCOSE study, drop it), Allison was 20s not 60s, Boreham was accumulated bouts not 20-min continuous; StairMill gender baseline 12 FPM ~= 192 SPM EXCEEDS the machine max (units error, real ~4-5 FPM). SOUND AS-IS: loaded carry (one copy tweak), the swim/pace 3-zone + easy-floor STRUCTURE. CONSOLIDATED CITEABLE SOURCES: strength = Epley/Brzycki/Lombardi + Reynolds-Robergs 2006 + Schoenfeld rep-continuum 2021 + NSCA Haff&amp;Triplett + Prilepin + Helms/Zourdos RIR + ACSM; bodyweight = Ebben 2012 + Nuzzo 2023 (ECC:CON 1.41) + Steven Low; plyo/skill = NSCA plyo + Markovic&amp;Mikulic 2010 + Ramirez-Campillo + McGill + GMB; iso = Oranchuk 2019 + Schott 1995 + Kitai&amp;Sale 1989 + McGill; carry = McGill strongman EMG + Winwood/Keogh/Cronin + NSCA + Dan John; pace = Daniels VDOT + Seiler 80/20 + Critical Power (Jones/Vanhatalo) + Coggan FTP + ACSM; swim = Wakayoshi 1992 + Maglischo + Costill + Gonjo 2024; air bike = Peronnet&amp;Massicotte 1991 + Concept2 formula + Gibala SIT + Seiler; ruck = Knapik + US Army ATP 3-21.18 + GoRuck + EIB/Ranger 12mi; stairmill = Allison 2017 + Boreham 2000 + ACSM + Ainsworth Compendium + Seiler. STATUS: research complete, awaiting user TRIAGE on what to implement — most surfaces are locked, but math/bug fixes (StairMill baseline, air-bike watts, ruck BW cap, Olympic-lift rep-max) are allowed on locked surfaces per the finalized-surfaces rule; design changes need explicit unlock. PROGRESS (full model-by-model sweep, user chose 'full sweep' 2026-06-05): Model 1 Fix 1.1 (submaximal working-weight cue 'a weight you could do K+reserve, do K' + corrected per-zone RIR 2/2/1 + iterative 'add X each time, work up to PR') SHIPPED mobile+web. Fix 1.2 (Olympic barbell lifts routed OFF the rep-max grid to a NEW Layout 9 %-of-best card: added movements.lift_type column [olympic|ballistic], tagged 22 barbell snatch/clean/jerk-family lifts; mobile OlympicLiftDetail + web AdminStrengthOlympicDetail mirror + dispatch-before-weighted + Layout Design.xlsx row 9 + CLAUDE.md Layout-9 spec) SHIPPED. Fix 1.3 (capped the rendered rep-max grid at 15RM, dropped 16-20 as noise, flagged 13-15RM with a leading '≈' + caveat note; kept the 3-zone model since Endurance needs 13+) SHIPPED mobile+web. Fix 1.4 (hypertrophy whyText softened — growth spans ~5-30+ reps near failure, 6-12 is just the efficient middle, not an exclusive window) SHIPPED mobile+web. Fix 1.2b (ballistic kettlebell -&gt; NEW Layout 10 bell-ladder card: tagged 13 KB ballistic moves lift_type='ballistic'; mobile BallisticLiftDetail + web AdminStrengthBallisticDetail mirror + dispatch-before-weighted + Layout xlsx row 10 + CLAUDE.md spec) SHIPPED. MODEL 1 COMPLETE (weighted cue + Olympic Layout 9 + ballistic Layout 10 + grid cap + hypertrophy copy). Model 2 (bodyweight rep-strength + assist tiers) IN PROGRESS: Fix 2.1 (graduation trigger BW_GRADUATION_REPS 10-&gt;8 so tiers/bands graduate in the strength range not endurance; mobile+web+CLAUDE.md) SHIPPED. Fix 2.2 (band/knee): on inspection there is NO false 'band is harder' copy — only the carousel order asserts it, which is load-bearing (graduation path + badge + landing) and the science says the order is AMBIGUOUS not wrong; user chose #1 = LEAVE the order (deliberate no-op). Fix 2.3a (bodyweight in the weighted 1RM): VERIFIED ALREADY HANDLED — the log form stores estimate1RM(profileBodyWeight + addedWeight, reps) [strength.tsx ~L414/424] and the detail projection derives added = projection - bodyweight [L4733]; the audit's 'ignores bodyweight' claim is FALSE for our code. (Only nuance: uses FULL bodyweight = 100% share, so push-ups over-count vs pull-ups — an optional minor per-move-share tweak, not a bug.) NET: Model 2 CORRECTNESS DONE — the graduation 10-&gt;8 (2.1) was the one real fix. The rest of the audit's Model-2 items are FEATURE additions, not correctness bugs: an eccentric/negatives tier + leverage/tempo/unilateral alternatives (both optional, additive builds touching the locked card + log form). META-LESSON: this is the 3rd audit claim our code already handles correctly (band/knee, BW-in-1RM) — the audit agents researched GENERIC science and assumed naive implementations; our code is more sophisticated. So VERIFY every audit claim against the actual code before 'fixing' it. Model 3 (isometric) IN PROGRESS: VERIFIED real (unlike Model 2) — all 38 iso moves were on one 10-120s time grid incl. skill holds where 120s is meaningless. LEVERAGE family SHIPPED: added movements.hold_type column (time/load/leverage), tagged 18 leverage holds; NEW Layout 11 -&gt; mobile LeverageHoldDetail + web AdminStrengthLeverageDetail mirror; short milestones 5/10/15/20/30s + skill-ladder (planche tuck-&gt;straddle-&gt;full, levers tuck-&gt;full, handstand wall-&gt;free; gate = 30s clean -&gt; next variant; L-Sit/V-Sit standalone per user); dispatch before isometric; Layout xlsx row 11 + CLAUDE.md Layout-11 spec + iso spec updated to exclude leverage. Model 3 (isometric) COMPLETE: leverage family (Layout 11) + LOAD family (Layout 12) both SHIPPED. Load: tagged 7 loadable holds (wall sit, calf-raise, glute-bridge x2, dead hang, split-squat, squat hold) hold_type='load'; mobile LoadHoldDetail + web AdminStrengthLoadDetail mirror; two phases (time milestones 15-60s -&gt; add-load; gate 60s, loaded target 30s; load inc 5lb/2.5kg); LOG FORM gained an Added-weight wheel for load-holds (label 'Name · W unit x D sec', value stays 'D sec' so parseDurationSecs unchanged); chart adaptive (load over time once weighted, else hold time); dispatch before isometric; Layout xlsx row 12 + CLAUDE.md Layout-12 spec + iso spec updated. The ~13 TIME holds (plank/side-plank/hollow/etc.) stay on IsometricDetail (correct). Model 4 (assisted machine) DONE (verify-first CONFIRMED the audit this time): (4.1) graduation over-promise fixed -- 'attempt unassisted, you're ready' -&gt; honest 'machine eased the hardest part, bridge with slow negatives + partial reps' (constant counterweight != real-rep readiness); (4.2) header 'Best Est. 1RM -- N assist' -&gt; 'Best -- N assist' (relative strength index, not a barbell 1RM); mobile+web, #3 info-disclaimer skipped per user. Model 5 (carry) DONE: verify-first verdict SOUND AS-IS (matches the audit's own 'SOUND AS-IS: loaded carry') -- one-axis-per-zone is correctly implemented AND shown (hero renders weight + distance as SEPARATE TickerNumbers, each with its own delta '+20 kg' vs 'same as your best', so 'push both axes at once' never reaches the user); the audit's only carry item (load+distance same session) is thus already handled, and the zone whyTexts already use the approved 'describe intent without the math' form. Another verify-first no-fix-needed (now: band/knee, BW-in-1RM, strength-log banner, carry). CARDIO SWEEP (user 'go on all 1-5', unlocked Pace+Swim): all 5 verify-first maps done via 5 parallel Explore agents. VERDICTS: (Ruck) REFUTED -- tiers are correctly labeled AND correctly absolute (match official GoRuck Light 20/Tough 35/Heavy 45; audit's 'our Tough=Heavy' + 'make BW-relative' both wrong); only real issue = no pack-weight safety cap (80lb=53%BW for a 150lb user) -&gt; AWAITING user soft-warning-vs-hard-cap pick. (StairMill) MOSTLY REFUTED -- 'FPM is a dial' false (it's derived=earned capacity), no units bug, peak-anchor by-design, Allison correctly documented; only real = 2 mis-cited studies (Honda 2014=glucose study; Boreham 2000=accumulated not 20-min continuous) -&gt; DONE: rewrote all 3 zone whyTexts to intent-only info-pill style (removes the citations, fixes the mis-cites; mobile+web) + corrected CLAUDE.md science tables + stale gender-baseline doc (code male 12/else 9, NOT 12/9/10), commit 7fcece9, web deployed. (Air Bike) CONFIRMED -- watts overlay cal/min x17.4 doesn't match the Assault console so '&gt;=X W' is unreadable + CLAUDE.md '17.4 industry-standard Assault/Echo' claim is FALSE -&gt; DROP the overlay (calibration needs a physical bike); also stale baseline doc (else 15 -&gt; code 13). (Pace) CONFIRMED -- single best-pace anchor + identical running offsets on every modality -&gt; add Critical Speed anchor (&gt;=2 efforts, fallback to single-pace), DEFER per-modality HR/power (needs HR integration, Phase 2). (Swim) CONFIRMED -- single-point Riegel CSS, fastest-biased (MIN), uniform 1.06 -&gt; 2-point linear CSS per stroke (fallback to Riegel under 2 distances). NEXT: Rucking (on pick) -&gt; Air Bike -&gt; Swim -&gt; Pace. OPTIONAL DEFERRED: BW eccentric/negatives tier + per-move-share BW 1RM (Model 2); web leverage pill carousel; assisted-log bare effective-1RM label; air-bike baseline doc fix (fold into Air Bike turn). === ROUND 2 QA FEEDBACK (2026-06-05), 6 items + overarching, NOT YET DONE: (1) Bench/weighted cue — each line must be SINGLE-LINE; restructure into bullet STEPS (work set / could-do-X-do-Y / add-each-time / work-up-to-PR / rest). (2) Power Clean / Olympic (Layout 9) cue — RESEARCH proper Olympic loading: express 'do X at ~50% (~Y lb)' or 'X x Y lb (~50% 1RM)' + a build-up-to-weight per-session progression; resolve how to pick the weight for a given rep/intensity (technique vs build vs peak) beyond 3 reps. (3) KB Swing / ballistic (Layout 10) — NEVER put attribution in the cue; make REST specific (research required rest / 'full rest', maybe = work time); does the bell-ladder benchmark apply to ALL bells incl 40kg? (4) Pull Up / BW consolidated (Layout 1) — shared chart wrongly mixes 13 light-band reps + 5 full-RX on ONE curve; SPLIT chart PER PILL/tier + update Layout xlsx. (5) Planche / leverage (Layout 11) — user wants the SWIMMING consolidation pattern: variant pill-swipe + tile grid (5 tiles), NOT separate per-variant pages. (6) Wall Sit / load (Layout 12) — 'Add load' is a CUE shown as a TITLE (fix title); NO target tile (build a 5-10 tile grid like Layout 1 but TIME-UNDER-TENSION tiles, added weight per tile); attribution-line format inconsistent. OVERARCHING (LOCKED DIRECTION): EVERY move that is a variation of another must follow the SWIMMING pattern end-to-end — DB naming 'Move [Variant]', consolidated detail w/ variant pill carousel, collapsed index/log row w/ variant badge. Read swimming impl end-to-end + replicate exactly (per-move design). ROUND-2 PROGRESS: [DONE] #1 cue format — user REJECTED bullets, so instead LOCKED ONE prose cue format SYSTEM-WIDE (one flowing sentence, commas not em-dashes, no bullets, no attribution-in-cue, numbers auto-emphasized w/ weights blue) behind a shared CueText component (mobile/src/components/CueText.tsx + web/src/components/CueText.jsx); swept EVERY coaching cue mobile+web (strength + cardio) onto it — zero em-dashes remain — then migrated the 4 hand-done cues (bench/ballistic/leverage/load) off inline spans onto CueText so there is literally ONE cue code path (commit db85128, web deployed). [DONE] #3 KB Swing -&gt; attribution removed from cue/benchmark (credit on its own line), concrete rest 'at least as long as the set takes (~1:1, power needs full recovery)', benchmark scoped to &lt;=32kg/70lb (hidden past the S&amp;S standard), last-bell now shows a 'top bell' state instead of a broken move-up-to-same. [DONE] #2 Power Clean / Olympic cue (Layout 9) -&gt; warm-up RAMP baked into the prose cue (empty bar -&gt; two loadable jumps at ~60% &amp; ~80% of the working weight via buildOlympicCue/olympicRamp, 0-2 rungs that collapse on light loads), working set restated as 'do X reps at Y lb, ~Z% of your best', PEAK = build to a heavy single PR; reps capped 1-3 BY DESIGN (no high-rep option — technique + bar speed collapse past ~3, cue says so). Also folded Olympic onto CueText + removed its em-dashes (its single-quoted static cues had been missed by the earlier backtick-only em-dash sweep). Mobile + web mirror + Layout-9 spec updated; user chose ramp-as-sentence over a chip row. REFINED after device test (user 'i barely understand it'): rephrased to an explicit STEP SEQUENCE ('Start with an empty bar, then N lb, then N lb, then do X reps at W lb, ~Z%...') so it reads step-by-step, AND added per-side PLATE CHIPS + 'N bar + ... per side' footer (platesForBarbellWeight, mirroring the weighted barbell card) so Olympic loads show plates like every other strength move. [DONE] #4 Pull-Up / BW consolidated chart -&gt; SPLIT per active tier: mobile chartData filters on bwTierFromVariantName(label)===bwActiveTier, web ===tier; PB reference line + caption follow the active tier; re-filters on pill swipe, never physically slides. Was wrongly blending ~13 light-band reps with ~5 full-RX reps on one curve. Updated CLAUDE.md BW spec item 5 (was 'shared across all tiers') + Layout Design.xlsx row 1 ('Consolidated chart' -&gt; 'Per-tier chart'). FOLLOW-UP CRASH FIX: the per-tier re-filter exposed a latent shared-LineChart bug -&gt; a PINNED tooltip stores an index, and when the dataset shrank on a tier swap that index went out of bounds, so points[activeIx] destructured undefined ('Invalid attempt to destructure non-iterable instance'). Fixed in mobile/src/components/LineChart.tsx (reset the pin on data.length change + bounds-guard the tooltip read), commit b3220f6 -- hardens EVERY mobile chart, not just bodyweight. RESEARCH BAKED IN: Olympic = 1-3 reps @ %1RM w/ warm-up ramp (Catalyst/NSCA/BarBend); KB power rest = 1:1 to 1:3 work:rest. [DONE] #6 Wall Sit / load holds (Layout 12) -&gt; rebuilt to look like Pull-Up Full RX: persistent TUT tile grid (10/20/30/45/60/90s) projecting the added weight to aim for at each duration via Rohmert's isometric-endurance curve (anchored on best loaded hold; heavier short, lighter long), tap a tile to drive the hero; build phase (no loaded efforts) shows bodyweight duration achievement + build cue; 'Add load' removed as the card TITLE (now in the cue); attribution -&gt; 'Rohmert curve · Oranchuk 2019 · ACSM'. Mobile + web mirror (AdminStrengthLoadDetail) + CLAUDE.md Layout-12 + Layout xlsx, end-to-end. [DONE] LAYOUT-OVERFLOW BUG found while testing the Full RX view: tile values wrapped mid-number (+107.5 -&gt; '+107.'/'5') and hero plate chips overflowed the card. Fixed mobile (numberOfLines+adjustsFontSizeToFit on tile values across BW/weighted/load grids + stretch in shared tileValueMono; on the BW/weighted-barbell/Olympic heroes the plates were then MOVED to their own single line below the number, label + chips in one row, NEVER wrapping, per user feedback that wrapping chips beside the number looked bad) + web (whitespace-nowrap on tile values; web plates already safe via flex-wrap + CSS default shrink). Cardio audited CLEAN. Root cause: RN flex-shrink defaults to 0 (CSS defaults to 1) so flexWrap never triggered on mobile plate blocks; tabular-nums keeps digit widths equal but does NOT stop wrapping. [DONE] #5 Planche/leverage swimming-consolidation -&gt; the 4 multi-variant leverage families (Planche, Front Lever, Back Lever, Handstand Hold) now run through the GENERIC FamilyConsolidatedDetail engine (the same Sled/Swimming pill carousel) on mobile -- NOT separate per-variant pages. User chose 'fit the generic engine (DB migration)'. DB migration (supabase/migrations-archive/20260605_consolidate_leverage_families.sql, applied via MCP): renamed each variant to 'Name [Variant]' bracket form, inserted a parent container row per family, linked children via parent_movement_id + variant_short_label (TUCK/STRADDLE/FULL/WALL/FREE), migrated 3 logged effort labels. Mobile code: LEVERAGE_LADDERS + leverageVariantLabel -&gt; bracket form; ladder strip hidden inside consolidated slots; FamilyConsolidatedDetail parent prop widened + SKILL badge for leverage parents (equipment=null). Carousel order easiest-&gt;hardest (Tuck-&gt;Straddle-&gt;Full, Wall-&gt;Freestanding); each slot = per-variant LeverageHoldDetail; index collapses each family to one row. Web coach mirror re-pointed to bracket names (AdminStrengthLeverageDetail ladders + lib/movements ISOMETRIC_LIST) -&gt; renders variants INDIVIDUALLY (web has no generic consolidation engine; a web pill carousel is deferred -- arguably clearer for read-only roster review anyway). CLAUDE.md Layout-11 spec rewritten (Family consolidation block + dispatch order). mobile committed 892c13e; web built+deployed + committed 50d5a10. OVERARCHING swimming pass: SATISFIED for strength -- enumerated the live movements table; leverage was the ONLY remaining true multi-variant family beyond the already-consolidated Swimming / Sled / BW-assist-tiers; grip/angle/stance paren movements confirmed DISTINCT (NOT merged, per user 'grip/angle stay distinct'). REMAINING T088: Model 4 (assisted machine) verify-first, then carry (Model 5) + cardio Models 6-11 (StairMill baseline, air-bike watts, ruck BW cap, pace critical-speed, swim 2-point CSS). OPTIONAL DEFERRED: BW eccentric/negatives tier + per-move-share BW 1RM (Model 2); web leverage pill carousel.</t>
+          <t>VERDICTS by severity. TIER A (correctness/safety): (A1) Olympic &amp; ballistic lifts (snatch, C&amp;J, power clean, KB swing/snatch) must NOT use rep-max math — a 20RM snatch is meaningless + suggests a dangerous practice; route to low-rep %1RM/velocity model. (A2) Rucking has NO bodyweight cap + mislabeled tiers (Tough=35lb is actually GoRuck HEAVY dry; true Tough=20/30lb by BW); 80lb ladder top = 53% BW for a 150lb user, past the ~1/3 BW safe limit — make tiers BW-relative + add ~1/3 BW hard cap. (A3) Plyometrics/jumps/jump-rope treated as max-reps — wrong; progress on OUTPUT (jump height/distance, box height) + contact budget + rest. (A4) StairMill: FPM is a machine SETTING not earned capacity (+ floor=16 vs 22 steps across models, peak-of-any-effort inflates); anchor on sustained held SPM / vertical m-per-min over a continuous block. TIER B (anchors mis-set): (B5) Bodyweight graduation 10 reps -&gt; ~5-8 (10 reps = endurance, ~70-75% 1RM). (B6) Isometric: tag axis time|load|leverage — time holds keep 2-min cap, loadable holds add load after ~30-60s, skill-leverage holds (planche/levers/flag/L-sit) drop the 120s grid -&gt; variant ladder. (B7) Pace cardio: anchor on Critical Speed (2-3 efforts) not single best pace; zones as %threshold per modality (power for ergs/bike, HR/RPE elliptical) not fixed running s/km offsets. (B8) Swim: replace Riegel single-point CSS with 2-point linear slope per stroke (1.06 is a running exponent, worse for fly/breast); kill 'fastest projection' (biased high); deepen VO2 to CSS-8..-10. (B9) Air bike: watts=cal/min*17.4 is arithmetically ok at 25% GE but 25% is optimistic AND doesn't match the console (~24.75 W/cal-min on Assault) so 'hold &gt;=X W' is unreadable — drop overlay or calibrate to console + name brand. (B10) Weighted 15/20RM tiles are guesses (cap grid ~10-12RM); + the T087 cue fix (submaximal + RIR + double progression). TIER C (copy/labels): hypertrophy '6-12' too strict (growth 5-30+ near failure); carry 'load+distance same session' (zones already do one-axis); assisted 'BW-assist-&gt;1RM' is a relative index not a true 1RM (counterweight is constant through ROM, pull-up hardest at bottom) — relabel + add reps/negatives; soften 'polarized 80/20 is best' (pyramidal = for recreational); CLAUDE.md air-bike '17.4 standard Assault/Echo conversion' claim is FALSE; StairMill cites Honda 2014 (a GLUCOSE study, drop it), Allison was 20s not 60s, Boreham was accumulated bouts not 20-min continuous; StairMill gender baseline 12 FPM ~= 192 SPM EXCEEDS the machine max (units error, real ~4-5 FPM). SOUND AS-IS: loaded carry (one copy tweak), the swim/pace 3-zone + easy-floor STRUCTURE. CONSOLIDATED CITEABLE SOURCES: strength = Epley/Brzycki/Lombardi + Reynolds-Robergs 2006 + Schoenfeld rep-continuum 2021 + NSCA Haff&amp;Triplett + Prilepin + Helms/Zourdos RIR + ACSM; bodyweight = Ebben 2012 + Nuzzo 2023 (ECC:CON 1.41) + Steven Low; plyo/skill = NSCA plyo + Markovic&amp;Mikulic 2010 + Ramirez-Campillo + McGill + GMB; iso = Oranchuk 2019 + Schott 1995 + Kitai&amp;Sale 1989 + McGill; carry = McGill strongman EMG + Winwood/Keogh/Cronin + NSCA + Dan John; pace = Daniels VDOT + Seiler 80/20 + Critical Power (Jones/Vanhatalo) + Coggan FTP + ACSM; swim = Wakayoshi 1992 + Maglischo + Costill + Gonjo 2024; air bike = Peronnet&amp;Massicotte 1991 + Concept2 formula + Gibala SIT + Seiler; ruck = Knapik + US Army ATP 3-21.18 + GoRuck + EIB/Ranger 12mi; stairmill = Allison 2017 + Boreham 2000 + ACSM + Ainsworth Compendium + Seiler. STATUS: research complete, awaiting user TRIAGE on what to implement — most surfaces are locked, but math/bug fixes (StairMill baseline, air-bike watts, ruck BW cap, Olympic-lift rep-max) are allowed on locked surfaces per the finalized-surfaces rule; design changes need explicit unlock. PROGRESS (full model-by-model sweep, user chose 'full sweep' 2026-06-05): Model 1 Fix 1.1 (submaximal working-weight cue 'a weight you could do K+reserve, do K' + corrected per-zone RIR 2/2/1 + iterative 'add X each time, work up to PR') SHIPPED mobile+web. Fix 1.2 (Olympic barbell lifts routed OFF the rep-max grid to a NEW Layout 9 %-of-best card: added movements.lift_type column [olympic|ballistic], tagged 22 barbell snatch/clean/jerk-family lifts; mobile OlympicLiftDetail + web AdminStrengthOlympicDetail mirror + dispatch-before-weighted + Layout Design.xlsx row 9 + CLAUDE.md Layout-9 spec) SHIPPED. Fix 1.3 (capped the rendered rep-max grid at 15RM, dropped 16-20 as noise, flagged 13-15RM with a leading '≈' + caveat note; kept the 3-zone model since Endurance needs 13+) SHIPPED mobile+web. Fix 1.4 (hypertrophy whyText softened — growth spans ~5-30+ reps near failure, 6-12 is just the efficient middle, not an exclusive window) SHIPPED mobile+web. Fix 1.2b (ballistic kettlebell -&gt; NEW Layout 10 bell-ladder card: tagged 13 KB ballistic moves lift_type='ballistic'; mobile BallisticLiftDetail + web AdminStrengthBallisticDetail mirror + dispatch-before-weighted + Layout xlsx row 10 + CLAUDE.md spec) SHIPPED. MODEL 1 COMPLETE (weighted cue + Olympic Layout 9 + ballistic Layout 10 + grid cap + hypertrophy copy). Model 2 (bodyweight rep-strength + assist tiers) IN PROGRESS: Fix 2.1 (graduation trigger BW_GRADUATION_REPS 10-&gt;8 so tiers/bands graduate in the strength range not endurance; mobile+web+CLAUDE.md) SHIPPED. Fix 2.2 (band/knee): on inspection there is NO false 'band is harder' copy — only the carousel order asserts it, which is load-bearing (graduation path + badge + landing) and the science says the order is AMBIGUOUS not wrong; user chose #1 = LEAVE the order (deliberate no-op). Fix 2.3a (bodyweight in the weighted 1RM): VERIFIED ALREADY HANDLED — the log form stores estimate1RM(profileBodyWeight + addedWeight, reps) [strength.tsx ~L414/424] and the detail projection derives added = projection - bodyweight [L4733]; the audit's 'ignores bodyweight' claim is FALSE for our code. (Only nuance: uses FULL bodyweight = 100% share, so push-ups over-count vs pull-ups — an optional minor per-move-share tweak, not a bug.) NET: Model 2 CORRECTNESS DONE — the graduation 10-&gt;8 (2.1) was the one real fix. The rest of the audit's Model-2 items are FEATURE additions, not correctness bugs: an eccentric/negatives tier + leverage/tempo/unilateral alternatives (both optional, additive builds touching the locked card + log form). META-LESSON: this is the 3rd audit claim our code already handles correctly (band/knee, BW-in-1RM) — the audit agents researched GENERIC science and assumed naive implementations; our code is more sophisticated. So VERIFY every audit claim against the actual code before 'fixing' it. Model 3 (isometric) IN PROGRESS: VERIFIED real (unlike Model 2) — all 38 iso moves were on one 10-120s time grid incl. skill holds where 120s is meaningless. LEVERAGE family SHIPPED: added movements.hold_type column (time/load/leverage), tagged 18 leverage holds; NEW Layout 11 -&gt; mobile LeverageHoldDetail + web AdminStrengthLeverageDetail mirror; short milestones 5/10/15/20/30s + skill-ladder (planche tuck-&gt;straddle-&gt;full, levers tuck-&gt;full, handstand wall-&gt;free; gate = 30s clean -&gt; next variant; L-Sit/V-Sit standalone per user); dispatch before isometric; Layout xlsx row 11 + CLAUDE.md Layout-11 spec + iso spec updated to exclude leverage. Model 3 (isometric) COMPLETE: leverage family (Layout 11) + LOAD family (Layout 12) both SHIPPED. Load: tagged 7 loadable holds (wall sit, calf-raise, glute-bridge x2, dead hang, split-squat, squat hold) hold_type='load'; mobile LoadHoldDetail + web AdminStrengthLoadDetail mirror; two phases (time milestones 15-60s -&gt; add-load; gate 60s, loaded target 30s; load inc 5lb/2.5kg); LOG FORM gained an Added-weight wheel for load-holds (label 'Name · W unit x D sec', value stays 'D sec' so parseDurationSecs unchanged); chart adaptive (load over time once weighted, else hold time); dispatch before isometric; Layout xlsx row 12 + CLAUDE.md Layout-12 spec + iso spec updated. The ~13 TIME holds (plank/side-plank/hollow/etc.) stay on IsometricDetail (correct). Model 4 (assisted machine) DONE (verify-first CONFIRMED the audit this time): (4.1) graduation over-promise fixed -- 'attempt unassisted, you're ready' -&gt; honest 'machine eased the hardest part, bridge with slow negatives + partial reps' (constant counterweight != real-rep readiness); (4.2) header 'Best Est. 1RM -- N assist' -&gt; 'Best -- N assist' (relative strength index, not a barbell 1RM); mobile+web, #3 info-disclaimer skipped per user. Model 5 (carry) DONE: verify-first verdict SOUND AS-IS (matches the audit's own 'SOUND AS-IS: loaded carry') -- one-axis-per-zone is correctly implemented AND shown (hero renders weight + distance as SEPARATE TickerNumbers, each with its own delta '+20 kg' vs 'same as your best', so 'push both axes at once' never reaches the user); the audit's only carry item (load+distance same session) is thus already handled, and the zone whyTexts already use the approved 'describe intent without the math' form. Another verify-first no-fix-needed (now: band/knee, BW-in-1RM, strength-log banner, carry). CARDIO SWEEP (user 'go on all 1-5', unlocked Pace+Swim): all 5 verify-first maps done via 5 parallel Explore agents. VERDICTS: (Ruck) REFUTED -- tiers are correctly labeled AND correctly absolute (match official GoRuck Light 20/Tough 35/Heavy 45; audit's 'our Tough=Heavy' + 'make BW-relative' both wrong); only real issue = no pack-weight safety cap (80lb=53%BW for a 150lb user) -&gt; AWAITING user soft-warning-vs-hard-cap pick. (StairMill) MOSTLY REFUTED -- 'FPM is a dial' false (it's derived=earned capacity), no units bug, peak-anchor by-design, Allison correctly documented; only real = 2 mis-cited studies (Honda 2014=glucose study; Boreham 2000=accumulated not 20-min continuous) -&gt; DONE: rewrote all 3 zone whyTexts to intent-only info-pill style (removes the citations, fixes the mis-cites; mobile+web) + corrected CLAUDE.md science tables + stale gender-baseline doc (code male 12/else 9, NOT 12/9/10), commit 7fcece9, web deployed. (Air Bike) CONFIRMED -- watts overlay cal/min x17.4 doesn't match the Assault console so '&gt;=X W' is unreadable + CLAUDE.md '17.4 industry-standard Assault/Echo' claim is FALSE -&gt; DROP the overlay (calibration needs a physical bike); also stale baseline doc (else 15 -&gt; code 13). (Pace) CONFIRMED -- single best-pace anchor + identical running offsets on every modality -&gt; add Critical Speed anchor (&gt;=2 efforts, fallback to single-pace), DEFER per-modality HR/power (needs HR integration, Phase 2). (Swim) CONFIRMED -- single-point Riegel CSS, fastest-biased (MIN), uniform 1.06 -&gt; 2-point linear CSS per stroke (fallback to Riegel under 2 distances). ALL 5 CARDIO MODELS DONE (user 'soft cap, finish all in one run'): (1) Rucking -&gt; SOFT bodyweight safety warning on the log form when pack &gt; ~1/3 BW (never blocks logging; tiers stay ABSOLUTE per verify-first -- they match official GoRuck), commit b569523. (2) StairMill -&gt; 2 mis-cited studies fixed by rewriting the 3 zone whyTexts to intent-only info-pill style (Honda 2014 = glucose study; Boreham 2000 = accumulated not continuous) + baseline doc corrected, commit 7fcece9. (3) Air Bike -&gt; watts overlay DROPPED (cal/min x17.4 is not a console standard + doesn't match the Assault display, so unverifiable; calsPerMinToWatts deleted mobile+web) + the false 'industry-standard conversion' CLAUDE.md claim removed, commit f05545c. (4) Swim -&gt; 2-point linear Critical Swim Speed with Riegel fallback (was single-point MIN-biased Riegel + running 1.06 exponent), commit da0a5a7. (5) Pace -&gt; Critical Speed zone anchor with fastest-pace fallback (was single best pace = too hard), commit 800f37c. All mobile + web mirror + CLAUDE.md; web deployed df75f088. T088 COMPLETE -- all 11 progression models (6 strength + 5 cardio) audited + corrected. DEFERRED (optional, NOT blocking): per-modality power/HR pace+erg zones (Phase 2, needs HR/power integration); BW eccentric/negatives tier + per-move-share BW 1RM (Model 2); web leverage pill carousel; assisted-log bare effective-1RM label. VERIFY-FIRST SCORECARD (8 of 11 had the audit at least partly wrong): audit WRONG/overblown on band-knee order, BW-in-1RM, strength-log banner (only Olympic/ballistic slipped), carry, Rucking tiers, StairMill headline (FPM-is-a-dial/units); audit RIGHT on Olympic rep-max, ballistic, Air Bike watts, Swim CSS, Pace anchor, StairMill citations, BW graduation reps. === ROUND 2 QA FEEDBACK (2026-06-05), 6 items + overarching, NOT YET DONE: (1) Bench/weighted cue — each line must be SINGLE-LINE; restructure into bullet STEPS (work set / could-do-X-do-Y / add-each-time / work-up-to-PR / rest). (2) Power Clean / Olympic (Layout 9) cue — RESEARCH proper Olympic loading: express 'do X at ~50% (~Y lb)' or 'X x Y lb (~50% 1RM)' + a build-up-to-weight per-session progression; resolve how to pick the weight for a given rep/intensity (technique vs build vs peak) beyond 3 reps. (3) KB Swing / ballistic (Layout 10) — NEVER put attribution in the cue; make REST specific (research required rest / 'full rest', maybe = work time); does the bell-ladder benchmark apply to ALL bells incl 40kg? (4) Pull Up / BW consolidated (Layout 1) — shared chart wrongly mixes 13 light-band reps + 5 full-RX on ONE curve; SPLIT chart PER PILL/tier + update Layout xlsx. (5) Planche / leverage (Layout 11) — user wants the SWIMMING consolidation pattern: variant pill-swipe + tile grid (5 tiles), NOT separate per-variant pages. (6) Wall Sit / load (Layout 12) — 'Add load' is a CUE shown as a TITLE (fix title); NO target tile (build a 5-10 tile grid like Layout 1 but TIME-UNDER-TENSION tiles, added weight per tile); attribution-line format inconsistent. OVERARCHING (LOCKED DIRECTION): EVERY move that is a variation of another must follow the SWIMMING pattern end-to-end — DB naming 'Move [Variant]', consolidated detail w/ variant pill carousel, collapsed index/log row w/ variant badge. Read swimming impl end-to-end + replicate exactly (per-move design). ROUND-2 PROGRESS: [DONE] #1 cue format — user REJECTED bullets, so instead LOCKED ONE prose cue format SYSTEM-WIDE (one flowing sentence, commas not em-dashes, no bullets, no attribution-in-cue, numbers auto-emphasized w/ weights blue) behind a shared CueText component (mobile/src/components/CueText.tsx + web/src/components/CueText.jsx); swept EVERY coaching cue mobile+web (strength + cardio) onto it — zero em-dashes remain — then migrated the 4 hand-done cues (bench/ballistic/leverage/load) off inline spans onto CueText so there is literally ONE cue code path (commit db85128, web deployed). [DONE] #3 KB Swing -&gt; attribution removed from cue/benchmark (credit on its own line), concrete rest 'at least as long as the set takes (~1:1, power needs full recovery)', benchmark scoped to &lt;=32kg/70lb (hidden past the S&amp;S standard), last-bell now shows a 'top bell' state instead of a broken move-up-to-same. [DONE] #2 Power Clean / Olympic cue (Layout 9) -&gt; warm-up RAMP baked into the prose cue (empty bar -&gt; two loadable jumps at ~60% &amp; ~80% of the working weight via buildOlympicCue/olympicRamp, 0-2 rungs that collapse on light loads), working set restated as 'do X reps at Y lb, ~Z% of your best', PEAK = build to a heavy single PR; reps capped 1-3 BY DESIGN (no high-rep option — technique + bar speed collapse past ~3, cue says so). Also folded Olympic onto CueText + removed its em-dashes (its single-quoted static cues had been missed by the earlier backtick-only em-dash sweep). Mobile + web mirror + Layout-9 spec updated; user chose ramp-as-sentence over a chip row. REFINED after device test (user 'i barely understand it'): rephrased to an explicit STEP SEQUENCE ('Start with an empty bar, then N lb, then N lb, then do X reps at W lb, ~Z%...') so it reads step-by-step, AND added per-side PLATE CHIPS + 'N bar + ... per side' footer (platesForBarbellWeight, mirroring the weighted barbell card) so Olympic loads show plates like every other strength move. [DONE] #4 Pull-Up / BW consolidated chart -&gt; SPLIT per active tier: mobile chartData filters on bwTierFromVariantName(label)===bwActiveTier, web ===tier; PB reference line + caption follow the active tier; re-filters on pill swipe, never physically slides. Was wrongly blending ~13 light-band reps with ~5 full-RX reps on one curve. Updated CLAUDE.md BW spec item 5 (was 'shared across all tiers') + Layout Design.xlsx row 1 ('Consolidated chart' -&gt; 'Per-tier chart'). FOLLOW-UP CRASH FIX: the per-tier re-filter exposed a latent shared-LineChart bug -&gt; a PINNED tooltip stores an index, and when the dataset shrank on a tier swap that index went out of bounds, so points[activeIx] destructured undefined ('Invalid attempt to destructure non-iterable instance'). Fixed in mobile/src/components/LineChart.tsx (reset the pin on data.length change + bounds-guard the tooltip read), commit b3220f6 -- hardens EVERY mobile chart, not just bodyweight. RESEARCH BAKED IN: Olympic = 1-3 reps @ %1RM w/ warm-up ramp (Catalyst/NSCA/BarBend); KB power rest = 1:1 to 1:3 work:rest. [DONE] #6 Wall Sit / load holds (Layout 12) -&gt; rebuilt to look like Pull-Up Full RX: persistent TUT tile grid (10/20/30/45/60/90s) projecting the added weight to aim for at each duration via Rohmert's isometric-endurance curve (anchored on best loaded hold; heavier short, lighter long), tap a tile to drive the hero; build phase (no loaded efforts) shows bodyweight duration achievement + build cue; 'Add load' removed as the card TITLE (now in the cue); attribution -&gt; 'Rohmert curve · Oranchuk 2019 · ACSM'. Mobile + web mirror (AdminStrengthLoadDetail) + CLAUDE.md Layout-12 + Layout xlsx, end-to-end. [DONE] LAYOUT-OVERFLOW BUG found while testing the Full RX view: tile values wrapped mid-number (+107.5 -&gt; '+107.'/'5') and hero plate chips overflowed the card. Fixed mobile (numberOfLines+adjustsFontSizeToFit on tile values across BW/weighted/load grids + stretch in shared tileValueMono; on the BW/weighted-barbell/Olympic heroes the plates were then MOVED to their own single line below the number, label + chips in one row, NEVER wrapping, per user feedback that wrapping chips beside the number looked bad) + web (whitespace-nowrap on tile values; web plates already safe via flex-wrap + CSS default shrink). Cardio audited CLEAN. Root cause: RN flex-shrink defaults to 0 (CSS defaults to 1) so flexWrap never triggered on mobile plate blocks; tabular-nums keeps digit widths equal but does NOT stop wrapping. [DONE] #5 Planche/leverage swimming-consolidation -&gt; the 4 multi-variant leverage families (Planche, Front Lever, Back Lever, Handstand Hold) now run through the GENERIC FamilyConsolidatedDetail engine (the same Sled/Swimming pill carousel) on mobile -- NOT separate per-variant pages. User chose 'fit the generic engine (DB migration)'. DB migration (supabase/migrations-archive/20260605_consolidate_leverage_families.sql, applied via MCP): renamed each variant to 'Name [Variant]' bracket form, inserted a parent container row per family, linked children via parent_movement_id + variant_short_label (TUCK/STRADDLE/FULL/WALL/FREE), migrated 3 logged effort labels. Mobile code: LEVERAGE_LADDERS + leverageVariantLabel -&gt; bracket form; ladder strip hidden inside consolidated slots; FamilyConsolidatedDetail parent prop widened + SKILL badge for leverage parents (equipment=null). Carousel order easiest-&gt;hardest (Tuck-&gt;Straddle-&gt;Full, Wall-&gt;Freestanding); each slot = per-variant LeverageHoldDetail; index collapses each family to one row. Web coach mirror re-pointed to bracket names (AdminStrengthLeverageDetail ladders + lib/movements ISOMETRIC_LIST) -&gt; renders variants INDIVIDUALLY (web has no generic consolidation engine; a web pill carousel is deferred -- arguably clearer for read-only roster review anyway). CLAUDE.md Layout-11 spec rewritten (Family consolidation block + dispatch order). mobile committed 892c13e; web built+deployed + committed 50d5a10. OVERARCHING swimming pass: SATISFIED for strength -- enumerated the live movements table; leverage was the ONLY remaining true multi-variant family beyond the already-consolidated Swimming / Sled / BW-assist-tiers; grip/angle/stance paren movements confirmed DISTINCT (NOT merged, per user 'grip/angle stay distinct'). REMAINING T088: Model 4 (assisted machine) verify-first, then carry (Model 5) + cardio Models 6-11 (StairMill baseline, air-bike watts, ruck BW cap, pace critical-speed, swim 2-point CSS). OPTIONAL DEFERRED: BW eccentric/negatives tier + per-move-share BW 1RM (Model 2); web leverage pill carousel.</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: close T087 (shipped via T088 Model-1 cue fix)
T087 (submaximal/RIR/double-progression strength cue) shipped as T088 Fix 1.1 on
mobile + web + CLAUDE.md. Status -> Done.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4684,9 +4684,9 @@
           <t>Mobile+Web</t>
         </is>
       </c>
-      <c r="E90" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E90" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>BRAINSTORM stage — do NOT implement until the model is agreed. Design a progression-aware strength cue that separates (a) the WORKING prescription (submaximal, RIR-based, day-to-day), (b) the PROGRESSION rule (when to bump load — e.g. double progression: add reps to top of range across all sets, then +smallest jump), (c) the PR ATTEMPT (one top set at the target, periodically). Affects the locked Weighted Standard next-target card + ADP_ZONE defaults (sets/RIR/rest). Plain-English, one decision at a time. RESEARCH DONE 2026-06-04 (deep-research harness returned empty; did it via WebSearch): EVIDENCE-DICTATED answer -&gt; working sets must be SUBMAXIMAL with ~2-3 reps in reserve, NOT the rep-max. (a) Strength gains are ~independent of proximity-to-failure (Refalo 2023 dose-response meta-regression; Schoenfeld) so no need to grind to max — leave reps in reserve. (b) Prilepin's table caps reps-per-set BELOW the single-set max at each %1RM (~85% -&gt; 2-4 reps/set, not 5) — the direct 'why you can't do 4-5 sets of 5 at your 5RM'. (c) Double progression confirmed (Plett/Schoenfeld PeerJ 2022 — rep AND load progression both work). (d) Dose zones match the ACSM position stand (strength &gt;=80% 1RM low reps long rest; hypertrophy 6-12RM 1-2min; endurance &lt;60% &gt;15 reps &lt;90s). SO: working weight ~= the 7-8RM (a couple reps in reserve), double-progress up to the 140 target, 140 = periodic TEST. Attribution credit for the prescription side: 'Prilepin · Helms/Zourdos RIR · ACSM' (+ optionally Schoenfeld). Cue redesign pending user go-ahead.</t>
+          <t>BRAINSTORM stage — do NOT implement until the model is agreed. Design a progression-aware strength cue that separates (a) the WORKING prescription (submaximal, RIR-based, day-to-day), (b) the PROGRESSION rule (when to bump load — e.g. double progression: add reps to top of range across all sets, then +smallest jump), (c) the PR ATTEMPT (one top set at the target, periodically). Affects the locked Weighted Standard next-target card + ADP_ZONE defaults (sets/RIR/rest). Plain-English, one decision at a time. RESEARCH DONE 2026-06-04 (deep-research harness returned empty; did it via WebSearch): EVIDENCE-DICTATED answer -&gt; working sets must be SUBMAXIMAL with ~2-3 reps in reserve, NOT the rep-max. (a) Strength gains are ~independent of proximity-to-failure (Refalo 2023 dose-response meta-regression; Schoenfeld) so no need to grind to max — leave reps in reserve. (b) Prilepin's table caps reps-per-set BELOW the single-set max at each %1RM (~85% -&gt; 2-4 reps/set, not 5) — the direct 'why you can't do 4-5 sets of 5 at your 5RM'. (c) Double progression confirmed (Plett/Schoenfeld PeerJ 2022 — rep AND load progression both work). (d) Dose zones match the ACSM position stand (strength &gt;=80% 1RM low reps long rest; hypertrophy 6-12RM 1-2min; endurance &lt;60% &gt;15 reps &lt;90s). SO: working weight ~= the 7-8RM (a couple reps in reserve), double-progress up to the 140 target, 140 = periodic TEST. Attribution credit for the prescription side: 'Prilepin · Helms/Zourdos RIR · ACSM' (+ optionally Schoenfeld). SHIPPED via T088 Model 1 Fix 1.1 (2026-06-05): the submaximal working-weight cue ('a weight you could do K+reserve, do K'), corrected per-zone RIR (2/2/1), and the iterative 'add X each time, work up to your PR' double-progression cue all landed on mobile + web (AdminStrengthWeightedDetail) + CLAUDE.md. T087 CLOSED 2026-06-05 — its deliverable IS T088's Model-1 cue fix.</t>
         </is>
       </c>
       <c r="H90" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(T080): coach-view efforts parity complete (mirror + family carousel)
Recorded the 2-agent parity cross-check verdict (all strength + cardio coach
mirrors current + matching, incl. the T088 cardio fixes; both audit "critical"
alarms were false on inspection) + the FamilyConsolidated coach carousel build that
closed the last gap. Mirror phase done; coaching add-ons remain deferred; non-effort
tabs tracked under T079 Phase 2.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -570,7 +570,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-05 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
+          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-06 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>STRUCTURE DECIDED 2026-06-04: keep ONE combined Efforts tab with an internal Strength|Cardio segmented toggle (dropped 'All', default Strength). LIST-VIEW read-only mirror DONE + deployed 2026-06-04 — removed the Add-effort form + backdate + button; AdminUserActivity is now read-only (207-&gt;193 lines). USER 2026-06-04: FINISH THE MIRROR BEFORE ADD-ONS. MAIN REMAINING = (1) DETAIL-SCREEN rebuild to mirror the athlete coaching surfaces, incremental: Strength Weighted Standard FIRST (validate with user), then other strength variants (bodyweight/assisted/carry/iso/sled), then cardio surfaces (pace/airbike/swim/ruck/stairmill/ergs/duration); (2) LIST variant-collapsing (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge like the athlete; coupled to the detail routes). DEFERRED until mirror complete: coaching add-ons (recency, stalled flag, frequency, PR timeline, balance, adherence). Detail rebuild notes: admin detail routes (AdminEffortDetail = bare 10-tile grid; AdminCardioDetail = old pace model w/ banned 'lower=faster') don't mirror the athlete coaching surfaces; KEEP the per-effort swipe-delete there. USER CORRECTION 2026-06-04: the coach is NOT fully read-only — they CAN delete efforts; only the athlete-style ADD/log form is excluded (that's the separate coach-input track). List view stays add-free; individual-effort delete lives in the detail screens. PROGRESS 2026-06-04: Strength Weighted Standard detail mirror DONE + deployed (new web/src/pages/admin/detail/AdminStrengthWeightedDetail.jsx, dispatched from AdminEffortDetail for barbell/dumbbell/kettlebell/machine/strongman; read-only + delete kept; rep-max projections + adp-zone pills + 20 tiles + next-target hero + chart + log). AWAITING user validation of this first variant before rolling out remaining strength variants (bodyweight/assisted/carry/iso/sled) + all cardio surfaces + list variant-collapsing.</t>
+          <t>STRUCTURE DECIDED 2026-06-04: keep ONE combined Efforts tab with an internal Strength|Cardio segmented toggle (dropped 'All', default Strength). LIST-VIEW read-only mirror DONE + deployed 2026-06-04 — removed the Add-effort form + backdate + button; AdminUserActivity is now read-only (207-&gt;193 lines). USER 2026-06-04: FINISH THE MIRROR BEFORE ADD-ONS. MAIN REMAINING = (1) DETAIL-SCREEN rebuild to mirror the athlete coaching surfaces, incremental: Strength Weighted Standard FIRST (validate with user), then other strength variants (bodyweight/assisted/carry/iso/sled), then cardio surfaces (pace/airbike/swim/ruck/stairmill/ergs/duration); (2) LIST variant-collapsing (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge like the athlete; coupled to the detail routes). DEFERRED until mirror complete: coaching add-ons (recency, stalled flag, frequency, PR timeline, balance, adherence). Detail rebuild notes: admin detail routes (AdminEffortDetail = bare 10-tile grid; AdminCardioDetail = old pace model w/ banned 'lower=faster') don't mirror the athlete coaching surfaces; KEEP the per-effort swipe-delete there. USER CORRECTION 2026-06-04: the coach is NOT fully read-only — they CAN delete efforts; only the athlete-style ADD/log form is excluded (that's the separate coach-input track). List view stays add-free; individual-effort delete lives in the detail screens. PROGRESS 2026-06-04: Strength Weighted Standard detail mirror DONE + deployed (new web/src/pages/admin/detail/AdminStrengthWeightedDetail.jsx, dispatched from AdminEffortDetail for barbell/dumbbell/kettlebell/machine/strongman; read-only + delete kept; rep-max projections + adp-zone pills + 20 tiles + next-target hero + chart + log). AWAITING user validation of this first variant before rolling out remaining strength variants (bodyweight/assisted/carry/iso/sled) + all cardio surfaces + list variant-collapsing. UPDATE 2026-06-06 — MIRROR COMPLETE. Ran a 2-agent parity cross-check (strength + cardio): ALL strength variant coach mirrors (weighted/bodyweight/assisted/carry/leverage/load/iso/Olympic/ballistic/repsonly) + ALL cardio mirrors (pace/ergs/swim/airbike/ruck/stairmill/beat-your-best) exist, are routed, and match the athlete — INCLUDING the T088 cardio fixes (StairMill citations, Air-Bike watts removal, Swim 2-point CSS, Pace Critical Speed all present in the coach mirrors). Both audits' 'critical' alarms were FALSE on verify-first inspection: 'Pace-CS-missing-on-coach' was an agent miss (it's at AdminCardioPaceDetail L275); 'FamilyConsolidatedDetail-missing' was the known-deferred carousel. Fixed 1 stale Air-Bike header doc-comment. THEN built the last gap — the FamilyConsolidated COACH carousel: new web/src/pages/admin/detail/AdminStrengthFamilyDetail.jsx (click variant pills + the selected child's AdminStrengthLeverageDetail with a new hideHeader prop) + AdminEffortDetail dispatch (a parent_movement_id parent with &gt;=2 children -&gt; family detail, child -&gt; per-variant) + AdminUserActivity catalog-driven family list-collapse (verified safe vs Sled/Swim, which also carry parent_movement_id: Sled branch runs first, Swimming is cardio-only). Web deployed (e226dc6f). List-collapsing now complete (BW tiers + Sled + Swim + admin families). Cosmetic 'drifts' (web click-toggle vs swipe pills, static numbers vs TickerNumber) are INTENTIONAL per the 'web stays simple' rule. REMAINING (deferred, now un-blocked): coaching ADD-ONS (recency, stalled flag, frequency, PR timeline, balance, adherence). Non-effort coach tabs (Sleep/Hydration/Heart/Bodyweight/Calories) parity = separate, tracked under T079 Phase 2.</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs(T080): mark Done — coach Efforts parity shipped, remaining add-ons descoped
User descoped stalled/frequency/balance/adherence ("no need for the rest"). T080
delivered: list mirror + family carousel + move-cards (graph + PR + recency) + card
click-affordance. Status -> Done.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4355,9 +4355,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E83" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
@@ -4367,7 +4367,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>STRUCTURE DECIDED 2026-06-04: keep ONE combined Efforts tab with an internal Strength|Cardio segmented toggle (dropped 'All', default Strength). LIST-VIEW read-only mirror DONE + deployed 2026-06-04 — removed the Add-effort form + backdate + button; AdminUserActivity is now read-only (207-&gt;193 lines). USER 2026-06-04: FINISH THE MIRROR BEFORE ADD-ONS. MAIN REMAINING = (1) DETAIL-SCREEN rebuild to mirror the athlete coaching surfaces, incremental: Strength Weighted Standard FIRST (validate with user), then other strength variants (bodyweight/assisted/carry/iso/sled), then cardio surfaces (pace/airbike/swim/ruck/stairmill/ergs/duration); (2) LIST variant-collapsing (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge like the athlete; coupled to the detail routes). DEFERRED until mirror complete: coaching add-ons (recency, stalled flag, frequency, PR timeline, balance, adherence). Detail rebuild notes: admin detail routes (AdminEffortDetail = bare 10-tile grid; AdminCardioDetail = old pace model w/ banned 'lower=faster') don't mirror the athlete coaching surfaces; KEEP the per-effort swipe-delete there. USER CORRECTION 2026-06-04: the coach is NOT fully read-only — they CAN delete efforts; only the athlete-style ADD/log form is excluded (that's the separate coach-input track). List view stays add-free; individual-effort delete lives in the detail screens. PROGRESS 2026-06-04: Strength Weighted Standard detail mirror DONE + deployed (new web/src/pages/admin/detail/AdminStrengthWeightedDetail.jsx, dispatched from AdminEffortDetail for barbell/dumbbell/kettlebell/machine/strongman; read-only + delete kept; rep-max projections + adp-zone pills + 20 tiles + next-target hero + chart + log). AWAITING user validation of this first variant before rolling out remaining strength variants (bodyweight/assisted/carry/iso/sled) + all cardio surfaces + list variant-collapsing. UPDATE 2026-06-06 — MIRROR COMPLETE. Ran a 2-agent parity cross-check (strength + cardio): ALL strength variant coach mirrors (weighted/bodyweight/assisted/carry/leverage/load/iso/Olympic/ballistic/repsonly) + ALL cardio mirrors (pace/ergs/swim/airbike/ruck/stairmill/beat-your-best) exist, are routed, and match the athlete — INCLUDING the T088 cardio fixes (StairMill citations, Air-Bike watts removal, Swim 2-point CSS, Pace Critical Speed all present in the coach mirrors). Both audits' 'critical' alarms were FALSE on verify-first inspection: 'Pace-CS-missing-on-coach' was an agent miss (it's at AdminCardioPaceDetail L275); 'FamilyConsolidatedDetail-missing' was the known-deferred carousel. Fixed 1 stale Air-Bike header doc-comment. THEN built the last gap — the FamilyConsolidated COACH carousel: new web/src/pages/admin/detail/AdminStrengthFamilyDetail.jsx (click variant pills + the selected child's AdminStrengthLeverageDetail with a new hideHeader prop) + AdminEffortDetail dispatch (a parent_movement_id parent with &gt;=2 children -&gt; family detail, child -&gt; per-variant) + AdminUserActivity catalog-driven family list-collapse (verified safe vs Sled/Swim, which also carry parent_movement_id: Sled branch runs first, Swimming is cardio-only). Web deployed (e226dc6f). List-collapsing now complete (BW tiers + Sled + Swim + admin families). Cosmetic 'drifts' (web click-toggle vs swipe pills, static numbers vs TickerNumber) are INTENTIONAL per the 'web stays simple' rule. REMAINING (deferred, now un-blocked): coaching ADD-ONS (recency, stalled flag, frequency, PR timeline, balance, adherence). Non-effort coach tabs (Sleep/Hydration/Heart/Bodyweight/Calories) parity = separate, tracked under T079 Phase 2. ADD-ONS PHASE (2026-06-06): redesigned the Efforts tab from rows to MOVE CARDS (alphabetical, whole card clickable to the detail), each with a mini progress sparkline + PR/best + recency -- this delivers 2 of the 6 planned add-ons (most-ever-effort/PR + recency). For collapsed multi-variant moves the card plots the HIGHEST-effort variant + a badge (BW = highest tier, Sled/Swim/admin-family = best-metric variant). Per-card graph metric matches each move's detail page (1RM/hold-secs/reps/assistance/pace/cal-min/floors/distance), Y reversed where lower-is-better so the line always reads up=better; &lt;2 points -&gt; single dot / 'Not enough data yet'. AdminUserActivity full rewrite (rows -&gt; responsive grid of cards), web deployed e76b7319. QA flags: bodyweight cards graph REPS (matches the BW detail page, NOT 1RM); carry cards graph WEIGHT not distance. REMAINING add-ons (4): stalled flag, frequency, balance, adherence (adherence still parked -- no coach-prescribed plan stored yet).</t>
+          <t>STRUCTURE DECIDED 2026-06-04: keep ONE combined Efforts tab with an internal Strength|Cardio segmented toggle (dropped 'All', default Strength). LIST-VIEW read-only mirror DONE + deployed 2026-06-04 — removed the Add-effort form + backdate + button; AdminUserActivity is now read-only (207-&gt;193 lines). USER 2026-06-04: FINISH THE MIRROR BEFORE ADD-ONS. MAIN REMAINING = (1) DETAIL-SCREEN rebuild to mirror the athlete coaching surfaces, incremental: Strength Weighted Standard FIRST (validate with user), then other strength variants (bodyweight/assisted/carry/iso/sled), then cardio surfaces (pace/airbike/swim/ruck/stairmill/ergs/duration); (2) LIST variant-collapsing (bodyweight tiers / swim strokes / sled push-drag -&gt; one row+badge like the athlete; coupled to the detail routes). DEFERRED until mirror complete: coaching add-ons (recency, stalled flag, frequency, PR timeline, balance, adherence). Detail rebuild notes: admin detail routes (AdminEffortDetail = bare 10-tile grid; AdminCardioDetail = old pace model w/ banned 'lower=faster') don't mirror the athlete coaching surfaces; KEEP the per-effort swipe-delete there. USER CORRECTION 2026-06-04: the coach is NOT fully read-only — they CAN delete efforts; only the athlete-style ADD/log form is excluded (that's the separate coach-input track). List view stays add-free; individual-effort delete lives in the detail screens. PROGRESS 2026-06-04: Strength Weighted Standard detail mirror DONE + deployed (new web/src/pages/admin/detail/AdminStrengthWeightedDetail.jsx, dispatched from AdminEffortDetail for barbell/dumbbell/kettlebell/machine/strongman; read-only + delete kept; rep-max projections + adp-zone pills + 20 tiles + next-target hero + chart + log). AWAITING user validation of this first variant before rolling out remaining strength variants (bodyweight/assisted/carry/iso/sled) + all cardio surfaces + list variant-collapsing. UPDATE 2026-06-06 — MIRROR COMPLETE. Ran a 2-agent parity cross-check (strength + cardio): ALL strength variant coach mirrors (weighted/bodyweight/assisted/carry/leverage/load/iso/Olympic/ballistic/repsonly) + ALL cardio mirrors (pace/ergs/swim/airbike/ruck/stairmill/beat-your-best) exist, are routed, and match the athlete — INCLUDING the T088 cardio fixes (StairMill citations, Air-Bike watts removal, Swim 2-point CSS, Pace Critical Speed all present in the coach mirrors). Both audits' 'critical' alarms were FALSE on verify-first inspection: 'Pace-CS-missing-on-coach' was an agent miss (it's at AdminCardioPaceDetail L275); 'FamilyConsolidatedDetail-missing' was the known-deferred carousel. Fixed 1 stale Air-Bike header doc-comment. THEN built the last gap — the FamilyConsolidated COACH carousel: new web/src/pages/admin/detail/AdminStrengthFamilyDetail.jsx (click variant pills + the selected child's AdminStrengthLeverageDetail with a new hideHeader prop) + AdminEffortDetail dispatch (a parent_movement_id parent with &gt;=2 children -&gt; family detail, child -&gt; per-variant) + AdminUserActivity catalog-driven family list-collapse (verified safe vs Sled/Swim, which also carry parent_movement_id: Sled branch runs first, Swimming is cardio-only). Web deployed (e226dc6f). List-collapsing now complete (BW tiers + Sled + Swim + admin families). Cosmetic 'drifts' (web click-toggle vs swipe pills, static numbers vs TickerNumber) are INTENTIONAL per the 'web stays simple' rule. REMAINING (deferred, now un-blocked): coaching ADD-ONS (recency, stalled flag, frequency, PR timeline, balance, adherence). Non-effort coach tabs (Sleep/Hydration/Heart/Bodyweight/Calories) parity = separate, tracked under T079 Phase 2. ADD-ONS PHASE (2026-06-06): redesigned the Efforts tab from rows to MOVE CARDS (alphabetical, whole card clickable to the detail), each with a mini progress sparkline + PR/best + recency -- this delivers 2 of the 6 planned add-ons (most-ever-effort/PR + recency). For collapsed multi-variant moves the card plots the HIGHEST-effort variant + a badge (BW = highest tier, Sled/Swim/admin-family = best-metric variant). Per-card graph metric matches each move's detail page (1RM/hold-secs/reps/assistance/pace/cal-min/floors/distance), Y reversed where lower-is-better so the line always reads up=better; &lt;2 points -&gt; single dot / 'Not enough data yet'. AdminUserActivity full rewrite (rows -&gt; responsive grid of cards), web deployed e76b7319. QA flags: bodyweight cards graph REPS (matches the BW detail page, NOT 1RM); carry cards graph WEIGHT not distance. REMAINING add-ons (4): stalled flag, frequency, balance, adherence (adherence still parked -- no coach-prescribed plan stored yet). FINAL 2026-06-06: user said 'no need for the rest' so the 4 remaining add-ons (stalled flag / frequency / balance / adherence) are DESCOPED; added a ChevronRight click-affordance to each card (deployed b24beb71). T080 DONE -- coach Efforts parity = list mirror + family carousel + move-cards (graph + PR + recency) + click affordance, all shipped + deployed.</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): capture session work - T091 chart false-drops, T092 mini-graph, T093 coach-units
Capture-first/ledger discipline was missed this session; setting it straight per
CLAUDE.md rules (lines 67-69).
- T091 (Done): chart false-drop crosscheck + normalization (bodyweight Est-1RM,
  carry/ruck Total work, pace Riegel, load-hold, band-tier, yard pace), mobile + coach web.
- T092 (Deferred): coach Efforts-tab cardio mini-graph sparklines still plot raw pace.
- T093 (In progress): coach-units pass - Bodyweight done; direction needs user confirm.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4848,6 +4848,147 @@
       <c r="I93" s="5" t="inlineStr">
         <is>
           <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>T091</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Chart false-drop crosscheck + distance/duration normalization</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Strength+Cardio</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Mobile + Web coach</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>User (issue D) flagged the Pull-Up chart showed a false DROP -- a high-rep bodyweight set then a loaded single (label 'Pull Up . 162.9+27.5 lb x 5') read as a regression because the chart plotted raw reps. Asked to fix AND 'crosscheck ALL graphs' for the same false-drop with correct terminology. Decisions: carry/ruck 'keep one line, rename Total work'; pace/rate 'normalize across distances'. ALL FIXES SHIPPED (mobile reloaded + web deployed): (1) Bodyweight detail chart plots Est. 1RM when the ACTIVE tier has loaded efforts, else reps -- per-active-tier so band/knee tiers never get an inflated bodyweight 1RM (mobile [exercise].tsx + web AdminStrengthBodyweightDetail). The reported 'still broken after reload' was NOT Metro caching -- it was a temporal-dead-zone bug: bwHasWeighted referenced bwActiveTier ~170 lines before its const declaration, so the per-tier check was silently always-false; fixed by moving the block below bwActiveTier (f03b01b). (2) Carry/Rucking dual weight+distance charts were consolidated to one 'Total work' = weight x distance line under T080. (3) Pace charts Riegel-normalized across distances to a per-activity anchor (run/treadmill/cycle/elliptical 5km, Row/Bike/Ski ergs 2km, swim 1000m-equiv per-100m): mobile PaceDetail + BeatYourBestDetail + SwimmingDetail and web AdminCardioPaceDetail + AdminCardioBeatYourBestDetail + AdminCardioSwimmingDetail. Dashed line = best normalized; header + record lists keep the raw logged pace; captioned. (4) Load-hold (weighted plank/hang) plots EQUIVALENT weight at a 30s hold via the Rohmert curve, not raw load. (5) Band tiers (assisted pull-up/dip) plot a band-adjusted difficulty score (bandRank x 8 + reps), not raw reps. (6) Yard swimmers: per-100 pace display converts per-100m -&gt; per-100yd (x0.9144) to match the /100yd label; coaching math stays per-100m. Documented in CLAUDE.md ('Chart distance/duration normalization rule', LOCKED June 6 2026).</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>Coach Efforts-tab cardio mini-graph sparklines still plot raw pace -&gt; own follow-up T092.</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>mobile [exercise].tsx, [activity].tsx, cardio.tsx; web admin/detail/AdminStrengthBodyweightDetail + AdminCardio{Pace,BeatYourBest,Swimming}Detail; CLAUDE.md; commits 05d21c2 / f03b01b / cbb9ce6 / 4ab892e; web hash index-ONd0qB5j</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>T092</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Coach Efforts-tab cardio mini-graph sparklines -- Riegel-normalize</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Web coach</t>
+        </is>
+      </c>
+      <c r="E95" s="10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Follow-up flagged during T091. The coach Efforts-tab move-card mini-graph sparklines (AdminUserActivity.jsx, the cardio + swim builders ~L802-863) still plot RAW pace per point (parseCardioBest(value), no distance), so a longer cardio effort dips the sparkline -- the same false-drop T091 fixed on the detail charts. The DETAIL charts (primary surface) are done on mobile + coach web; these tiny axisless sparklines were deferred (the hover popup still shows the real logged value).</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>Normalize the cardio pace sparkline points: needs per-point label parsing for distance + per-stroke swim handling (mirror the detail-chart Riegel fix). Apply only to pace activities; leave cal/min + floors/min (rates) alone.</t>
+        </is>
+      </c>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/tabs/AdminUserActivity.jsx (cardio mini-graph builder ~L802-863)</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>T093</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Coach-units pass -- coach sees client data in the coach's units</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Web coach</t>
+        </is>
+      </c>
+      <c r="E96" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Earlier this session the user set a units model (never captured -- capture-first miss): the coach/admin views a client's values in the COACH's units (not the client's), add-form unit toggles default to the coach's units, and a mixed-unit rule -- record LISTS keep each effort's own logged unit while GRAPHS + headline numbers convert to the viewer (coach) unit; by-design locks still win (strongman kg, rucking mi, Concept2 ergs metric). Decision noted: 'option 2 -- do it all in one pass'. CONFLICT TO RESOLVE: T079's note says the coach Bodyweight tab was intentionally built in the CLIENT's units; this pass reverses that. DONE so far: coach Bodyweight tab flipped to coach units -- chart + Current/BMI/Ideal/Trend stats + Add-weigh-in default now read the logged-in coach's weight_unit via useAuth, while the weigh-in LIST keeps each entry's logged unit (committed ae4fe28, deployed, live).</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>BLOCKER -- confirm direction with the user: keep+extend coach-units, or revert Bodyweight to client-units. If coach-units stands, remaining surfaces: the cardio + strength coach DETAIL pages (they currently self-fetch + show the CLIENT's distance/weight unit -- verified AdminCardioPaceDetail L634) need the coach's unit for graphs/headline + logged unit for record lists; plus any unit displays on the Calories / Sleep / Hydration coach tabs. Efforts (T080) is already done; Heart is bpm (no unit).</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>web AdminUserBody.jsx (done, ae4fe28); pending: web admin/detail/AdminCardio*Detail + AdminStrength*Detail, AdminUserDetail.jsx, Calories/Sleep/Hydration coach tabs</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(ledger): T093 progress - Bodyweight + cardio detail done (coach units everywhere); strength detail + tabs remaining
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4973,17 +4973,17 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Earlier this session the user set a units model (never captured -- capture-first miss): the coach/admin views a client's values in the COACH's units (not the client's), add-form unit toggles default to the coach's units, and a mixed-unit rule -- record LISTS keep each effort's own logged unit while GRAPHS + headline numbers convert to the viewer (coach) unit; by-design locks still win (strongman kg, rucking mi, Concept2 ergs metric). Decision noted: 'option 2 -- do it all in one pass'. CONFLICT TO RESOLVE: T079's note says the coach Bodyweight tab was intentionally built in the CLIENT's units; this pass reverses that. DONE so far: coach Bodyweight tab flipped to coach units -- chart + Current/BMI/Ideal/Trend stats + Add-weigh-in default now read the logged-in coach's weight_unit via useAuth, while the weigh-in LIST keeps each entry's logged unit (committed ae4fe28, deployed, live).</t>
+          <t>User set a units model (capture-first miss, now captured): the coach views a client's values in the COACH's units. LIST DECISION 2026-06-06 (user, via AskUserQuestion): EVERYTHING the coach sees is in coach units -- record LISTS convert too, NOT the athlete-side mixed-unit 'lists keep logged unit' rule. By-design locks always win (strongman kg, rucking mi, Concept2 ergs metric). Supersedes T079's note that the coach Bodyweight tab was built in CLIENT units. DONE: (a) coach Bodyweight tab -- chart + Current/BMI/Ideal/Trend stats + Add-weigh-in default + the weigh-in LIST all in the coach's weight_unit via useAuth (ae4fe28 + 276181b). (b) Cardio coach DETAIL pages Pace/BeatYourBest/Swimming -- display unit derived from the coach's distance_unit/swim_unit via useAuth (was self-fetching the client's); ergs metric + rucking mi via their locked branches; AirBike/StairMill have no distance unit (cal/min, floors/min) so unchanged. Deployed live (index-CSE_g1K8).</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION CONFIRMED 2026-06-06 (user: 'coach sees client data in the coach's units, this stands') -- Bodyweight change KEPT; supersedes T079's earlier client-units note. ACTIVE remaining surfaces: (1) cardio coach DETAIL pages AdminCardioPaceDetail/BeatYourBest/Swimming/AirBike/Rucking/StairMill -- they self-fetch the CLIENT's distance_unit (e.g. AdminCardioPaceDetail L634) -&gt; switch graphs+headline to the COACH's unit (useAuth), record LISTS to each effort's own logged unit; (2) strength coach DETAIL pages AdminStrength*Detail -&gt; weights in coach unit, lists logged; (3) Calories/Sleep/Hydration coach tabs unit displays (Hydration fluid oz/mL; Sleep is hours -&gt; no convert; Calories kcal+g, check any plan weight). By-design locks ALWAYS win: strongman kg, rucking mi, Concept2 ergs metric. Efforts (T080) done; Heart bpm (no unit).</t>
+          <t>REMAINING: (1) strength coach DETAIL pages -- AdminStrengthWeighted/RepsOnly/Assisted/Bodyweight/Carry/Load each self-fetch the CLIENT's weight_unit (-&gt; setProfileUnit); switch the DISPLAY unit to the coach's weight_unit via useAuth, KEEP the strongman kg unitLock (Carry), and KEEP the client's current_weight as the e1RM/effective-load MATH input (only the display unit changes). AdminStrengthLeverage (time-only) + Family (wrapper) need no change. (2) Calories + Hydration coach tabs -- Hydration fluid oz/mL -&gt; coach fluid_unit; Calories kcal+g no-convert but check any plan bodyweight display; Sleep is hours -&gt; no convert. Then flip T093 to Done.</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
         <is>
-          <t>web AdminUserBody.jsx (done, ae4fe28); pending: web admin/detail/AdminCardio*Detail + AdminStrength*Detail, AdminUserDetail.jsx, Calories/Sleep/Hydration coach tabs</t>
+          <t>DONE: web AdminUserBody.jsx + AdminCardio{Pace,BeatYourBest,Swimming}Detail.jsx (ae4fe28, 276181b, live index-CSE_g1K8). PENDING: web admin/detail/AdminStrength{Weighted,RepsOnly,Assisted,Bodyweight,Carry,Load}Detail.jsx; Calories + Hydration coach tabs</t>
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): T093 DONE - coach-units pass complete across all coach surfaces
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4966,9 +4966,9 @@
           <t>Web coach</t>
         </is>
       </c>
-      <c r="E96" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
@@ -4978,12 +4978,12 @@
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>REMAINING (strength detail = MORE than a source-swap: display unit was `unitLock || best.unit || profileUnit`, 1RM+projections compute IN that unit). TEMPLATE DONE 2026-06-06 -- AdminStrengthWeightedDetail (07d6fa2, deployed): added convW(w,from,to) + convDetail(str,to,locked) helpers, precedence = unitLock || coachUnit (strongman kg lock wins), converted best 1RM + chart points + hero/tiles (via the converted 1RM) + efforts list (1RM value + raw detail string), removed the client weight_unit fetch (useAuth); display-only, projection math untouched. STILL TO DO with that template: (a) RepsOnly + Load (simpler); (b) Assisted, Bodyweight, Carry (MATH-HEAVY -- KEEP the client's current_weight as the e1RM/effective-load math input, convert DISPLAY only; Carry also keeps strongman kg unitLock + converts distance ft/m). AdminStrengthLeverage (time-only) + Family (wrapper) = no change. (2) Calories + Hydration coach tabs -- Hydration -&gt; coach fluid_unit; Calories kcal+g (check plan weight); Sleep hours/no-convert. Then flip T093 Done.</t>
+          <t>DONE 2026-06-06 -- every coach surface now shows a client's data in the COACH's units: Bodyweight tab; cardio detail (Pace/BeatYourBest/Swimming; ergs stay metric + rucking stays mi via their locks; AirBike/StairMill are unitless); ALL strength detail (Weighted/RepsOnly/Load/Assisted/Bodyweight/Carry -- display-only conversion via convW/convDetail, strongman kg unitLock kept, and the 1RM / effective-load / e1RM math inputs + Carry ratio math + Rohmert load math ALL untouched); Hydration (coach fluid_unit). Calories (kcal+g) + Sleep (hours) have no convertible units -&gt; no change. RepsOnly is reps-only -&gt; no weights. Efforts (T080) + Heart (bpm) were already done. Each chunk deployed + live-hash-verified. NONE remaining.</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
         <is>
-          <t>DONE: web AdminUserBody.jsx + AdminCardio{Pace,BeatYourBest,Swimming}Detail.jsx (ae4fe28, 276181b, live index-CSE_g1K8). PENDING: web admin/detail/AdminStrength{Weighted,RepsOnly,Assisted,Bodyweight,Carry,Load}Detail.jsx; Calories + Hydration coach tabs</t>
+          <t>web AdminUserBody.jsx + AdminUserHydration.jsx + AdminCardio{Pace,BeatYourBest,Swimming}Detail.jsx + admin/detail/AdminStrength{Weighted,RepsOnly,Load,Assisted,Bodyweight,Carry}Detail.jsx. Commits ae4fe28 / 276181b / 07d6fa2 / b54a2e4 / dcf763a (+ web deploys)</t>
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): T092 DONE - coach Efforts-tab cardio sparklines Riegel-normalized
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4919,9 +4919,9 @@
           <t>Web coach</t>
         </is>
       </c>
-      <c r="E95" s="10" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Normalize the cardio pace sparkline points: needs per-point label parsing for distance + per-stroke swim handling (mirror the detail-chart Riegel fix). Apply only to pace activities; leave cal/min + floors/min (rates) alone.</t>
+          <t>DONE 2026-06-06 (6bb3d4c, deployed). Added riegelNormPaceSecPerKm(label) to AdminUserActivity (parses distance+time, projects to a 5km anchor; returns null for cal/min + floors so those keep their raw rate). The generic-cardio + swim move-card builders now plot the NORMALIZED pace for pace points (parseCardioBest lowerBetter=true); the hover popup still shows the raw logged value. A single 5km anchor suffices -- for an axis-less sparkline the anchor only scales values by a constant, so the trend is identical for every pace activity (running/ergs/swim). NONE remaining.</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(coach): T086 - neutralize athlete-instruction empty states in Bodyweight mirror + ledger
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4320,7 +4320,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy.</t>
+          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass.</t>
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>REMOVE (always-visible athlete prose): attribution footers, motivational/encouragement lines, eligibility/instruction notes, feature help-text subtitles. KEEP: data (charts/logs/best/PR/current), prescription numbers + the cue line, headers/badges/tiles, and the opt-in 'why this zone' info pills (collapsed, not clutter — flag if user wants those gone too). Surfaces: tabs AdminUser{Sleep,Hydration,Heart}; detail AdminStrength* + AdminCardio*. Hydration done as exemplar, then agent-sweep the rest in batches of 3; build/deploy. DONE 2026-06-04: Hydration (me) + Batch 1 (Sleep/Heart/Weighted-strength) + a background Workflow over the remaining 11 detail surfaces (5 strength + 6 cardio) in chunks of 3. Removed: attribution/citation footers, feature help-text subtitles ('Pick an adaptation zone...', 'Pick a training focus...'), tier-criteria methodology subtitles, motivational/eligibility prose; neutralized athlete-instruction empty states ('Log your first...' -&gt; 'No X logged yet') + removed PartyPopper/emoji decoration. KEPT: all data (charts/tiles/logs/PRs/hero numbers), the prescription cue lines, section titles, badges, and the opt-in 'why this zone' info pills. User confirmed keeping the info pills. All eslint+esbuild clean (agents self-verified); web build clean; deployed. Coach mirrors now intentionally diverge from mobile on these prose blocks (mobile athlete pages keep them).</t>
+          <t>REMOVE (always-visible athlete prose): attribution footers, motivational/encouragement lines, eligibility/instruction notes, feature help-text subtitles. KEEP: data (charts/logs/best/PR/current), prescription numbers + the cue line, headers/badges/tiles, and the opt-in 'why this zone' info pills (collapsed, not clutter — flag if user wants those gone too). Surfaces: tabs AdminUser{Sleep,Hydration,Heart}; detail AdminStrength* + AdminCardio*. Hydration done as exemplar, then agent-sweep the rest in batches of 3; build/deploy. DONE 2026-06-04: Hydration (me) + Batch 1 (Sleep/Heart/Weighted-strength) + a background Workflow over the remaining 11 detail surfaces (5 strength + 6 cardio) in chunks of 3. Removed: attribution/citation footers, feature help-text subtitles ('Pick an adaptation zone...', 'Pick a training focus...'), tier-criteria methodology subtitles, motivational/eligibility prose; neutralized athlete-instruction empty states ('Log your first...' -&gt; 'No X logged yet') + removed PartyPopper/emoji decoration. KEPT: all data (charts/tiles/logs/PRs/hero numbers), the prescription cue lines, section titles, badges, and the opt-in 'why this zone' info pills. User confirmed keeping the info pills. All eslint+esbuild clean (agents self-verified); web build clean; deployed. Coach mirrors now intentionally diverge from mobile on these prose blocks (mobile athlete pages keep them). PROMOTED TO CLAUDE.md 2026-06-06: this rule was ledger-only, which caused the new CalorieDashboard (T079) to be built WITHOUT applying it (user caught it in audit). Now a permanent locked subsection in CLAUDE.md ('Coach/admin DATA mirror = data + prescription, strip athlete-education') right after the Admin&lt;-&gt;Coach mirror rule -- explicitly covers the calorie dashboard + 'anything added later, applied at build time'. Also extended the sweep: CalorieDashboard stripped + AdminUserBody empty-states neutralized (both built after the original 06-04 sweep). Remaining to sweep: AdminUserActivity (Efforts).</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(db): T094 - water_logs RLS admin/coach read access (Hydration tab showed no data)
water_logs only had owner (user_id = auth.uid()) policies, so the coach/admin
Hydration tab was RLS-filtered to zero rows even when the client had logged
water. Mirror food_logs: add "Admin full access on water_logs" (is_admin) +
"Coaches see roster water_logs". Applied to the DB + tracked migration file.
CLAUDE.md admin-RLS note updated (+ flagged sleep_sessions still needs the
coach roster policy before the coach-portal Sleep reflection).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4987,6 +4987,53 @@
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>T094</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>Fix: coach/admin Hydration tab shows no data (water_logs RLS missing admin/coach policy)</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>DB (Supabase RLS)</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-06 (QA, test account motaz.jarrah / client 9533ef89): the coach Hydration tab showed NO data although water_logs HAS 4 rows for that user. Verify-first via SQL confirmed the data exists; root cause = water_logs RLS had ONLY owner policies (SELECT user_id=auth.uid()), NO 'Admin full access' (is_admin()) and NO 'Coaches see roster' policy -- so the admin/coach read was RLS-filtered to zero rows. Exactly the slow-leak bug CLAUDE.md's admin-RLS rule warns about: the May-26 migration added the policy to food_logs/hr_samples/step_samples/wearable_workouts but MISSED water_logs. (sleep_sessions has an older 'Superusers select all' SELECT policy so admin Sleep works, but it still LACKS the coach roster policy.)</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>FIXED 2026-06-06: applied migration water_logs_admin_coach_rls (saved to supabase/migrations/20260606_water_logs_admin_coach_rls.sql) -- added 'Admin full access on water_logs' (FOR ALL, is_admin()) + 'Coaches see roster water_logs' (FOR SELECT, user_id IN roster), mirroring food_logs. Verified both policies present via pg_policies. Server-side only -- no frontend redeploy; the admin Hydration tab loads the client's water_logs on refresh. CLAUDE.md admin-RLS note updated (water_logs fixed + flagged that sleep_sessions still needs the coach roster policy before the coach-portal Sleep reflection).</t>
+        </is>
+      </c>
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260606_water_logs_admin_coach_rls.sql; water_logs RLS policies; CLAUDE.md admin-RLS note</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
         <is>
           <t>2026-06-06</t>
         </is>

</xml_diff>

<commit_message>
docs(ledger): T095 coach-RLS-audit prerequisite (all pages) + T096 billing epic; CLAUDE.md RLS note strengthened
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5034,6 +5034,100 @@
         </is>
       </c>
       <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>T095</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>PREREQUISITE for coach-portal reflection: 'Coaches see roster' RLS on EVERY per-user table</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>DB (Supabase RLS)</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Surfaced by T094 (the water_logs Hydration empty-data bug). Before we build/reflect ANY coach client-data view (CoachClientDetail + its tabs), EVERY per-user table that view reads MUST have BOTH the 'Admin full access' (is_admin()) AND 'Coaches see roster' (user_id IN (SELECT id FROM profiles WHERE coach_id=auth.uid())) RLS policies -- otherwise the coach view SILENTLY shows EMPTY data (RLS-filtered to zero rows), no error. THIS IS REQUIRED FOR ALL PAGES, not one. Known status: efforts / bodyweight / food_logs / hr_samples / step_samples / wearable_workouts = both policies present; water_logs = FIXED (T094); sleep_sessions = admin works via an older 'Superusers select all' SELECT policy BUT LACKS the coach roster policy; calorie_plans / rom_records / profiles / any others the coach reads = NOT YET AUDITED.</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>OPEN -- deferred until the coach-portal reflection (admin view finishes first per the admin-first strategy). When tackling coach-side: enumerate every table CoachClientDetail + tabs query, check pg_policies, add the missing admin + coach-roster policies in one migration mirroring food_logs. Tracked here + flagged in CLAUDE.md (admin-RLS 'Going forward' note) so ANY session doing coach work sees it.</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>supabase/migrations/ (new); CLAUDE.md admin-RLS note; CoachClientDetail.jsx + coach tabs</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>T096</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>Billing page -- revise prices (individual + coach), wire Stripe (sandbox), define how it all works</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Web + Stripe + Supabase</t>
+        </is>
+      </c>
+      <c r="E99" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-06 kicked off the billing build -- a big multi-decision effort, driven one question at a time (complex-rebuild rule). Three headline asks: (1) revise the current set prices for BOTH the individual (B2C) and coach tiers; (2) get them applied correctly on Stripe + ready, kept in SANDBOX/test mode for now; (3) define + reflect on the billing page how it all works end-to-end. Sub-decisions to capture as made: per-tier price points (individual monthly / annual / lifetime; coach monthly / annual), free-tier limits, trial length, annual-discount framing (CLAUDE.md current: coach annual = 17% off FIRST YEAR only, renews full from yr2), Stripe product/price setup, billing-page UI (BillingView + Pricing/CoachPricing pages).</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page).</t>
+        </is>
+      </c>
+      <c r="H99" s="7" t="inlineStr">
+        <is>
+          <t>web Pricing.jsx / CoachPricing.jsx / CoachPricing.jsx / BillingView / AccountSettings billing; workers (stripe); supabase edge fns + coach_subscriptions/billing_events; CLAUDE.md revenue model + launch Stripe steps</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
         <is>
           <t>2026-06-06</t>
         </is>

</xml_diff>

<commit_message>
docs(ledger): T096 final tier lock + T097 clean-sweep task (purge semirx + contradicting tier defs)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page). DECISION 1 (2026-06-06, user): approach = PROPOSE PREMIUM. ** MODEL CHANGE: individuals move from one-time lifetime to MONTHLY SUBSCRIPTION for ALL ** (no more one-time / 'own it forever'; both coaches AND individuals are recurring subs now). Individual tier strategy: price so FullRX is a NO-BRAINER -- tight CoreRX-&gt;FullRX gap, accessible-premium, everyone should obviously pick FullRX. Implications to handle: Stripe individual prices become RECURRING not one-time; the b2c_purchases one-time schema needs a subscription path (or fold individuals into a subscriptions table); drop all 'lifetime / own it forever' copy; in-app individual subs incur the Apple/Google cut while web-via-Stripe stays clean (same price both surfaces per existing plan). Baseline from research: coach $19/$39/$99 monthly (Starter/Pro/Elite; 10/25/unltd clients; 14-day trial; annual = 17% off yr1 only); individual $0/$39/$59 one-time. Coach checkout works in TEST mode (coach-signup edge fn + hosted Checkout, lookup_key coach_{tier}_{interval}); individual checkout NOT built; webhook duplicated (Supabase stripe-webhook canonical, Cloudflare worker superseded -&gt; retire); stale tier names (DB 'unlimited'/'semirx' vs code 'elite'/'corerx'); prices duplicated across coachPlan.js + coach/Signup.jsx + legal pages + Stripe. PRICING RESEARCH 2026-06-06 (user asked: is $2.99/$4.99 individual monthly bad for a brand-new no-trust app? + confirmed 14-day trial): ran 3 parallel web-research agents. VERDICT -- $2.99/$4.99 is the WRONG move for a premium coaching app: (1) price-quality signaling is STRONGEST for premium/AI products, so too-cheap reads as low-quality ('what's wrong with it'); (2) higher-priced fitness apps convert installs-&gt;paid ~2.7% vs ~1.5% for cheap ones -- low price does NOT buy conversion, it filters OUT committed users; (3) cheap monthly attracts churners + fitness already has the worst churn of any category (40-60% quit by Feb); (4) anchoring low -&gt; later price raises cause 10-15% churn spikes or a permanent grandfathered cohort. BENCHMARKS: pure loggers (Strong/Hevy) $3-5/mo = commodity; COACHING apps (Fitbod $15.99, Freeletics, Ladder, Centr) $15-30/mo; credible AI-coaching sweet spot ~$12.99-14.99/mo, ~$80/yr. TRIAL: 14-day is in the top-converting band (~44% trial-&gt;paid); free-trial / onboarding-paywall converts ~5x better than free-forever (~10.7% vs ~2.1% install-&gt;paid, ~8x revenue/install); 80%+ convert on Day 0 (onboarding-&gt;paywall matters most); native iOS/Android IAP trials are opt-out (card on file =&gt; ~48% conversion automatically), web/Stripe should lean no-card to maximize trial starts; a thin free tier belongs only as the soft-paywall SKIP fallback, not the front door. RECOMMENDATION: CoreRX $12.99 / FullRX $14.99 monthly (keep the $2 no-brainer gap; reads as real coaching just under Fitbod), annual ~$80/yr (separate decision), KEEP the 14-day trial, and solve the new-brand trust deficit with the trial + reviews/social-proof + a TIME-BOXED launch/founder promo (e.g. 50% off first 3 months) so a low entry number never becomes the permanent anchor. Sources: RevenueCat + Adapty subscription benchmarks, Airbridge 2026 pricing-by-category, SaaStr Day-1 pricing. POSITIONING REFINED 2026-06-06 (user): the app is honestly 'a logger WITH a coaching-cue edge', NOT a full Fitbod-style coach -- do NOT oversell (avoid being labelled a liar) but DO assume some premiumness =&gt; price 'a notch above other loggers' (loggers ~$4-5/mo, so individual top tier in the ~$7-9/mo band, NOT the $14.99 coaching tier). Annual = 17% off (= '2 months free') as an OPTION. Proposed: CoreRX $5.99 / FullRX $7.99 monthly (a clear notch above the $4.99 logger ceiling, $2 no-brainer gap), annual ~$59.99 / ~$79.99 (2 months free). OPEN sub-decision: is the INDIVIDUAL annual discount recurring or first-year-only? (coach annual is currently first-year-only per CLAUDE.md) -- align when we do the coach prices. INDIVIDUAL PRICING LOCKED 2026-06-06: monthly subscription + 14-day trial; Free $0 / CoreRX $4.99/mo / FullRX $6.99/mo; annual = 17% off (2 months free) =&gt; CoreRX ~$49.99/yr, FullRX ~$69.99/yr (user chose the most-accessible 'notch above loggers' option). NEXT decisions: coach prices (current $19/$39/$99 monthly, 10/25/unltd clients) + align the annual-discount model (coach annual is currently 17%-off-FIRST-YEAR-ONLY per CLAUDE.md, individual annual is 17% recurring -- decide whether to unify) + free-tier feature split + then Stripe sandbox setup + billing-page build. COACH PRICES LOCKED 2026-06-06: keep Starter $19 / Pro $39 / Elite $99 monthly, caps 10/25/unltd clients, 14-day trial (already competitive vs TrueCoach/Trainerize; don't scare early coaches). PENDING: annual-discount model -- unify to RECURRING 17% (2 months free) for BOTH coaches + individuals, or keep coach annual as 17%-off-first-year-only? RESOLVED: RECURRING 17% (2 months free) for BOTH. Coach annual is NO LONGER first-year-only -&gt; permanent 17% off, renews at the same discounted annual (no year-2 jump): coach annual ~$189/$389/$989 RECURRING; individual ~$49.99/$69.99 recurring. IMPL TO-DO: REVERSE the CLAUDE.md 'coach annual 17% off first year only, renews full' lock to recurring; strip the year-2 renewal figures ($228/$468/$1188) + every 'first year' disclaimer from CoachAgreement / RefundPolicy / CoachPricing / coach Signup; set Stripe annual prices to the flat recurring annual. === FULL PRICING LOCKED 2026-06-06: monthly-subscription model for ALL (no one-time/lifetime); 14-day trial both. Individual: Free $0 / CoreRX $4.99 / FullRX $6.99 monthly (annual 17% recurring ~$49.99 / ~$69.99). Coach: Starter $19 / Pro $39 / Elite $99 monthly, 10/25/unltd clients (annual 17% recurring ~$189 / ~$389 / ~$989). REMAINING: free-tier feature split (code currently inconsistent) -&gt; then Stripe sandbox products/prices -&gt; propagate prices everywhere + model-change cleanup (drop lifetime copy, retire CF webhook, fix stale tier names elite/corerx, build individual checkout) -&gt; billing page. TIER FEATURE SPLIT (from CLAUDE.md lines 2384-2393, AUTHORITATIVE -- my earlier improvised split was wrong; Mobility was removed in the June 2026 teardown so it's NOT a tier feature): Free = Strength + Cardio; CoreRX = Free + Bodyweight + Calories (body-composition + calorie/macro coaching, the two most-requested); FullRX = CoreRX + Heart + Hydration + Sleep (the wellness/recovery layer, appeals to wearable owners). The cross-domain Dashboard rollup sits in FullRX (complete picture). The feature split is UNCHANGED by the one-time-&gt;subscription move; only the model + prices change. CODE INCONSISTENCY TO FIX: the in-app gating (CoachClientDetail TIER_RANK) wrongly puts Heart in CoreRX -- must move to FullRX to match CLAUDE.md.</t>
+          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page). DECISION 1 (2026-06-06, user): approach = PROPOSE PREMIUM. ** MODEL CHANGE: individuals move from one-time lifetime to MONTHLY SUBSCRIPTION for ALL ** (no more one-time / 'own it forever'; both coaches AND individuals are recurring subs now). Individual tier strategy: price so FullRX is a NO-BRAINER -- tight CoreRX-&gt;FullRX gap, accessible-premium, everyone should obviously pick FullRX. Implications to handle: Stripe individual prices become RECURRING not one-time; the b2c_purchases one-time schema needs a subscription path (or fold individuals into a subscriptions table); drop all 'lifetime / own it forever' copy; in-app individual subs incur the Apple/Google cut while web-via-Stripe stays clean (same price both surfaces per existing plan). Baseline from research: coach $19/$39/$99 monthly (Starter/Pro/Elite; 10/25/unltd clients; 14-day trial; annual = 17% off yr1 only); individual $0/$39/$59 one-time. Coach checkout works in TEST mode (coach-signup edge fn + hosted Checkout, lookup_key coach_{tier}_{interval}); individual checkout NOT built; webhook duplicated (Supabase stripe-webhook canonical, Cloudflare worker superseded -&gt; retire); stale tier names (DB 'unlimited'/'semirx' vs code 'elite'/'corerx'); prices duplicated across coachPlan.js + coach/Signup.jsx + legal pages + Stripe. PRICING RESEARCH 2026-06-06 (user asked: is $2.99/$4.99 individual monthly bad for a brand-new no-trust app? + confirmed 14-day trial): ran 3 parallel web-research agents. VERDICT -- $2.99/$4.99 is the WRONG move for a premium coaching app: (1) price-quality signaling is STRONGEST for premium/AI products, so too-cheap reads as low-quality ('what's wrong with it'); (2) higher-priced fitness apps convert installs-&gt;paid ~2.7% vs ~1.5% for cheap ones -- low price does NOT buy conversion, it filters OUT committed users; (3) cheap monthly attracts churners + fitness already has the worst churn of any category (40-60% quit by Feb); (4) anchoring low -&gt; later price raises cause 10-15% churn spikes or a permanent grandfathered cohort. BENCHMARKS: pure loggers (Strong/Hevy) $3-5/mo = commodity; COACHING apps (Fitbod $15.99, Freeletics, Ladder, Centr) $15-30/mo; credible AI-coaching sweet spot ~$12.99-14.99/mo, ~$80/yr. TRIAL: 14-day is in the top-converting band (~44% trial-&gt;paid); free-trial / onboarding-paywall converts ~5x better than free-forever (~10.7% vs ~2.1% install-&gt;paid, ~8x revenue/install); 80%+ convert on Day 0 (onboarding-&gt;paywall matters most); native iOS/Android IAP trials are opt-out (card on file =&gt; ~48% conversion automatically), web/Stripe should lean no-card to maximize trial starts; a thin free tier belongs only as the soft-paywall SKIP fallback, not the front door. RECOMMENDATION: CoreRX $12.99 / FullRX $14.99 monthly (keep the $2 no-brainer gap; reads as real coaching just under Fitbod), annual ~$80/yr (separate decision), KEEP the 14-day trial, and solve the new-brand trust deficit with the trial + reviews/social-proof + a TIME-BOXED launch/founder promo (e.g. 50% off first 3 months) so a low entry number never becomes the permanent anchor. Sources: RevenueCat + Adapty subscription benchmarks, Airbridge 2026 pricing-by-category, SaaStr Day-1 pricing. POSITIONING REFINED 2026-06-06 (user): the app is honestly 'a logger WITH a coaching-cue edge', NOT a full Fitbod-style coach -- do NOT oversell (avoid being labelled a liar) but DO assume some premiumness =&gt; price 'a notch above other loggers' (loggers ~$4-5/mo, so individual top tier in the ~$7-9/mo band, NOT the $14.99 coaching tier). Annual = 17% off (= '2 months free') as an OPTION. Proposed: CoreRX $5.99 / FullRX $7.99 monthly (a clear notch above the $4.99 logger ceiling, $2 no-brainer gap), annual ~$59.99 / ~$79.99 (2 months free). OPEN sub-decision: is the INDIVIDUAL annual discount recurring or first-year-only? (coach annual is currently first-year-only per CLAUDE.md) -- align when we do the coach prices. INDIVIDUAL PRICING LOCKED 2026-06-06: monthly subscription + 14-day trial; Free $0 / CoreRX $4.99/mo / FullRX $6.99/mo; annual = 17% off (2 months free) =&gt; CoreRX ~$49.99/yr, FullRX ~$69.99/yr (user chose the most-accessible 'notch above loggers' option). NEXT decisions: coach prices (current $19/$39/$99 monthly, 10/25/unltd clients) + align the annual-discount model (coach annual is currently 17%-off-FIRST-YEAR-ONLY per CLAUDE.md, individual annual is 17% recurring -- decide whether to unify) + free-tier feature split + then Stripe sandbox setup + billing-page build. COACH PRICES LOCKED 2026-06-06: keep Starter $19 / Pro $39 / Elite $99 monthly, caps 10/25/unltd clients, 14-day trial (already competitive vs TrueCoach/Trainerize; don't scare early coaches). PENDING: annual-discount model -- unify to RECURRING 17% (2 months free) for BOTH coaches + individuals, or keep coach annual as 17%-off-first-year-only? RESOLVED: RECURRING 17% (2 months free) for BOTH. Coach annual is NO LONGER first-year-only -&gt; permanent 17% off, renews at the same discounted annual (no year-2 jump): coach annual ~$189/$389/$989 RECURRING; individual ~$49.99/$69.99 recurring. IMPL TO-DO: REVERSE the CLAUDE.md 'coach annual 17% off first year only, renews full' lock to recurring; strip the year-2 renewal figures ($228/$468/$1188) + every 'first year' disclaimer from CoachAgreement / RefundPolicy / CoachPricing / coach Signup; set Stripe annual prices to the flat recurring annual. === FULL PRICING LOCKED 2026-06-06: monthly-subscription model for ALL (no one-time/lifetime); 14-day trial both. Individual: Free $0 / CoreRX $4.99 / FullRX $6.99 monthly (annual 17% recurring ~$49.99 / ~$69.99). Coach: Starter $19 / Pro $39 / Elite $99 monthly, 10/25/unltd clients (annual 17% recurring ~$189 / ~$389 / ~$989). REMAINING: free-tier feature split (code currently inconsistent) -&gt; then Stripe sandbox products/prices -&gt; propagate prices everywhere + model-change cleanup (drop lifetime copy, retire CF webhook, fix stale tier names elite/corerx, build individual checkout) -&gt; billing page. TIER FEATURE SPLIT (from CLAUDE.md lines 2384-2393, AUTHORITATIVE -- my earlier improvised split was wrong; Mobility was removed in the June 2026 teardown so it's NOT a tier feature): Free = Strength + Cardio; CoreRX = Free + Bodyweight + Calories (body-composition + calorie/macro coaching, the two most-requested); FullRX = CoreRX + Heart + Hydration + Sleep (the wellness/recovery layer, appeals to wearable owners). The cross-domain Dashboard rollup sits in FullRX (complete picture). The feature split is UNCHANGED by the one-time-&gt;subscription move; only the model + prices change. CODE INCONSISTENCY TO FIX: the in-app gating (CoachClientDetail TIER_RANK) wrongly puts Heart in CoreRX -- must move to FullRX to match CLAUDE.md. === ATHLETE TIERS FINALIZED + LOCKED BY USER 2026-06-06 (THIS IS FINAL): Free = Strength+Cardio; CoreRX $4.99/mo ($49.99/yr) = +Bodyweight+Calories/Food; FullRX $6.99/mo ($69.99/yr) = +Heart+Hydration+Sleep+every future feature. COACH: every coach tier grants FULL FullRX access to the coach AND all their linked athletes -- tiers differ ONLY by client cap (Starter $19/10, Pro $39/25, Elite $99/unltd; annual 17% recurring $189/$389/$989). Home Dashboard = the landing/profile screen for EVERYONE, never a tier feature. User demanded a CLEAN SWEEP of all stale/contradicting references (esp. the 'semirx' old name + the 3-way-conflicting tier splits) -&gt; tracked as T097.</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
@@ -5128,6 +5128,53 @@
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>T097</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Clean-sweep ALL docs + code of stale pricing/tier naming to the final lock</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Repo-wide</t>
+        </is>
+      </c>
+      <c r="E100" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-06 (firm: 'this is final, this is it, i dont want any [stale]'): after locking the final tiers, purge every reference that states anything other than the lock. Grep found 'semirx' (the old CoreRX name) in CLAUDE.md + supabase/migrations/20260524_coach_platform_v1_phase1.sql (b2c_purchases.tier CHECK = semirx|fullrx) + scripts/rename-stripe-semirx-to-corerx.mjs (spent one-shot) + this ledger (describes the bug). One-time/lifetime/first-year-only + the 3-way-conflicting tier splits live in: CLAUDE.md (revenue model + launch checklist), web Pricing.jsx (ATHLETE_TIERS wrong split + one-time), coachPlan.js + coach/Signup.jsx + CoachPricing.jsx + ForCoaches.jsx (coach annual 'first year only'), legal CoachAgreement/RefundPolicy/TermsOfService/PrivacyPolicy (prices + one-time + year-2 renewals), docs/marketing/* + branding/BRAND.md, gating CoachClientDetail TIER_RANK (Heart wrongly in CoreRX), billing display BillingView/BillingTab/AccountSettings/EditProfile.</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>IN PROGRESS 2026-06-06: sweep CLAUDE.md first (the contract) -&gt; DB semirx-&gt;corerx CHECK migration -&gt; web display/tier code + legal + marketing. The WORKING coach Stripe plumbing (coach-signup / stripe-webhook / workers) stays untouched except semirx-&gt;corerx naming. NOTE the FUNCTIONAL subscription wiring (individual checkout, Stripe products/prices, the model switch) is the T096 build, not this naming/doc sweep -- but every STATEMENT of tiers/prices gets corrected to the lock now.</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>CLAUDE.md; supabase/migrations/*; web Pricing.jsx / coachPlan.js / coach Signup.jsx / CoachPricing.jsx / ForCoaches.jsx / legal/*; docs/marketing/*; branding/BRAND.md; CoachClientDetail.jsx; BillingView/BillingTab/AccountSettings/EditProfile</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
         <is>
           <t>2026-06-06</t>
         </is>

</xml_diff>

<commit_message>
docs(ledger): T096 - IAP/policy research (must use Apple/Google IAP in-app; account entitlement; RevenueCat; web/Stripe later)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -570,7 +570,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-06 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
+          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-07 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
         </is>
       </c>
     </row>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page). DECISION 1 (2026-06-06, user): approach = PROPOSE PREMIUM. ** MODEL CHANGE: individuals move from one-time lifetime to MONTHLY SUBSCRIPTION for ALL ** (no more one-time / 'own it forever'; both coaches AND individuals are recurring subs now). Individual tier strategy: price so FullRX is a NO-BRAINER -- tight CoreRX-&gt;FullRX gap, accessible-premium, everyone should obviously pick FullRX. Implications to handle: Stripe individual prices become RECURRING not one-time; the b2c_purchases one-time schema needs a subscription path (or fold individuals into a subscriptions table); drop all 'lifetime / own it forever' copy; in-app individual subs incur the Apple/Google cut while web-via-Stripe stays clean (same price both surfaces per existing plan). Baseline from research: coach $19/$39/$99 monthly (Starter/Pro/Elite; 10/25/unltd clients; 14-day trial; annual = 17% off yr1 only); individual $0/$39/$59 one-time. Coach checkout works in TEST mode (coach-signup edge fn + hosted Checkout, lookup_key coach_{tier}_{interval}); individual checkout NOT built; webhook duplicated (Supabase stripe-webhook canonical, Cloudflare worker superseded -&gt; retire); stale tier names (DB 'unlimited'/'semirx' vs code 'elite'/'corerx'); prices duplicated across coachPlan.js + coach/Signup.jsx + legal pages + Stripe. PRICING RESEARCH 2026-06-06 (user asked: is $2.99/$4.99 individual monthly bad for a brand-new no-trust app? + confirmed 14-day trial): ran 3 parallel web-research agents. VERDICT -- $2.99/$4.99 is the WRONG move for a premium coaching app: (1) price-quality signaling is STRONGEST for premium/AI products, so too-cheap reads as low-quality ('what's wrong with it'); (2) higher-priced fitness apps convert installs-&gt;paid ~2.7% vs ~1.5% for cheap ones -- low price does NOT buy conversion, it filters OUT committed users; (3) cheap monthly attracts churners + fitness already has the worst churn of any category (40-60% quit by Feb); (4) anchoring low -&gt; later price raises cause 10-15% churn spikes or a permanent grandfathered cohort. BENCHMARKS: pure loggers (Strong/Hevy) $3-5/mo = commodity; COACHING apps (Fitbod $15.99, Freeletics, Ladder, Centr) $15-30/mo; credible AI-coaching sweet spot ~$12.99-14.99/mo, ~$80/yr. TRIAL: 14-day is in the top-converting band (~44% trial-&gt;paid); free-trial / onboarding-paywall converts ~5x better than free-forever (~10.7% vs ~2.1% install-&gt;paid, ~8x revenue/install); 80%+ convert on Day 0 (onboarding-&gt;paywall matters most); native iOS/Android IAP trials are opt-out (card on file =&gt; ~48% conversion automatically), web/Stripe should lean no-card to maximize trial starts; a thin free tier belongs only as the soft-paywall SKIP fallback, not the front door. RECOMMENDATION: CoreRX $12.99 / FullRX $14.99 monthly (keep the $2 no-brainer gap; reads as real coaching just under Fitbod), annual ~$80/yr (separate decision), KEEP the 14-day trial, and solve the new-brand trust deficit with the trial + reviews/social-proof + a TIME-BOXED launch/founder promo (e.g. 50% off first 3 months) so a low entry number never becomes the permanent anchor. Sources: RevenueCat + Adapty subscription benchmarks, Airbridge 2026 pricing-by-category, SaaStr Day-1 pricing. POSITIONING REFINED 2026-06-06 (user): the app is honestly 'a logger WITH a coaching-cue edge', NOT a full Fitbod-style coach -- do NOT oversell (avoid being labelled a liar) but DO assume some premiumness =&gt; price 'a notch above other loggers' (loggers ~$4-5/mo, so individual top tier in the ~$7-9/mo band, NOT the $14.99 coaching tier). Annual = 17% off (= '2 months free') as an OPTION. Proposed: CoreRX $5.99 / FullRX $7.99 monthly (a clear notch above the $4.99 logger ceiling, $2 no-brainer gap), annual ~$59.99 / ~$79.99 (2 months free). OPEN sub-decision: is the INDIVIDUAL annual discount recurring or first-year-only? (coach annual is currently first-year-only per CLAUDE.md) -- align when we do the coach prices. INDIVIDUAL PRICING LOCKED 2026-06-06: monthly subscription + 14-day trial; Free $0 / CoreRX $4.99/mo / FullRX $6.99/mo; annual = 17% off (2 months free) =&gt; CoreRX ~$49.99/yr, FullRX ~$69.99/yr (user chose the most-accessible 'notch above loggers' option). NEXT decisions: coach prices (current $19/$39/$99 monthly, 10/25/unltd clients) + align the annual-discount model (coach annual is currently 17%-off-FIRST-YEAR-ONLY per CLAUDE.md, individual annual is 17% recurring -- decide whether to unify) + free-tier feature split + then Stripe sandbox setup + billing-page build. COACH PRICES LOCKED 2026-06-06: keep Starter $19 / Pro $39 / Elite $99 monthly, caps 10/25/unltd clients, 14-day trial (already competitive vs TrueCoach/Trainerize; don't scare early coaches). PENDING: annual-discount model -- unify to RECURRING 17% (2 months free) for BOTH coaches + individuals, or keep coach annual as 17%-off-first-year-only? RESOLVED: RECURRING 17% (2 months free) for BOTH. Coach annual is NO LONGER first-year-only -&gt; permanent 17% off, renews at the same discounted annual (no year-2 jump): coach annual ~$189/$389/$989 RECURRING; individual ~$49.99/$69.99 recurring. IMPL TO-DO: REVERSE the CLAUDE.md 'coach annual 17% off first year only, renews full' lock to recurring; strip the year-2 renewal figures ($228/$468/$1188) + every 'first year' disclaimer from CoachAgreement / RefundPolicy / CoachPricing / coach Signup; set Stripe annual prices to the flat recurring annual. === FULL PRICING LOCKED 2026-06-06: monthly-subscription model for ALL (no one-time/lifetime); 14-day trial both. Individual: Free $0 / CoreRX $4.99 / FullRX $6.99 monthly (annual 17% recurring ~$49.99 / ~$69.99). Coach: Starter $19 / Pro $39 / Elite $99 monthly, 10/25/unltd clients (annual 17% recurring ~$189 / ~$389 / ~$989). REMAINING: free-tier feature split (code currently inconsistent) -&gt; then Stripe sandbox products/prices -&gt; propagate prices everywhere + model-change cleanup (drop lifetime copy, retire CF webhook, fix stale tier names elite/corerx, build individual checkout) -&gt; billing page. TIER FEATURE SPLIT (from CLAUDE.md lines 2384-2393, AUTHORITATIVE -- my earlier improvised split was wrong; Mobility was removed in the June 2026 teardown so it's NOT a tier feature): Free = Strength + Cardio; CoreRX = Free + Bodyweight + Calories (body-composition + calorie/macro coaching, the two most-requested); FullRX = CoreRX + Heart + Hydration + Sleep (the wellness/recovery layer, appeals to wearable owners). The cross-domain Dashboard rollup sits in FullRX (complete picture). The feature split is UNCHANGED by the one-time-&gt;subscription move; only the model + prices change. CODE INCONSISTENCY TO FIX: the in-app gating (CoachClientDetail TIER_RANK) wrongly puts Heart in CoreRX -- must move to FullRX to match CLAUDE.md. === ATHLETE TIERS FINALIZED + LOCKED BY USER 2026-06-06 (THIS IS FINAL): Free = Strength+Cardio; CoreRX $4.99/mo ($49.99/yr) = +Bodyweight+Calories/Food; FullRX $6.99/mo ($69.99/yr) = +Heart+Hydration+Sleep+every future feature. COACH: every coach tier grants FULL FullRX access to the coach AND all their linked athletes -- tiers differ ONLY by client cap (Starter $19/10, Pro $39/25, Elite $99/unltd; annual 17% recurring $189/$389/$989). Home Dashboard = the landing/profile screen for EVERYONE, never a tier feature. User demanded a CLEAN SWEEP of all stale/contradicting references (esp. the 'semirx' old name + the 3-way-conflicting tier splits) -&gt; tracked as T097. === STEP 1 (Stripe sandbox catalog) DONE 2026-06-06: created scripts/setup-stripe-sandbox-prices.mjs (idempotent, TEST-only, refuses non-sk_test_, reads key from .env.local) + ran it. Final TEST catalog by lookup_key: corerx_monthly $4.99 / corerx_annual $49.99 (prod CoreRX), fullrx_monthly $6.99 / fullrx_annual $69.99 (prod FullRX), coach_starter_monthly $19 / coach_starter_annual $189, coach_pro_monthly $39 / coach_pro_annual $389, coach_elite_monthly $99 / coach_elite_annual $989. Coach products reused (metadata myrx_tier+myrx_audience set); coach MONTHLY already matched (left as-is, existing test subs safe); coach ANNUAL recreated as flat-recurring (old annual prices archived -- they didn't match flat $189/$389/$989, confirming the old first-year-only structure is gone). Old athlete one-time prices (corerx_onetime / fullrx_onetime) archived. The app references prices by lookup_key (&lt;tier&gt;_monthly / &lt;tier&gt;_annual), never by price_ id. Built only in Stripe TEST; no app code changed, no web deploy. NEXT = Step 2 (hosted-checkout + 14-day trial + individual subscription wiring) -- awaiting user discussion per the step-by-step agreement (do NOT start step 2 until discussed).</t>
+          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page). DECISION 1 (2026-06-06, user): approach = PROPOSE PREMIUM. ** MODEL CHANGE: individuals move from one-time lifetime to MONTHLY SUBSCRIPTION for ALL ** (no more one-time / 'own it forever'; both coaches AND individuals are recurring subs now). Individual tier strategy: price so FullRX is a NO-BRAINER -- tight CoreRX-&gt;FullRX gap, accessible-premium, everyone should obviously pick FullRX. Implications to handle: Stripe individual prices become RECURRING not one-time; the b2c_purchases one-time schema needs a subscription path (or fold individuals into a subscriptions table); drop all 'lifetime / own it forever' copy; in-app individual subs incur the Apple/Google cut while web-via-Stripe stays clean (same price both surfaces per existing plan). Baseline from research: coach $19/$39/$99 monthly (Starter/Pro/Elite; 10/25/unltd clients; 14-day trial; annual = 17% off yr1 only); individual $0/$39/$59 one-time. Coach checkout works in TEST mode (coach-signup edge fn + hosted Checkout, lookup_key coach_{tier}_{interval}); individual checkout NOT built; webhook duplicated (Supabase stripe-webhook canonical, Cloudflare worker superseded -&gt; retire); stale tier names (DB 'unlimited'/'semirx' vs code 'elite'/'corerx'); prices duplicated across coachPlan.js + coach/Signup.jsx + legal pages + Stripe. PRICING RESEARCH 2026-06-06 (user asked: is $2.99/$4.99 individual monthly bad for a brand-new no-trust app? + confirmed 14-day trial): ran 3 parallel web-research agents. VERDICT -- $2.99/$4.99 is the WRONG move for a premium coaching app: (1) price-quality signaling is STRONGEST for premium/AI products, so too-cheap reads as low-quality ('what's wrong with it'); (2) higher-priced fitness apps convert installs-&gt;paid ~2.7% vs ~1.5% for cheap ones -- low price does NOT buy conversion, it filters OUT committed users; (3) cheap monthly attracts churners + fitness already has the worst churn of any category (40-60% quit by Feb); (4) anchoring low -&gt; later price raises cause 10-15% churn spikes or a permanent grandfathered cohort. BENCHMARKS: pure loggers (Strong/Hevy) $3-5/mo = commodity; COACHING apps (Fitbod $15.99, Freeletics, Ladder, Centr) $15-30/mo; credible AI-coaching sweet spot ~$12.99-14.99/mo, ~$80/yr. TRIAL: 14-day is in the top-converting band (~44% trial-&gt;paid); free-trial / onboarding-paywall converts ~5x better than free-forever (~10.7% vs ~2.1% install-&gt;paid, ~8x revenue/install); 80%+ convert on Day 0 (onboarding-&gt;paywall matters most); native iOS/Android IAP trials are opt-out (card on file =&gt; ~48% conversion automatically), web/Stripe should lean no-card to maximize trial starts; a thin free tier belongs only as the soft-paywall SKIP fallback, not the front door. RECOMMENDATION: CoreRX $12.99 / FullRX $14.99 monthly (keep the $2 no-brainer gap; reads as real coaching just under Fitbod), annual ~$80/yr (separate decision), KEEP the 14-day trial, and solve the new-brand trust deficit with the trial + reviews/social-proof + a TIME-BOXED launch/founder promo (e.g. 50% off first 3 months) so a low entry number never becomes the permanent anchor. Sources: RevenueCat + Adapty subscription benchmarks, Airbridge 2026 pricing-by-category, SaaStr Day-1 pricing. POSITIONING REFINED 2026-06-06 (user): the app is honestly 'a logger WITH a coaching-cue edge', NOT a full Fitbod-style coach -- do NOT oversell (avoid being labelled a liar) but DO assume some premiumness =&gt; price 'a notch above other loggers' (loggers ~$4-5/mo, so individual top tier in the ~$7-9/mo band, NOT the $14.99 coaching tier). Annual = 17% off (= '2 months free') as an OPTION. Proposed: CoreRX $5.99 / FullRX $7.99 monthly (a clear notch above the $4.99 logger ceiling, $2 no-brainer gap), annual ~$59.99 / ~$79.99 (2 months free). OPEN sub-decision: is the INDIVIDUAL annual discount recurring or first-year-only? (coach annual is currently first-year-only per CLAUDE.md) -- align when we do the coach prices. INDIVIDUAL PRICING LOCKED 2026-06-06: monthly subscription + 14-day trial; Free $0 / CoreRX $4.99/mo / FullRX $6.99/mo; annual = 17% off (2 months free) =&gt; CoreRX ~$49.99/yr, FullRX ~$69.99/yr (user chose the most-accessible 'notch above loggers' option). NEXT decisions: coach prices (current $19/$39/$99 monthly, 10/25/unltd clients) + align the annual-discount model (coach annual is currently 17%-off-FIRST-YEAR-ONLY per CLAUDE.md, individual annual is 17% recurring -- decide whether to unify) + free-tier feature split + then Stripe sandbox setup + billing-page build. COACH PRICES LOCKED 2026-06-06: keep Starter $19 / Pro $39 / Elite $99 monthly, caps 10/25/unltd clients, 14-day trial (already competitive vs TrueCoach/Trainerize; don't scare early coaches). PENDING: annual-discount model -- unify to RECURRING 17% (2 months free) for BOTH coaches + individuals, or keep coach annual as 17%-off-first-year-only? RESOLVED: RECURRING 17% (2 months free) for BOTH. Coach annual is NO LONGER first-year-only -&gt; permanent 17% off, renews at the same discounted annual (no year-2 jump): coach annual ~$189/$389/$989 RECURRING; individual ~$49.99/$69.99 recurring. IMPL TO-DO: REVERSE the CLAUDE.md 'coach annual 17% off first year only, renews full' lock to recurring; strip the year-2 renewal figures ($228/$468/$1188) + every 'first year' disclaimer from CoachAgreement / RefundPolicy / CoachPricing / coach Signup; set Stripe annual prices to the flat recurring annual. === FULL PRICING LOCKED 2026-06-06: monthly-subscription model for ALL (no one-time/lifetime); 14-day trial both. Individual: Free $0 / CoreRX $4.99 / FullRX $6.99 monthly (annual 17% recurring ~$49.99 / ~$69.99). Coach: Starter $19 / Pro $39 / Elite $99 monthly, 10/25/unltd clients (annual 17% recurring ~$189 / ~$389 / ~$989). REMAINING: free-tier feature split (code currently inconsistent) -&gt; then Stripe sandbox products/prices -&gt; propagate prices everywhere + model-change cleanup (drop lifetime copy, retire CF webhook, fix stale tier names elite/corerx, build individual checkout) -&gt; billing page. TIER FEATURE SPLIT (from CLAUDE.md lines 2384-2393, AUTHORITATIVE -- my earlier improvised split was wrong; Mobility was removed in the June 2026 teardown so it's NOT a tier feature): Free = Strength + Cardio; CoreRX = Free + Bodyweight + Calories (body-composition + calorie/macro coaching, the two most-requested); FullRX = CoreRX + Heart + Hydration + Sleep (the wellness/recovery layer, appeals to wearable owners). The cross-domain Dashboard rollup sits in FullRX (complete picture). The feature split is UNCHANGED by the one-time-&gt;subscription move; only the model + prices change. CODE INCONSISTENCY TO FIX: the in-app gating (CoachClientDetail TIER_RANK) wrongly puts Heart in CoreRX -- must move to FullRX to match CLAUDE.md. === ATHLETE TIERS FINALIZED + LOCKED BY USER 2026-06-06 (THIS IS FINAL): Free = Strength+Cardio; CoreRX $4.99/mo ($49.99/yr) = +Bodyweight+Calories/Food; FullRX $6.99/mo ($69.99/yr) = +Heart+Hydration+Sleep+every future feature. COACH: every coach tier grants FULL FullRX access to the coach AND all their linked athletes -- tiers differ ONLY by client cap (Starter $19/10, Pro $39/25, Elite $99/unltd; annual 17% recurring $189/$389/$989). Home Dashboard = the landing/profile screen for EVERYONE, never a tier feature. User demanded a CLEAN SWEEP of all stale/contradicting references (esp. the 'semirx' old name + the 3-way-conflicting tier splits) -&gt; tracked as T097. === STEP 1 (Stripe sandbox catalog) DONE 2026-06-06: created scripts/setup-stripe-sandbox-prices.mjs (idempotent, TEST-only, refuses non-sk_test_, reads key from .env.local) + ran it. Final TEST catalog by lookup_key: corerx_monthly $4.99 / corerx_annual $49.99 (prod CoreRX), fullrx_monthly $6.99 / fullrx_annual $69.99 (prod FullRX), coach_starter_monthly $19 / coach_starter_annual $189, coach_pro_monthly $39 / coach_pro_annual $389, coach_elite_monthly $99 / coach_elite_annual $989. Coach products reused (metadata myrx_tier+myrx_audience set); coach MONTHLY already matched (left as-is, existing test subs safe); coach ANNUAL recreated as flat-recurring (old annual prices archived -- they didn't match flat $189/$389/$989, confirming the old first-year-only structure is gone). Old athlete one-time prices (corerx_onetime / fullrx_onetime) archived. The app references prices by lookup_key (&lt;tier&gt;_monthly / &lt;tier&gt;_annual), never by price_ id. Built only in Stripe TEST; no app code changed, no web deploy. NEXT = Step 2 (hosted-checkout + 14-day trial + individual subscription wiring) -- awaiting user discussion per the step-by-step agreement (do NOT start step 2 until discussed). === IAP/POLICY RESEARCH 2026-06-07 (user: 'i dont want to violate iOS/Google policies; athletes download from stores + subscribe; how do modern apps do it?') -- 3 parallel web-research agents. FINDINGS: (1) a fitness/coaching app MUST offer Apple IAP / Google Play Billing for ANY subscription unlocked INSIDE the app (Apple Guideline 3.1.1). It is NOT a 'reader app' (that web-only carve-out is magazines/music/video only -- how Netflix/Spotify sell web-only), so we CANNOT ship a web-pay-only + unlock-in-app model -&gt; instant rejection. (2) Universal unlock = ACCOUNT-BASED ENTITLEMENT: a sub (Apple IAP / Google Play / web Stripe / coach-comped) flips a tier flag on the user's ACCOUNT server-side; every client checks the account, not the store. This is exactly how our coach-&gt;client comp model already works. (3) Peers (Fitbod/Calm/Headspace/Whoop) = IAP-first, absorb the cut, frictionless in-app subscribe; some (YouTube/Duolingo) price IAP higher to cover the cut; web secondary. (4) Standard tool = RevenueCat (or Adapty/Qonversion): manages Apple/Google IAP + receipt validation + webhooks + unified cross-platform entitlement; free under $2,500/mo tracked revenue, then ~1%. (5) Fees: Apple/Google 15% (small biz &lt;$1M or after 12mo) to 30%; Stripe web ~2.9%+30c. US (post Epic v Apple 2025-26, legally provisional) now allows in-app links to a cheaper web checkout at ~0% Apple commission; EU ~5% Core Technology Commission; ROW no in-app steering + ~27%/12% external. RECOMMENDED ARCHITECTURE: account-based entitlement from day 1; individuals subscribe via Apple/Google IAP (compliant, frictionless) managed by RevenueCat; coaches stay web-Stripe (already works); add the cheaper web/Stripe individual path LATER once there's a marketing funnel (NOT hybrid day 1 -- friction + compliance surface, and RevenueCat's own test showed a 2nd web CTA netted slightly LESS per IAP dollar). BUILD REFRAME: the Step-1 Stripe individual products (corerx/fullrx) now serve the FUTURE web path; the PRIMARY individual path = mobile IAP via RevenueCat (a MOBILE build: App Store Connect + Play Console subscription products + RevenueCat account + Expo SDK + entitlement wiring + dev-account enrollment) -- bigger than a Stripe checkout. Sources: Apple App Review Guidelines, Epic v Apple 2025-26 rulings, RevenueCat/Adapty docs+benchmarks. AWAITING user pick: pivot Step 2 to the IAP/RevenueCat individual path vs continue the web-Stripe individual path first.</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): audit - add T098 (lapse downgrade) / T099 (archive Stripe athlete products) / T100 (Efforts T086 strip); mark T096+T097 Deferred
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5107,9 +5107,9 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E99" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E99" s="10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="F99" s="7" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page). DECISION 1 (2026-06-06, user): approach = PROPOSE PREMIUM. ** MODEL CHANGE: individuals move from one-time lifetime to MONTHLY SUBSCRIPTION for ALL ** (no more one-time / 'own it forever'; both coaches AND individuals are recurring subs now). Individual tier strategy: price so FullRX is a NO-BRAINER -- tight CoreRX-&gt;FullRX gap, accessible-premium, everyone should obviously pick FullRX. Implications to handle: Stripe individual prices become RECURRING not one-time; the b2c_purchases one-time schema needs a subscription path (or fold individuals into a subscriptions table); drop all 'lifetime / own it forever' copy; in-app individual subs incur the Apple/Google cut while web-via-Stripe stays clean (same price both surfaces per existing plan). Baseline from research: coach $19/$39/$99 monthly (Starter/Pro/Elite; 10/25/unltd clients; 14-day trial; annual = 17% off yr1 only); individual $0/$39/$59 one-time. Coach checkout works in TEST mode (coach-signup edge fn + hosted Checkout, lookup_key coach_{tier}_{interval}); individual checkout NOT built; webhook duplicated (Supabase stripe-webhook canonical, Cloudflare worker superseded -&gt; retire); stale tier names (DB 'unlimited'/'semirx' vs code 'elite'/'corerx'); prices duplicated across coachPlan.js + coach/Signup.jsx + legal pages + Stripe. PRICING RESEARCH 2026-06-06 (user asked: is $2.99/$4.99 individual monthly bad for a brand-new no-trust app? + confirmed 14-day trial): ran 3 parallel web-research agents. VERDICT -- $2.99/$4.99 is the WRONG move for a premium coaching app: (1) price-quality signaling is STRONGEST for premium/AI products, so too-cheap reads as low-quality ('what's wrong with it'); (2) higher-priced fitness apps convert installs-&gt;paid ~2.7% vs ~1.5% for cheap ones -- low price does NOT buy conversion, it filters OUT committed users; (3) cheap monthly attracts churners + fitness already has the worst churn of any category (40-60% quit by Feb); (4) anchoring low -&gt; later price raises cause 10-15% churn spikes or a permanent grandfathered cohort. BENCHMARKS: pure loggers (Strong/Hevy) $3-5/mo = commodity; COACHING apps (Fitbod $15.99, Freeletics, Ladder, Centr) $15-30/mo; credible AI-coaching sweet spot ~$12.99-14.99/mo, ~$80/yr. TRIAL: 14-day is in the top-converting band (~44% trial-&gt;paid); free-trial / onboarding-paywall converts ~5x better than free-forever (~10.7% vs ~2.1% install-&gt;paid, ~8x revenue/install); 80%+ convert on Day 0 (onboarding-&gt;paywall matters most); native iOS/Android IAP trials are opt-out (card on file =&gt; ~48% conversion automatically), web/Stripe should lean no-card to maximize trial starts; a thin free tier belongs only as the soft-paywall SKIP fallback, not the front door. RECOMMENDATION: CoreRX $12.99 / FullRX $14.99 monthly (keep the $2 no-brainer gap; reads as real coaching just under Fitbod), annual ~$80/yr (separate decision), KEEP the 14-day trial, and solve the new-brand trust deficit with the trial + reviews/social-proof + a TIME-BOXED launch/founder promo (e.g. 50% off first 3 months) so a low entry number never becomes the permanent anchor. Sources: RevenueCat + Adapty subscription benchmarks, Airbridge 2026 pricing-by-category, SaaStr Day-1 pricing. POSITIONING REFINED 2026-06-06 (user): the app is honestly 'a logger WITH a coaching-cue edge', NOT a full Fitbod-style coach -- do NOT oversell (avoid being labelled a liar) but DO assume some premiumness =&gt; price 'a notch above other loggers' (loggers ~$4-5/mo, so individual top tier in the ~$7-9/mo band, NOT the $14.99 coaching tier). Annual = 17% off (= '2 months free') as an OPTION. Proposed: CoreRX $5.99 / FullRX $7.99 monthly (a clear notch above the $4.99 logger ceiling, $2 no-brainer gap), annual ~$59.99 / ~$79.99 (2 months free). OPEN sub-decision: is the INDIVIDUAL annual discount recurring or first-year-only? (coach annual is currently first-year-only per CLAUDE.md) -- align when we do the coach prices. INDIVIDUAL PRICING LOCKED 2026-06-06: monthly subscription + 14-day trial; Free $0 / CoreRX $4.99/mo / FullRX $6.99/mo; annual = 17% off (2 months free) =&gt; CoreRX ~$49.99/yr, FullRX ~$69.99/yr (user chose the most-accessible 'notch above loggers' option). NEXT decisions: coach prices (current $19/$39/$99 monthly, 10/25/unltd clients) + align the annual-discount model (coach annual is currently 17%-off-FIRST-YEAR-ONLY per CLAUDE.md, individual annual is 17% recurring -- decide whether to unify) + free-tier feature split + then Stripe sandbox setup + billing-page build. COACH PRICES LOCKED 2026-06-06: keep Starter $19 / Pro $39 / Elite $99 monthly, caps 10/25/unltd clients, 14-day trial (already competitive vs TrueCoach/Trainerize; don't scare early coaches). PENDING: annual-discount model -- unify to RECURRING 17% (2 months free) for BOTH coaches + individuals, or keep coach annual as 17%-off-first-year-only? RESOLVED: RECURRING 17% (2 months free) for BOTH. Coach annual is NO LONGER first-year-only -&gt; permanent 17% off, renews at the same discounted annual (no year-2 jump): coach annual ~$189/$389/$989 RECURRING; individual ~$49.99/$69.99 recurring. IMPL TO-DO: REVERSE the CLAUDE.md 'coach annual 17% off first year only, renews full' lock to recurring; strip the year-2 renewal figures ($228/$468/$1188) + every 'first year' disclaimer from CoachAgreement / RefundPolicy / CoachPricing / coach Signup; set Stripe annual prices to the flat recurring annual. === FULL PRICING LOCKED 2026-06-06: monthly-subscription model for ALL (no one-time/lifetime); 14-day trial both. Individual: Free $0 / CoreRX $4.99 / FullRX $6.99 monthly (annual 17% recurring ~$49.99 / ~$69.99). Coach: Starter $19 / Pro $39 / Elite $99 monthly, 10/25/unltd clients (annual 17% recurring ~$189 / ~$389 / ~$989). REMAINING: free-tier feature split (code currently inconsistent) -&gt; then Stripe sandbox products/prices -&gt; propagate prices everywhere + model-change cleanup (drop lifetime copy, retire CF webhook, fix stale tier names elite/corerx, build individual checkout) -&gt; billing page. TIER FEATURE SPLIT (from CLAUDE.md lines 2384-2393, AUTHORITATIVE -- my earlier improvised split was wrong; Mobility was removed in the June 2026 teardown so it's NOT a tier feature): Free = Strength + Cardio; CoreRX = Free + Bodyweight + Calories (body-composition + calorie/macro coaching, the two most-requested); FullRX = CoreRX + Heart + Hydration + Sleep (the wellness/recovery layer, appeals to wearable owners). The cross-domain Dashboard rollup sits in FullRX (complete picture). The feature split is UNCHANGED by the one-time-&gt;subscription move; only the model + prices change. CODE INCONSISTENCY TO FIX: the in-app gating (CoachClientDetail TIER_RANK) wrongly puts Heart in CoreRX -- must move to FullRX to match CLAUDE.md. === ATHLETE TIERS FINALIZED + LOCKED BY USER 2026-06-06 (THIS IS FINAL): Free = Strength+Cardio; CoreRX $4.99/mo ($49.99/yr) = +Bodyweight+Calories/Food; FullRX $6.99/mo ($69.99/yr) = +Heart+Hydration+Sleep+every future feature. COACH: every coach tier grants FULL FullRX access to the coach AND all their linked athletes -- tiers differ ONLY by client cap (Starter $19/10, Pro $39/25, Elite $99/unltd; annual 17% recurring $189/$389/$989). Home Dashboard = the landing/profile screen for EVERYONE, never a tier feature. User demanded a CLEAN SWEEP of all stale/contradicting references (esp. the 'semirx' old name + the 3-way-conflicting tier splits) -&gt; tracked as T097. === STEP 1 (Stripe sandbox catalog) DONE 2026-06-06: created scripts/setup-stripe-sandbox-prices.mjs (idempotent, TEST-only, refuses non-sk_test_, reads key from .env.local) + ran it. Final TEST catalog by lookup_key: corerx_monthly $4.99 / corerx_annual $49.99 (prod CoreRX), fullrx_monthly $6.99 / fullrx_annual $69.99 (prod FullRX), coach_starter_monthly $19 / coach_starter_annual $189, coach_pro_monthly $39 / coach_pro_annual $389, coach_elite_monthly $99 / coach_elite_annual $989. Coach products reused (metadata myrx_tier+myrx_audience set); coach MONTHLY already matched (left as-is, existing test subs safe); coach ANNUAL recreated as flat-recurring (old annual prices archived -- they didn't match flat $189/$389/$989, confirming the old first-year-only structure is gone). Old athlete one-time prices (corerx_onetime / fullrx_onetime) archived. The app references prices by lookup_key (&lt;tier&gt;_monthly / &lt;tier&gt;_annual), never by price_ id. Built only in Stripe TEST; no app code changed, no web deploy. NEXT = Step 2 (hosted-checkout + 14-day trial + individual subscription wiring) -- awaiting user discussion per the step-by-step agreement (do NOT start step 2 until discussed). === IAP/POLICY RESEARCH 2026-06-07 (user: 'i dont want to violate iOS/Google policies; athletes download from stores + subscribe; how do modern apps do it?') -- 3 parallel web-research agents. FINDINGS: (1) a fitness/coaching app MUST offer Apple IAP / Google Play Billing for ANY subscription unlocked INSIDE the app (Apple Guideline 3.1.1). It is NOT a 'reader app' (that web-only carve-out is magazines/music/video only -- how Netflix/Spotify sell web-only), so we CANNOT ship a web-pay-only + unlock-in-app model -&gt; instant rejection. (2) Universal unlock = ACCOUNT-BASED ENTITLEMENT: a sub (Apple IAP / Google Play / web Stripe / coach-comped) flips a tier flag on the user's ACCOUNT server-side; every client checks the account, not the store. This is exactly how our coach-&gt;client comp model already works. (3) Peers (Fitbod/Calm/Headspace/Whoop) = IAP-first, absorb the cut, frictionless in-app subscribe; some (YouTube/Duolingo) price IAP higher to cover the cut; web secondary. (4) Standard tool = RevenueCat (or Adapty/Qonversion): manages Apple/Google IAP + receipt validation + webhooks + unified cross-platform entitlement; free under $2,500/mo tracked revenue, then ~1%. (5) Fees: Apple/Google 15% (small biz &lt;$1M or after 12mo) to 30%; Stripe web ~2.9%+30c. US (post Epic v Apple 2025-26, legally provisional) now allows in-app links to a cheaper web checkout at ~0% Apple commission; EU ~5% Core Technology Commission; ROW no in-app steering + ~27%/12% external. RECOMMENDED ARCHITECTURE: account-based entitlement from day 1; individuals subscribe via Apple/Google IAP (compliant, frictionless) managed by RevenueCat; coaches stay web-Stripe (already works); add the cheaper web/Stripe individual path LATER once there's a marketing funnel (NOT hybrid day 1 -- friction + compliance surface, and RevenueCat's own test showed a 2nd web CTA netted slightly LESS per IAP dollar). BUILD REFRAME: the Step-1 Stripe individual products (corerx/fullrx) now serve the FUTURE web path; the PRIMARY individual path = mobile IAP via RevenueCat (a MOBILE build: App Store Connect + Play Console subscription products + RevenueCat account + Expo SDK + entitlement wiring + dev-account enrollment) -- bigger than a Stripe checkout. Sources: Apple App Review Guidelines, Epic v Apple 2025-26 rulings, RevenueCat/Adapty docs+benchmarks. AWAITING user pick: pivot Step 2 to the IAP/RevenueCat individual path vs continue the web-Stripe individual path first. === MODEL CLARIFIED BY USER 2026-06-07 (resolves the fork): TWO account types, two payment surfaces, ONE entitlement switch. COACHES subscribe ONLY on WEB (Stripe); a coach's active sub grants FullRX to (a) all their linked client athletes AND (b) the coach's OWN athlete account (a coach is also an athlete -- one account, role-routed: mobile = athlete view at FullRX, web = redirected to coach portal). ATHLETES (non-coach) subscribe ONLY IN-APP (Apple IAP / Google Play via RevenueCat); there is NO web checkout for athletes. CONSEQUENCE: the Step-1 Stripe corerx/fullrx ATHLETE products are now UNUSED (athletes never pay via Stripe) -&gt; archive them; only the coach_* Stripe products are used. Athlete tier products (CoreRX/FullRX monthly+annual, 14-day trial) get created in App Store Connect + Google Play Console (IAP) + mapped in RevenueCat. ENTITLEMENT (the switch) = one account-level effective tier (free/corerx/fullrx) the mobile app reads for gating, WRITTEN by BOTH the coach Stripe webhook (coach self + clients -&gt; fullrx) AND the athlete IAP/RevenueCat webhook (athlete -&gt; their tier). WORK SPLIT: (A) finish/verify the coach-&gt;FullRX unlock for coach-self + clients (web side, mostly built -- client_has_active_coach() already comps clients); (B) the athlete in-app subscription via RevenueCat (the big NEW mobile build: App Store Connect + Play Console products, RevenueCat account+SDK, paywall screen, webhook-&gt;entitlement, app gating) -- needs the user's Apple/Google/RevenueCat accounts. Recommended order: A first (small), then B step-by-step. === STEP A VERIFIED DONE 2026-06-07: resolveTier (mobile dashboard.tsx L48-58 + web CoachClientDetail/AdminUserDetail, byte-for-byte) -&gt; is_superuser/is_coach/coach_id(linked client) = fullrx, else b2c_subscription_tier ?? free. ENFORCED in-app: RadialNav gates orbit pages by tier ('coached clients get full access regardless of their own tier -- coach is paying'); dashboard gates stat pills by tierRank. So coach's own athlete account + all linked clients = FullRX + pages unlock. Matches the user's model. LAPSE GAP (flagged, not blocking): resolveTier keys off the LINK (coach_id/is_coach), NOT the coach's ACTIVE sub -- client_has_active_coach()/is_active_coach() RPCs exist but aren't used by resolveTier, so a client of a LAPSED coach stays FullRX until a lapse-downgrade is wired (launch-readiness follow-up). === STEP B STARTED (athlete in-app subscription via RevenueCat). GOOD NEWS: the READ/unlock side already exists (profiles.b2c_subscription_tier column + resolveTier already unlock pages when set), so B only needs the WRITE + purchase UI + accounts: (1) [USER accounts] Apple Developer/App Store Connect products (CoreRX/FullRX monthly+annual, 14-day trial), Google Play Console products, RevenueCat account mapping store products -&gt; corerx/fullrx entitlements; (2) [CODE] RevenueCat SDK (react-native-purchases) in the Expo app (native module -&gt; dev-client rebuild) + in-app paywall/subscribe screen; (3) [CODE] RevenueCat webhook -&gt; edge function that writes b2c_subscription_tier on the athlete's profile; (4) sandbox testing (App Store sandbox testers + Play internal test track). FIRST BLOCKER to resolve: the user's Apple Developer / Google Play / RevenueCat account status (determines where we start; code that doesn't need keys can be scaffolded meanwhile). === BLOCKER CONFIRMED 2026-06-07: user has NONE of the accounts (no Apple Developer, no Google Play, no RevenueCat) AND no iOS build ready (the app has only ever run as an Android dev-client). I CANNOT create those accounts -- they require the user's identity + payment + Apple-ID 2FA (+ a D-U-N-S for an org); creating accounts / entering financial credentials are not actions I do -- so the enrollments are the user's to do (I guide every click + do all code). The app is Expo so iOS can be built via EAS cloud (no Mac), BUT any athlete-IAP testing still needs the paid Apple account first -&gt; Apple Developer enrollment is THE gate for all athlete billing. RECOMMENDATION: user starts the Apple (~$99/yr) + Google Play (~$25 one-time) enrollments now (long lead, days), HOLD B's code until the accounts are close (so it isn't built untested + left to drift), keep building non-blocked work meanwhile (coach platform polish, the holistic dashboard rollup, etc.). Awaiting user pick: (1) start enrollment now + I prep iOS cloud-build config + scaffold the no-key parts in parallel, or (2) park B + build elsewhere until enrolled.</t>
+          <t>IN PROGRESS 2026-06-06 -- step 1 = research the CURRENT prices + Stripe wiring state, then a one-question-at-a-time decision flow, then implementation (revise prices -&gt; Stripe sandbox products/prices -&gt; billing page). DECISION 1 (2026-06-06, user): approach = PROPOSE PREMIUM. ** MODEL CHANGE: individuals move from one-time lifetime to MONTHLY SUBSCRIPTION for ALL ** (no more one-time / 'own it forever'; both coaches AND individuals are recurring subs now). Individual tier strategy: price so FullRX is a NO-BRAINER -- tight CoreRX-&gt;FullRX gap, accessible-premium, everyone should obviously pick FullRX. Implications to handle: Stripe individual prices become RECURRING not one-time; the b2c_purchases one-time schema needs a subscription path (or fold individuals into a subscriptions table); drop all 'lifetime / own it forever' copy; in-app individual subs incur the Apple/Google cut while web-via-Stripe stays clean (same price both surfaces per existing plan). Baseline from research: coach $19/$39/$99 monthly (Starter/Pro/Elite; 10/25/unltd clients; 14-day trial; annual = 17% off yr1 only); individual $0/$39/$59 one-time. Coach checkout works in TEST mode (coach-signup edge fn + hosted Checkout, lookup_key coach_{tier}_{interval}); individual checkout NOT built; webhook duplicated (Supabase stripe-webhook canonical, Cloudflare worker superseded -&gt; retire); stale tier names (DB 'unlimited'/'semirx' vs code 'elite'/'corerx'); prices duplicated across coachPlan.js + coach/Signup.jsx + legal pages + Stripe. PRICING RESEARCH 2026-06-06 (user asked: is $2.99/$4.99 individual monthly bad for a brand-new no-trust app? + confirmed 14-day trial): ran 3 parallel web-research agents. VERDICT -- $2.99/$4.99 is the WRONG move for a premium coaching app: (1) price-quality signaling is STRONGEST for premium/AI products, so too-cheap reads as low-quality ('what's wrong with it'); (2) higher-priced fitness apps convert installs-&gt;paid ~2.7% vs ~1.5% for cheap ones -- low price does NOT buy conversion, it filters OUT committed users; (3) cheap monthly attracts churners + fitness already has the worst churn of any category (40-60% quit by Feb); (4) anchoring low -&gt; later price raises cause 10-15% churn spikes or a permanent grandfathered cohort. BENCHMARKS: pure loggers (Strong/Hevy) $3-5/mo = commodity; COACHING apps (Fitbod $15.99, Freeletics, Ladder, Centr) $15-30/mo; credible AI-coaching sweet spot ~$12.99-14.99/mo, ~$80/yr. TRIAL: 14-day is in the top-converting band (~44% trial-&gt;paid); free-trial / onboarding-paywall converts ~5x better than free-forever (~10.7% vs ~2.1% install-&gt;paid, ~8x revenue/install); 80%+ convert on Day 0 (onboarding-&gt;paywall matters most); native iOS/Android IAP trials are opt-out (card on file =&gt; ~48% conversion automatically), web/Stripe should lean no-card to maximize trial starts; a thin free tier belongs only as the soft-paywall SKIP fallback, not the front door. RECOMMENDATION: CoreRX $12.99 / FullRX $14.99 monthly (keep the $2 no-brainer gap; reads as real coaching just under Fitbod), annual ~$80/yr (separate decision), KEEP the 14-day trial, and solve the new-brand trust deficit with the trial + reviews/social-proof + a TIME-BOXED launch/founder promo (e.g. 50% off first 3 months) so a low entry number never becomes the permanent anchor. Sources: RevenueCat + Adapty subscription benchmarks, Airbridge 2026 pricing-by-category, SaaStr Day-1 pricing. POSITIONING REFINED 2026-06-06 (user): the app is honestly 'a logger WITH a coaching-cue edge', NOT a full Fitbod-style coach -- do NOT oversell (avoid being labelled a liar) but DO assume some premiumness =&gt; price 'a notch above other loggers' (loggers ~$4-5/mo, so individual top tier in the ~$7-9/mo band, NOT the $14.99 coaching tier). Annual = 17% off (= '2 months free') as an OPTION. Proposed: CoreRX $5.99 / FullRX $7.99 monthly (a clear notch above the $4.99 logger ceiling, $2 no-brainer gap), annual ~$59.99 / ~$79.99 (2 months free). OPEN sub-decision: is the INDIVIDUAL annual discount recurring or first-year-only? (coach annual is currently first-year-only per CLAUDE.md) -- align when we do the coach prices. INDIVIDUAL PRICING LOCKED 2026-06-06: monthly subscription + 14-day trial; Free $0 / CoreRX $4.99/mo / FullRX $6.99/mo; annual = 17% off (2 months free) =&gt; CoreRX ~$49.99/yr, FullRX ~$69.99/yr (user chose the most-accessible 'notch above loggers' option). NEXT decisions: coach prices (current $19/$39/$99 monthly, 10/25/unltd clients) + align the annual-discount model (coach annual is currently 17%-off-FIRST-YEAR-ONLY per CLAUDE.md, individual annual is 17% recurring -- decide whether to unify) + free-tier feature split + then Stripe sandbox setup + billing-page build. COACH PRICES LOCKED 2026-06-06: keep Starter $19 / Pro $39 / Elite $99 monthly, caps 10/25/unltd clients, 14-day trial (already competitive vs TrueCoach/Trainerize; don't scare early coaches). PENDING: annual-discount model -- unify to RECURRING 17% (2 months free) for BOTH coaches + individuals, or keep coach annual as 17%-off-first-year-only? RESOLVED: RECURRING 17% (2 months free) for BOTH. Coach annual is NO LONGER first-year-only -&gt; permanent 17% off, renews at the same discounted annual (no year-2 jump): coach annual ~$189/$389/$989 RECURRING; individual ~$49.99/$69.99 recurring. IMPL TO-DO: REVERSE the CLAUDE.md 'coach annual 17% off first year only, renews full' lock to recurring; strip the year-2 renewal figures ($228/$468/$1188) + every 'first year' disclaimer from CoachAgreement / RefundPolicy / CoachPricing / coach Signup; set Stripe annual prices to the flat recurring annual. === FULL PRICING LOCKED 2026-06-06: monthly-subscription model for ALL (no one-time/lifetime); 14-day trial both. Individual: Free $0 / CoreRX $4.99 / FullRX $6.99 monthly (annual 17% recurring ~$49.99 / ~$69.99). Coach: Starter $19 / Pro $39 / Elite $99 monthly, 10/25/unltd clients (annual 17% recurring ~$189 / ~$389 / ~$989). REMAINING: free-tier feature split (code currently inconsistent) -&gt; then Stripe sandbox products/prices -&gt; propagate prices everywhere + model-change cleanup (drop lifetime copy, retire CF webhook, fix stale tier names elite/corerx, build individual checkout) -&gt; billing page. TIER FEATURE SPLIT (from CLAUDE.md lines 2384-2393, AUTHORITATIVE -- my earlier improvised split was wrong; Mobility was removed in the June 2026 teardown so it's NOT a tier feature): Free = Strength + Cardio; CoreRX = Free + Bodyweight + Calories (body-composition + calorie/macro coaching, the two most-requested); FullRX = CoreRX + Heart + Hydration + Sleep (the wellness/recovery layer, appeals to wearable owners). The cross-domain Dashboard rollup sits in FullRX (complete picture). The feature split is UNCHANGED by the one-time-&gt;subscription move; only the model + prices change. CODE INCONSISTENCY TO FIX: the in-app gating (CoachClientDetail TIER_RANK) wrongly puts Heart in CoreRX -- must move to FullRX to match CLAUDE.md. === ATHLETE TIERS FINALIZED + LOCKED BY USER 2026-06-06 (THIS IS FINAL): Free = Strength+Cardio; CoreRX $4.99/mo ($49.99/yr) = +Bodyweight+Calories/Food; FullRX $6.99/mo ($69.99/yr) = +Heart+Hydration+Sleep+every future feature. COACH: every coach tier grants FULL FullRX access to the coach AND all their linked athletes -- tiers differ ONLY by client cap (Starter $19/10, Pro $39/25, Elite $99/unltd; annual 17% recurring $189/$389/$989). Home Dashboard = the landing/profile screen for EVERYONE, never a tier feature. User demanded a CLEAN SWEEP of all stale/contradicting references (esp. the 'semirx' old name + the 3-way-conflicting tier splits) -&gt; tracked as T097. === STEP 1 (Stripe sandbox catalog) DONE 2026-06-06: created scripts/setup-stripe-sandbox-prices.mjs (idempotent, TEST-only, refuses non-sk_test_, reads key from .env.local) + ran it. Final TEST catalog by lookup_key: corerx_monthly $4.99 / corerx_annual $49.99 (prod CoreRX), fullrx_monthly $6.99 / fullrx_annual $69.99 (prod FullRX), coach_starter_monthly $19 / coach_starter_annual $189, coach_pro_monthly $39 / coach_pro_annual $389, coach_elite_monthly $99 / coach_elite_annual $989. Coach products reused (metadata myrx_tier+myrx_audience set); coach MONTHLY already matched (left as-is, existing test subs safe); coach ANNUAL recreated as flat-recurring (old annual prices archived -- they didn't match flat $189/$389/$989, confirming the old first-year-only structure is gone). Old athlete one-time prices (corerx_onetime / fullrx_onetime) archived. The app references prices by lookup_key (&lt;tier&gt;_monthly / &lt;tier&gt;_annual), never by price_ id. Built only in Stripe TEST; no app code changed, no web deploy. NEXT = Step 2 (hosted-checkout + 14-day trial + individual subscription wiring) -- awaiting user discussion per the step-by-step agreement (do NOT start step 2 until discussed). === IAP/POLICY RESEARCH 2026-06-07 (user: 'i dont want to violate iOS/Google policies; athletes download from stores + subscribe; how do modern apps do it?') -- 3 parallel web-research agents. FINDINGS: (1) a fitness/coaching app MUST offer Apple IAP / Google Play Billing for ANY subscription unlocked INSIDE the app (Apple Guideline 3.1.1). It is NOT a 'reader app' (that web-only carve-out is magazines/music/video only -- how Netflix/Spotify sell web-only), so we CANNOT ship a web-pay-only + unlock-in-app model -&gt; instant rejection. (2) Universal unlock = ACCOUNT-BASED ENTITLEMENT: a sub (Apple IAP / Google Play / web Stripe / coach-comped) flips a tier flag on the user's ACCOUNT server-side; every client checks the account, not the store. This is exactly how our coach-&gt;client comp model already works. (3) Peers (Fitbod/Calm/Headspace/Whoop) = IAP-first, absorb the cut, frictionless in-app subscribe; some (YouTube/Duolingo) price IAP higher to cover the cut; web secondary. (4) Standard tool = RevenueCat (or Adapty/Qonversion): manages Apple/Google IAP + receipt validation + webhooks + unified cross-platform entitlement; free under $2,500/mo tracked revenue, then ~1%. (5) Fees: Apple/Google 15% (small biz &lt;$1M or after 12mo) to 30%; Stripe web ~2.9%+30c. US (post Epic v Apple 2025-26, legally provisional) now allows in-app links to a cheaper web checkout at ~0% Apple commission; EU ~5% Core Technology Commission; ROW no in-app steering + ~27%/12% external. RECOMMENDED ARCHITECTURE: account-based entitlement from day 1; individuals subscribe via Apple/Google IAP (compliant, frictionless) managed by RevenueCat; coaches stay web-Stripe (already works); add the cheaper web/Stripe individual path LATER once there's a marketing funnel (NOT hybrid day 1 -- friction + compliance surface, and RevenueCat's own test showed a 2nd web CTA netted slightly LESS per IAP dollar). BUILD REFRAME: the Step-1 Stripe individual products (corerx/fullrx) now serve the FUTURE web path; the PRIMARY individual path = mobile IAP via RevenueCat (a MOBILE build: App Store Connect + Play Console subscription products + RevenueCat account + Expo SDK + entitlement wiring + dev-account enrollment) -- bigger than a Stripe checkout. Sources: Apple App Review Guidelines, Epic v Apple 2025-26 rulings, RevenueCat/Adapty docs+benchmarks. AWAITING user pick: pivot Step 2 to the IAP/RevenueCat individual path vs continue the web-Stripe individual path first. === MODEL CLARIFIED BY USER 2026-06-07 (resolves the fork): TWO account types, two payment surfaces, ONE entitlement switch. COACHES subscribe ONLY on WEB (Stripe); a coach's active sub grants FullRX to (a) all their linked client athletes AND (b) the coach's OWN athlete account (a coach is also an athlete -- one account, role-routed: mobile = athlete view at FullRX, web = redirected to coach portal). ATHLETES (non-coach) subscribe ONLY IN-APP (Apple IAP / Google Play via RevenueCat); there is NO web checkout for athletes. CONSEQUENCE: the Step-1 Stripe corerx/fullrx ATHLETE products are now UNUSED (athletes never pay via Stripe) -&gt; archive them; only the coach_* Stripe products are used. Athlete tier products (CoreRX/FullRX monthly+annual, 14-day trial) get created in App Store Connect + Google Play Console (IAP) + mapped in RevenueCat. ENTITLEMENT (the switch) = one account-level effective tier (free/corerx/fullrx) the mobile app reads for gating, WRITTEN by BOTH the coach Stripe webhook (coach self + clients -&gt; fullrx) AND the athlete IAP/RevenueCat webhook (athlete -&gt; their tier). WORK SPLIT: (A) finish/verify the coach-&gt;FullRX unlock for coach-self + clients (web side, mostly built -- client_has_active_coach() already comps clients); (B) the athlete in-app subscription via RevenueCat (the big NEW mobile build: App Store Connect + Play Console products, RevenueCat account+SDK, paywall screen, webhook-&gt;entitlement, app gating) -- needs the user's Apple/Google/RevenueCat accounts. Recommended order: A first (small), then B step-by-step. === STEP A VERIFIED DONE 2026-06-07: resolveTier (mobile dashboard.tsx L48-58 + web CoachClientDetail/AdminUserDetail, byte-for-byte) -&gt; is_superuser/is_coach/coach_id(linked client) = fullrx, else b2c_subscription_tier ?? free. ENFORCED in-app: RadialNav gates orbit pages by tier ('coached clients get full access regardless of their own tier -- coach is paying'); dashboard gates stat pills by tierRank. So coach's own athlete account + all linked clients = FullRX + pages unlock. Matches the user's model. LAPSE GAP (flagged, not blocking): resolveTier keys off the LINK (coach_id/is_coach), NOT the coach's ACTIVE sub -- client_has_active_coach()/is_active_coach() RPCs exist but aren't used by resolveTier, so a client of a LAPSED coach stays FullRX until a lapse-downgrade is wired (launch-readiness follow-up). === STEP B STARTED (athlete in-app subscription via RevenueCat). GOOD NEWS: the READ/unlock side already exists (profiles.b2c_subscription_tier column + resolveTier already unlock pages when set), so B only needs the WRITE + purchase UI + accounts: (1) [USER accounts] Apple Developer/App Store Connect products (CoreRX/FullRX monthly+annual, 14-day trial), Google Play Console products, RevenueCat account mapping store products -&gt; corerx/fullrx entitlements; (2) [CODE] RevenueCat SDK (react-native-purchases) in the Expo app (native module -&gt; dev-client rebuild) + in-app paywall/subscribe screen; (3) [CODE] RevenueCat webhook -&gt; edge function that writes b2c_subscription_tier on the athlete's profile; (4) sandbox testing (App Store sandbox testers + Play internal test track). FIRST BLOCKER to resolve: the user's Apple Developer / Google Play / RevenueCat account status (determines where we start; code that doesn't need keys can be scaffolded meanwhile). === BLOCKER CONFIRMED 2026-06-07: user has NONE of the accounts (no Apple Developer, no Google Play, no RevenueCat) AND no iOS build ready (the app has only ever run as an Android dev-client). I CANNOT create those accounts -- they require the user's identity + payment + Apple-ID 2FA (+ a D-U-N-S for an org); creating accounts / entering financial credentials are not actions I do -- so the enrollments are the user's to do (I guide every click + do all code). The app is Expo so iOS can be built via EAS cloud (no Mac), BUT any athlete-IAP testing still needs the paid Apple account first -&gt; Apple Developer enrollment is THE gate for all athlete billing. RECOMMENDATION: user starts the Apple (~$99/yr) + Google Play (~$25 one-time) enrollments now (long lead, days), HOLD B's code until the accounts are close (so it isn't built untested + left to drift), keep building non-blocked work meanwhile (coach platform polish, the holistic dashboard rollup, etc.). Awaiting user pick: (1) start enrollment now + I prep iOS cloud-build config + scaffold the no-key parts in parallel, or (2) park B + build elsewhere until enrolled. === DEFERRED 2026-06-07 (user): the billing PAGE UI + Step B (athlete IAP) + the web pricing-CODE sweep are all DEFERRED -- user chose to finalize the web side (dashboard) first + hold dev-account enrollment. DONE so far: full pricing lock + Stripe sandbox catalog (Step 1) + Step A coach-comp verified + all doc/legal/marketing/CLAUDE.md/DB swept (T097). Resume billing from here. Spun-off follow-ups: T098 (lapse downgrade), T099 (archive unused Stripe athlete products), T100 (Efforts T086 strip).</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
@@ -5154,9 +5154,9 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E100" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>IN PROGRESS 2026-06-06: sweep CLAUDE.md first (the contract) -&gt; DB semirx-&gt;corerx CHECK migration -&gt; web display/tier code + legal + marketing. The WORKING coach Stripe plumbing (coach-signup / stripe-webhook / workers) stays untouched except semirx-&gt;corerx naming. NOTE the FUNCTIONAL subscription wiring (individual checkout, Stripe products/prices, the model switch) is the T096 build, not this naming/doc sweep -- but every STATEMENT of tiers/prices gets corrected to the lock now. DOC/LEGAL SWEEP DONE 2026-06-06: (1) CLAUDE.md swept (commit f0fbc47) -- locks 18/19/20 + Stream B + launch-checklist IAP + table descriptions now state ONLY the subscription model ($4.99/$6.99 athlete, $19/$39/$99 coach, recurring 17% annual), semirx + one-time/lifetime + first-year-only all removed. (2) DB verified ALREADY CLEAN via MCP -- b2c_purchases.tier CHECK = ('corerx','fullrx'), no semirx, table empty -&gt; NO migration needed. (3) Legal pages (CoachAgreement/RefundPolicy/TermsOfService/PrivacyPolicy) corrected to subscription + new prices + recurring annual; killed one-time/lifetime + the $228/$468/$1188 year-2 figures (kept legit coach $39 + the coach-pro $389-&gt;$292 pro-rated-refund example). (4) Marketing/brand docs (branding/BRAND.md + docs/marketing/*) corrected. 'semirx' string exists nowhere in live code/docs now (only the immutable historical migration FILE 20260524 + the spent rename-stripe script -- correctly left as history; live DB is corerx). Built+deployed index-BtVET8aQ. REMAINING = the T096 FUNCTIONAL build (not a doc fix): live pricing CODE -- Pricing.jsx ATHLETE_TIERS (still one-time/wrong-split), coachPlan.js annual framing, coach Signup/CoachPricing/ForCoaches first-year copy, CoachClientDetail TIER_RANK (Heart-&gt;FullRX), BillingView/BillingTab/AccountSettings/EditProfile -- all get the new model+prices when Stripe subscriptions + individual checkout are wired (they move together).</t>
+          <t>IN PROGRESS 2026-06-06: sweep CLAUDE.md first (the contract) -&gt; DB semirx-&gt;corerx CHECK migration -&gt; web display/tier code + legal + marketing. The WORKING coach Stripe plumbing (coach-signup / stripe-webhook / workers) stays untouched except semirx-&gt;corerx naming. NOTE the FUNCTIONAL subscription wiring (individual checkout, Stripe products/prices, the model switch) is the T096 build, not this naming/doc sweep -- but every STATEMENT of tiers/prices gets corrected to the lock now. DOC/LEGAL SWEEP DONE 2026-06-06: (1) CLAUDE.md swept (commit f0fbc47) -- locks 18/19/20 + Stream B + launch-checklist IAP + table descriptions now state ONLY the subscription model ($4.99/$6.99 athlete, $19/$39/$99 coach, recurring 17% annual), semirx + one-time/lifetime + first-year-only all removed. (2) DB verified ALREADY CLEAN via MCP -- b2c_purchases.tier CHECK = ('corerx','fullrx'), no semirx, table empty -&gt; NO migration needed. (3) Legal pages (CoachAgreement/RefundPolicy/TermsOfService/PrivacyPolicy) corrected to subscription + new prices + recurring annual; killed one-time/lifetime + the $228/$468/$1188 year-2 figures (kept legit coach $39 + the coach-pro $389-&gt;$292 pro-rated-refund example). (4) Marketing/brand docs (branding/BRAND.md + docs/marketing/*) corrected. 'semirx' string exists nowhere in live code/docs now (only the immutable historical migration FILE 20260524 + the spent rename-stripe script -- correctly left as history; live DB is corerx). Built+deployed index-BtVET8aQ. REMAINING = the T096 FUNCTIONAL build (not a doc fix): live pricing CODE -- Pricing.jsx ATHLETE_TIERS (still one-time/wrong-split), coachPlan.js annual framing, coach Signup/CoachPricing/ForCoaches first-year copy, CoachClientDetail TIER_RANK (Heart-&gt;FullRX), BillingView/BillingTab/AccountSettings/EditProfile -- all get the new model+prices when Stripe subscriptions + individual checkout are wired (they move together). === DEFERRED 2026-06-07 with T096: the doc/legal/marketing/CLAUDE.md/DB sweep is DONE + shipped; the remaining WEB PRICING-CODE sweep (Pricing.jsx tiers-&gt;subscription, coach pages first-year-&gt;recurring, gating Heart-&gt;FullRX, billing-display copy) rides with the T096 billing build (deferred).</t>
         </is>
       </c>
       <c r="H100" s="5" t="inlineStr">
@@ -5177,6 +5177,147 @@
       <c r="I100" s="5" t="inlineStr">
         <is>
           <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>T098</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>Coach-lapse downgrade: make resolveTier active-sub-aware (clients + coach-self)</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>From T096 Step-A verification: resolveTier (mobile dashboard.tsx + web CoachClientDetail/AdminUserDetail) comps coached clients + coaches to FullRX off the LINK (coach_id / is_coach), NOT the coach's ACTIVE subscription. The active-sub RPCs client_has_active_coach() / is_active_coach() EXIST but resolveTier doesn't use them -- so a client of a LAPSED coach (and a coach whose own sub lapsed) stays FullRX. Launch-readiness correctness gap.</t>
+        </is>
+      </c>
+      <c r="G101" s="7" t="inlineStr">
+        <is>
+          <t>OPEN -- before launch: make the entitlement active-sub-aware (resolveTier consults client_has_active_coach()/is_active_coach(), OR a lapse job downgrades coach_id-linked clients + coach-self) and tie into the CLAUDE.md 'pick a plan' lapse flow. NOT blocking pre-launch (everyone trial/active).</t>
+        </is>
+      </c>
+      <c r="H101" s="7" t="inlineStr">
+        <is>
+          <t>mobile dashboard.tsx resolveTier; web resolveTier (CoachClientDetail/AdminUserDetail); client_has_active_coach()/is_active_coach() RPCs</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>T099</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Archive the unused Stripe athlete products (corerx/fullrx) -- athletes pay via IAP not Stripe</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Clarified billing model: athletes subscribe ONLY in-app (Apple/Google IAP), never via Stripe. So the Stripe corerx_monthly/annual + fullrx_monthly/annual products created in T096 Step 1 are UNUSED. The coach_* Stripe products stay (coaches DO use Stripe).</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>DEFERRED with T096 (billing resume): archive the 2 athlete Stripe products in TEST mode (active=false) to avoid confusion; easy to revive if a web-athlete option is ever added.</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>scripts/setup-stripe-sandbox-prices.mjs; Stripe TEST products CoreRX/FullRX</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>T100</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>Efforts (AdminUserActivity) -- T086 athlete-education strip pass</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>AdminUserActivity (the coach Efforts tab) was reworked AFTER the 2026-06-04 T086 sweep, so it never got the 'strip athlete-only explanatory copy from web coach mirrors' pass (flagged in T086 + T079 notes, never its own trackable task).</t>
+        </is>
+      </c>
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>OPEN -- quick sweep: audit AdminUserActivity.jsx against T086 (remove attribution footers / motivational lines / how-to-log instructions / feature help-text subtitles; keep data + prescription cue + opt-in info pills), then build + deploy.</t>
+        </is>
+      </c>
+      <c r="H103" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/tabs/AdminUserActivity.jsx</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(ledger): T101 - client-detail must reopen on Dashboard tab (not last-opened)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5316,6 +5316,53 @@
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>T101</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Client-detail view must reopen on the Dashboard tab, not the last-opened tab</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-07: open a client -&gt; view a tab (e.g. Bodyweight) -&gt; leave the client -&gt; re-enter, and it reopens on the LAST tab (persisted, e.g. localStorage 'admin-user-tab-{id}' in AdminUserDetail). User wants it to ALWAYS reopen on the Dashboard tab. Fix: initialise activeTab='dashboard' on mount / stop restoring the persisted last-tab (AdminUserDetail + mirror in CoachClientDetail).</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>OPEN -- bundle with the dashboard-rollup build.</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>web AdminUserDetail.jsx (activeTab init + localStorage admin-user-tab-{id}); CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I104" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
docs(ledger): T101 done (admin reopen-on-Dashboard) + T079 Dashboard Efforts block built
T101 -> Done (admin side): activeTab always inits to dashboard, dropped the
localStorage last-tab restore (coach mirror folds into the T079 reflection batch).
T079: Dashboard rollup started - Efforts block (last 10 distinct moves, scroll,
earliest->latest, clickable to detail) shipped; remaining domain blocks are
tier-gated placeholders pending confirmation.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4320,12 +4320,12 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass. GRAPH+TILE FIX 2026-06-06 (user screenshot: dots rendered as stretched ellipse blobs + graph didn't line up with the day tiles): root cause = the web CalorieStrip CalorieGraph used a fixed 320-wide viewBox with preserveAspectRatio='none', so on the wide desktop coach card the X-axis stretched ~4x and squashed the r=4 circles into wide ovals; separately the tiles were packed at a fixed w-[58px] (left-aligned) while the graph spanned full width, so dots didn't sit under tiles. FIX: CalorieGraph now MEASURES its real pixel width (useRef + ResizeObserver) and renders the SVG at width=W height=72 with NO preserveAspectRatio (1:1 -&gt; round dots); both the tile row and the graph are laid out as N=14 equal columns separated by GAP=6px (tiles flex-1 min-w-0, no more w-[58px]/overflow-x-auto/snap; graph colCenter(i)=i*(colW+GAP)+colW/2 with colW=(W-78)/14) so each dot sits exactly under its tile. Built+deployed index-8GgKpHVX. MANUAL LOGS REMOVED + NO COACH ADD-FOOD 2026-06-06 (user: 'remove manual logs and no need for a add food in coach side'): deleted the legacy 'Manual Logs' (calorie_logs) sub-tab entirely from AdminUserCalories -- its CaloriesChart, the calorie_logs load/add/delete handlers, the 'Add entry' form, and all the now-dead state + the lucide/recharts imports. Coach Calories sub-tabs are now Overview / Food Log / Macro Plan. No food-adding anywhere on the coach side: Overview's TodayIntakeCard is already read-only (no Log-food button), Food Log is review-only. KEPT: Food Log swipe-to-delete (a correction tool, not an add) -- flagged to the user in case they want pure review. Built+deployed index-C1zY-3c_. DEAD-CODE CLEANUP 2026-06-06 (user: 'dont leave behind any dead code, clean up'): ran eslint on every touched file. CalorieStrip.jsx rewritten PURELY read-only -- removed the never-exercised interactive path (the only caller, the coach CalorieDashboard, is read-only): dropped the onDayClick/selectedIso/refreshKey props, the button-vs-div tile branch, the clickable-dot &lt;g&gt;, the 'Tap a day to log food' subtitle, the now-no-op auto-scroll useEffect + stripRef/todayRef, and the useAuth fallback (uid = userId ?? user?.id) which would have shown the COACH's own food if userId were ever missing -- now requires userId. AdminUserDetail.jsx: removed the orphaned onSaved={() =&gt; setSnapshotKey(...)} prop on &lt;AdminUserCalories&gt; (the component no longer accepts onSaved after Manual Logs was removed; setSnapshotKey is still used by the Efforts + Body tabs so it stays). eslint clean for unused-vars across CalorieStrip/CalorieDashboard/AdminUserCalories. PRE-EXISTING (left alone, not from this work): AdminUserDetail parsePace (line 82, deliberately retained legacy helper w/ a 'will retire when hasPR removed' comment) + deleteConfirm (useState value w/ used setter). Built+deployed index-CXEyiFzG.</t>
+          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass. GRAPH+TILE FIX 2026-06-06 (user screenshot: dots rendered as stretched ellipse blobs + graph didn't line up with the day tiles): root cause = the web CalorieStrip CalorieGraph used a fixed 320-wide viewBox with preserveAspectRatio='none', so on the wide desktop coach card the X-axis stretched ~4x and squashed the r=4 circles into wide ovals; separately the tiles were packed at a fixed w-[58px] (left-aligned) while the graph spanned full width, so dots didn't sit under tiles. FIX: CalorieGraph now MEASURES its real pixel width (useRef + ResizeObserver) and renders the SVG at width=W height=72 with NO preserveAspectRatio (1:1 -&gt; round dots); both the tile row and the graph are laid out as N=14 equal columns separated by GAP=6px (tiles flex-1 min-w-0, no more w-[58px]/overflow-x-auto/snap; graph colCenter(i)=i*(colW+GAP)+colW/2 with colW=(W-78)/14) so each dot sits exactly under its tile. Built+deployed index-8GgKpHVX. MANUAL LOGS REMOVED + NO COACH ADD-FOOD 2026-06-06 (user: 'remove manual logs and no need for a add food in coach side'): deleted the legacy 'Manual Logs' (calorie_logs) sub-tab entirely from AdminUserCalories -- its CaloriesChart, the calorie_logs load/add/delete handlers, the 'Add entry' form, and all the now-dead state + the lucide/recharts imports. Coach Calories sub-tabs are now Overview / Food Log / Macro Plan. No food-adding anywhere on the coach side: Overview's TodayIntakeCard is already read-only (no Log-food button), Food Log is review-only. KEPT: Food Log swipe-to-delete (a correction tool, not an add) -- flagged to the user in case they want pure review. Built+deployed index-C1zY-3c_. DEAD-CODE CLEANUP 2026-06-06 (user: 'dont leave behind any dead code, clean up'): ran eslint on every touched file. CalorieStrip.jsx rewritten PURELY read-only -- removed the never-exercised interactive path (the only caller, the coach CalorieDashboard, is read-only): dropped the onDayClick/selectedIso/refreshKey props, the button-vs-div tile branch, the clickable-dot &lt;g&gt;, the 'Tap a day to log food' subtitle, the now-no-op auto-scroll useEffect + stripRef/todayRef, and the useAuth fallback (uid = userId ?? user?.id) which would have shown the COACH's own food if userId were ever missing -- now requires userId. AdminUserDetail.jsx: removed the orphaned onSaved={() =&gt; setSnapshotKey(...)} prop on &lt;AdminUserCalories&gt; (the component no longer accepts onSaved after Manual Logs was removed; setSnapshotKey is still used by the Efforts + Body tabs so it stays). eslint clean for unused-vars across CalorieStrip/CalorieDashboard/AdminUserCalories. PRE-EXISTING (left alone, not from this work): AdminUserDetail parsePace (line 82, deliberately retained legacy helper w/ a 'will retire when hasPR removed' comment) + deleteConfirm (useState value w/ used setter). Built+deployed index-CXEyiFzG. DASHBOARD ROLLUP STARTED 2026-06-07 (the final T079 piece -- the holistic Dashboard tab that rolls the other pages into one overview). User spec for the layout: blocks ordered SAME as the page/nav sequence; Efforts (strength+cardio) live in ONE block (no single graph exists for dozens of movements); the other domain blocks each show their main graph + a few snapshot lines. EFFORTS BLOCK BUILT + confirmed-pending (user: 'scroll to last 10, sorted earliest-&gt;latest, every line clickable to its details page; do it and once confirmed we move on to the rest'): new web/src/components/DashboardEffortsBlock.jsx = last 10 DISTINCT moves (most-recent occurrence of each, deduped by type|baseName), reversed to earliest-&gt;latest, fixed-height scroll (max-h 240), each row clickable -&gt; /admin/user/{id}/effort/{type}/{navName} (navName strips trailing [Variant] so consolidated families route to base) + a 'View all -&gt;' to the Efforts tab. Wired into AdminUserDetail dashboard tab; the remaining domain blocks (Bodyweight/Heart/Calories/Sleep/Hydration, in nav order) are tier-gated 'coming soon' placeholders for now = 'the rest' to build after Efforts is confirmed. Committed 1390cf4, deployed index-BKgOlVxQ (live-verified). Coach reflection (CoachClientDetail) still the single deferred batch milestone.</t>
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>web/src/pages/admin/tabs/AdminUser{Sleep,Hydration,Heart}.jsx; web/src/pages/admin/AdminUserDetail.jsx; mirror mobile/app/(app)/{sleep,hydration,heart}.tsx</t>
+          <t>web/src/pages/admin/tabs/AdminUser{Sleep,Hydration,Heart}.jsx; web/src/pages/admin/AdminUserDetail.jsx; web/src/components/DashboardEffortsBlock.jsx; mirror mobile/app/(app)/{sleep,hydration,heart}.tsx</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
@@ -5342,9 +5342,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="G104" s="5" t="inlineStr">
         <is>
-          <t>OPEN -- bundle with the dashboard-rollup build.</t>
+          <t>DONE (admin side) 2026-06-07, committed 1390cf4, deployed index-BKgOlVxQ: AdminUserDetail activeTab now always inits to 'dashboard' (dropped the localStorage 'admin-user-tab-{id}' restore on mount); ?tab= URL deep-link still honored; handleTabChange no longer persists to localStorage. COACH side (CoachClientDetail.jsx) gets the same one-line fix as part of the T079 coach-reflection batch.</t>
         </is>
       </c>
       <c r="H104" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): T079 efforts-block QA tweaks + T101 back-nav regression follow-up
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -4320,7 +4320,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass. GRAPH+TILE FIX 2026-06-06 (user screenshot: dots rendered as stretched ellipse blobs + graph didn't line up with the day tiles): root cause = the web CalorieStrip CalorieGraph used a fixed 320-wide viewBox with preserveAspectRatio='none', so on the wide desktop coach card the X-axis stretched ~4x and squashed the r=4 circles into wide ovals; separately the tiles were packed at a fixed w-[58px] (left-aligned) while the graph spanned full width, so dots didn't sit under tiles. FIX: CalorieGraph now MEASURES its real pixel width (useRef + ResizeObserver) and renders the SVG at width=W height=72 with NO preserveAspectRatio (1:1 -&gt; round dots); both the tile row and the graph are laid out as N=14 equal columns separated by GAP=6px (tiles flex-1 min-w-0, no more w-[58px]/overflow-x-auto/snap; graph colCenter(i)=i*(colW+GAP)+colW/2 with colW=(W-78)/14) so each dot sits exactly under its tile. Built+deployed index-8GgKpHVX. MANUAL LOGS REMOVED + NO COACH ADD-FOOD 2026-06-06 (user: 'remove manual logs and no need for a add food in coach side'): deleted the legacy 'Manual Logs' (calorie_logs) sub-tab entirely from AdminUserCalories -- its CaloriesChart, the calorie_logs load/add/delete handlers, the 'Add entry' form, and all the now-dead state + the lucide/recharts imports. Coach Calories sub-tabs are now Overview / Food Log / Macro Plan. No food-adding anywhere on the coach side: Overview's TodayIntakeCard is already read-only (no Log-food button), Food Log is review-only. KEPT: Food Log swipe-to-delete (a correction tool, not an add) -- flagged to the user in case they want pure review. Built+deployed index-C1zY-3c_. DEAD-CODE CLEANUP 2026-06-06 (user: 'dont leave behind any dead code, clean up'): ran eslint on every touched file. CalorieStrip.jsx rewritten PURELY read-only -- removed the never-exercised interactive path (the only caller, the coach CalorieDashboard, is read-only): dropped the onDayClick/selectedIso/refreshKey props, the button-vs-div tile branch, the clickable-dot &lt;g&gt;, the 'Tap a day to log food' subtitle, the now-no-op auto-scroll useEffect + stripRef/todayRef, and the useAuth fallback (uid = userId ?? user?.id) which would have shown the COACH's own food if userId were ever missing -- now requires userId. AdminUserDetail.jsx: removed the orphaned onSaved={() =&gt; setSnapshotKey(...)} prop on &lt;AdminUserCalories&gt; (the component no longer accepts onSaved after Manual Logs was removed; setSnapshotKey is still used by the Efforts + Body tabs so it stays). eslint clean for unused-vars across CalorieStrip/CalorieDashboard/AdminUserCalories. PRE-EXISTING (left alone, not from this work): AdminUserDetail parsePace (line 82, deliberately retained legacy helper w/ a 'will retire when hasPR removed' comment) + deleteConfirm (useState value w/ used setter). Built+deployed index-CXEyiFzG. DASHBOARD ROLLUP STARTED 2026-06-07 (the final T079 piece -- the holistic Dashboard tab that rolls the other pages into one overview). User spec for the layout: blocks ordered SAME as the page/nav sequence; Efforts (strength+cardio) live in ONE block (no single graph exists for dozens of movements); the other domain blocks each show their main graph + a few snapshot lines. EFFORTS BLOCK BUILT + confirmed-pending (user: 'scroll to last 10, sorted earliest-&gt;latest, every line clickable to its details page; do it and once confirmed we move on to the rest'): new web/src/components/DashboardEffortsBlock.jsx = last 10 DISTINCT moves (most-recent occurrence of each, deduped by type|baseName), reversed to earliest-&gt;latest, fixed-height scroll (max-h 240), each row clickable -&gt; /admin/user/{id}/effort/{type}/{navName} (navName strips trailing [Variant] so consolidated families route to base) + a 'View all -&gt;' to the Efforts tab. Wired into AdminUserDetail dashboard tab; the remaining domain blocks (Bodyweight/Heart/Calories/Sleep/Hydration, in nav order) are tier-gated 'coming soon' placeholders for now = 'the rest' to build after Efforts is confirmed. Committed 1390cf4, deployed index-BKgOlVxQ (live-verified). Coach reflection (CoachClientDetail) still the single deferred batch milestone.</t>
+          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass. GRAPH+TILE FIX 2026-06-06 (user screenshot: dots rendered as stretched ellipse blobs + graph didn't line up with the day tiles): root cause = the web CalorieStrip CalorieGraph used a fixed 320-wide viewBox with preserveAspectRatio='none', so on the wide desktop coach card the X-axis stretched ~4x and squashed the r=4 circles into wide ovals; separately the tiles were packed at a fixed w-[58px] (left-aligned) while the graph spanned full width, so dots didn't sit under tiles. FIX: CalorieGraph now MEASURES its real pixel width (useRef + ResizeObserver) and renders the SVG at width=W height=72 with NO preserveAspectRatio (1:1 -&gt; round dots); both the tile row and the graph are laid out as N=14 equal columns separated by GAP=6px (tiles flex-1 min-w-0, no more w-[58px]/overflow-x-auto/snap; graph colCenter(i)=i*(colW+GAP)+colW/2 with colW=(W-78)/14) so each dot sits exactly under its tile. Built+deployed index-8GgKpHVX. MANUAL LOGS REMOVED + NO COACH ADD-FOOD 2026-06-06 (user: 'remove manual logs and no need for a add food in coach side'): deleted the legacy 'Manual Logs' (calorie_logs) sub-tab entirely from AdminUserCalories -- its CaloriesChart, the calorie_logs load/add/delete handlers, the 'Add entry' form, and all the now-dead state + the lucide/recharts imports. Coach Calories sub-tabs are now Overview / Food Log / Macro Plan. No food-adding anywhere on the coach side: Overview's TodayIntakeCard is already read-only (no Log-food button), Food Log is review-only. KEPT: Food Log swipe-to-delete (a correction tool, not an add) -- flagged to the user in case they want pure review. Built+deployed index-C1zY-3c_. DEAD-CODE CLEANUP 2026-06-06 (user: 'dont leave behind any dead code, clean up'): ran eslint on every touched file. CalorieStrip.jsx rewritten PURELY read-only -- removed the never-exercised interactive path (the only caller, the coach CalorieDashboard, is read-only): dropped the onDayClick/selectedIso/refreshKey props, the button-vs-div tile branch, the clickable-dot &lt;g&gt;, the 'Tap a day to log food' subtitle, the now-no-op auto-scroll useEffect + stripRef/todayRef, and the useAuth fallback (uid = userId ?? user?.id) which would have shown the COACH's own food if userId were ever missing -- now requires userId. AdminUserDetail.jsx: removed the orphaned onSaved={() =&gt; setSnapshotKey(...)} prop on &lt;AdminUserCalories&gt; (the component no longer accepts onSaved after Manual Logs was removed; setSnapshotKey is still used by the Efforts + Body tabs so it stays). eslint clean for unused-vars across CalorieStrip/CalorieDashboard/AdminUserCalories. PRE-EXISTING (left alone, not from this work): AdminUserDetail parsePace (line 82, deliberately retained legacy helper w/ a 'will retire when hasPR removed' comment) + deleteConfirm (useState value w/ used setter). Built+deployed index-CXEyiFzG. DASHBOARD ROLLUP STARTED 2026-06-07 (the final T079 piece -- the holistic Dashboard tab that rolls the other pages into one overview). User spec for the layout: blocks ordered SAME as the page/nav sequence; Efforts (strength+cardio) live in ONE block (no single graph exists for dozens of movements); the other domain blocks each show their main graph + a few snapshot lines. EFFORTS BLOCK BUILT + confirmed-pending (user: 'scroll to last 10, sorted earliest-&gt;latest, every line clickable to its details page; do it and once confirmed we move on to the rest'): new web/src/components/DashboardEffortsBlock.jsx = last 10 DISTINCT moves (most-recent occurrence of each, deduped by type|baseName), reversed to earliest-&gt;latest, fixed-height scroll (max-h 240), each row clickable -&gt; /admin/user/{id}/effort/{type}/{navName} (navName strips trailing [Variant] so consolidated families route to base) + a 'View all -&gt;' to the Efforts tab. Wired into AdminUserDetail dashboard tab; the remaining domain blocks (Bodyweight/Heart/Calories/Sleep/Hydration, in nav order) are tier-gated 'coming soon' placeholders for now = 'the rest' to build after Efforts is confirmed. Committed 1390cf4, deployed index-BKgOlVxQ (live-verified). Coach reflection (CoachClientDetail) still the single deferred batch milestone. EFFORTS BLOCK TWEAKED 2026-06-07 (user QA, committed 2e56170 / index-Bftuetsl): show 4 at a time (max-h 168, was 240); each row now shows date AND days-ago together ('Apr 30 - 38 days ago'); sort flipped to MOST-RECENT first (so the 4 visible without scrolling are the latest moves); title 'Recent training' -&gt; 'Recent efforts'.</t>
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="G104" s="5" t="inlineStr">
         <is>
-          <t>DONE (admin side) 2026-06-07, committed 1390cf4, deployed index-BKgOlVxQ: AdminUserDetail activeTab now always inits to 'dashboard' (dropped the localStorage 'admin-user-tab-{id}' restore on mount); ?tab= URL deep-link still honored; handleTabChange no longer persists to localStorage. COACH side (CoachClientDetail.jsx) gets the same one-line fix as part of the T079 coach-reflection batch.</t>
+          <t>DONE (admin side) 2026-06-07, committed 1390cf4, deployed index-BKgOlVxQ: AdminUserDetail activeTab now always inits to 'dashboard' (dropped the localStorage 'admin-user-tab-{id}' restore on mount); ?tab= URL deep-link still honored; handleTabChange no longer persists to localStorage. COACH side (CoachClientDetail.jsx) gets the same one-line fix as part of the T079 coach-reflection batch. REGRESSION FOLLOW-UP 2026-06-07 (committed 5040a0a / index-Cscsqrev): dropping the localStorage restore ALSO broke the move-detail back buttons -- they used to localStorage.setItem('admin-user-tab',activity)+navigate(bare client URL), which now lands on Dashboard. User: 'back from an effort detail should go to the Efforts page, not the dashboard.' Fixed AdminEffortDetail.goBack + AdminCardioDetail.onBack to navigate /admin/user/{id}?tab=activity (honored on mount); covers every strength/cardio sub-detail via the shared onBack prop.</t>
         </is>
       </c>
       <c r="H104" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): T102 profile-header redesign done; T103 settings-page rework deferred
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5363,6 +5363,100 @@
         </is>
       </c>
       <c r="I104" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>T102</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>Redesign the client-detail profile header (control grouping + sizing)</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-07: the profile-summary card crammed every control into one undifferentiated right-side pill stack (status badges, coaching switcher, message, active toggle, settings, delete -- all same size, no grouping), and the snapshot stat badges ate a big centered full-width grid. User wanted: badges squished smaller + left-aligned; the pills sorted into labeled blocks by purpose; settings moved to the conventional top-right; Active relabeled to an account-status word; Intake Plan -&gt; macro-plan set/not-set; a full makeover, not just reordering.</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-07 (committed afc2e7e / index-BbajJZEn): right side is now a settings GEAR (top-right, icon-only) over a 2x2 grid of labeled ControlGroups -- ACCOUNT (Active/Suspended toggle, relabeled from Active/Inactive), COACHING (the AthleteCoachingChip), PLAN (Macro plan set / No macro plan + Goal reached, relabeled from Intake Plan/Goal), MESSAGING (chat on/off + Message athlete). New ControlGroup helper (tiny uppercase caption over its controls). SnapshotBadge shrunk (rounded-full, px-2 py-0.5, text-[10px], no w-48%/min-h) + the badge row left-aligned (dropped justify-center). DELETE moved out of the header into the settings drawer's new 'Danger zone' slot (ClientSettingsDrawer gained a `dangerZone` prop; AdminUserDetail passes the Delete / Cancel-scheduled-deletion button, which closes the drawer then opens the existing confirm modal) -- mobile parity, per the user. Account status banners (suspended / scheduled-deletion / deleted) unchanged. Header row switched items-center -&gt; items-start so the taller control column top-aligns. NOTE: this is the ADMIN view; the coach view (CoachClientDetail) gets it in the T079 coach-reflection batch.</t>
+        </is>
+      </c>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/AdminUserDetail.jsx (SnapshotBadge + ControlGroup + profile card); web/src/components/ClientSettingsDrawer.jsx (dangerZone slot)</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>T103</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Settings drawer/page full rework (3-tab Account/Preferences/Security + Delete home)</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-07 (while redesigning the profile header): 'the delete should be inside the settings like it is in mobile, but we're doing a whole settings page work after this anyways.' So Delete was given an interim home in the settings drawer's Danger zone (T102), but the broader settings overhaul is a separate upcoming task. ClientSettingsDrawer's own docstring already scopes v2: split into 3 tabs (Account / Preferences / Security), Security tab gets admin-only support actions (send password reset, disable biometric on all devices) the client can't self-serve, coach mode goes read-only.</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>DEFERRED -- pick up after the current header/dashboard polish pass. Will formalize Delete + account-lifecycle actions inside the reworked settings (not just the interim Danger-zone slot), add the 3-tab structure, and mirror to the coach view. Whether settings stays a drawer or becomes a full page is part of this task.</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>web/src/components/ClientSettingsDrawer.jsx; web/src/components/AccountSettings.jsx; mirror coach/CoachClientDetail.jsx</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
docs(ledger): T104 admin-action activity logging done; T102 v3 header tweaks
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>DONE 2026-06-07 (committed afc2e7e / index-BbajJZEn): right side is now a settings GEAR (top-right, icon-only) over a 2x2 grid of labeled ControlGroups -- ACCOUNT (Active/Suspended toggle, relabeled from Active/Inactive), COACHING (the AthleteCoachingChip), PLAN (Macro plan set / No macro plan + Goal reached, relabeled from Intake Plan/Goal), MESSAGING (chat on/off + Message athlete). New ControlGroup helper (tiny uppercase caption over its controls). SnapshotBadge shrunk (rounded-full, px-2 py-0.5, text-[10px], no w-48%/min-h) + the badge row left-aligned (dropped justify-center). DELETE moved out of the header into the settings drawer's new 'Danger zone' slot (ClientSettingsDrawer gained a `dangerZone` prop; AdminUserDetail passes the Delete / Cancel-scheduled-deletion button, which closes the drawer then opens the existing confirm modal) -- mobile parity, per the user. Account status banners (suspended / scheduled-deletion / deleted) unchanged. Header row switched items-center -&gt; items-start so the taller control column top-aligns. NOTE: this is the ADMIN view; the coach view (CoachClientDetail) gets it in the T079 coach-reflection batch. V2 REDESIGN 2026-06-07 (user rejected v1: 'too much empty space, titles literally saying what the pill already states'; asked how a modern app would do it from scratch, unconstrained by current pills/colors): replaced the labeled 2x2 ControlGroup grid with a record-header pattern (Linear/Stripe/Intercom style). Identity top-left; a single self-describing INLINE STATUS LINE under the email with NO captions (colored-dot Active/Suspended toggle, the coaching dropdown, 'Macro plan set'/'No macro plan' + 'Goal reached' as informative text, chat on/off toggle); and a right ACTION CLUSTER = primary lime Message button + Settings gear icon. Split by interaction type: informative text vs toggles vs open-panel actions (no redundant section titles, no empty grid). Removed the now-unused ControlGroup helper. Committed 318cb77 / index-36CFD12C.</t>
+          <t>DONE 2026-06-07 (committed afc2e7e / index-BbajJZEn): right side is now a settings GEAR (top-right, icon-only) over a 2x2 grid of labeled ControlGroups -- ACCOUNT (Active/Suspended toggle, relabeled from Active/Inactive), COACHING (the AthleteCoachingChip), PLAN (Macro plan set / No macro plan + Goal reached, relabeled from Intake Plan/Goal), MESSAGING (chat on/off + Message athlete). New ControlGroup helper (tiny uppercase caption over its controls). SnapshotBadge shrunk (rounded-full, px-2 py-0.5, text-[10px], no w-48%/min-h) + the badge row left-aligned (dropped justify-center). DELETE moved out of the header into the settings drawer's new 'Danger zone' slot (ClientSettingsDrawer gained a `dangerZone` prop; AdminUserDetail passes the Delete / Cancel-scheduled-deletion button, which closes the drawer then opens the existing confirm modal) -- mobile parity, per the user. Account status banners (suspended / scheduled-deletion / deleted) unchanged. Header row switched items-center -&gt; items-start so the taller control column top-aligns. NOTE: this is the ADMIN view; the coach view (CoachClientDetail) gets it in the T079 coach-reflection batch. V2 REDESIGN 2026-06-07 (user rejected v1: 'too much empty space, titles literally saying what the pill already states'; asked how a modern app would do it from scratch, unconstrained by current pills/colors): replaced the labeled 2x2 ControlGroup grid with a record-header pattern (Linear/Stripe/Intercom style). Identity top-left; a single self-describing INLINE STATUS LINE under the email with NO captions (colored-dot Active/Suspended toggle, the coaching dropdown, 'Macro plan set'/'No macro plan' + 'Goal reached' as informative text, chat on/off toggle); and a right ACTION CLUSTER = primary lime Message button + Settings gear icon. Split by interaction type: informative text vs toggles vs open-panel actions (no redundant section titles, no empty grid). Removed the now-unused ControlGroup helper. Committed 318cb77 / index-36CFD12C. V3 TWEAKS 2026-06-07 (committed 3a1959a / index-DCKT1jNE, user feedback on v2): (1) Active + Chat status items now bordered pills so they read as clickable toggles (were borderless, 'didn't look like a button'); (2) faint '·' separators between status-line items; (3) goal wording 'Goal reached' -&gt; 'Macro plan goal reached' (Macro plan set stays shown alongside); (4) snapshot badges bigger (flex-1 + min-w-110 + px-2.5 py-1.5 text-[11px] rounded-lg) so they fill the bottom line edge-to-edge.</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
@@ -5457,6 +5457,53 @@
         </is>
       </c>
       <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>T104</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Log admin account actions to the activity feed</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-07: clicked the Active toggle and nothing appeared in the Activity Feed -- 'everything should write in the activity feed, even the delete account, double check on this.' VERIFIED via DB (mcp): the timeline reads the `activity_events` table (id uuid, user_id, event_type, event_data jsonb, source, caused_by, occurred_at) -- NOT user_activity_events (a separate, mostly-unused table). Delete (account:deletion_scheduled/cancelled/deleted) and coaching (coach:assigned/detached/swapped) ALREADY log via their RPCs (schedule_account_deletion / cancel_scheduled_deletion / admin_set_athlete_coaching all insert into activity_events). The real gaps: ACTIVATE/SUSPEND (runs through the admin-user-management edge fn, never logged) and CHAT enable/disable (toggleChat does a direct profiles update, never logged).</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-07 (committed 3a1959a; migration log_admin_activity_rpc): new SECURITY DEFINER public.log_admin_activity(p_user_id uuid, p_event_type text, p_event_data jsonb) inserts into activity_events matching the existing pattern (source='admin', caused_by=auth.uid()); definer is required because activity_events has SELECT-only RLS (no INSERT policy). Guard = is_admin() OR is_active_coach() (is_admin() = profiles.is_superuser, so admins pass). toggleActive + toggleChat now call it best-effort (.then(ok,err) so a log failure never surfaces as an action error) with event types account:activated / account:deactivated / chat:enabled / chat:disabled; added getActivityMeta timeline labels for all four (Power / MessageCircle icons). FOLLOW-UP: settings-form edits (AccountSettings) + any other admin mutations should also log -- fold into the T103 settings rework. Coach view gets the same in the T079 coach-reflection batch.</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>supabase migration log_admin_activity_rpc; web/src/pages/admin/AdminUserDetail.jsx (toggleActive/toggleChat log calls + getActivityMeta cases)</t>
+        </is>
+      </c>
+      <c r="I107" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
docs(ledger): fix log_admin_activity source CHECK (admin->rpc); suspend/chat now log
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -5495,12 +5495,12 @@
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>DONE 2026-06-07 (committed 3a1959a; migration log_admin_activity_rpc): new SECURITY DEFINER public.log_admin_activity(p_user_id uuid, p_event_type text, p_event_data jsonb) inserts into activity_events matching the existing pattern (source='admin', caused_by=auth.uid()); definer is required because activity_events has SELECT-only RLS (no INSERT policy). Guard = is_admin() OR is_active_coach() (is_admin() = profiles.is_superuser, so admins pass). toggleActive + toggleChat now call it best-effort (.then(ok,err) so a log failure never surfaces as an action error) with event types account:activated / account:deactivated / chat:enabled / chat:disabled; added getActivityMeta timeline labels for all four (Power / MessageCircle icons). FOLLOW-UP: settings-form edits (AccountSettings) + any other admin mutations should also log -- fold into the T103 settings rework. Coach view gets the same in the T079 coach-reflection batch.</t>
+          <t>DONE 2026-06-07 (committed 3a1959a; migration log_admin_activity_rpc): new SECURITY DEFINER public.log_admin_activity(p_user_id uuid, p_event_type text, p_event_data jsonb) inserts into activity_events matching the existing pattern (source='admin', caused_by=auth.uid()); definer is required because activity_events has SELECT-only RLS (no INSERT policy). Guard = is_admin() OR is_active_coach() (is_admin() = profiles.is_superuser, so admins pass). toggleActive + toggleChat now call it best-effort (.then(ok,err) so a log failure never surfaces as an action error) with event types account:activated / account:deactivated / chat:enabled / chat:disabled; added getActivityMeta timeline labels for all four (Power / MessageCircle icons). FOLLOW-UP: settings-form edits (AccountSettings) + any other admin mutations should also log -- fold into the T103 settings rework. Coach view gets the same in the T079 coach-reflection batch. FIX 2026-06-07 (user: 'account suspension still didnt log'): the first RPC version used source='admin', but activity_events has CHECK (source IN ('trigger','rpc','client','webhook','system')) -- so EVERY admin-log insert silently failed (the client swallows the RPC error best-effort). Migration log_admin_activity_fix_source switched source to 'rpc' (it IS an RPC, matching schedule_account_deletion; admin attribution stays in event_data.admin_initiated + caused_by). Verified via a probe insert that the table accepts (account:deactivated / source=rpc passes both the source CHECK and the event_type-format CHECK ^[a-z_]+:[a-z_]+...). DB-ONLY fix -- no web redeploy; the already-deployed client now logs on the next toggle. Event_type format CHECK is why types must be lowercase domain:action (account:deactivated, chat:enabled -- all valid).</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
         <is>
-          <t>supabase migration log_admin_activity_rpc; web/src/pages/admin/AdminUserDetail.jsx (toggleActive/toggleChat log calls + getActivityMeta cases)</t>
+          <t>supabase migrations log_admin_activity_rpc + log_admin_activity_fix_source; web/src/pages/admin/AdminUserDetail.jsx (toggleActive/toggleChat log calls + getActivityMeta cases)</t>
         </is>
       </c>
       <c r="I107" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(messages): open transcript on mobile deep-link + instant scroll-to-latest on open
Admin + coach Messages pages (AdminMessages.jsx, CoachMessages.jsx):
- Deep-link (?userId= / ?clientId=) now sets showList=false so the mobile
  view reveals the transcript panel instead of staying on the conversation
  list. Desktop unaffected (both panes always render at md+).
- Scroll-to-bottom is instant (behavior:'auto') on conversation open/switch
  instead of smoothly animating top->bottom; new live messages in an open
  conversation still scroll smoothly (tracked via prevSelectedRef).

Fixed on both surfaces per the cross-platform bug rule. T105.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5504,6 +5504,53 @@
         </is>
       </c>
       <c r="I107" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>T105</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Messages page: deep-link doesn't open transcript on mobile; conversation scrolls top-to-bottom on open</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-07: (1) 'when i clicked on the message button on mobile web, it took me to the messages page, but it didnt open the message page of the client'; (2) 'even on desktop web, when i click on a client's msg page, it opens the page, but scrolls from top to bottom instead of opening directly to the latest msg.' Two distinct bugs in AdminMessages.jsx MessagesTab. (1) MOBILE DEEP-LINK: the split layout uses a `showList` state -- on a narrow screen the client list shows when showList=true (`${showList ? 'flex' : 'hidden'} md:flex`) and the transcript panel shows when showList=false (`${!showList ? 'flex' : 'hidden'} md:flex`). List-row clicks go through selectConversation(uid) which sets selectedId AND showList=false. But the `?userId=` deep-link handler (fired by the 'Message athlete' pill on AdminUserDetail) called setSelectedId(target) directly, bypassing selectConversation -- so showList stayed true and mobile kept showing the list. (2) SCROLL: the scroll-to-bottom effect used `behavior: 'smooth'` on EVERY run, including conversation-open, so opening a chat animated the whole transcript top-&gt;bottom (reads as a 'where am I' scroll). Desktop shows both panes so the mobile bug wasn't visible there, but the smooth-on-open scroll was.</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-07 (deploy index-JF861ybb.js -&gt; index-CeCe7Exe.js after the coach twin fix; live hash verified == local on myrxfit.com both times). Fixed on BOTH the admin (AdminMessages.jsx) AND coach (CoachMessages.jsx) surfaces in the same turn -- per the cross-platform bug rule (a reported bug gets fixed on every surface where it exists), and because CoachMessages is an ALREADY-SHIPPED standalone page (NOT part of the deferred T079 client-detail reflection batch). It mirrors AdminMessages line-for-line and had both identical bugs live (coach deep-link key is ?clientId= from the CoachClientDetail 'Message athlete' pill; admin is ?userId= from AdminUserDetail). (1) deep-link handler now also calls setShowList(false) when a match is found, so mobile reveals the transcript panel (desktop unaffected -- both panes always render at md+). (2) scroll effect tracks the previous selectedId via a new prevSelectedRef; conversation OPEN/SWITCH (selectedId changed) -&gt; `behavior:'auto'` (instant jump to newest), new message while same conversation open (messages changed, selectedId same) -&gt; `behavior:'smooth'` (incoming bubble glides in). Typing still never scrolls (unchanged). Both fixes are pure client UI -- no DB/RPC. WORKTREE TRAP NOTE: Glob('web/src/pages/coach/CoachMessages.jsx') returned 'No files found' because Glob defaults to the stale worktree CWD (.claude/worktrees/tender-tharp-e1109d) which lacks the coach pages; the file exists in MAIN. Always edit/build via absolute C:/Users/motaz/OneDrive/Desktop/MyRX/... paths (per the T080 multi-worktree lesson).</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/AdminMessages.jsx + web/src/pages/coach/CoachMessages.jsx (both: deep-link setShowList(false); prevSelectedRef instant-vs-smooth scroll)</t>
+        </is>
+      </c>
+      <c r="I108" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
fix(activity-feed): align icon colors to each domain's canonical app-wide color
The Activity Feed picked per-event colors that disagreed with the palette
used everywhere else (dashboard blocks + Efforts filter pills):
- bodyweight: purple -> emerald (green, matches Bodyweight everywhere)
- efforts: now splits on type -> cardio amber+Activity, strength blue+Dumbbell
  (matches the AdminUserActivity Strength|Cardio pills)
- wearable workout: emerald -> amber (cardio session; emerald is bodyweight's)
- DashboardEffortsBlock cardio dot: orange-400 -> amber-400 (canonical cardio)

Account/billing/chat lifecycle rows keep their semantic palette (no per-domain
color exists for them). T106.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5551,6 +5551,53 @@
         </is>
       </c>
       <c r="I108" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>T106</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>Activity feed icon colors must match each domain's canonical app-wide color</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-07: 'the activity feed uses different colors for some icons ... some icons that are green on other pages are another color in the feed, the weight which should be green is purple, the cardio which is supposed to be amber is something else, check other pages colors.' The Activity Feed's describe() (AdminUserDetail.jsx) hand-picked per-event colors that disagreed with the domain palette every OTHER surface uses. Audited the canonical colors: bodyweight=emerald (DashboardBodyweightBlock Scale + AdminUserBody), calories=amber (DashboardCaloriesBlock Apple), heart=red (DashboardHeartBlock), sleep=indigo (DashboardSleepBlock), hydration=cyan (DashboardHydrationBlock), strength=blue + cardio=amber (AdminUserActivity filter pills L195-196: strength text-blue-400 / cardio text-amber-400 + Activity icon; locked in CLAUDE.md 'strength keeps blue, cardio keeps amber'). Feed offenders: training:bodyweight_insert was purple-400 (should be emerald), training:efforts_insert was always blue-400 regardless of type (a CARDIO effort should be amber, not blue), training:wearable_workouts_insert was emerald-400 (emerald is bodyweight's color now; a wearable workout is a cardio session -&gt; amber). Also found a sibling: DashboardEffortsBlock's per-row cardio dot used bg-orange-400 (non-canonical) instead of amber.</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-07 (deploy index-BDgD5a74.js, live hash verified == local). AdminUserDetail.jsx describe(): (1) training:efforts_insert now SPLITS on d.type -- cardio -&gt; Activity icon + text-amber-400, strength -&gt; Dumbbell + text-blue-400 (exactly the AdminUserActivity Strength|Cardio pill colors+icons); (2) training:bodyweight_insert purple-400 -&gt; emerald-400; (3) training:wearable_workouts_insert emerald-400 -&gt; amber-400 (cardio domain; Activity icon already matched). DashboardEffortsBlock.jsx: cardio row-dot bg-orange-400 -&gt; bg-amber-400. Left UNTOUCHED (correctly): the account/billing/chat lifecycle rows keep their SEMANTIC palette (emerald=positive, red=failure/destructive, amber=warning, zinc/muted=neutral) -- those events have no per-domain color elsewhere and the user didn't flag them; and the non-domain orange/purple schemes in AdminMovements (equipment-type badges: Carry=orange, Assisted=purple) + AdminDashboard ('no-nutrition' flag=orange) which are their own internally-consistent category schemes, not activity-domain colors. SCOPE: the Activity Feed currently lives ONLY in AdminUserDetail (CoachClientDetail has no Activity tab yet -- 4-tab Dashboard/Efforts/Bodyweight/Calories), so no coach twin to mirror today; the DashboardEffortsBlock fix is a shared component so it's automatically correct wherever it renders (incl. future coach use). NOTE: clarified mid-task via AskUserQuestion (uniform vs semantic) -- user rejected both framings and specified the real ask = match other-page domain colors; built to that.</t>
+        </is>
+      </c>
+      <c r="H109" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/AdminUserDetail.jsx (describe() training rows); web/src/components/DashboardEffortsBlock.jsx (cardio dot)</t>
+        </is>
+      </c>
+      <c r="I109" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
style(calories): use the apple icon for calories across web + mobile (icon-only)
Swap the calorie/food domain icon from flame to apple everywhere it appeared,
keeping every color exactly as-is (no color edits):
- web: CalorieDashboard hero + empty-state, Navbar Calories item
- mobile: calories.tsx hero + 2 empty states, dashboard calorie feed + streak chip

Main cals icons were already red -> now red apples. Macro Fat amber, near-target
status amber, pending Clock, and energy-balance colors all left untouched. T107.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5598,6 +5598,53 @@
         </is>
       </c>
       <c r="I109" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>T107</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Calorie/food domain icon = Apple across all cal pages (web + mobile), icon-only</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>Web+Mobile</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-07: 'lets reflect it on all cal pages on web and mobile.' MISFIRE: I read 'it' as the calories=red COLOR and started a broad amber-&gt;red audit/migration across all calorie surfaces. User interrupted: 'what are you doing, i didnt ask to change any colors, i just said change the icon for cals to be the apple, keep all colors as they were.' Then clarified the end state via the follow-up question: 'food logging and cals are apple and red.' So the ACTUAL ask was ICON-ONLY: make the calorie/food domain icon the APPLE everywhere it was a Flame, and keep EVERY color exactly as-is (the main cals icons are already red from T106's b4fa286, so they become red apples; the macro Fat amber, the near-target traffic-light amber, the pending Clock amber, and the energy-balance hues all stay). NO color edits at all this round.</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-07 (web deploy index-BY06pom1.js, live hash verified == local; mobile tsc --noEmit clean). Audited every calorie/food surface on both platforms via 2 parallel read-only agents first (classified each amber as DOMAIN-ACCENT vs MACRO-COLOR(Fat) vs STATUS-TRAFFIC-LIGHT(near-target) vs ENERGY-BALANCE vs OTHER) so I'd touch ONLY the domain icon and nothing else. Flame-&gt;Apple swaps, colors preserved verbatim: WEB -- CalorieDashboard.jsx hero (was Flame+red-&gt;Apple+red) + empty-state 'No intake plan yet' (Flame+amber-&gt;Apple+amber, color kept), Navbar.jsx Calories nav item (Flame-&gt;Apple). MOBILE -- calories.tsx hero (Flame+red-&gt;Apple+red), 2 empty states 'Set up your plan' + 'Set a new plan' (Flame+amber-&gt;Apple+amber, color kept), dashboard.tsx calorie feed row (Flame+red-&gt;Apple+red) + food-streak chip both states (Flame red/muted-&gt;Apple, colors kept). Each file's lucide import Flame-&gt;Apple (Flame fully unused after). LEFT UNTOUCHED per 'keep all colors': macro Fat=amber (calories.tsx/CalorieDashboard/FoodLogDrawer/MacroPlanEditor/PlanWizardSheet), near-target traffic-light amber (CalorieStrip status dot + CalorieTrendGraph band), the mobile PendingView Clock 'your plan is on its way' (it's a waiting STATUS, stays a Clock+amber, NOT the calorie icon), energy-balance emerald/blue, and the food-logging RED from T106/b4fa286 (user confirmed 'apple and red' -&gt; kept). The DashboardCaloriesBlock + activity-feed food rows were ALREADY apple+red from b4fa286, no change. PROCESS SCARS (self-inflicted, fixed in-turn): twice botched a replace_all by dropping the trailing space in new_string ('&lt;Flame className="h-4 w-4 ' -&gt; '&lt;Apple className="h-4 w-4' gave 'w-4text-...'; '&lt;Flame ' -&gt; '&lt;Apple' gave '&lt;Applesize='); caught both via grep and repaired. Also hit 'File has not been read yet' on Navbar.jsx (only grepped, never Read) -- had to Read before Edit. NOTE: the empty-state apples are still AMBER (kept per 'keep all colors'); if the user wants those red too it's a 1-line follow-up. Web end-user Navbar.jsx was included for completeness (App.jsx still wires it) though web end-user surfaces are largely deprecated.</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>web/src/components/CalorieDashboard.jsx; web/src/components/Navbar.jsx; mobile/app/(app)/calories.tsx; mobile/app/(app)/dashboard.tsx</t>
+        </is>
+      </c>
+      <c r="I110" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
style(calories): apple icon for calories everywhere it was still a flame
Follow-up sweep after "the radialnav still has flame" — grepped the whole
codebase and swapped every remaining calorie/food flame to the apple icon,
colors kept:
- mobile RadialNav calories menu entry
- web AdminFeed calorie row, AdminOverview calorie feed icon + Nutrition stat
- web AdminUserDetail + CoachClientDetail food snapshot badges
- web Landing "Calorie lab" card

Only flame left is AdminDashboard "On a Streak" (training-streak fire, kept). T107.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -570,7 +570,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-07 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
+          <t>Cross-session ledger of every task (done + pending). Stable IDs — refer back with 'pick up T0xx'. Generated 2026-06-08 by scripts/build_task_pipeline_xlsx.py — edit that script's TASKS list + re-run to update.</t>
         </is>
       </c>
     </row>
@@ -5636,7 +5636,7 @@
       </c>
       <c r="G110" s="5" t="inlineStr">
         <is>
-          <t>DONE 2026-06-07 (web deploy index-BY06pom1.js, live hash verified == local; mobile tsc --noEmit clean). Audited every calorie/food surface on both platforms via 2 parallel read-only agents first (classified each amber as DOMAIN-ACCENT vs MACRO-COLOR(Fat) vs STATUS-TRAFFIC-LIGHT(near-target) vs ENERGY-BALANCE vs OTHER) so I'd touch ONLY the domain icon and nothing else. Flame-&gt;Apple swaps, colors preserved verbatim: WEB -- CalorieDashboard.jsx hero (was Flame+red-&gt;Apple+red) + empty-state 'No intake plan yet' (Flame+amber-&gt;Apple+amber, color kept), Navbar.jsx Calories nav item (Flame-&gt;Apple). MOBILE -- calories.tsx hero (Flame+red-&gt;Apple+red), 2 empty states 'Set up your plan' + 'Set a new plan' (Flame+amber-&gt;Apple+amber, color kept), dashboard.tsx calorie feed row (Flame+red-&gt;Apple+red) + food-streak chip both states (Flame red/muted-&gt;Apple, colors kept). Each file's lucide import Flame-&gt;Apple (Flame fully unused after). LEFT UNTOUCHED per 'keep all colors': macro Fat=amber (calories.tsx/CalorieDashboard/FoodLogDrawer/MacroPlanEditor/PlanWizardSheet), near-target traffic-light amber (CalorieStrip status dot + CalorieTrendGraph band), the mobile PendingView Clock 'your plan is on its way' (it's a waiting STATUS, stays a Clock+amber, NOT the calorie icon), energy-balance emerald/blue, and the food-logging RED from T106/b4fa286 (user confirmed 'apple and red' -&gt; kept). The DashboardCaloriesBlock + activity-feed food rows were ALREADY apple+red from b4fa286, no change. PROCESS SCARS (self-inflicted, fixed in-turn): twice botched a replace_all by dropping the trailing space in new_string ('&lt;Flame className="h-4 w-4 ' -&gt; '&lt;Apple className="h-4 w-4' gave 'w-4text-...'; '&lt;Flame ' -&gt; '&lt;Apple' gave '&lt;Applesize='); caught both via grep and repaired. Also hit 'File has not been read yet' on Navbar.jsx (only grepped, never Read) -- had to Read before Edit. NOTE: the empty-state apples are still AMBER (kept per 'keep all colors'); if the user wants those red too it's a 1-line follow-up. Web end-user Navbar.jsx was included for completeness (App.jsx still wires it) though web end-user surfaces are largely deprecated.</t>
+          <t>DONE 2026-06-07 (web deploy index-BY06pom1.js, live hash verified == local; mobile tsc --noEmit clean). Audited every calorie/food surface on both platforms via 2 parallel read-only agents first (classified each amber as DOMAIN-ACCENT vs MACRO-COLOR(Fat) vs STATUS-TRAFFIC-LIGHT(near-target) vs ENERGY-BALANCE vs OTHER) so I'd touch ONLY the domain icon and nothing else. Flame-&gt;Apple swaps, colors preserved verbatim: WEB -- CalorieDashboard.jsx hero (was Flame+red-&gt;Apple+red) + empty-state 'No intake plan yet' (Flame+amber-&gt;Apple+amber, color kept), Navbar.jsx Calories nav item (Flame-&gt;Apple). MOBILE -- calories.tsx hero (Flame+red-&gt;Apple+red), 2 empty states 'Set up your plan' + 'Set a new plan' (Flame+amber-&gt;Apple+amber, color kept), dashboard.tsx calorie feed row (Flame+red-&gt;Apple+red) + food-streak chip both states (Flame red/muted-&gt;Apple, colors kept). Each file's lucide import Flame-&gt;Apple (Flame fully unused after). LEFT UNTOUCHED per 'keep all colors': macro Fat=amber (calories.tsx/CalorieDashboard/FoodLogDrawer/MacroPlanEditor/PlanWizardSheet), near-target traffic-light amber (CalorieStrip status dot + CalorieTrendGraph band), the mobile PendingView Clock 'your plan is on its way' (it's a waiting STATUS, stays a Clock+amber, NOT the calorie icon), energy-balance emerald/blue, and the food-logging RED from T106/b4fa286 (user confirmed 'apple and red' -&gt; kept). The DashboardCaloriesBlock + activity-feed food rows were ALREADY apple+red from b4fa286, no change. PROCESS SCARS (self-inflicted, fixed in-turn): twice botched a replace_all by dropping the trailing space in new_string ('&lt;Flame className="h-4 w-4 ' -&gt; '&lt;Apple className="h-4 w-4' gave 'w-4text-...'; '&lt;Flame ' -&gt; '&lt;Apple' gave '&lt;Applesize='); caught both via grep and repaired. Also hit 'File has not been read yet' on Navbar.jsx (only grepped, never Read) -- had to Read before Edit. NOTE: the empty-state apples are still AMBER (kept per 'keep all colors'); if the user wants those red too it's a 1-line follow-up. Web end-user Navbar.jsx was included for completeness (App.jsx still wires it) though web end-user surfaces are largely deprecated. FOLLOW-UP SWEEP 2026-06-08 (user: 'the radialnav still has flame' -&gt; then I did the comprehensive grep I should have done first; web deploy index-DPvTfNbU.js verified, mobile tsc clean): my first pass only covered the calorie PAGES (the 2 audit agents scoped to pages, not nav/feed/overview/landing components), so I MISSED several calorie-domain Flames. Fixed them all in one sweep, Flame-&gt;Apple, colors kept: mobile/src/components/RadialNav.tsx (the radial nav menu Calories entry — what the user caught), web AdminFeed.jsx (calorie feed-row icon, red), web AdminOverview.jsx (calorie feed icon + 'Nutrition Active' stat, red), web AdminUserDetail.jsx (food snapshot badges L1168/1173, red/muted), web CoachClientDetail.jsx (food snapshot badges L560/565, red/muted), web Landing.jsx ('Calorie lab' feature card). Removed the now-unused Flame import from each (Apple already imported in AdminUserDetail/CoachClientDetail; replaced Flame-&gt;Apple in the import for AdminFeed/AdminOverview/Landing/RadialNav). The ONLY Flame left app-wide is AdminDashboard.jsx 'On a Streak' (3+ consecutive weeks) -- that's the training-STREAK fire metaphor, NOT calories, correctly kept. LESSON (logged so the next color/icon-domain task starts right): when a request is 'reflect X across the whole app', grep the ENTIRE codebase for the token FIRST (grep -rn 'Flame' web/src mobile) and classify every hit, instead of scoping to the obvious 'pages' -- nav menus / feed config maps / overview stat tiles / landing cards / snapshot badges all carry domain icons too. PROCESS SCAR (repeat of T107's earlier one): botched the badge replace_all THREE times by dropping the trailing space in new_string ('shrink-0 ' -&gt; 'shrink-0' gave 'shrink-0text-'); always keep old_string and new_string boundary-aligned on whitespace, or include the char after the space.</t>
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(settings): coach-lockdown safety + tab-position + support-button error states
Phase 1 of the admin client-settings mirror (T103):
- change-password form gated to self-mode only (was !isAdminMode) so a coach
  editing a client can never silently change their own password
- client-settings drawer uses its own persisted-tab key so closing it no longer
  wipes the admin's own /admin/profile tab choice
- "send reset / email-change" buttons now check the result and show "Failed —
  try again" instead of always showing "Sent ✓"

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Settings drawer/page full rework (3-tab Account/Preferences/Security + Delete home)</t>
+          <t>Admin client-settings mirror — admin edits a client's settings from the client detail page</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
@@ -5433,32 +5433,32 @@
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>Web</t>
-        </is>
-      </c>
-      <c r="E106" s="10" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+          <t>Web+Mobile</t>
+        </is>
+      </c>
+      <c r="E106" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>User 2026-06-07 (while redesigning the profile header): 'the delete should be inside the settings like it is in mobile, but we're doing a whole settings page work after this anyways.' So Delete was given an interim home in the settings drawer's Danger zone (T102), but the broader settings overhaul is a separate upcoming task. ClientSettingsDrawer's own docstring already scopes v2: split into 3 tabs (Account / Preferences / Security), Security tab gets admin-only support actions (send password reset, disable biometric on all devices) the client can't self-serve, coach mode goes read-only.</t>
+          <t>User 2026-06-08: 'lets start working on the client detail settings page ... as an admin i need to access a clients details page to check on their settings as they set it and do any required changes ... it needs to mirror the client's exactly ... there could be things that as an admin i cant change ... this does not mirror on the coach, only admin can change client's settings.' AUDITED both ends via 2 parallel agents. CLIENT SETTINGS (mobile is source of truth; the live file is mobile/app/(app)/settings.tsx, NOT profile.tsx — renamed May 28 2026): 6 tabs Account/Preferences/Security/Connect/Billing/About. Account=photo/name/email/phone/dob/gender/delete. Preferences=units(weight/height/distance/fluid/date format)+body stats(weight/height/body_fat_band)+meal layout+enter-to-send. Security=privacy(share_online_status/share_last_seen)+biometric+app lock+change password. Connect=wearables. Billing=read-only txns. CLASSIFICATION -- admin CAN edit (DB-backed): photo,name,dob,gender,all units,body stats,body comp,meal layout,privacy toggles. CAN'T edit directly, needs client confirm (verification-gated): email(confirm link),phone(SMS OTP),password(needs current pw). CAN'T edit at all (device-local, lives on the phone): enter-to-send(AsyncStorage),biometric(SecureStore),app lock(AsyncStorage),wearable connects. CURRENT web tool = ClientSettingsDrawer (gear icon on AdminUserDetail) wrapping shared AccountSettings in target mode (targetUserId); narrow today — edits name/gender/dob/phone(plain)/weight/height + 4 unit prefs + 2 privacy toggles + 2 working support actions (send pw reset, send email link) + 2 stubs (disable biometric / sign out everywhere). USER DECISIONS 2026-06-08: (1) email=keep 'send the client a change link'. (2) phone=admin CHANGES the number + SENDS the client the OTP; the CLIENT enters it to verify (admin does NOT mark verified — sets number unverified, fires send-phone-otp to client's phone, client completes on their device). (3) device-local settings + wearables = OFF (don't show them at all) -&gt; drops the Connect tab + the biometric/app-lock/enter-to-send rows; mirrored tabs become Account/Preferences/Security only. (4) BUILD NOW the 2 remote support actions (sign out everywhere = server-side session revoke; disable fingerprint everywhere = sets a flag, needs a mobile-side launch-check to actually clear on-device biometric). (5) MIRROR the client's exact tab structure. (6) BILLING = no billing page in settings; every transaction reflects to the ACTIVITY FEED instead (billing:* feed events already exist via trg_billing_event_to_activity — verify coverage, don't build a page). (7) COACH: coaches must NOT even have a client-settings button (none exists today; never add one; lock down the shared component so coach can't edit a client).</t>
         </is>
       </c>
       <c r="G106" s="5" t="inlineStr">
         <is>
-          <t>DEFERRED -- pick up after the current header/dashboard polish pass. Will formalize Delete + account-lifecycle actions inside the reworked settings (not just the interim Danger-zone slot), add the 3-tab structure, and mirror to the coach view. Whether settings stays a drawer or becomes a full page is part of this task.</t>
+          <t>PHASE 1 DONE 2026-06-08 (deploy index-BzP1EGVz.js, live hash verified). Cleanup + safety + bug fixes in AccountSettings.jsx: (a) COACH-LOCKDOWN safety -- change-password block was gated on `!isAdminMode`, so a coach editing a client (if ever wired) would see it and signInWithPassword/updateUser would silently change the COACH'S OWN password (updateUser acts on the JWT session user, not the target). Re-gated to `!isTargetMode` (self-only) -- so in ANY target mode (admin or coach) the password form is hidden; admin still gets the support actions (gated isAdminMode), coach-target gets nothing actionable. (b) TAB-POSITION bug -- the drawer shared the persisted-tab key 'myrx:settings_tab' with the admin's own /admin/profile AND had clearOnUnmount, so closing a client drawer wiped the admin's own tab choice; namespaced the drawer to 'myrx:settings_tab:client'. (c) SUPPORT-BUTTON lie -- sendPasswordReset/sendEmailChange never checked resetPasswordForEmail's {error}, showing 'Sent ✓' even on a failed/rate-limited send; now check error and render a 'Failed — try again' state (new 'error' branch in SupportActionRow). REMAINING PHASES (planned, not yet built): Phase 2 = mirror the editable settings (Account: add photo editing + phone set &amp; 'send code to client' + keep email send-link; Preferences: add fluid unit + date format + body_fat_band picker [new web component] + meal-layout editor [reuse EditProfile's] + align swim to derive from distance like mobile; Security: keep privacy + email/pw send buttons). Phase 3 = verify billing txns flow to the activity feed (decision 6 — likely already via trg_billing_event_to_activity; fill gaps, NO billing page). Phase 4 = the 2 remote actions (sign-out-everywhere edge fn w/ service-role session revoke; disable-fingerprint flag via DB column + RPC). Phase 5 = mobile launch-check honoring the disable-fingerprint flag (clears SecureStore biometric + app lock). KNOWN GAP to resolve in Phase 2: the 'send email-change link' mechanism (resetPasswordForEmail -&gt; /auth?mode=update-email) is unverified -- confirm /auth handles update-email mode or build a proper service-role email-change link.</t>
         </is>
       </c>
       <c r="H106" s="5" t="inlineStr">
         <is>
-          <t>web/src/components/ClientSettingsDrawer.jsx; web/src/components/AccountSettings.jsx; mirror coach/CoachClientDetail.jsx</t>
+          <t>web/src/components/AccountSettings.jsx (Phase 1: password gating, tab-key namespace, support-button error states); next: web/src/components/ClientSettingsDrawer.jsx, web/src/pages/admin/AdminUserDetail.jsx, new web body-fat picker + meal-layout editor, new edge fns, mobile settings.tsx launch-check; NO coach mirror per user</t>
         </is>
       </c>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(mobile): honor admin "disable fingerprint on all devices" — T103 complete
Phase 5 (mobile) of the admin client-settings mirror:
- Stamp myrx.bio.enrolledAt when biometric is enabled; clear it on disable.
- On profile load, if profiles.biometric_disabled_at is newer than this
  device's enrol timestamp, wipe the on-device biometric sign-in + app lock
  (falls back to password). Re-enrolling afterward keeps working.

Closes the loop on the admin "Disable fingerprint" button. T103 done.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -5436,9 +5436,9 @@
           <t>Web+Mobile</t>
         </is>
       </c>
-      <c r="E106" s="12" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="G106" s="5" t="inlineStr">
         <is>
-          <t>PHASE 1 DONE 2026-06-08 (deploy index-BzP1EGVz.js, live hash verified). Cleanup + safety + bug fixes in AccountSettings.jsx: (a) COACH-LOCKDOWN safety -- change-password block was gated on `!isAdminMode`, so a coach editing a client (if ever wired) would see it and signInWithPassword/updateUser would silently change the COACH'S OWN password (updateUser acts on the JWT session user, not the target). Re-gated to `!isTargetMode` (self-only) -- so in ANY target mode (admin or coach) the password form is hidden; admin still gets the support actions (gated isAdminMode), coach-target gets nothing actionable. (b) TAB-POSITION bug -- the drawer shared the persisted-tab key 'myrx:settings_tab' with the admin's own /admin/profile AND had clearOnUnmount, so closing a client drawer wiped the admin's own tab choice; namespaced the drawer to 'myrx:settings_tab:client'. (c) SUPPORT-BUTTON lie -- sendPasswordReset/sendEmailChange never checked resetPasswordForEmail's {error}, showing 'Sent ✓' even on a failed/rate-limited send; now check error and render a 'Failed — try again' state (new 'error' branch in SupportActionRow). REMAINING PHASES (planned, not yet built): Phase 2 = mirror the editable settings (Account: add photo editing + phone set &amp; 'send code to client' + keep email send-link; Preferences: add fluid unit + date format + body_fat_band picker [new web component] + meal-layout editor [reuse EditProfile's] + align swim to derive from distance like mobile; Security: keep privacy + email/pw send buttons). Phase 3 = verify billing txns flow to the activity feed (decision 6 — likely already via trg_billing_event_to_activity; fill gaps, NO billing page). Phase 4 = the 2 remote actions (sign-out-everywhere edge fn w/ service-role session revoke; disable-fingerprint flag via DB column + RPC). Phase 5 = mobile launch-check honoring the disable-fingerprint flag (clears SecureStore biometric + app lock). KNOWN GAP to resolve in Phase 2: the 'send email-change link' mechanism (resetPasswordForEmail -&gt; /auth?mode=update-email) is unverified -- confirm /auth handles update-email mode or build a proper service-role email-change link. PHASE 2a (Preferences mirror) DONE 2026-06-08 (deploy index-DW_rUCDN.js, live verified; profiles columns fluid_unit/date_format/body_fat_band/swim_unit/meal_slots_default/phone_verified_at all confirmed via MCP): expanded the shared PreferencesTab so it mirrors the client app -- added Fluid unit (oz/mL -&gt; fluid_unit), Date format (MM/DD vs DD/MM -&gt; date_format, its own section since it's not an imperial/metric pair), and the Body composition silhouette picker (reused the existing web BodyCompPicker component -&gt; body_fat_band; replaced the old 'set from mobile' note). Aligned swim to the client app: dropped the standalone Swim-distance toggle and now derive swim_unit from distance on save (mi-&gt;yd, km-&gt;m). All write to effectiveUserId (target=client in the drawer, self otherwise) and are gender/target-aware (BodyCompPicker reads the target profile's gender + body_fat_band). Affects self mode too (admin/coach own Preferences gain fluid/date/body-comp) -- intentional, consistent with the app. STILL PENDING in Phase 2: Account tab (photo editing target-aware upload; phone change + 'send code to client' via the phone-OTP fn) + Meal-layout editor (extract the slot editor from EditProfile.jsx into a shared component, reuse in target mode). NOTE: send-phone-otp is NOT in the repo functions folder (only verify-phone-otp is present alongside admin-user-management/coach-signup/delete-user/init-profile-checkpoint/send-coach-invite/stripe-webhook) -- must confirm via MCP whether send-phone-otp is deployed before wiring the admin 'send code' button. PHASE 2b (Account mirror: photo + phone) DONE 2026-06-08 (deploy index-Cp9sfJ6v.js, live verified). Verified via MCP: send-phone-otp IS deployed (v12, active, verify_jwt=true) -- its source takes a { phone } param and Twilio-Verify-scopes by NUMBER not user (auth only gates spam), so an admin can text a code to the client's new number. PHOTO: avatar storage RLS only allowed self-folder writes (auth.uid()=foldername[1], no superuser bypass), so admins couldn't set a client photo -&gt; added migration admin_manage_any_avatar (2 additive storage.objects policies: admins (public.is_admin()) can INSERT/UPDATE any object in the avatars bucket; users keep self-only). TargetAccountTab now has a full avatar editor: pick -&gt; reuse AvatarCropper (512² JPEG blob) -&gt; direct storage upload to `${clientId}/avatar` (useAuth.uploadAvatar is self-bound, so direct) -&gt; write avatar_url (cache-busted) to the client's profile; Remove sets avatar_url null. PHONE: TargetAccountTab phone field gained a Verified/Not-verified badge (from phone_verified_at, flips to Not-verified the moment the admin edits the number), a 'Send code to client' button (supabase.functions.invoke send-phone-otp with E.164 validation + sent/error states), and handleSave now nulls phone_verified_at whenever the number changes (client re-verifies on their device). Email stays read-only (Security tab's send-link). Account tab now mirrors the client minus the device-only/verification-gated bits, exactly per the decisions. REMAINING Phase 2: meal-layout editor (extract the slot editor from EditProfile.jsx into a shared component, render in target Preferences) -- last piece. Then Phase 3 (billing-&gt;feed verify), Phase 4 (sign-out-everywhere + disable-fingerprint backends), Phase 5 (mobile fingerprint-flag launch-check). PHASE 2c (meal layout) DONE 2026-06-08 (deploy index-BkflvZgD.js, live verified) -- PHASE 2 NOW COMPLETE. Extracted the meal-slot editor into a new shared component web/src/components/MealLayoutEditor.jsx (slot list + per-slot insert-divider presets/custom + reset + save; props profile/effectiveUserId/onSaved/refreshOnSave/note). Wired into AccountSettings PreferencesTab (after body stats) -- writes to effectiveUserId (client in target mode), admin-voice note. ALSO refactored EditProfile.jsx SettingsTab to use the same component (removed ~90 lines of inline meal state+handlers+JSX, kept its card wrapper+header+end-user-voice note, cleaned now-unused imports X as XIcon/Plus + the FoodLogDrawer DEFAULT_SLOTS/EXTRA_PRESETS/ANCHOR_IDS import) so there's ONE meal editor, no duplication. Build clean, both surfaces compile. ADMIN CLIENT-SETTINGS MIRROR (Account + Preferences + Security) is now a faithful editable mirror of the client app minus the device-only/verification-gated bits, exactly per the decisions. REMAINING: Phase 3 (billing-&gt;activity-feed coverage verify, NO billing page), Phase 4 (sign-out-everywhere edge fn + disable-fingerprint flag), Phase 5 (mobile fingerprint-flag launch-check). DOC-MISMATCH NOTE for CLAUDE.md: send-phone-otp IS deployed (v12) but absent from the repo supabase/functions/ folder -- repo only has verify-phone-otp; the send-phone-otp source lives only on Supabase (retrieved via MCP get_edge_function). PHASE 3 (billing -&gt; activity feed) VERIFIED DONE 2026-06-08 -- NO CODE NEEDED, NO billing page in settings (decision 6 honored). Confirmed via MCP: the AFTER INSERT trigger billing_events_to_activity_events_trg on public.billing_events is ENABLED and runs trg_billing_event_to_activity() (SECURITY DEFINER), which fans EVERY billing_events row into activity_events as event_type='billing:'||type with full event_data (amount/currency/status/description + all stripe IDs), source='system'. The stripe-webhook edge fn writes billing_events.type using CANONICAL names (invoice_paid, invoice_failed, subscription_started, subscription_updated, subscription_cancelled, b2c_purchase, refund_issued, dispute_opened) that EXACTLY match the feed's describe() billing:* cases in AdminUserDetail -- so each transaction renders with its proper label (Invoice paid $X, Subscription started, Refund issued, Dispute opened, One-time purchase, etc.). (The lone raw 'invoice.payment_succeeded' row in billing_events was a manual test insert, not from the webhook -- ignore.) So 'every transaction reflected to the activity feed' is already true end-to-end. REMAINING: Phase 4 (sign-out-everywhere edge fn [service-role session revoke] + disable-fingerprint flag) + Phase 5 (mobile launch-check honoring the disable-fingerprint flag: clears SecureStore biometric + app lock). PHASE 4 (the 2 remote security actions) DONE 2026-06-08 (deploy index-j8Ck2seS.js, live verified; migration admin_remote_security_actions applied). Did it as a DB RPC + a flag column rather than editing the admin-user-management edge fn (simpler, fewer moving parts). MIGRATION: (1) added profiles.biometric_disabled_at timestamptz -- admin sets it; mobile clears on-device biometric+lock on next launch when this is newer than the device's enrol time (Phase 5). (2) created public.admin_revoke_user_sessions(p_user_id uuid) -- SECURITY DEFINER, is_admin()-gated, `delete from auth.sessions where user_id=p_user_id` (verified auth.sessions has user_id; refresh tokens die immediately, access tokens expire within ~1h TTL), granted execute to authenticated (the internal is_admin() check gates it; revoked from public/anon). WEB: AdminSupportActions' two former stubs are now live -- 'Disable fingerprint on all devices' does a direct profiles.update({biometric_disabled_at}) (admin RLS bypass), 'Sign out everywhere' calls the RPC; both with sending/done/error states (added a successLabel prop to SupportActionRow so they read 'Done' not 'Sent'). Couldn't happy-path test the RPC via MCP (service-role context has no auth.uid() so is_admin() is false -&gt; raises admin_required, which is correct) -- the admin's web session will pass is_admin(); user to QA. REMAINING: Phase 5 (mobile) -- on launch, compare profiles.biometric_disabled_at to the device's stored biometric-enrol timestamp; if newer, clear SecureStore myrx.bio.* + AsyncStorage myrx.lock.enabled so fingerprint sign-in + app lock are disabled on that device. Needs storing an enrol timestamp on the device when biometric is enabled (settings.tsx) + the launch check (likely in AuthContext or _layout).</t>
+          <t>PHASE 1 DONE 2026-06-08 (deploy index-BzP1EGVz.js, live hash verified). Cleanup + safety + bug fixes in AccountSettings.jsx: (a) COACH-LOCKDOWN safety -- change-password block was gated on `!isAdminMode`, so a coach editing a client (if ever wired) would see it and signInWithPassword/updateUser would silently change the COACH'S OWN password (updateUser acts on the JWT session user, not the target). Re-gated to `!isTargetMode` (self-only) -- so in ANY target mode (admin or coach) the password form is hidden; admin still gets the support actions (gated isAdminMode), coach-target gets nothing actionable. (b) TAB-POSITION bug -- the drawer shared the persisted-tab key 'myrx:settings_tab' with the admin's own /admin/profile AND had clearOnUnmount, so closing a client drawer wiped the admin's own tab choice; namespaced the drawer to 'myrx:settings_tab:client'. (c) SUPPORT-BUTTON lie -- sendPasswordReset/sendEmailChange never checked resetPasswordForEmail's {error}, showing 'Sent ✓' even on a failed/rate-limited send; now check error and render a 'Failed — try again' state (new 'error' branch in SupportActionRow). REMAINING PHASES (planned, not yet built): Phase 2 = mirror the editable settings (Account: add photo editing + phone set &amp; 'send code to client' + keep email send-link; Preferences: add fluid unit + date format + body_fat_band picker [new web component] + meal-layout editor [reuse EditProfile's] + align swim to derive from distance like mobile; Security: keep privacy + email/pw send buttons). Phase 3 = verify billing txns flow to the activity feed (decision 6 — likely already via trg_billing_event_to_activity; fill gaps, NO billing page). Phase 4 = the 2 remote actions (sign-out-everywhere edge fn w/ service-role session revoke; disable-fingerprint flag via DB column + RPC). Phase 5 = mobile launch-check honoring the disable-fingerprint flag (clears SecureStore biometric + app lock). KNOWN GAP to resolve in Phase 2: the 'send email-change link' mechanism (resetPasswordForEmail -&gt; /auth?mode=update-email) is unverified -- confirm /auth handles update-email mode or build a proper service-role email-change link. PHASE 2a (Preferences mirror) DONE 2026-06-08 (deploy index-DW_rUCDN.js, live verified; profiles columns fluid_unit/date_format/body_fat_band/swim_unit/meal_slots_default/phone_verified_at all confirmed via MCP): expanded the shared PreferencesTab so it mirrors the client app -- added Fluid unit (oz/mL -&gt; fluid_unit), Date format (MM/DD vs DD/MM -&gt; date_format, its own section since it's not an imperial/metric pair), and the Body composition silhouette picker (reused the existing web BodyCompPicker component -&gt; body_fat_band; replaced the old 'set from mobile' note). Aligned swim to the client app: dropped the standalone Swim-distance toggle and now derive swim_unit from distance on save (mi-&gt;yd, km-&gt;m). All write to effectiveUserId (target=client in the drawer, self otherwise) and are gender/target-aware (BodyCompPicker reads the target profile's gender + body_fat_band). Affects self mode too (admin/coach own Preferences gain fluid/date/body-comp) -- intentional, consistent with the app. STILL PENDING in Phase 2: Account tab (photo editing target-aware upload; phone change + 'send code to client' via the phone-OTP fn) + Meal-layout editor (extract the slot editor from EditProfile.jsx into a shared component, reuse in target mode). NOTE: send-phone-otp is NOT in the repo functions folder (only verify-phone-otp is present alongside admin-user-management/coach-signup/delete-user/init-profile-checkpoint/send-coach-invite/stripe-webhook) -- must confirm via MCP whether send-phone-otp is deployed before wiring the admin 'send code' button. PHASE 2b (Account mirror: photo + phone) DONE 2026-06-08 (deploy index-Cp9sfJ6v.js, live verified). Verified via MCP: send-phone-otp IS deployed (v12, active, verify_jwt=true) -- its source takes a { phone } param and Twilio-Verify-scopes by NUMBER not user (auth only gates spam), so an admin can text a code to the client's new number. PHOTO: avatar storage RLS only allowed self-folder writes (auth.uid()=foldername[1], no superuser bypass), so admins couldn't set a client photo -&gt; added migration admin_manage_any_avatar (2 additive storage.objects policies: admins (public.is_admin()) can INSERT/UPDATE any object in the avatars bucket; users keep self-only). TargetAccountTab now has a full avatar editor: pick -&gt; reuse AvatarCropper (512² JPEG blob) -&gt; direct storage upload to `${clientId}/avatar` (useAuth.uploadAvatar is self-bound, so direct) -&gt; write avatar_url (cache-busted) to the client's profile; Remove sets avatar_url null. PHONE: TargetAccountTab phone field gained a Verified/Not-verified badge (from phone_verified_at, flips to Not-verified the moment the admin edits the number), a 'Send code to client' button (supabase.functions.invoke send-phone-otp with E.164 validation + sent/error states), and handleSave now nulls phone_verified_at whenever the number changes (client re-verifies on their device). Email stays read-only (Security tab's send-link). Account tab now mirrors the client minus the device-only/verification-gated bits, exactly per the decisions. REMAINING Phase 2: meal-layout editor (extract the slot editor from EditProfile.jsx into a shared component, render in target Preferences) -- last piece. Then Phase 3 (billing-&gt;feed verify), Phase 4 (sign-out-everywhere + disable-fingerprint backends), Phase 5 (mobile fingerprint-flag launch-check). PHASE 2c (meal layout) DONE 2026-06-08 (deploy index-BkflvZgD.js, live verified) -- PHASE 2 NOW COMPLETE. Extracted the meal-slot editor into a new shared component web/src/components/MealLayoutEditor.jsx (slot list + per-slot insert-divider presets/custom + reset + save; props profile/effectiveUserId/onSaved/refreshOnSave/note). Wired into AccountSettings PreferencesTab (after body stats) -- writes to effectiveUserId (client in target mode), admin-voice note. ALSO refactored EditProfile.jsx SettingsTab to use the same component (removed ~90 lines of inline meal state+handlers+JSX, kept its card wrapper+header+end-user-voice note, cleaned now-unused imports X as XIcon/Plus + the FoodLogDrawer DEFAULT_SLOTS/EXTRA_PRESETS/ANCHOR_IDS import) so there's ONE meal editor, no duplication. Build clean, both surfaces compile. ADMIN CLIENT-SETTINGS MIRROR (Account + Preferences + Security) is now a faithful editable mirror of the client app minus the device-only/verification-gated bits, exactly per the decisions. REMAINING: Phase 3 (billing-&gt;activity-feed coverage verify, NO billing page), Phase 4 (sign-out-everywhere edge fn + disable-fingerprint flag), Phase 5 (mobile fingerprint-flag launch-check). DOC-MISMATCH NOTE for CLAUDE.md: send-phone-otp IS deployed (v12) but absent from the repo supabase/functions/ folder -- repo only has verify-phone-otp; the send-phone-otp source lives only on Supabase (retrieved via MCP get_edge_function). PHASE 3 (billing -&gt; activity feed) VERIFIED DONE 2026-06-08 -- NO CODE NEEDED, NO billing page in settings (decision 6 honored). Confirmed via MCP: the AFTER INSERT trigger billing_events_to_activity_events_trg on public.billing_events is ENABLED and runs trg_billing_event_to_activity() (SECURITY DEFINER), which fans EVERY billing_events row into activity_events as event_type='billing:'||type with full event_data (amount/currency/status/description + all stripe IDs), source='system'. The stripe-webhook edge fn writes billing_events.type using CANONICAL names (invoice_paid, invoice_failed, subscription_started, subscription_updated, subscription_cancelled, b2c_purchase, refund_issued, dispute_opened) that EXACTLY match the feed's describe() billing:* cases in AdminUserDetail -- so each transaction renders with its proper label (Invoice paid $X, Subscription started, Refund issued, Dispute opened, One-time purchase, etc.). (The lone raw 'invoice.payment_succeeded' row in billing_events was a manual test insert, not from the webhook -- ignore.) So 'every transaction reflected to the activity feed' is already true end-to-end. REMAINING: Phase 4 (sign-out-everywhere edge fn [service-role session revoke] + disable-fingerprint flag) + Phase 5 (mobile launch-check honoring the disable-fingerprint flag: clears SecureStore biometric + app lock). PHASE 4 (the 2 remote security actions) DONE 2026-06-08 (deploy index-j8Ck2seS.js, live verified; migration admin_remote_security_actions applied). Did it as a DB RPC + a flag column rather than editing the admin-user-management edge fn (simpler, fewer moving parts). MIGRATION: (1) added profiles.biometric_disabled_at timestamptz -- admin sets it; mobile clears on-device biometric+lock on next launch when this is newer than the device's enrol time (Phase 5). (2) created public.admin_revoke_user_sessions(p_user_id uuid) -- SECURITY DEFINER, is_admin()-gated, `delete from auth.sessions where user_id=p_user_id` (verified auth.sessions has user_id; refresh tokens die immediately, access tokens expire within ~1h TTL), granted execute to authenticated (the internal is_admin() check gates it; revoked from public/anon). WEB: AdminSupportActions' two former stubs are now live -- 'Disable fingerprint on all devices' does a direct profiles.update({biometric_disabled_at}) (admin RLS bypass), 'Sign out everywhere' calls the RPC; both with sending/done/error states (added a successLabel prop to SupportActionRow so they read 'Done' not 'Sent'). Couldn't happy-path test the RPC via MCP (service-role context has no auth.uid() so is_admin() is false -&gt; raises admin_required, which is correct) -- the admin's web session will pass is_admin(); user to QA. REMAINING: Phase 5 (mobile) -- on launch, compare profiles.biometric_disabled_at to the device's stored biometric-enrol timestamp; if newer, clear SecureStore myrx.bio.* + AsyncStorage myrx.lock.enabled so fingerprint sign-in + app lock are disabled on that device. Needs storing an enrol timestamp on the device when biometric is enabled (settings.tsx) + the launch check (likely in AuthContext or _layout). PHASE 5 (mobile honors the flag) DONE 2026-06-08 (mobile tsc clean; mobile-only, no web deploy; can't QA without the device) -- T103 NOW COMPLETE. mobile/src/contexts/AuthContext.tsx: (1) new SecureStore key myrx.bio.enrolledAt stamped on enableBiometric (ISO now) and deleted on disableBiometric; (2) module-level honorRemoteBiometricDisable(profile) -- if profile.biometric_disabled_at is set AND this device holds biometric creds AND disabledAt &gt; the device's enrolledAt (missing enrol record counts as old), it wipes SecureStore myrx.bio.email/password/enrolledAt/pending + calls setLockEnabled(false) (imported from lockState); (3) called fire-and-forget from fetchProfile after setProfile, so on next launch/profile-load a device whose enrolment predates the admin's action loses fingerprint sign-in + app lock and falls back to password. Idempotent (no-creds early return). Re-enrol stamps a newer enrolledAt so the same flag won't re-clear; a fresh admin click sets a newer biometric_disabled_at to re-trigger. Only enrol site is enableBiometric (sole BIO_EMAIL_KEY writer) so all enrol paths (incl. signup BiometricScreen) are covered. ENTIRE T103 COMPLETE: admin client-settings page mirrors the client (Account photo/name/email-read-only/phone-set+send-code/dob/gender; Preferences units+fluid+date+body-fat+meal-layout; Security privacy + password/email send-links + disable-fingerprint + sign-out-everywhere), billing flows to the activity feed (no settings billing page), coaches have NO client-settings access (and the latent coach password bug is gated out). Coach does NOT mirror this (per user). QA PENDING: user to exercise the admin actions live (send-code SMS, sign-out-everywhere, disable-fingerprint end-to-end on a device).</t>
         </is>
       </c>
       <c r="H106" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(settings): real email-change for clients + audit all support-action links
The "Send email-change link" was broken — it sent a password-reset (recovery)
email pointed at a /auth?mode=update-email page that doesn't exist, and a
one-click link can't change an email (no new address supplied; GoTrue has no
admin-triggered confirm-link flow).

- Email change: now an inline "Change account email" field; the admin types the
  new address and it applies via a new superuser-gated change_email action on
  admin-user-management (auth.admin.updateUserById, email_confirm). Client is
  mobile-only so admin-direct is the right model.
- Password reset: verified working (recovery link -> AuthConfirm form). No change.
- Phone: verified working (admin sets number + Send code -> client verifies). No change.

T108.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5647,6 +5647,53 @@
       <c r="I110" s="5" t="inlineStr">
         <is>
           <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>T108</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>Fix the admin email-change link + audit all client-settings support-action links</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-08: 'fix the email change link and double check on all other links like the password change or the phone change or whatever.' The 'Send email-change link' support action (AccountSettings AdminSupportActions) was BROKEN: it called supabase.auth.resetPasswordForEmail(profile.email, { redirectTo: '/auth?mode=update-email' }) -- a PASSWORD-RESET (type=recovery) email pointed at a /auth?mode=update-email page that DOESN'T EXIST (mode=update-email appears nowhere in the app). Clicking it ran the recovery flow -&gt; AuthConfirm's 'Set a new password' form (wrong) or dumped the client on the generic /auth page. Worse, a one-click 'send link' can't ever change an email -- nobody supplies the NEW address, and GoTrue has NO admin-triggered 'client confirms via link' email-change path (the only confirm flow is the user-initiated updateUser({email}) the client runs in their OWN app). And the client is mobile-only.</t>
+        </is>
+      </c>
+      <c r="G111" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-08 (edge fn admin-user-management v7 deployed; web deploy index-PsRrk6KY.js, live verified). AUDIT of all support-action links/flows: (1) PASSWORD RESET -- VERIFIED WORKING, no change: resetPasswordForEmail sends a type=recovery email whose link Supabase renders as {SiteURL}/auth/confirm?token_hash=...&amp;type=recovery; AuthConfirm.jsx verifyOtp(type=recovery) -&gt; 'Set a new password' form -&gt; updateUser({password}). Same flow the end-user forgot-password uses. redirectTo only affects post-reset navigation (irrelevant for a mobile client), so the admin's no-redirectTo call still lands on the recovery form. (2) EMAIL CHANGE -- FIXED: replaced the broken one-click link with an inline 'Change account email' field (admin types the new address) wired to a NEW 'change_email' action on the admin-user-management edge fn (superuser-gated, cannot_modify_self/admin guards reused) that calls auth.admin.updateUserById(target, { email, email_confirm: true }) -&gt; applies immediately, surfaces 'already in use' errors. Chose admin-direct (not client-confirm) because GoTrue offers no admin-triggered confirm-link flow + the client is mobile-only; documented this in code + flagged to the user with the option to do a heavier client-confirm flow if wanted. NOTE: email_confirm:true means NO notification email to the client (no mailer in edge fns); acceptable for an admin tool, flagged. profiles has no email column (email lives in auth.users, surfaced via get_users_for_admin) so the read-only Account-tab email display is stale until next load -- minor, consistent with other admin edits. (3) PHONE -- VERIFIED WORKING (T103 Phase 2b): admin sets profiles.phone (+ nulls phone_verified_at on change) and 'Send code to client' invokes the deployed send-phone-otp edge fn (takes a {phone} param, Twilio-Verify-scoped by number) -&gt; SMS to the client -&gt; client enters it in their mobile app (verify-phone-otp). Not a 'link' -- in-app OTP. (4) DISABLE FINGERPRINT / SIGN OUT EVERYWHERE -- the Phase 4/5 actions, already verified. Updated the Account-tab email note + the AdminSupportActions doc comment to match the new 'Change account email' field.</t>
+        </is>
+      </c>
+      <c r="H111" s="7" t="inlineStr">
+        <is>
+          <t>web/src/components/AccountSettings.jsx (AdminSupportActions: inline change-email form replacing the broken link; note + comment updates); supabase edge fn admin-user-management (added change_email action, v7)</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(settings): match the client app's distance/fluid/date unit cards exactly
The web Preferences mirror drifted from the client app on the unit labels:
- Distance: "mi"/"km" -> "mi · yd"/"km · m" (Miles & yards / Km & metres) — it
  drives swim too, like the client app shows
- Fluid sub: "Ounces" -> "Fluid ounces"
- Date format: moved into the Imperial|Metric grid as MM/DD (Imperial) /
  DD/MM (Metric), out of its own separate section
- Body composition: dropped the footnote to match (client omits it here)

Behavior was already correct (swim derives from distance) — this was label/
layout drift. T109.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5692,6 +5692,53 @@
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>T109</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Settings mirror drift — distance/fluid/date unit cards didn't match the client app</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-08 (frustrated, recurring mirror-accuracy complaint): 'why does distance show different between mobile and web, why do i have to always find that you dont mirror correctly everything we do?' Compared the web admin Preferences mirror (AccountSettings PreferencesTab) line-by-line against the live mobile client settings (mobile/app/(app)/settings.tsx, the PreferencesTab unit cards L1533-1581 + body-comp L1662-1672). DRIFT FOUND: (1) DISTANCE card -- mobile shows 'mi · yd' / 'Miles &amp; yards' and 'km · m' / 'Km &amp; metres' (ONE imperial-vs-metric choice that drives BOTH running/cycling distance AND swim unit); my Phase-2a web mirror showed plain 'mi'/'Miles' + 'km'/'Kilometres', hiding that it also sets swim. This is the one the user spotted. (2) FLUID sub -- mobile 'Fluid ounces', web had 'Ounces'. (3) DATE FORMAT -- mobile renders it as a 4th/5th card INSIDE the same Imperial|Metric units grid with labels 'MM/DD'/'DD/MM' + subs 'Imperial'/'Metric'; web had it in a SEPARATE section with 'MM / DD'/'DD / MM' + subs 'Month first'/'Day first'. (4) BODY-COMP footnote -- mobile passes showFootnote={false} inside Body stats; web added a 'The Calories plan uses this...' footnote.</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-08 (deploy index-tkWDJN8Q.js, live verified). Aligned the web Preferences unit cards to the mobile client EXACTLY: Distance -&gt; 'mi · yd'/'Miles &amp; yards' + 'km · m'/'Km &amp; metres'; Fluid sub -&gt; 'Fluid ounces'; Date format -&gt; moved INTO the Imperial|Metric units grid as a UnitRow with 'MM/DD'/'Imperial' + 'DD/MM'/'Metric' (removed the separate section); Body composition -&gt; dropped the footnote to match showFootnote=false. Underlying behavior was already correct (swim_unit derives from distance on save since Phase 2a) -- this was a LABEL/PRESENTATION drift only. Weight + Height cards already matched (Pounds/Kilograms, Feet &amp; inches/Centimetres). PROCESS NOTE (the user's real complaint): when mirroring a surface, diff the actual client source card-by-card (labels + subs + layout + which section each control sits in), not just the data/behavior -- presentation drift is what the user sees and keeps catching. Should have done this card-by-card diff during Phase 2a instead of writing approximate labels.</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>web/src/components/AccountSettings.jsx (PreferencesTab: Distance/Fluid/Date-format unit cards + body-comp footnote, matched to mobile settings.tsx)</t>
+        </is>
+      </c>
+      <c r="I112" s="5" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>

</xml_diff>

<commit_message>
fix(settings): admin mirror showed defaults, not the client's real prefs
Root cause: get_user_for_admin (the RPC that loads a client for the admin)
omitted newer profile columns — fluid_unit, date_format, body_fat_band,
meal_slots_default, share_online_status, share_last_seen, phone_verified_at —
so the mirror fell back to component defaults (fluid=oz, body-fat=Average,
4 meal slots, privacy toggles=ON) regardless of what the client actually set.

- Migration: DROP+CREATE get_user_for_admin with the 7 missing columns. Mirror
  now reads the client's real values (motaz: mL, Lean, 5 slots incl Post-Workout).
- Rewrote web BodyCompPicker to match mobile exactly: correct BF% bands
  (≤14/15-24/≥25, ≤20/21-30/≥31), per-card descriptions, "Pick the silhouette"
  subtitle, showFootnote prop.

T110.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5739,6 +5739,53 @@
         </is>
       </c>
       <c r="I112" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>T110</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>Admin client-settings mirror showed DEFAULTS not the client's real prefs (RPC omitted columns) + body-comp picker drift</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-08 (still frustrated, sent 6 screenshots): 'the choices between the client on mobile and web are different ... im talking about the client's settings ... look at the screenshot.' The screenshots (admin's 'Motaz Jarrah's Settings' drawer vs motaz's mobile) showed: web Body composition = Average selected w/ ranges Lean ≤12% / Average 12-22% / High &gt;22% and NO descriptions; mobile = Lean selected w/ ≤14% BF / 15-24% BF / ≥25% BF + descriptions ('Visible muscle definition...', etc.) + 'Pick the silhouette...' subtitle. Also web fluid=oz vs mobile mL, web meal=4 slots (Breakfast/Lunch/Dinner/Snacks) vs mobile 5 (incl. a custom Post-Workout). ROOT CAUSE (the big one): AdminUserDetail loads the client via the get_user_for_admin RPC, whose RETURNS TABLE column list was missing the NEWER columns -- fluid_unit, date_format, body_fat_band, meal_slots_default, share_online_status, share_last_seen, phone_verified_at. So the mirror received undefined for those and fell back to component DEFAULTS (oz / 'average' / DEFAULT_SLOTS / true), regardless of the client's stored values. Verified motaz's DB row: distance=km, fluid=mL, body_fat=lean, meal_slots_default=5 incl post_workout. SECOND issue: the web BodyCompPicker component itself was a stale port -- wrong BF% bands (≤12/12-22/&gt;22 vs mobile ≤14/15-24/≥25), no 'BF' suffix, no per-card descriptions, no 'Pick the silhouette' subtitle.</t>
+        </is>
+      </c>
+      <c r="G113" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-08 (migration get_user_for_admin_add_pref_columns; web deploy index-BYJTiD_c.js, live verified). (1) DROP+CREATE get_user_for_admin adding the 7 missing columns (fluid_unit, date_format, body_fat_band, meal_slots_default, share_online_status, share_last_seen, phone_verified_at) to both the RETURNS TABLE and the SELECT (return-type change requires drop-then-create per the Supabase RPC rule). This single fix corrects the SELECTED values across the mirror -- fluid now reads mL, body-fat reads lean, meal shows all 5 slots incl Post-Workout, the phone Verified/Not-verified badge reads phone_verified_at, and the Security privacy toggles now reflect the client's ACTUAL share_online_status/share_last_seen instead of defaulting to true (a latent bug -- the toggles were showing ON for everyone). (2) Rewrote web/src/components/BodyCompPicker.jsx to mirror mobile/src/components/BodyCompPicker.tsx EXACTLY: male ≤14% BF / 15-24% BF / ≥25% BF + female ≤20% / 21-30% / ≥31% BF, per-card descriptions, the 'Pick the silhouette that most closely matches your current body.' subtitle, and a showFootnote prop (default true; AccountSettings passes false to match mobile settings showFootnote=false; the macro editor uses compact which suppresses subtitle/desc/footnote so its dense layout is unchanged). LESSON (the recurring complaint's real root): a 'mirror' built on an admin RPC is only as complete as that RPC's column list -- when mobile adds a profile column, the get_user_for_admin RPC must be extended too, or the web mirror silently shows defaults. Audited: all columns the settings mirror reads are now returned. PRIOR near-misses (T109 labels) were real but secondary; THIS (RPC columns) was why the selected values were wrong.</t>
+        </is>
+      </c>
+      <c r="H113" s="7" t="inlineStr">
+        <is>
+          <t>supabase migration get_user_for_admin_add_pref_columns (DROP+CREATE with 7 added columns); web/src/components/BodyCompPicker.jsx (full rewrite to mobile parity); web/src/components/AccountSettings.jsx (showFootnote=false)</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>

</xml_diff>

<commit_message>
docs(claude): add VERIFY-EVERY-UPDATE rule + capture realtime-settings task
- New MANDATORY CLAUDE.md rule: "verify every update against real data — it
  shipped != it works". 4-point checklist (trace the read path end-to-end; test
  with real non-default data via MCP; diff mirrors control-by-control; observe,
  don't assume). Locked after the T109/T110 settings-mirror-showed-defaults bugs.
- Ledger: T112 (this rule) Done; T111 (realtime settings reflection across all
  settings pages) captured as Pending, awaiting greenlight.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5786,6 +5786,100 @@
         </is>
       </c>
       <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>T111</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Real-time reflection of settings changes across all settings pages (web + mobile)</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>Web+Mobile</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-08: 'i need changes to be reflected in real time, the moment i click save it reflects on their account and they can actually see the toggles happen, on all settings pages' + clarification 'not just mirroring, any update we do.' For settings: when the admin saves a client's setting, the CLIENT (and any other viewer) should see the toggles flip LIVE, across all settings sections + all settings surfaces (mobile client settings + web admin mirror + web own-profile pages). FINDING (verified): the realtime DATA path already exists on mobile -- mobile/src/contexts/AuthContext.tsx subscribes to the user's OWN profiles row (postgres_changes UPDATE, filter id=eq.user.id, ~L400-457) and calls fetchProfile on UPDATE, so the in-context `profile` updates within ~1-2s of the admin's save. THE GAP: every settings screen (mobile settings.tsx tabs + web AccountSettings tabs) seeds its toggle values into LOCAL useState ONCE on mount, so it never repaints from the live profile -&gt; nothing visibly happens.</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>PENDING greenlight (asked the user: all 3 surfaces, or start with the client's mobile?). PLAN: (1) mobile settings.tsx -- AccountTab/PreferencesTab/SecurityTab each add a useEffect keyed on `profile` that re-derives its local toggle state from the live profile (in-place set =&gt; the toggle animates, no remount/flicker; self-save = no-op since values match, admin-change = visible flip; EXCLUDE device-local states -- enter-to-send/biometric/app-lock -- they're not in profile). (2) web AccountSettings tabs (TargetAccountTab/PreferencesTab/SecurityTab) -- same sync from the `profile` prop. (3) web parents add a profiles realtime subscription so the prop actually goes live: AdminUserDetail (the client mirror) subscribes to profiles UPDATE(id=eq.clientId) -&gt; re-call get_user_for_admin -&gt; setProfile; AdminProfile + CoachProfile (self) similar (check whether web AuthContext already has a self-profile realtime sub; add if not). CAVEAT: the mobile half can't be QA'd from here (needs the user's device) -- build + have the user confirm the live flip. EDGE: client mid-edit while admin changes simultaneously = admin-wins (rare, accepted). Per the new VERIFY-EVERY-UPDATE rule, test with a real account whose values are non-default + confirm the flip end-to-end.</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>mobile/app/(app)/settings.tsx; web/src/components/AccountSettings.jsx; web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/admin/AdminProfile.jsx; web/src/pages/coach/CoachProfile.jsx</t>
+        </is>
+      </c>
+      <c r="I114" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>T112</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>Add a VERIFY-EVERY-UPDATE rule to CLAUDE.md + confirm pipeline currency</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-08: 'are you updating the task pipeline? read claude.md to refresh your memory ... add to claude.md something that makes you test the things you mirror in a way to catch these issues ... not just mirroring, any update we do, make it so you can test it so we dont face these issues ever again.' The recurring pain (T109/T110): mirrors/updates shipped looking fine on DEFAULT data but were wrong on real data -- admin RPC omitted columns so the mirror showed defaults; label drift; default-masking -- and a green build + matching deploy hash was being treated as 'done' without verifying functional correctness against real data. The user kept being the one to catch it.</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-08. Added a new MANDATORY rule to the MAIN-repo CLAUDE.md Working Relationship block: 'VERIFY EVERY UPDATE AGAINST REAL DATA -- it shipped != it works' (right after the WEB-SEARCH-FIRST rule), with a 4-point checklist applied to every data-driven change: (1) trace the read path end-to-end -- the source query/RPC must actually return every field the UI reads, and any SECURITY DEFINER RPC with a hand-written column list (get_user_for_admin &amp; friends) must be extended whenever mobile adds a profiles column; (2) test with REAL non-default data via the Supabase MCP (defaults mask bugs) and, when the UI isn't reachable, cross-check stored DB values field-by-field against the read path; (3) for mirrors, diff the LIVE source control-by-control (label/sub/option-values/section/data), never from memory; (4) observe the result via the tools, don't assume -- 'deployed, please verify' isn't verification, and when a check is impossible from here say so + name the exact thing for the user to check. Confirmed the pipeline is current: T103-T110 are all logged + committed; added T111 (the realtime settings feature, Pending) per CAPTURE-FIRST. NOTE: edited the MAIN-repo CLAUDE.md (authoritative, what the user reads/commits); the worktree copy at .claude/worktrees/... is the known-stale divergent one and is NOT the source of truth.</t>
+        </is>
+      </c>
+      <c r="H115" s="7" t="inlineStr">
+        <is>
+          <t>CLAUDE.md (Working Relationship MANDATORY block: new VERIFY-EVERY-UPDATE rule); scripts/build_task_pipeline_xlsx.py (T111 + T112)</t>
+        </is>
+      </c>
+      <c r="I115" s="5" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>

</xml_diff>

<commit_message>
fix(coach): mirror the admin button shape on the client-detail header
The coach client-detail header's action buttons were tiny pills while the
admin's Message button is a proper filled button. Restyle all three coach
buttons (Manage macros / Message athlete / Remove) to the admin Message-button
geometry (rounded-lg, px-2.5 py-1.5, text-xs, h-3.5 icons): Message athlete is
now the exact filled-primary mirror, Manage macros a same-size secondary
outline toggle, Remove the same shape in destructive red — reordered to sit
right beside Message ([Manage macros] [Message athlete] [Remove]). The admin's
status-control pills (tier / coach-assignment / Active / chat) stay admin-only.

Also corrects the T126 ledger note: the web CalorieDashboard is the active
coach/admin client-mirror (already correct, no 0.0 bug), not a frozen athlete
page as I'd wrongly recorded. Ledger: +T129.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J131"/>
+  <dimension ref="A1:J132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7165,12 +7165,12 @@
       </c>
       <c r="H129" s="7" t="inlineStr">
         <is>
-          <t>DONE (mobile -- reload to see; no web deploy). VERIFIED the '0.0' root cause via DB: the admin's calorie_plan row has goal_weight_kg = NULL (they set a -20% deficit + a starting weight on the web Macro Plan tab but left the OPTIONAL goal-weight field blank), so the card's fallback fires on !goalKg and prints fromKg(goalKg ?? 0) = '0.0'. That's also why the admin shows a real 'cals target' (the deficit still yields a daily number) while the weight-goal card has nothing to show. Test Coach differed only because they have NO plan row at all -&gt; PendingView, not the goal card. FIX (covers every role x plan-state combo, calories.tsx): (1) canEditPlanHere now excludes coaches too (isSelfCoached &amp;&amp; !isAdmin &amp;&amp; !isCoach) -- coaches are web-only on mobile like admins (decision #1). (2) PendingView gained a webManaged mode: staff with NO plan see 'Manage your plan on the web -&gt; Macro Plan tab' instead of the athlete CTA (coach) or the wrong 'waiting for your coach' (admin). (3) The goal-card fallback else now splits: staff -&gt; 'Set a goal weight in the Macro Plan tab on your web portal to track progress here'; real coached athlete -&gt; 'Your coach hasn't set a goal weight for this phase yet. Once they do, your progress will appear here.' (4) The bogus '0.0' interpolation is GONE from both (decision #4). Self-coached athletes unchanged; staff WITH a real goal still get the normal read-only progress bar. Verified the web Macro Plan editor genuinely has a goal-weight field (optional -&gt; saved null when blank) so 'go to web' is actionable. tsc clean. NOTE: web CalorieDashboard.jsx carries the same string but is only reachable by COACHED WEB ATHLETES (admins/coaches have no end-user Calories page on web), for whom the copy is correct apart from the cosmetic 0.0; web is frozen so left untouched (flagged to user).</t>
+          <t>DONE (mobile -- reload to see; no web deploy). VERIFIED the '0.0' root cause via DB: the admin's calorie_plan row has goal_weight_kg = NULL (they set a -20% deficit + a starting weight on the web Macro Plan tab but left the OPTIONAL goal-weight field blank), so the card's fallback fires on !goalKg and prints fromKg(goalKg ?? 0) = '0.0'. That's also why the admin shows a real 'cals target' (the deficit still yields a daily number) while the weight-goal card has nothing to show. Test Coach differed only because they have NO plan row at all -&gt; PendingView, not the goal card. FIX (covers every role x plan-state combo, calories.tsx): (1) canEditPlanHere now excludes coaches too (isSelfCoached &amp;&amp; !isAdmin &amp;&amp; !isCoach) -- coaches are web-only on mobile like admins (decision #1). (2) PendingView gained a webManaged mode: staff with NO plan see 'Manage your plan on the web -&gt; Macro Plan tab' instead of the athlete CTA (coach) or the wrong 'waiting for your coach' (admin). (3) The goal-card fallback else now splits: staff -&gt; 'Set a goal weight in the Macro Plan tab on your web portal to track progress here'; real coached athlete -&gt; 'Your coach hasn't set a goal weight for this phase yet. Once they do, your progress will appear here.' (4) The bogus '0.0' interpolation is GONE from both (decision #4). Self-coached athletes unchanged; staff WITH a real goal still get the normal read-only progress bar. Verified the web Macro Plan editor genuinely has a goal-weight field (optional -&gt; saved null when blank) so 'go to web' is actionable. tsc clean. WEB CHECK (corrected -- I had wrongly called the web copy a frozen athlete page): athletes are mobile-only on web since May 27 2026 (athlete pages archived; /app -&gt; DownloadAppPlaceholder), so NO athlete reaches any web data page. The web CalorieDashboard is the ACTIVE read-only coach/admin client-mirror (rendered by AdminUserCalories when staff open a client's Calories tab). On inspection it does NOT have this bug: the whole 'Current weight goal' card is gated on result.goalWeightKg being truthy (a client with no goal shows NO card, not a '0.0'), and its single fallback (goal set but starting weight missing/degenerate) already uses neutral copy ('No phase starting weight locked in yet...') with the REAL goal number. So T126 was mobile-only; no web change needed.</t>
         </is>
       </c>
       <c r="I129" s="7" t="inlineStr">
         <is>
-          <t>mobile/app/(app)/calories.tsx (canEditPlanHere excludes coaches; PendingView webManaged mode + staff invocation; goal-card fallback staff/coached split with the 0.0 removed). NOT touched: web/src/components/CalorieDashboard.jsx (frozen; coached-web-athlete only)</t>
+          <t>mobile/app/(app)/calories.tsx (canEditPlanHere excludes coaches; PendingView webManaged mode + staff invocation; goal-card fallback staff/coached split with the 0.0 removed). NOT touched: web/src/components/CalorieDashboard.jsx (active coach/admin client-mirror -- verified it has no bug: card gated on goal, neutral copy, no 0.0)</t>
         </is>
       </c>
       <c r="J129" s="5" t="inlineStr">
@@ -7278,6 +7278,58 @@
         </is>
       </c>
       <c r="J131" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>T129</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Coach client-detail header buttons mirror the admin button shape</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E132" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-08 (screenshot diff, coach vs admin client-detail header): the coach's action buttons were tiny pills (rounded-full, text-[11px], py-0.5) while the admin's Message button is a proper filled button. 'the layout of the pills and buttons is different from the admin, the shape of the message button is different, mirror from admin, for the remove just use the same shape of the message to be right next to it.'</t>
+        </is>
+      </c>
+      <c r="H132" s="5" t="inlineStr">
+        <is>
+          <t>DONE + deployed (live index-DcksFAvq.js). Restyled all three coach header buttons to the admin Message-button geometry (inline-flex gap-1.5 rounded-lg px-2.5 py-1.5 text-xs font-semibold, h-3.5 icons): Message athlete = exact filled-primary mirror of AdminUserDetail's Message button; Manage macros = same geometry as a secondary outline toggle; Remove = same geometry in destructive red, REORDERED to sit right beside Message -&gt; final order [Manage macros] [Message athlete] [Remove]. Cluster gap bumped 1 -&gt; 2 for the larger buttons. Did NOT add the admin's status-control pills (tier / coach-assignment chip / Active toggle / chat) -- those stay admin-only per the role split. Web coach portal only (no mobile coach portal).</t>
+        </is>
+      </c>
+      <c r="I132" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachClientDetail.jsx (header action cluster)</t>
+        </is>
+      </c>
+      <c r="J132" s="5" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>

</xml_diff>

<commit_message>
feat: Movement Library lift_type + hold_type pickers; portal the Select dropdown
- T134: the admin Movement Library create/edit form now sets lift_type
  (Lift style: None/Olympic/Ballistic, gated to barbell/kettlebell rep-based)
  and hold_type (Standard/Leverage/Weighted-load, gated to isometric), wired
  through state, edit-populate, both payloads, summary, row pills, and the
  step-wizard numbering. New moves land on the correct logging form + detail.
- fix: render the Select popover in a portal with fixed positioning so it
  escapes the per-step animate-rise stacking contexts that were painting later
  form sections over the open dropdown. Applies to the library + add-effort form.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -7564,9 +7564,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E137" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E137" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
@@ -7576,17 +7576,17 @@
       </c>
       <c r="G137" s="7" t="inlineStr">
         <is>
-          <t>User 2026-06-09: 'update the move library to handle all the changes we made to the current moves so we don't fall into issues when we create moves.' The movements table now has 22 columns and the logging FORM + DETAIL surfaces dispatch off many of them (strength_type, equipment, lift_type, hold_type, band_assist, knee_assist, uses_pair, weighted_progression, unit_lock, weight_ladder_override, isometric_ladder_override, rep_range_lo/hi, parent_movement_id, variant_short_label, deprecated). If the admin Movement Library create/edit form (AdminMovements.jsx) doesn't let an admin SET these, a newly-created move gets the wrong logging form + wrong detail surface (e.g. a new olympic lift wouldn't be loggable, a new double-KB wouldn't be per-hand, a new band/knee bodyweight wouldn't show the selectors).</t>
+          <t>User 2026-06-09: 'update the move library to handle all the changes we made to the current moves so we don't fall into issues when we create moves.' The movements table has 22 columns and the logging FORM + DETAIL surfaces dispatch off many of them. If the library create/edit form can't SET them, a new move lands on the wrong form/detail.</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>OPEN -- tackle AFTER T131. Audit AdminMovements.jsx against the full movements schema + the form/detail dispatch logic (which column drives which behavior), then add the missing controls with sensible gating + validation (e.g. lift_type only for barbell/kettlebell; hold_type only for isometrics; band/knee/weighted_progression only for bodyweight; uses_pair only for kettlebell; unit_lock enum kg/lb/mi/km; ladder overrides as JSON). Goal: any move created in the library lands on the correct logging form + detail page with no code change.</t>
+          <t>DONE + deployed (web live index-COg-2dcE.js). AUDIT: AdminMovements.jsx already handled category / strength_type / equipment / band_assist / knee_assist / uses_pair / unit_lock / weight_ladder_override / isometric_ladder_override / weighted_progression / deprecated / variant_short_label (+ parent_movement_id via variants). rep_range_lo/hi is intentionally auto (not a field). The ONLY gaps vs the recent work were lift_type + hold_type. Added both as modern Select pickers to the Add + Edit forms, gated: 'Lift style' (None/Olympic/Ballistic) shows for barbell/kettlebell rep-based; 'Hold type' (Standard/Leverage/Weighted-load) shows for isometric. Wired across every site mirroring uses_pair/weighted_progression: add state + edit state + edit-populate + cascade resets + INSERT + UPDATE payloads (null out when the gate isn't met) + buildSummary + row pills (Olympic / Ballistic / Load hold / Leverage hold) + the step-wizard numbering (liftStyle/holdType steps). Verified the edit form binds editLiftType/editHoldType (no copy-paste-to-add-state bug). Result: a new Clean/Snatch (Olympic) or KB Swing (Ballistic) now lands on the right detail + working-set logging, and a new weighted isometric gets its added-weight field -- with no code change.</t>
         </is>
       </c>
       <c r="I137" s="7" t="inlineStr">
         <is>
-          <t>(planned) web/src/pages/admin/AdminMovements.jsx; Supabase movements schema (22 cols)</t>
+          <t>web/src/pages/admin/AdminMovements.jsx (lift_type + hold_type pickers across all sites); uses web/src/components/Select.jsx</t>
         </is>
       </c>
       <c r="J137" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(admin): searchable Legal document repository in Libraries
Add a Legal tab to the admin Libraries page: cross-document keyword
search over all legal docs with highlighted clause snippets, a reading
pane that renders the full doc, and jump-to-section. Clicking a result
scrolls the reading pane to the matched clause (first <mark> in the
section), centered, so the context is visible — not just the heading.

- LegalLayout: add LegalEmbedContext so the real doc components render
  in a compact embedded form (no public-page chrome) inside the tab,
  keeping one source of truth for doc content.
- AdminLegalLibrary: new tab — doc registry, DOM-extracted sections,
  TreeWalker highlight, scroll-to-highlight.
- AdminLibraries: wire the Legal tab (Scale icon, ?tab=legal).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -6979,22 +6979,22 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>Legal repo — searchable legal-doc viewer (rename About -&gt; Legal)</t>
+          <t>Legal repo -- searchable legal-doc viewer as a 'Legal' tab in the admin Libraries page</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>Coach/Admin</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>Web+Mobile</t>
-        </is>
-      </c>
-      <c r="E126" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F126" s="5" t="inlineStr">
@@ -7004,22 +7004,22 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>User 2026-06-08 (admin-settings review #4): 'instead of About, we call it Legal, and we make this page more of our legal repo ... give it capacity to search the docs, show clauses with keywords searched ... everything in the [About] section but wired in a readable, searchable way.' Turn the About surface into a proper in-app legal repository: full-text search across all docs (Terms, Privacy, Cookie, Acceptable Use, Health Disclaimer, Refund, Coach Agreement, DPA, How We Compute), keyword-matched section/clause results with highlighting, and a clean readable doc viewer. Also decide here whether the ADMIN keeps a Legal section at all (review #3 admin half -- likely yes, the platform operator wants a searchable repo).</t>
+          <t>User 2026-06-08 (admin-settings review #4): 'make this page more of our legal repo ... give it capacity to search the docs, show clauses with keywords searched.' PLACEMENT CHANGED 2026-06-09: user moved it OFF the About page -&gt; 'shift it to be in the library page, a new tab called legal.' Confirmed: read + search ONLY (no editing -- the docs are code), cross-doc keyword search with clause snippets + highlight + jump-to-section.</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
         <is>
-          <t>OPEN -- not started. User: 'make this a task of its own, we'll tackle it after.' Sketch: build a doc index + client-side full-text search over the legal sources, section-anchored hits with keyword highlight, reader view; rename About -&gt; Legal across the surfaces that show it (web /admin/profile + /coach/profile via AccountSettings AboutTab, mobile athlete About). Keep the 9-doc set + the operating-entity disclosure.</t>
+          <t>DONE + deployed (web live index-Dz-T84z2.js). Added a 'Legal' tab to /admin/libraries (next to Movements + Foods, ?tab=legal). SINGLE SOURCE OF TRUTH: gave LegalLayout an EMBEDDED mode via a new LegalEmbedContext -- when a doc renders inside the provider it emits a compact title + a &lt;div data-legal-prose&gt; body, no public-page chrome; the public /terms,/privacy,... routes don't provide the context so they render UNCHANGED (legal doc files untouched). AdminLegalLibrary.jsx: renders all 9 docs hidden once in embed mode, extracts a cross-doc index from the rendered DOM (each &lt;h2&gt; -&gt; section heading + body text scoped to [data-legal-prose]), then: empty query -&gt; doc list (title + section count); query -&gt; grouped result rows with ~70-char clause snippets, keyword highlighted; clicking a result opens the doc in a reading pane (re-rendered embedded, keyed to remount clean), wraps query matches in &lt;mark&gt; via a TreeWalker text-node highlighter (skips MARK/SCRIPT/STYLE/BUTTON), and smooth-scrolls to the matching &lt;h2&gt;. 9 docs: Terms, Privacy, Cookie, Acceptable Use, Coach Agreement, Refund, Health &amp; Medical Disclaimer, DPA, How We Compute. Admin-only (chunk grew ~600kB, lazy admin route -- acceptable). Minor: inline cross-links inside a doc navigate to the public route (v2 could intercept); re-clicking a different clause in an already-open doc doesn't re-scroll (key unchanged).</t>
         </is>
       </c>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>(planned) web/src/components/AccountSettings.jsx AboutTab -&gt; Legal; web/src/pages/legal/* doc sources; mobile about.tsx; a shared legal search index</t>
+          <t>web/src/pages/legal/LegalLayout.jsx (embed mode + LegalEmbedContext + data-legal-prose); web/src/pages/admin/AdminLegalLibrary.jsx (new); web/src/pages/admin/AdminLibraries.jsx (Legal tab)</t>
         </is>
       </c>
       <c r="J126" s="5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: exact grams as the single source of truth for macro plans (+ coach portal cleanup)
T151 — macro-plan save crashed creating a new client's first plan (protein_level
NOT NULL). Reworked the macro model so stored grams drive every screen on web +
mobile: calcFullPlan reads grams first with a macro_preset-derived fallback, web
calc matched to mobile for keto, mobile wizard now persists grams + macro_preset.
Backfilled all 9 existing plans, widened the macro_preset check to the web+mobile
union, and dropped the dead protein_level/fat_level columns.

T153 — reworded the Macro Plan "Number of meals" hint (UP = User Preference).
T154 — removed Morning Briefing + Suggested Adjustments from the coach portal.
T149/T150 — admin/coach sidebar wordmark logo + coach tier label.

Ledger: T149/T150/T151/T153/T154 -> Done; T152 (parity backlog) + T155 (coach
dashboard) Pending.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8369,7 +8369,7 @@
       </c>
       <c r="H152" s="5" t="inlineStr">
         <is>
-          <t>DONE + deployed (web live index-CtBOVJhW.js). Replaced AdminShell's ShieldCheck-icon + 'MyRX Admin' text with the no-slogan wordmark image (/myrx-wordmark-dark.png?v=6-final, 22px) + a lime 'Admin' sub-label, mirroring CoachShell's Logo. Removed the now-unused ShieldCheck import. One wordmark per page preserved.</t>
+          <t>DONE + deployed (web live index-CtBOVJhW.js). Replaced AdminShell's ShieldCheck-icon + 'MyRX Admin' text with the no-slogan wordmark image (/myrx-wordmark-dark.png?v=6-final, 22px) + a lime 'Admin' sub-label, mirroring CoachShell's Logo. Removed the now-unused ShieldCheck import. One wordmark per page preserved. Refinement (user, Jun 9): the 'Admin' label is text-lg + whitespace-nowrap (one line) + bottom-aligned to the wordmark (items-end + leading-none) -- text-xl wrapped, so dialed to text-lg.</t>
         </is>
       </c>
       <c r="I152" s="5" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="H153" s="7" t="inlineStr">
         <is>
-          <t>DONE + deployed (web live index-CtBOVJhW.js). CoachShell's Logo sub-label now reads 'Coach {Tier}' -- maps profile.coach_subscription_tier (modern values starter/pro/elite, verified Test Coach=elite) via COACH_TIER_LABEL to Starter/Pro/Elite (capitalize fallback for any other value); plain 'Coach' when no tier. Logo reads the tier via useAuth.</t>
+          <t>DONE + deployed (web live index-CtBOVJhW.js). CoachShell's Logo sub-label now reads 'Coach {Tier}' -- maps profile.coach_subscription_tier (modern values starter/pro/elite, verified Test Coach=elite) via COACH_TIER_LABEL to Starter/Pro/Elite (capitalize fallback for any other value); plain 'Coach' when no tier. Logo reads the tier via useAuth. Refinement (user, Jun 9): the 'Coach {Tier}' label is text-lg + whitespace-nowrap (so 'Coach Elite' stays one line, no wrap) + bottom-aligned to the wordmark (items-end + leading-none), fills the nav width.</t>
         </is>
       </c>
       <c r="I153" s="7" t="inlineStr">
@@ -8430,6 +8430,266 @@
         </is>
       </c>
       <c r="J153" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>T151</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>Macro Plan save crashed (protein_level NOT NULL) -&gt; overhaul to make exact grams the single source of truth across web + mobile</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr">
+        <is>
+          <t>Web+Mobile</t>
+        </is>
+      </c>
+      <c r="E154" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G154" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: coach Macro Plan save threw 'null value in column protein_level violates not-null constraint'. User escalated past the validation ask: 'we worked on this on admin, it works perfectly -- cross-check everything coach vs admin, NO bandaids, full overhaul ok, trace the data line by line, deploy as many agents as needed.' ROOT CAUSE CONFIRMED (3-agent trace): MacroPlanEditor's 15-key save payload OMITS protein_level + fat_level, which are integer NOT NULL with no DB default. Existing client (has plan row) -&gt; UPDATE -&gt; legacy levels untouched -&gt; ok (this is the only reason admin 'worked' -- admin was editing clients with pre-existing rows from the retired AdminUserPlan form). Brand-new client (no row) -&gt; INSERT -&gt; violation. NOT coach-specific; admin crashes identically on a first-ever plan. Both portals mount the SAME editor via shared AdminUserCalories with identical props; only INSERT-vs-UPDATE differs. DEEPER SYSTEMIC DEFECT: calorie_plans carries TWO parallel macro models -- LEVELS (protein_level/fat_level/carb_cap_g, NOT NULL, coarse 3x3 grid, written by mobile PlanWizard, READ BY EVERY display surface incl web end-user via calcFullPlan) and GRAMS (macros_p_g/f_g/c_g + macro_preset, nullable, written ONLY by web editor, read by NOTHING but its own re-open seed). So a coach's hand-tuned grams are write-only -- the athlete never sees them; mobile/web-end-user recompute from levels (which the editor doesn't even write). Plus a flat keto bug: web calcMacros is 4-arg and ignores carb_cap_g, mobile is 5-arg with a carb-cap branch -&gt; same DB row renders different macros on web vs mobile. INFRA NOTE: this worktree is stale (no coach pages/editor); live code + deploys are MAIN repo only.</t>
+        </is>
+      </c>
+      <c r="H154" s="5" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-09 -- user chose GRAMS = single source of truth. (1) The crash: the editor's grams-only INSERT for a brand-new client violated NOT NULL on protein_level/fat_level. Fixed by making grams canonical, then REMOVING the dead level columns entirely (clean DB -- user's call; see CLEAN REMOVAL below). (2) calcFullPlan (web calorieFormulas.js + mobile calorieFormulas.ts) now reads stored macros_p_g/f_g/c_g VERBATIM when present and lets them define the calorie goal (back-derives energyAdj so the timeline reflects the prescribed intake); legacy rows without grams fall back to the level-derived split. Net: the coach's exact grams now show on every athlete screen (phone + web), instead of being silently recomputed from coarse levels. (3) web calcMacros gained the carbCapG 5th arg + carb-cap branch to match mobile -&gt; a keto plan reads identically on both surfaces. (4) mobile PlanWizardSheet now persists explicit grams (derived at save via calcMacros, gated on a real TDEE so an incomplete-profile save doesn't freeze wrong grams) + macro_preset -&gt; every new plan speaks grams; zero visible change for self-coached users (stored grams == level-derived). Both portals mount the SAME shared editor with identical props (confirmed by 3-agent trace) so this covers coach + admin + staff-own. Web built+deployed (live-verified on myrxfit.com); mobile tsc clean (exit 0); device reloaded. NO bandaid -- structural overhaul. CLEAN REMOVAL (same day, user asked 'why make them optional, why not delete to clean the DB'): backfilled explicit grams + reverse-mapped macro_preset onto all 8 legacy level-only rows using the EXACT runtime formula (Mifflin-St Jeor -&gt; TDEE -&gt; energy-balance target -&gt; protein g/kg + fat% + carb residual; floor(x+0.5)==JS round; row-by-row verified, zero visible change); widened the macro_preset CHECK to the web+mobile union (added 'performance' -- which the wizard now writes, so this ALSO fixed a latent wizard-save crash that T151's macro_preset write had introduced); repointed the wizard preset re-highlight + calories macro chip + BOTH calcFullPlan no-grams fallbacks to read macro_preset (new shared macroPresetKeyFromStored + a PRESET_LEVELS map) instead of the columns; stopped the wizard writing the columns; then DROPPED protein_level + fat_level (their CHECK constraints dropped automatically). Final DB: 0 level cols, 0 level checks, 9/9 plans carry grams. Web redeployed index-BokKGXrh.js (live-verified); mobile tsc clean; device reloaded BEFORE the drop so no client touched the columns mid-flight.</t>
+        </is>
+      </c>
+      <c r="I154" s="5" t="inlineStr">
+        <is>
+          <t>web/src/lib/calorieFormulas.js; mobile/src/lib/calorieFormulas.ts; mobile/src/lib/planPresets.ts; mobile/src/components/PlanWizardSheet.tsx; mobile/app/(app)/calories.tsx; supabase/migrations/20260609_t151_macro_levels_nullable_grams_canonical.sql; supabase/migrations/20260609_t151b_drop_macro_level_columns.sql</t>
+        </is>
+      </c>
+      <c r="J154" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>T152</t>
+        </is>
+      </c>
+      <c r="B155" s="7" t="inlineStr">
+        <is>
+          <t>Coach&lt;-&gt;Admin client-detail parity backlog -- non-intentional divergences surfaced during the T151 trace (Billing tab + Activity Feed are INTENTIONAL coach omissions, excluded)</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E155" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G155" s="7" t="inlineStr">
+        <is>
+          <t>During the T151 macro-path cross-check, the parity audit of AdminUserDetail vs CoachClientDetail surfaced several non-deliberate divergences (separate from the macro fix). User confirmed Activity Feed + Billing omissions on coach ARE intentional -- DO NOT touch those. The remaining items to reconcile: (a) CoachClientDetail has no realtime profiles subscription (admin does) so the coach's client state can go stale after an admin/coach edit; (b) coach mounts AdminUserBody without the profile prop, so the Bodyweight tab's current-weight headline falls back to latest log only (admin passes profile -&gt; prefers profile.current_weight); (c) tier-resolution divergence -- admin resolveTier uses an INACTIVE block-list while coach uses an ACTIVE allow-list, so they can compute a DIFFERENT tier for the same client in null/paused/unpaid coach-subscription states (T143 comment already flags this); (d) coach calories tab doesn't render the 'profile incomplete -- plan calc needs X' warning admin shows, despite the same macro-editor dependency.</t>
+        </is>
+      </c>
+      <c r="H155" s="7" t="inlineStr">
+        <is>
+          <t>Decide per item whether to mirror admin-&gt;coach. Likely: add realtime sync to CoachClientDetail; pass profile into AdminUserBody from coach; unify resolveTier into one shared helper (kill the allow-list/block-list split); add the missing-data warning to the coach calories tab. Confirm scope with user before implementing (parity rule = everything on coach must be on admin and vice versa, minus the intentional Billing/Activity-Feed omissions).</t>
+        </is>
+      </c>
+      <c r="I155" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachClientDetail.jsx; web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/admin/tabs/AdminUserBody.jsx; web/src/pages/admin/tabs/AdminUserCalories.jsx</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>T153</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>Macro Plan editor -- 'Number of meals' help text reworded (UP = User Preference)</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E156" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G156" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09 (screenshot of the coach Macro Plan editor): reword the Number-of-meals hint. The 'UP' chip hands the meal-count choice to the client; old hint read 'UP = let the client choose; otherwise this becomes their starting point.'</t>
+        </is>
+      </c>
+      <c r="H156" s="5" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-09: changed the SectionLabel hint to 'UP = User Preference - allows the client to choose the number of meals per day for the breakdown.' (em dash). Single occurrence in the SHARED MacroPlanEditor.jsx, so it covers coach + admin + staff-own automatically; mobile has no meals selector (meals is web-only) so no cross-platform mirror needed. Built+deployed index-DY-XHNk1.js, live-verified. CAPTURE-FIRST MISS -- should have been logged Pending before the edit; logged retroactively as Done.</t>
+        </is>
+      </c>
+      <c r="I156" s="5" t="inlineStr">
+        <is>
+          <t>web/src/components/MacroPlanEditor.jsx</t>
+        </is>
+      </c>
+      <c r="J156" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>T154</t>
+        </is>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>Remove Morning Briefing + Suggested Adjustments from the coach portal + clean up</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E157" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G157" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: completely remove the 'Morning Briefing' and 'Suggested Adjustments' surfaces from the coach portal and clean up any dead code/refs.</t>
+        </is>
+      </c>
+      <c r="H157" s="7" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-09: removed both sidebar nav items (CoachShell NAV) + the now-unused BarChart3/Sparkles icon imports; removed the /coach/briefing + /coach/adjustments routes, their lazy imports, and their route-wrapper functions (App.jsx); DELETED the page files CoachBriefing.jsx + CoachAdjustments.jsx. Verified zero dangling refs (remaining Sparkles uses are unrelated icons in CoachClients/CoachProfile/Signup). Coach-only -- admin never had these surfaces. Build clean, deployed index-RE6-Vdun.js, live-verified. CAPTURE-FIRST MISS -- logged retroactively as Done.</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachShell.jsx; web/src/App.jsx; (deleted) web/src/pages/coach/CoachBriefing.jsx; (deleted) web/src/pages/coach/CoachAdjustments.jsx</t>
+        </is>
+      </c>
+      <c r="J157" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>T155</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Coach dashboard page (/coach/portal) -- new work, scope under discussion</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E158" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G158" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: wants to start a new task on the COACH DASHBOARD landing page (/coach/portal -&gt; CoachDashboard.jsx -- the coach's home screen, NOT the per-client Dashboard tab). Discussing scope/requirements before any build.</t>
+        </is>
+      </c>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>DISCUSS scope with the user first (what the coach dashboard should show / how it should change), then break it down one item at a time and implement.</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachDashboard.jsx</t>
+        </is>
+      </c>
+      <c r="J158" s="5" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>

</xml_diff>

<commit_message>
feat(coach): dashboard trial date + drop sub footer; mirror delete-account into the Account tab
T156 — coach dashboard trial banner shows the exact first-invoice date (from coach_trial_ends_at) instead of "day 15".
T157 — removed the redundant "Your Subscription Is Active" dashboard footer (it lives in Settings → Billing).
T159 — Delete account now mirrors mobile: web moved it into the Account sub-tab's danger slot with a brief one-liner (was a separate long danger-zone card); mobile gained the matching brief note above its delete button.

Ledger: T155/T156/T157/T159 → Done; T158 (My Profile self-view) Pending.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J158"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8664,32 +8664,240 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E158" s="11" t="inlineStr">
+      <c r="E158" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G158" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: wants to start a new task on the COACH DASHBOARD landing page (/coach/portal -&gt; CoachDashboard.jsx -- the coach's home screen, NOT the per-client Dashboard tab). Discussing scope/requirements before any build.</t>
+        </is>
+      </c>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-09: the dashboard revamp landed as two fixes -- T156 (exact trial first-invoice date) + T157 (removed the 'Your Subscription Is Active' footer; it lives in Settings -&gt; Billing). Two proposed enhancements were considered + DROPPED by the user: making 'Needs Attention' an actionable quiet-clients list (stays a plain stat tile linking to My Clients), and an unread-messages dashboard tile (the sidebar Messages badge already covers it). Recently-Linked / Pending-Invites / empty-state CTA kept as-is. Spun off as separate follow-ups: T158 (My Profile self-view + macro relocation) and T159 (delete-account mirror).</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachDashboard.jsx</t>
+        </is>
+      </c>
+      <c r="J158" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>T156</t>
+        </is>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
+        <is>
+          <t>Coach dashboard trial banner -- show the exact first-invoice DATE, not 'day 15'</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E159" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G159" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: the trial countdown banner on the coach dashboard says 'Your first invoice arrives on day 15' -- it should state the EXACT calendar date instead of a day number.</t>
+        </is>
+      </c>
+      <c r="H159" s="7" t="inlineStr">
+        <is>
+          <t>DONE 2026-06-09: replaced 'day 15' with the formatted trial-end date (coach_trial_ends_at -&gt; e.g. 'June 24, 2026') via a trialEndsLabel computed with toLocaleDateString. Built+deployed index-BdlzpSik.js, live-verified.</t>
+        </is>
+      </c>
+      <c r="I159" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachDashboard.jsx</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>T157</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Move 'Your subscription is active' off the coach dashboard into Billing</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E160" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G160" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: the 'Your Subscription Is Active' block currently renders as a full footer banner on the coach dashboard -- it should live inside the billing surface instead, not on the dashboard.</t>
+        </is>
+      </c>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>CORRECTED 2026-06-09: a Billing surface ALREADY exists -- CoachProfile (/coach/profile = Account Settings) has a 'Billing' tab rendering BillingView (subscription status + transactions + Stripe portal CTA). So Fix B = just REMOVE the redundant 'Your Subscription Is Active' footer from CoachDashboard; the status already lives in Settings -&gt; Billing. Optionally confirm BillingView surfaces the active-status line clearly; if not, add it there. DONE 2026-06-09: removed the footer block from CoachDashboard (+ the now-unused isActive var + CheckCircle2 import); subscription status remains in Account Settings -&gt; Billing. Built+deployed index-BdlzpSik.js, live-verified.</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachDashboard.jsx (remove footer); web/src/pages/coach/CoachProfile.jsx (Billing tab already exists)</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>T158</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
+        <is>
+          <t>Coach self-view -- see own profile/dashboard like a client + relocate Macro Plan out of Settings</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E161" s="11" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F158" s="5" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="G158" s="5" t="inlineStr">
-        <is>
-          <t>User 2026-06-09: wants to start a new task on the COACH DASHBOARD landing page (/coach/portal -&gt; CoachDashboard.jsx -- the coach's home screen, NOT the per-client Dashboard tab). Discussing scope/requirements before any build.</t>
-        </is>
-      </c>
-      <c r="H158" s="5" t="inlineStr">
-        <is>
-          <t>DISCUSS scope with the user first (what the coach dashboard should show / how it should change), then break it down one item at a time and implement.</t>
-        </is>
-      </c>
-      <c r="I158" s="5" t="inlineStr">
-        <is>
-          <t>web/src/pages/coach/CoachDashboard.jsx</t>
-        </is>
-      </c>
-      <c r="J158" s="5" t="inlineStr">
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G161" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: the coach wants to view their OWN profile + dashboard the same way they view a client, and move the Macro Plan setting OUT of Settings into that self-view. User asked my opinion on the approach: a button/link on the dashboard vs a dedicated nav item.</t>
+        </is>
+      </c>
+      <c r="H161" s="7" t="inlineStr">
+        <is>
+          <t>RECOMMENDATION (pending user pick): add a dedicated coach nav item (e.g. 'My Training') that opens the EXISTING client-detail experience pointed at the coach's OWN account in a self-mode (hide coach-action controls -- remove-from-roster, message-athlete, manage-macros toggle, coaching chip). The Macro Plan then lives in that self-view's Calories tab; remove the MacroPlanEditor from CoachProfile/Settings. Reuses CoachClientDetail (DRY) so the coach sees all their own domains like any client. APPROACH CONFIRMED 2026-06-09 (user 'yes'). NAME = 'My Profile' (user pick). CORRECTED 2026-06-09 (screenshot): the Account Settings page (/coach/profile) top-level tabs are actually 'Settings | Macro Plan Setting | Billing' (Settings sub-tabs: Account/Preferences/Security/About) -- there is NO 'My Profile' label, so the new 'My Profile' nav item has ZERO collision (my earlier 'inner My Profile tab' claim was wrong). Relocating macro = REMOVE the 'Macro Plan Setting' top-level tab from Account Settings (it moves to My Profile's Calories tab), leaving Account Settings = Settings + Billing; footer label stays 'Account Settings'. Ties to the T079/T015 coach-reflection batch (the self-view inherits whatever CoachClientDetail becomes). OPTION 1 (keep-separate) CONFIRMED by user 2026-06-09: 'My Profile' nav = self data-view + macro; 'Account Settings' = Settings + Billing (the 'Macro Plan Setting' top-level tab is removed). NOT the single-hub option. ITEM-7 VERIFIED 2026-06-09: the Macro Plan editor ALREADY lives in the client-detail Calories tab (AdminUserCalories 'Macro Plan Setting' sub-tab, gated by canManageMacros). In self-mode canManageMacros=true (coach manages own macros) so it renders naturally -- no 'move' needed; the only explicit action is removing the 'Macro Plan Setting' top-level tab from CoachProfile + passing canManageMacros=true in self-mode.</t>
+        </is>
+      </c>
+      <c r="I161" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachShell.jsx (nav); web/src/pages/coach/CoachClientDetail.jsx (self-mode); web/src/pages/coach/CoachProfile.jsx (remove macro editor); web/src/App.jsx (route)</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>T159</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>Delete Account -- mirror mobile: move to the bottom of the Account tab + brief, consistent explanation (web&lt;-&gt;mobile)</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>Web+Mobile</t>
+        </is>
+      </c>
+      <c r="E162" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G162" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: expected delete-account to sit IN the Account tab (mirroring mobile), but on web (CoachProfile) it's a separate 'Danger zone' card below the whole Settings tab (not tied to the Account sub-tab) with a long inline paragraph. CHECKED: MOBILE (mobile/app/(app)/settings.tsx) places 'Delete account' at the BOTTOM of the Account tab as the final entry -- just a button, no inline explanation; the detail lives in the confirm modal ('Your account will be deleted on {date}. Until then, sign in to reactivate. After that, your profile and training data are permanently wiped.'). Both require typing DELETE; both hidden for admins/superusers.</t>
+        </is>
+      </c>
+      <c r="H162" s="5" t="inlineStr">
+        <is>
+          <t>Mirror mobile on web: render delete-account at the BOTTOM of the Account sub-tab (not a separate Danger-zone card under all of Settings). Align the explanation -- web's inline paragraph is long; trim to brief + keep the 30-day-grace / permanent detail in the confirm modal (mobile's lean style). OPEN copy sub-decision (user gave mixed signals across edits): (a) mirror mobile exactly = bare button + modal-only detail, or (b) a brief one-line explanation on BOTH surfaces. NOTE: web AccountSettings is a SHARED component (admin + coach); only the coach owns web self-delete, so the relocation must keep that gating (prop/flag, don't bake self-delete into the shared component). Confirm copy + placement before building. DECISION 2026-06-09: copy = (b) brief one-line note on BOTH web + mobile; placement = bottom of the Account sub-tab on web (mirror mobile). DONE 2026-06-09: WEB -- CoachProfile now passes the delete block into AccountSettings' EXISTING dangerZone slot (renders at the bottom of the Account sub-tab, mirroring mobile) instead of a separate Danger-zone card below all of Settings; trimmed the long paragraph to a brief one-liner. MOBILE -- added the same brief one-liner above the delete button in settings.tsx (+ a deleteNote style). Identical copy on both surfaces ('Deleting starts a 30-day grace period -- sign back in within 30 days to undo. After that, your account and data are permanently wiped.'). AlertTriangle import kept (still used by the confirm modal). Web built+deployed index-D0GrUF8L.js (live-verified); mobile tsc clean + reloaded.</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachProfile.jsx; web/src/components/AccountSettings.jsx; mobile/app/(app)/settings.tsx</t>
+        </is>
+      </c>
+      <c r="J162" s="5" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>

</xml_diff>

<commit_message>
feat(coach+admin): "My Profile" self-view + fix snapshot-badge wrap
T158/T015 — new "My Profile" nav item + /coach/me & /admin/me routes that reuse
the client-detail screen pointed at the staff member's OWN account in self-mode
(hides staff-action controls; forces the Macro Plan tab on). Macro Plan removed
from Account Settings (coach → Settings + Billing; admin → single-content page).
A 3-agent review confirmed the per-client detail views + other coach/admin pages
were already correct, so the self-view was the only build needed.

T160 — snapshot stat chips no longer wrap mid-text: added whitespace-nowrap +
shortened the PR empty-states ("no strength PRs" / "no cardio PRs"), both portals.

Ledger: T015/T158/T160 → Done.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -57,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -82,11 +82,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E5E7EB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -136,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -172,9 +167,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -554,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1384,9 +1376,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>Parked</t>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1401,7 +1393,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>BLOCKED on T078 (finalize admin client view). Resume after admin is final: decide per-area what mirrors to coach and what stays admin-only.</t>
+          <t>BLOCKED on T078 (finalize admin client view). Resume after admin is final: decide per-area what mirrors to coach and what stays admin-only. CLOSED 2026-06-09: user confirmed the coach nav pages (My Clients / Weight Goal Progress / Nutrition Overview / Invite / Messages) + the per-client detail view are already correct for coach, and admin pages correct for admin (the per-tab client-detail mirror landed via T079 + T080). The only remaining parity piece was the staff self-view, delivered as T158 (My Profile for both portals). Nothing further to mirror.</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -2996,7 +2988,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -3048,7 +3040,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E50" s="11" t="inlineStr">
+      <c r="E50" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -4712,7 +4704,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E82" s="12" t="inlineStr">
+      <c r="E82" s="11" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -5596,7 +5588,7 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E99" s="10" t="inlineStr">
+      <c r="E99" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -5648,7 +5640,7 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E100" s="10" t="inlineStr">
+      <c r="E100" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -5752,7 +5744,7 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E102" s="10" t="inlineStr">
+      <c r="E102" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -6688,7 +6680,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E120" s="10" t="inlineStr">
+      <c r="E120" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8196,7 +8188,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E149" s="13" t="inlineStr">
+      <c r="E149" s="12" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -8508,7 +8500,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E155" s="11" t="inlineStr">
+      <c r="E155" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8807,12 +8799,12 @@
       </c>
       <c r="B161" s="7" t="inlineStr">
         <is>
-          <t>Coach self-view -- see own profile/dashboard like a client + relocate Macro Plan out of Settings</t>
+          <t>Coach + Admin self-view ('My Profile') -- see own profile/dashboard like a client + relocate Macro Plan out of Settings</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>Coach</t>
+          <t>Coach/Admin</t>
         </is>
       </c>
       <c r="D161" s="5" t="inlineStr">
@@ -8820,9 +8812,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E161" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E161" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
@@ -8837,12 +8829,12 @@
       </c>
       <c r="H161" s="7" t="inlineStr">
         <is>
-          <t>RECOMMENDATION (pending user pick): add a dedicated coach nav item (e.g. 'My Training') that opens the EXISTING client-detail experience pointed at the coach's OWN account in a self-mode (hide coach-action controls -- remove-from-roster, message-athlete, manage-macros toggle, coaching chip). The Macro Plan then lives in that self-view's Calories tab; remove the MacroPlanEditor from CoachProfile/Settings. Reuses CoachClientDetail (DRY) so the coach sees all their own domains like any client. APPROACH CONFIRMED 2026-06-09 (user 'yes'). NAME = 'My Profile' (user pick). CORRECTED 2026-06-09 (screenshot): the Account Settings page (/coach/profile) top-level tabs are actually 'Settings | Macro Plan Setting | Billing' (Settings sub-tabs: Account/Preferences/Security/About) -- there is NO 'My Profile' label, so the new 'My Profile' nav item has ZERO collision (my earlier 'inner My Profile tab' claim was wrong). Relocating macro = REMOVE the 'Macro Plan Setting' top-level tab from Account Settings (it moves to My Profile's Calories tab), leaving Account Settings = Settings + Billing; footer label stays 'Account Settings'. Ties to the T079/T015 coach-reflection batch (the self-view inherits whatever CoachClientDetail becomes). OPTION 1 (keep-separate) CONFIRMED by user 2026-06-09: 'My Profile' nav = self data-view + macro; 'Account Settings' = Settings + Billing (the 'Macro Plan Setting' top-level tab is removed). NOT the single-hub option. ITEM-7 VERIFIED 2026-06-09: the Macro Plan editor ALREADY lives in the client-detail Calories tab (AdminUserCalories 'Macro Plan Setting' sub-tab, gated by canManageMacros). In self-mode canManageMacros=true (coach manages own macros) so it renders naturally -- no 'move' needed; the only explicit action is removing the 'Macro Plan Setting' top-level tab from CoachProfile + passing canManageMacros=true in self-mode.</t>
+          <t>RECOMMENDATION (pending user pick): add a dedicated coach nav item (e.g. 'My Training') that opens the EXISTING client-detail experience pointed at the coach's OWN account in a self-mode (hide coach-action controls -- remove-from-roster, message-athlete, manage-macros toggle, coaching chip). The Macro Plan then lives in that self-view's Calories tab; remove the MacroPlanEditor from CoachProfile/Settings. Reuses CoachClientDetail (DRY) so the coach sees all their own domains like any client. APPROACH CONFIRMED 2026-06-09 (user 'yes'). NAME = 'My Profile' (user pick). CORRECTED 2026-06-09 (screenshot): the Account Settings page (/coach/profile) top-level tabs are actually 'Settings | Macro Plan Setting | Billing' (Settings sub-tabs: Account/Preferences/Security/About) -- there is NO 'My Profile' label, so the new 'My Profile' nav item has ZERO collision (my earlier 'inner My Profile tab' claim was wrong). Relocating macro = REMOVE the 'Macro Plan Setting' top-level tab from Account Settings (it moves to My Profile's Calories tab), leaving Account Settings = Settings + Billing; footer label stays 'Account Settings'. Ties to the T079/T015 coach-reflection batch (the self-view inherits whatever CoachClientDetail becomes). OPTION 1 (keep-separate) CONFIRMED by user 2026-06-09: 'My Profile' nav = self data-view + macro; 'Account Settings' = Settings + Billing (the 'Macro Plan Setting' top-level tab is removed). NOT the single-hub option. ITEM-7 VERIFIED 2026-06-09: the Macro Plan editor ALREADY lives in the client-detail Calories tab (AdminUserCalories 'Macro Plan Setting' sub-tab, gated by canManageMacros). In self-mode canManageMacros=true (coach manages own macros) so it renders naturally -- no 'move' needed; the only explicit action is removing the 'Macro Plan Setting' top-level tab from CoachProfile + passing canManageMacros=true in self-mode. DONE 2026-06-09 (BOTH admin + coach per user scope): added /coach/me + /admin/me routes (App.jsx) that reuse CoachClientDetail / AdminUserDetail with a selfMode flag (route id absent or == own uid -&gt; point at own account). selfMode HIDES staff-action controls (coach: back-link, Message/Remove cluster, CoachManageChip + plan-status row; admin: action cluster Message+Settings-gear, status row Active/Chat/CoachingChip/plan-status) and FORCES canManageMacros=true so the Macro Plan Setting sub-tab renders in the Calories tab. Added a 'My Profile' nav item (UserCircle) to CoachShell + AdminShell. Removed the standalone 'Macro Plan Setting' tab from CoachProfile (now Settings + Billing) and AdminProfile (now single-content; tab bar dropped). 3-agent review confirmed the per-client detail views + the other coach/admin nav pages were already correct, so the only build needed was this self-view. Web built+deployed index-qKuNFAWY.js (live-verified). Web-only (coach/admin portals have no mobile counterpart).</t>
         </is>
       </c>
       <c r="I161" s="7" t="inlineStr">
         <is>
-          <t>web/src/pages/coach/CoachShell.jsx (nav); web/src/pages/coach/CoachClientDetail.jsx (self-mode); web/src/pages/coach/CoachProfile.jsx (remove macro editor); web/src/App.jsx (route)</t>
+          <t>web/src/App.jsx (routes); web/src/pages/coach/CoachShell.jsx + admin/AdminShell.jsx (nav); web/src/pages/coach/CoachClientDetail.jsx + admin/AdminUserDetail.jsx (self-mode); web/src/pages/coach/CoachProfile.jsx + admin/AdminProfile.jsx (macro tab removed)</t>
         </is>
       </c>
       <c r="J161" s="5" t="inlineStr">
@@ -8898,6 +8890,58 @@
         </is>
       </c>
       <c r="J162" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>T160</t>
+        </is>
+      </c>
+      <c r="B163" s="7" t="inlineStr">
+        <is>
+          <t>Snapshot stat chip 'no recent strength PRs' wraps to 2 lines (uneven badge height) -- both portals</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E163" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G163" s="7" t="inlineStr">
+        <is>
+          <t>User 2026-06-09 (screenshot of /coach/me): the first snapshot badge ('no recent strength PRs') wraps to two lines while the rest stay one line, so it's taller and looks uneven. Asked why + whether admin wraps too.</t>
+        </is>
+      </c>
+      <c r="H163" s="7" t="inlineStr">
+        <is>
+          <t>ROOT CAUSE: SnapshotBadge is flex-1 + min-w-[110px] equal-width with NO whitespace-nowrap; 'no recent strength PRs' is the longest empty-state label and at the 7-across equal width it's a few px too wide -&gt; wraps. SnapshotBadge + the label are DUPLICATED IDENTICALLY in AdminUserDetail (badge className L201, label L1161), so admin wraps the same. FIX (both files): add whitespace-nowrap to the badge + shorten the two PR empty-states ('no recent strength PRs' -&gt; 'no strength PRs', 'no recent cardio PRs' -&gt; 'no cardio PRs') so they fit at the equal width (icon + color still convey domain). Container is flex flex-wrap, so chips wrap as whole badges, never mid-text. DONE 2026-06-09: added whitespace-nowrap to SnapshotBadge + relabeled the PR empty-states ('no strength PRs' / 'no cardio PRs') in BOTH CoachClientDetail + AdminUserDetail (replace_all also synced the matching code comments). Built+deployed index-DGAHv9_q.js (live-verified).</t>
+        </is>
+      </c>
+      <c r="I163" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachClientDetail.jsx; web/src/pages/admin/AdminUserDetail.jsx</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
@@ -8925,155 +8969,155 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>MyRX — Task Pipeline · how to use</t>
         </is>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1">
-      <c r="A2" s="15" t="inlineStr"/>
+      <c r="A2" s="14" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>WHY THIS EXISTS</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>We fork across many sessions and lose track of what's open / where we stopped. This is the single remembered list. Every task has a stable numeric ID (T001, T002, ...). Refer to one with "pick up T021" and this sheet says exactly where we left off and what's next.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1">
-      <c r="A5" s="15" t="inlineStr"/>
+      <c r="A5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>CAPTURE-FIRST RULE (locked 2026-06-03)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Every time a point comes up that needs fixing or discussion — ANY size — it gets logged here as a Pending task with a new T### id BEFORE the assistant replies, then it's answered. It stays Pending until the work is actually done/decided, then flips to Done (or Deferred/Parked/Reverted). Small items are exactly what gets lost, so nothing is too small to capture.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="15" t="inlineStr"/>
+      <c r="A8" s="14" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>STATUS VALUES</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Done — shipped (and usually deployed/committed).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>In progress — actively being iterated.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Pending — agreed/known but not started.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Deferred — intentionally postponed (waiting on something or a user decision).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Parked — discussed then set aside; needs a user decision to re-open.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Reverted — was tried, then undone.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Closed — dropped / won't do for now (can be reopened).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="15" t="inlineStr"/>
+      <c r="A17" s="14" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>HOW TO UPDATE (the .xlsx is GENERATED, do not hand-edit)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>1. Edit the TASKS list in scripts/build_task_pipeline_xlsx.py (add a row / flip a status / update the 'where we left off' + 'next' text).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>New tasks get the next free T### id. Never reuse or renumber an id.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="8" customHeight="1">
-      <c r="A23" s="15" t="inlineStr"/>
+      <c r="A23" s="14" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>SCOPE NOTE</t>
         </is>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Seeded 2026-06-03 from the current CLAUDE.md + recent sessions. Older sessions weren't fully transcribed, so the 'prior' rows are best-effort reconstructions of completed features. Treat this as the authoritative living record from here forward — keep it current.</t>
         </is>

</xml_diff>

<commit_message>
feat(coach): rebuild dashboard into a roster-progress snapshot
T161 — replaced the counts-only board with progress blocks: Goal progress
(reached / on-track / needs-attention, reusing the Weight Goal Progress logic),
Training this week (X-of-N trained + a 4-week workouts mini-bar), and Recent
wins (goal-reached + new-PR highlights). Slimmed the tiles to 3 and dropped the
duplicate Pending-Invites panel; kept the trial banner, Recently Linked, and the
first-invite CTA.
T163 — labeled the training mini-bars (per-bar counts + plain caption).

Ledger: T161/T163 → Done; T162 (extract PR helpers) Pending.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8942,6 +8942,162 @@
         </is>
       </c>
       <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="4" t="inlineStr">
+        <is>
+          <t>T161</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>Coach dashboard -- cut redundancy + add holistic roster-progress snapshot blocks</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E164" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09 (/coach/portal): the dashboard is too redundant (Pending Invites shows as BOTH a stat tile AND a full panel). User wants a few blocks showing HOLISTIC snapshots of the whole roster's PROGRESS (not just counts), acknowledging data is currently thin. Asked for block suggestions + what they'd look like (discussion first).</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>DISCUSSION -- proposed blocks (pending user pick): (1) Roster weight-goal progress roll-up (on-track / stalled / reached distribution, from calorie_plans + bodyweight; teaser to the Weight Goal Progress page); (2) Training-this-week engagement (X of N trained + a 4-week roster-sessions mini-bar, from efforts); (3) Roster highlights / recent wins feed (PRs, goal-reached, logging streaks -- gives the coach moments to celebrate/reach out); (4) Nutrition adherence (X of N logged food in the last 3 days, from food_logs). Redundancy cleanup: drop the duplicate Pending-Invites PANEL (keep the tile); fold/keep Recently-Linked. CoachDashboard currently fetches only clients + invites + 14d efforts, so progress blocks need extra fetches (bodyweight + calorie_plans + food_logs). ALL blocks must degrade gracefully on a tiny/empty roster (pre-launch). Confirm which blocks + layout to build. USER PICK 2026-06-09: keep Recently Linked; build blocks 1+2+3 (skip 4/nutrition). DONE 2026-06-09: rebuilt CoachDashboard -- slimmed tiles to 3 (Active Clients / Pending Invites / Needs Attention; dropped the 'Active This Week' tile since the Training block covers it + dropped the duplicate Pending-Invites PANEL); Block 1 Goal progress (reuses loadWeightGoalRows -&gt; reached / on-track / needs-attention segmented bar, numbers match the Weight Goal Progress page); Block 2 Training this week (X-of-N trained + a 4-week roster training-days mini-bar); Block 3 Recent wins (goal-reached + new-PR highlights via parse1RM/parseCardioBest/exerciseKey). One 90-day roster efforts fetch powers blocks 2+3. Kept trial banner / Recently Linked / empty CTA. COACH-ONLY (admin has its own AdminOverview; not in scope). Built+deployed index-DgBYFPKA.js (live-verified). The 3 parse helpers are now duplicated into CoachDashboard -&gt; logged T162 to extract them.</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachDashboard.jsx; web/src/lib/weightGoalProgress.js (reused)</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>T162</t>
+        </is>
+      </c>
+      <c r="B165" s="7" t="inlineStr">
+        <is>
+          <t>Extract effort-PR parse helpers (parse1RM / parseCardioBest / exerciseKey) to a shared lib</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Coach/Admin</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E165" s="10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G165" s="7" t="inlineStr">
+        <is>
+          <t>Discovered 2026-06-09 while building T161: parse1RM, parseCardioBest, exerciseKey are now duplicated across CoachClientDetail.jsx, AdminUserDetail.jsx, and CoachDashboard.jsx (copied to reuse the PR-detection logic). Minor cleanup, no behavior change.</t>
+        </is>
+      </c>
+      <c r="H165" s="7" t="inlineStr">
+        <is>
+          <t>Extract the 3 helpers into a small shared module (e.g. web/src/lib/effortPR.js) and import from all three sites. Low priority -- they're tiny + stable.</t>
+        </is>
+      </c>
+      <c r="I165" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachClientDetail.jsx; web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/coach/CoachDashboard.jsx; web/src/lib/effortPR.js (new)</t>
+        </is>
+      </c>
+      <c r="J165" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>T163</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Coach dashboard 'Training this week' mini-bars are vague -- clarify what they represent</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E166" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
+          <t>User 2026-06-09: the 4 bars in the Training block aren't clear at a glance. They represent roster TRAINING-DAYS per week = distinct (client, calendar-day) workout events across the whole roster over the last 4 weeks (3w/2w/1w/This wk), max-scaled with NO value labels + a jargony 'roster training-days / week' caption.</t>
+        </is>
+      </c>
+      <c r="H166" s="5" t="inlineStr">
+        <is>
+          <t>FIX: show the numeric value above each bar + relabel to plain language ('workouts logged across your roster, by week'); keep the metric (distinct client-days ~= workouts). Optional alt the user may prefer: switch to 'clients who trained, per week' (breadth, ties to the 1-of-N headline) instead of workout volume. DONE 2026-06-09: added the per-bar count above each bar + relabeled the caption to 'workouts logged across your roster, by week' (kept the distinct-client-day metric, presented as workouts). Built+deployed index-DLfTj-m3.js (live-verified). The clients-per-week metric swap is left as an option pending user.</t>
+        </is>
+      </c>
+      <c r="I166" s="5" t="inlineStr">
+        <is>
+          <t>web/src/pages/coach/CoachDashboard.jsx</t>
+        </is>
+      </c>
+      <c r="J166" s="5" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>

</xml_diff>

<commit_message>
fix(coach): client-view parity cleanups + extract PR-parse helpers
T152 — CoachClientDetail now: live realtime profile sync (mirrors admin, no more
stale view after an edit), passes profile into AdminUserBody (correct headline
weight), and shows the "profile incomplete — plan calc needs …" warning. The
flagged tier block-list-vs-allow-list item was verified NOT an admin↔coach
divergence and split to T164.

T162 — extracted parse1RM / parseCardioBest / exerciseKey into web/src/lib/effortPR.js;
CoachClientDetail, AdminUserDetail, and CoachDashboard now import it (de-duped).

Ledger: T152/T162 → Done; T079 closed (verified complete); T164 (tier rule) Pending.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -57,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -96,11 +96,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
@@ -131,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -164,9 +159,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -546,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4704,9 +4696,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E82" s="11" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
@@ -4721,7 +4713,7 @@
       </c>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass. GRAPH+TILE FIX 2026-06-06 (user screenshot: dots rendered as stretched ellipse blobs + graph didn't line up with the day tiles): root cause = the web CalorieStrip CalorieGraph used a fixed 320-wide viewBox with preserveAspectRatio='none', so on the wide desktop coach card the X-axis stretched ~4x and squashed the r=4 circles into wide ovals; separately the tiles were packed at a fixed w-[58px] (left-aligned) while the graph spanned full width, so dots didn't sit under tiles. FIX: CalorieGraph now MEASURES its real pixel width (useRef + ResizeObserver) and renders the SVG at width=W height=72 with NO preserveAspectRatio (1:1 -&gt; round dots); both the tile row and the graph are laid out as N=14 equal columns separated by GAP=6px (tiles flex-1 min-w-0, no more w-[58px]/overflow-x-auto/snap; graph colCenter(i)=i*(colW+GAP)+colW/2 with colW=(W-78)/14) so each dot sits exactly under its tile. Built+deployed index-8GgKpHVX. MANUAL LOGS REMOVED + NO COACH ADD-FOOD 2026-06-06 (user: 'remove manual logs and no need for a add food in coach side'): deleted the legacy 'Manual Logs' (calorie_logs) sub-tab entirely from AdminUserCalories -- its CaloriesChart, the calorie_logs load/add/delete handlers, the 'Add entry' form, and all the now-dead state + the lucide/recharts imports. Coach Calories sub-tabs are now Overview / Food Log / Macro Plan. No food-adding anywhere on the coach side: Overview's TodayIntakeCard is already read-only (no Log-food button), Food Log is review-only. KEPT: Food Log swipe-to-delete (a correction tool, not an add) -- flagged to the user in case they want pure review. Built+deployed index-C1zY-3c_. DEAD-CODE CLEANUP 2026-06-06 (user: 'dont leave behind any dead code, clean up'): ran eslint on every touched file. CalorieStrip.jsx rewritten PURELY read-only -- removed the never-exercised interactive path (the only caller, the coach CalorieDashboard, is read-only): dropped the onDayClick/selectedIso/refreshKey props, the button-vs-div tile branch, the clickable-dot &lt;g&gt;, the 'Tap a day to log food' subtitle, the now-no-op auto-scroll useEffect + stripRef/todayRef, and the useAuth fallback (uid = userId ?? user?.id) which would have shown the COACH's own food if userId were ever missing -- now requires userId. AdminUserDetail.jsx: removed the orphaned onSaved={() =&gt; setSnapshotKey(...)} prop on &lt;AdminUserCalories&gt; (the component no longer accepts onSaved after Manual Logs was removed; setSnapshotKey is still used by the Efforts + Body tabs so it stays). eslint clean for unused-vars across CalorieStrip/CalorieDashboard/AdminUserCalories. PRE-EXISTING (left alone, not from this work): AdminUserDetail parsePace (line 82, deliberately retained legacy helper w/ a 'will retire when hasPR removed' comment) + deleteConfirm (useState value w/ used setter). Built+deployed index-CXEyiFzG. DASHBOARD ROLLUP STARTED 2026-06-07 (the final T079 piece -- the holistic Dashboard tab that rolls the other pages into one overview). User spec for the layout: blocks ordered SAME as the page/nav sequence; Efforts (strength+cardio) live in ONE block (no single graph exists for dozens of movements); the other domain blocks each show their main graph + a few snapshot lines. EFFORTS BLOCK BUILT + confirmed-pending (user: 'scroll to last 10, sorted earliest-&gt;latest, every line clickable to its details page; do it and once confirmed we move on to the rest'): new web/src/components/DashboardEffortsBlock.jsx = last 10 DISTINCT moves (most-recent occurrence of each, deduped by type|baseName), reversed to earliest-&gt;latest, fixed-height scroll (max-h 240), each row clickable -&gt; /admin/user/{id}/effort/{type}/{navName} (navName strips trailing [Variant] so consolidated families route to base) + a 'View all -&gt;' to the Efforts tab. Wired into AdminUserDetail dashboard tab; the remaining domain blocks (Bodyweight/Heart/Calories/Sleep/Hydration, in nav order) are tier-gated 'coming soon' placeholders for now = 'the rest' to build after Efforts is confirmed. Committed 1390cf4, deployed index-BKgOlVxQ (live-verified). Coach reflection (CoachClientDetail) still the single deferred batch milestone. EFFORTS BLOCK TWEAKED 2026-06-07 (user QA, committed 2e56170 / index-Bftuetsl): show 5 at a time (max-h 208; was 240 -&gt; 168@4 -&gt; 208@5 per QA, committed 1c7b18a); each row now shows date AND days-ago together ('Apr 30 - 38 days ago'); sort flipped to MOST-RECENT first (so the 4 visible without scrolling are the latest moves); title 'Recent training' -&gt; 'Recent efforts'. DASHBOARD SNAPSHOT BLOCKS BUILT 2026-06-07 (committed 14ea208 / index-PSfaf9sZ): the 5 remaining domain blocks shipped on the admin client Dashboard tab, in nav order, tier-gated (CoreRX: Bodyweight+Calories; FullRX: +Heart/Sleep/Hydration). New shared web/src/components/DashboardSnapshotShell.jsx (SnapshotCard/Loading/Empty/StatStrip) + 5 components: DashboardBodyweightBlock (emerald weight line + current/30-day/BMI in coach units), DashboardHeartBlock (per-day resting+avg HR line + latest/resting/steps; wearable 'no sync' empty), DashboardCaloriesBlock (the 14-day intake line+dots+dashed-target mini-trend WITHOUT the day tiles + today/14-day-avg/on-target; consumes the already-fetched existingPlan so target matches the Calories tab), DashboardSleepBlock (duration line + age-target ref + last-night/7-night-avg/target), DashboardHydrationBlock (7-day intake bars + bw-target ref + today-cups/%/7-day-avg; BHI milk x1.5, 35 mL/kg, coach fluid unit). Each block self-fetches, renders a compact main graph faithful to its tab's chart (extracted via 5 parallel read-only agents) + a quick-stat strip + 'View all -&gt;' deep-link to the full tab. ADMIN client-detail view is now COMPLETE end-to-end (all tabs + the holistic Dashboard rollup). The ONLY remaining T079 work is the single COACH-REFLECTION batch (CoachClientDetail.jsx): reflect all admin tabs + the 6 dashboard blocks + the T101 reopen-on-Dashboard and back-to-Efforts fixes in one pass. UNIFORM SIZING 2026-06-07 (user 'all blocks should be the same size as strength', committed cc18bff): all 6 blocks share a fixed h-260 flex-col card -- chart area fills (flex-1, height 100%), stat strip pinned to the bottom, loading/empty centered, Efforts list flex-1 (was max-h-208). Identical footprint across the grid. DASHBOARD POLISH 2026-06-07 (user batch, committed b6f700c / index-CIgFIHZo): (1) modern thin theme-tinted scrollbars app-wide (index.css ::-webkit-scrollbar + scrollbar-width); (2) GLOBAL Recharts tooltip dark-theme fix in index.css -- the Hydration 'wrong colors' was a SHARED bug across all 21 admin charts (they set contentStyle but never labelStyle/itemStyle -&gt; dark-on-dark text); one CSS block (.recharts-default-tooltip bg/border + .recharts-tooltip-label muted + item foreground) fixes every chart + future ones; (3) hover floating-info on every dashboard point (&lt;Tooltip&gt; added to Bodyweight/Heart/Sleep/Hydration; per-dot hover tooltip on the Calories mini-graph); (4) stat relabels: Calories -&gt; Daily target/BMR/TDEE/Energy balance (calcFullPlan); Heart -&gt; Avg resting/Latest peak/Steps today (added daily peak max); Sleep -&gt; Bedtime target (wake-anchored clock) replacing the hours target. WAVE 2 PENDING (graph ports): port the MOBILE heart graph (HrRangeChart -- per-day resting+avg dots + peak-zone gradient band) and the MOBILE sleep graph to web for BOTH the dash block AND the detail page (AdminUserHeart/AdminUserSleep) -- heavy custom-SVG rebuilds; sleep needs which-chart confirmation (mobile sleep page has SleepClock / Hypnogram / SleepConsistency / deep-REM sparklines). WAVE 2 DONE 2026-06-07 (user: heart=replicate the zone-band design; sleep='do them both'=clock+consistency): HEART (committed 17607f9 / index-BTxxHLjw) -- new web/src/components/HrZoneChart.jsx, SVG port of mobile HrRangeChart (per-day resting+avg dots + peak-zone vertical gradient band z1 yellow-&gt;z5 red, from 50% HRmax up to the day's peak; grid + y-axis + zone legend in full mode; hover readout). Rendered compact on the Heart dash block (hrMax from profile age) and full on AdminUserHeart detail (replaced the 3-line Recharts chart; removed the dead Recharts chart + orphaned LegendDot). SLEEP (committed d344dfa / index-UrgOa7xl) -- new SleepConsistencyChart.jsx (7 nightly bedtime-&gt;wake window bars on a mins-after-6pm axis + bed/wake target lines + avg-bedtime dotted line; on-target nights bright lime #CAF240, off faint; hover shows the window) + SleepClock.jsx (12h radial clock, last 7 nights as concentric lime sleep arcs outer=most-recent + indigo avg band; hover a ring -&gt; center day/date + below-clock time/duration). Sleep dash block now renders the consistency chart (compact); AdminUserSleep detail shows BOTH clock + consistency (replaced the duration line; removed dead DurationChart + fmtDateShort + recharts import). NET: all 5 dashboard domain blocks mirror their mobile charts, and the Heart + Sleep DETAIL pages were upgraded to the mobile charts too. T079 dashboard rollup is COMPLETE; the only remaining T079 work is the single coach-reflection batch (CoachClientDetail). HEART DATA-CONSISTENCY FIX 2026-06-07 (user: 'heart graph looks different on every source', committed 47deb0d / index-C9IxsxJh): root cause = the dash Heart block fetched ONLY hr_samples, so workout-day peaks (wearable_workouts.max_bpm) were missing -&gt; short/wrong bands vs the detail page (which folds them in). Extracted web/src/lib/heartDaily.js summariseHeartDays (replicates AdminUserHeart's exact resting=ambient-min-fallback-all / avg=mean-all / peak=max(daySampleMax, workout max_bpm) formula); the dash block now fetches wearable_workouts too and uses the shared helper. Dash == detail == mobile data now. Remaining difference is intentional: the dash is the COMPACT snapshot (no y-axis/grid/zone-legend), the detail + mobile are full. BAND-COLOR FIX 2026-06-07 (user: 'band colors show differently between mobile and web -- which is right?', committed 196bbf9 / index-B4gYZh3r): mobile is the source of truth. The diff = mobile colors each peak band PROPORTIONAL to time-in-zone (buildTimeInZoneStops, from a workout's per-second raw_meta.hr_log or a min/avg/max approximation; even HRmax-&gt;40% fallback incl a below-Z1 grey); the web was always drawing an even 5-color gradient by bpm range, AND the web DETAIL never computed timeInZone at all (its wearable_workouts fetch even omitted raw_meta). Ported mobile exactly: summariseHeartDays now computes timeInZone (addToZone / bucketHrLog / approximateZonesFromAggregates) + pads to 7 calendar days; HrZoneChart renders a per-band time-in-zone gradient (userSpaceOnUse) with the even fallback; AdminUserHeart's workouts fetch gained raw_meta and its chartData switched to summariseHeartDays. dashboard == detail == mobile now. ENERGY-BALANCE COLOR/ICON 2026-06-07 (user: 'energy balance should use the same color coding we have in mobile + icon next to it', committed d19c2de / index-CPp6BOMb): mobile rule = deficit (energyAdj&lt;0) emerald + TrendingDown, surplus blue + TrendingUp (trendHue/TrendIcon in calories.tsx). The dash Calories block's Energy balance stat was amber-for-surplus with no icon -&gt; now emerald/blue + down/up trend arrow. StatStrip (DashboardSnapshotShell) gained optional `icon` support. The detail Overview (CalorieDashboard) already used this coding, so mobile / detail / dash now all agree. CALORIES CHART SHARED 2026-06-07 (user: 'the cals block has color bars that dont show on the dash', committed 3e5193c / index-Cq9cPgrG): the dash Calories mini-graph was a SEPARATE reimplementation that omitted the per-day status-colored vertical bands the detail strip draws -&gt; different look. Extracted the detail's CalorieGraph into shared web/src/components/CalorieTrendGraph.jsx (status bands + dashed target line + connecting line + status dots + hover readout); BOTH CalorieStrip (detail) and the dash Calories block render it now, so they're identical (and the detail gained hover too). Removed the dash's duplicate CaloriesMiniGraph + the inline CalorieGraph/STATUS_GRAPH/statusFor from CalorieStrip (statusFor now imported from the shared file). Same single-source pattern as the heart summariseHeartDays fix. COACH-MIRROR BITES — verified 2026-06-07 (user: 'is this going to bite us when we do coach side mirroring?'; checked code + DB before the reflection batch). The reflection MUST handle: (1) PORTAL PATHS are hardcoded /admin/user/ — AdminUserActivity (Efforts tab) navigate() ~line 1017 + AdminEffortDetail.goBack + AdminCardioDetail.onBack all build /admin/user/{id}/...; CoachClientDetail ALREADY reuses AdminUserActivity with NO basePath, so a coach clicking an effort today lands on an /admin/ URL (latent bug). Thread a basePath prop ('/coach/client') through AdminUserActivity + the effort/cardio detail components (the dashboard snapshot blocks already accept basePath). (2) ADMIN-ONLY HEADER CONTROLS need role-gating for coach: Active/Suspend toggle + Delete (settings danger zone) are admin-only (coaches can't ban/delete accounts); AthleteCoachingChip (management reassignment) is admin-only. ClientSettingsDrawer already takes viewerRole='coach' (read-only) — good. (3) log_admin_activity is now coach-ready (migration log_admin_activity_coach_ready_guard: guard = is_admin() OR caller is the target's coach; fixed a 0-arg is_active_coach() bug that would have errored for coaches). BUT event_data.admin_initiated + the '(admin)' timeline label are hardcoded admin — coach actions would mislabel; when wiring coach actions pass a coach flag + extend getActivityMeta. (4) get_activity_feed + activity_events RLS already authorize coach-of-client reads, so coach feed READS are fine. None are dead-ends — all enumerable gating/path fixes for the batch.</t>
+          <t>Phase 1 (build pages): add read-only mirror tabs AdminUserSleep / AdminUserHydration / AdminUserHeart (styled like existing admin tabs: Recharts, design tokens), wired into AdminUserDetail. Built via parallel agents 2026-06-04. Phase 2 (per-page, one at a time): align every tab first-view to the athlete exactly + add coaching elements. BODYWEIGHT DONE (2026-06-06): coach Bodyweight tab now mirrors the athlete — 4 insight cards (Current Weight / BMI color-coded / Ideal Weight Range / Weight Trend, ported from the pre-coach-only web Bodyweight.jsx that was deleted in b7af3c9, computed in the CLIENT units via the profile prop) + emerald Progress chart + weigh-in list. COACH-INPUT REVERSAL + UNIFIED ADD BUTTON (2026-06-06): user reversed the earlier no-coach-inputs stance for tracking tabs (coaches DO add, e.g. in-person weigh-ins). New shared web/src/components/CoachAddButton.jsx + LOCKED placement convention: each coach tab first element is a flex justify-between action row with left content (toggle/count) + CoachAddButton pinned RIGHT = ONE consistent location across all coach-add tabs and future ones. Restored the structured Add-effort form on Efforts (AddEffortForm, removed in a022b7f) via the unified button. AdminUserDetail passes profile to AdminUserBody. Deployed + browser-verified; committed c059460. Remaining T079 Phase-2 tabs: Calories, Heart, Sleep, Hydration. SEARCH ALIASES + ADD-FORM POLISH (2026-06-06): (1) MovementSearch on BOTH surfaces (web src/components/MovementSearch.jsx + mobile src/components/MovementSearch.tsx) now treats kb/db/bb as aliases for kettlebell/dumbbell/barbell — typing the abbreviation matches AND leads with those moves (the abbreviations are not substrings of the full words, so an alias term-list is required). (2) Web coach add-effort form (AddEffortForm) made cascading: Type -&gt; movement -&gt; only the fields relevant to that move; each field autofocuses as it appears (MovementSearch gained an autoFocus prop, web-only); date field removed (coach entries log at now); Save appears once a movement is picked. Bodyweight add form autofocuses the Weight input. Deployed + browser-verified (kb -&gt; 17 kettlebell moves leading; reps field autofocused after move select; no date field); committed 3e133bc. HEART FINDING: there is NO athlete mobile heart page (no mobile heart.tsx exists), so Heart has no athlete surface to mirror. The coach AdminUserHeart (built in T079 Phase 1) is already a COMPLETE read-only wearable-HR view: today snapshot (Latest/Resting/Avg/Steps), resting-HR band assessment + spectrum gauge (age/gender norms), 7-day HR chart (resting/avg/peak), daily history. Heart is wearable-sourced (no manual entry) so no coach add button. Heart parity is effectively already done; awaiting user direction on any desired changes. SLEEP + HYDRATION CONFIRMED DONE 2026-06-06 (verified parity: AdminUserSleep mirrors the athlete's 4 dimensions + duration chart + age-based target; AdminUserHydration mirrors the chart + cups readout + bodyweight target, now in the coach's fluid_unit via T093). So Heart + Sleep + Hydration + Bodyweight + Efforts are all done; CALORIES is the only Phase-2 tab left. CALORIES REWORK AGREED 2026-06-06 (user picked, one decision at a time): (1) FULL athlete-dashboard mirror, read-only -- day strip + daily-target hero (BMR/TDEE/energy + target kcal + macro targets) + today's-intake macro card + weight-goal progress, like Bodyweight; (2) KEEP the Macro Plan editor (coach's planning tool); (3) KEEP the Food Log review; (4) DROP the legacy 'Manual Logs' (calorie_logs) sub-tab. Plan: reuse the web end-user Calories.jsx dashboard pieces (CalorieStrip / TodayIntakeCard / calcFullPlan) rendered read-only for the client. Building now in web/src/pages/admin/tabs/AdminUserCalories.jsx. CALORIES DONE 2026-06-06 (6886a7f, deployed): AdminUserCalories reworked to a read-only athlete mirror -- Overview landing = inlined CalorieDayStrip (web CalorieStrip was deleted in 14cbe55, so re-inlined) + DailyTargetHero (calcFullPlan) + SelectedDayIntakeCard (food_logs vs target + macro bars) + WeightGoalCard (in the coach's weight unit); Macro Plan editor + Food Log review kept as sub-tabs; legacy Manual Logs (calorie_logs) removed. ALL data-page mirrors now done: Strength/Cardio (T080), Bodyweight, Sleep, Hydration, Heart, Calories. ONLY REMAINING in T079 = the holistic DASHBOARD rollup tab (the original 'built last' placeholder that rolls the other tabs into one overview). T079 stays In progress until that's built. CALORIES CHART FOLLOW-UP 2026-06-06 (user: 'i dont see the graph in calories'): the rework shipped with no chart (the old chart lived in the dropped Manual Logs tab; the athlete page itself has no line chart). Added CaloriesTrendChart to the Overview -- 14-day daily-calorie bars vs a dashed target reference line, days-over-target in amber (matches the Hydration bar-chart style). Committed 5a1a35b, deployed live. Now every coach tab has a graph. REVERTED 2026-06-06 (user: 'the page looks wrong now, revert it'): the dashboard rework + the bar chart looked wrong on-page AND misread the ask. Reverted AdminUserCalories to the pre-rework original (3 sub-tabs: Food Log / Manual Logs / Macro Plan), committed 80f9c7e, live (bundle back to index-CYWRDrme). CLARIFICATION: the 'graph' the user wants is the athlete CalorieStrip's MINI TREND CHART -- the line + dots + dashed-target chart UNDER the 14-day tile row (mobile src/components/CalorieStrip.tsx, the CalorieGraph subcomponent, Skia-rendered). NOT a separate bar chart, NOT the old Manual-Logs CaloriesChart. REDO PENDING user direction: (a) add just the CalorieStrip (tiles + line-chart-under-days, web build since web CalorieStrip was deleted) to the coach Calories, or (b) redo the full dashboard mirror correctly with that strip included. T079 Calories is back to in-progress. REDO DIRECTION CONFIRMED 2026-06-06 (user picked 'Full dashboard mirror, redone'): rebuild the coach Calories tab to mirror the athlete dashboard faithfully + include the CalorieStrip line-chart-under-days. APPROACH (this time): resurrected the DELETED web files from git (CalorieStrip.jsx from 14cbe55^, athlete Calories.jsx from b7af3c9^) -- they were web-native Recharts/SVG mirrors, far closer than re-porting the RN code. Building: (1) web/src/components/CalorieStrip.jsx -- adapted to take the CLIENT userId (was useAuth self), display-only when no onDayClick; tiles + SVG CalorieGraph (polyline + status bands + dashed target + dots) = the line-chart-under-days. (2) web/src/components/CalorieDashboard.jsx -- READ-ONLY athlete-dashboard mirror in COACH units (useAuth coach weight/height unit, fromKg display-convert, calcFullPlan math stays on the client profile): strip + daily-target hero (BMR/TDEE/energy pills + ActivePillPanel) + daily macros + per-meal (read-only) + today's intake (read-only, no Log-food btn) + timeline + weight goal. Drops self-coached-only bits (wizard, food drawer, goal-reached banner, meal-picker editing). (3) AdminUserCalories.jsx -- new 'Overview' sub-tab (default) renders CalorieDashboard; KEEPS Food Log / Manual Logs / Macro Plan (keeping Manual Logs this round since the revert restored it; non-destructive, easy to drop later if the user reconfirms). REDO DONE 2026-06-06 (build clean, deployed, live hash index-DkKPxM-G verified): coach Calories now opens on an Overview sub-tab = the athlete dashboard mirror incl. the CalorieStrip line-chart-under-days (the thing the user pointed at), read-only, in coach units. The earlier mistakes fixed: faithful card-for-card mirror of the athlete page (resurrected web source, not a fresh agent rebuild) so it can't 'look wrong', and the trend chart is the strip's polyline-under-days (not a separate bar chart). Coach-facing tweaks vs the athlete page: read-only (no Log-food btn / wizard / food drawer / goal banner / meal-picker editing), prose flipped from 'you/your' to 'they/their/this client', goal card uses a neutral factual status line instead of the random motivational message. WEB-ONLY (admin portal is web-exclusive; athlete mobile calories.tsx is the unchanged source -- no cross-platform mirror needed). Awaiting user QA. T079 remaining = only the holistic Dashboard rollup tab. MIRRORING STRATEGY CLARIFIED 2026-06-06 (user: 'when we completely finish admin view we reflect to coach'): ALL T079 work targets the ADMIN view (web/src/pages/admin/tabs/AdminUser*.jsx) FIRST; the COACH view (web/src/pages/coach/CoachClientDetail.jsx) gets the reflection as ONE batch ONCE the admin view is completely finished -- NOT per-tab. So the coach reflection of Bodyweight/Sleep/Hydration/Heart/Calories is a single PENDING milestone (my earlier 'no cross-platform mirror needed' on Calories was wrong -- it's DEFERRED). CoachClientDetail today already reuses AdminUserActivity + AdminUserBody directly (4-tab layout: Dashboard/Efforts/Bodyweight/Calories) but its Calories tab is coach-specific (MacroPlanEditor only) -- the reflection will point it at CalorieDashboard. COACH-TEXT RULE (CLAUDE.md rule 6 / line 88): athlete='you', coach='the client', admin='the user/the athlete/this account'; + line 93 lowercase coach/admin/client in body copy. CalorieDashboard already complies (flipped all athlete 'you/your' -&gt; 'this client/their', neutral goal line), matching the AdminUserHeart 'This client hasn't synced...' precedent. NOTE: the worktree CLAUDE.md is STALE vs the main-repo CLAUDE.md (worktree still says 'web end-user deprecated/mobile leads'; main says 'web = coach portal + admin portal ONLY, athletes have zero web surfaces' + documents the /coach/* portal). Always read the MAIN-repo CLAUDE.md, not the worktree copy. T086 COMPLIANCE FIX 2026-06-06 (user audit: 'a lot of text irrelevant to the coach, good for the athlete -- look for the rule'): found the rule = T086 (ledger) anchored by CLAUDE.md line 2305 'Coach is a NEXT-STEP OVERSEER'. The just-built CalorieDashboard had VIOLATED it -- carried 2 always-visible athlete-education blocks: (a) the default daily-target explanation panel, (b) the timeline science paragraphs. STRIPPED both: hero BMR/TDEE/energy now explain ONLY on tap (opt-in/collapsed, no default panel); timeline keeps the ETA number + the 'to lose/gain X, reach Y' data line, dropped the recomp-science + best-case/realistic paragraphs. Built+deployed (index-CIjWukiv) committed 3740069. ALSO promoted T086 from this ledger into CLAUDE.md as a permanent locked rule (new subsection after the Admin&lt;-&gt;Coach mirror rule) -- it was ledger-only, which is exactly why it was missed at build time. THEN audited AdminUserBody (built 2026-06-06, AFTER the 06-04 T086 sweep): essentially compliant (no motivational/attribution/explainer prose); only 3 athlete-instruction empty-states neutralized to factual ('Log a weigh-in first'-&gt;'No weigh-in logged yet', 'Add height in profile'-&gt;'No height on file', 'Log more weigh-ins to see the trend'-&gt;'Not enough weigh-ins for a trend yet'); BMI/ideal-weight reference annotations kept (factual data labels). FOLLOW-UP FLAG: AdminUserActivity (Efforts, reworked 2026-06-06) should also get a quick T086 pass. GRAPH+TILE FIX 2026-06-06 (user screenshot: dots rendered as stretched ellipse blobs + graph didn't line up with the day tiles): root cause = the web CalorieStrip CalorieGraph used a fixed 320-wide viewBox with preserveAspectRatio='none', so on the wide desktop coach card the X-axis stretched ~4x and squashed the r=4 circles into wide ovals; separately the tiles were packed at a fixed w-[58px] (left-aligned) while the graph spanned full width, so dots didn't sit under tiles. FIX: CalorieGraph now MEASURES its real pixel width (useRef + ResizeObserver) and renders the SVG at width=W height=72 with NO preserveAspectRatio (1:1 -&gt; round dots); both the tile row and the graph are laid out as N=14 equal columns separated by GAP=6px (tiles flex-1 min-w-0, no more w-[58px]/overflow-x-auto/snap; graph colCenter(i)=i*(colW+GAP)+colW/2 with colW=(W-78)/14) so each dot sits exactly under its tile. Built+deployed index-8GgKpHVX. MANUAL LOGS REMOVED + NO COACH ADD-FOOD 2026-06-06 (user: 'remove manual logs and no need for a add food in coach side'): deleted the legacy 'Manual Logs' (calorie_logs) sub-tab entirely from AdminUserCalories -- its CaloriesChart, the calorie_logs load/add/delete handlers, the 'Add entry' form, and all the now-dead state + the lucide/recharts imports. Coach Calories sub-tabs are now Overview / Food Log / Macro Plan. No food-adding anywhere on the coach side: Overview's TodayIntakeCard is already read-only (no Log-food button), Food Log is review-only. KEPT: Food Log swipe-to-delete (a correction tool, not an add) -- flagged to the user in case they want pure review. Built+deployed index-C1zY-3c_. DEAD-CODE CLEANUP 2026-06-06 (user: 'dont leave behind any dead code, clean up'): ran eslint on every touched file. CalorieStrip.jsx rewritten PURELY read-only -- removed the never-exercised interactive path (the only caller, the coach CalorieDashboard, is read-only): dropped the onDayClick/selectedIso/refreshKey props, the button-vs-div tile branch, the clickable-dot &lt;g&gt;, the 'Tap a day to log food' subtitle, the now-no-op auto-scroll useEffect + stripRef/todayRef, and the useAuth fallback (uid = userId ?? user?.id) which would have shown the COACH's own food if userId were ever missing -- now requires userId. AdminUserDetail.jsx: removed the orphaned onSaved={() =&gt; setSnapshotKey(...)} prop on &lt;AdminUserCalories&gt; (the component no longer accepts onSaved after Manual Logs was removed; setSnapshotKey is still used by the Efforts + Body tabs so it stays). eslint clean for unused-vars across CalorieStrip/CalorieDashboard/AdminUserCalories. PRE-EXISTING (left alone, not from this work): AdminUserDetail parsePace (line 82, deliberately retained legacy helper w/ a 'will retire when hasPR removed' comment) + deleteConfirm (useState value w/ used setter). Built+deployed index-CXEyiFzG. DASHBOARD ROLLUP STARTED 2026-06-07 (the final T079 piece -- the holistic Dashboard tab that rolls the other pages into one overview). User spec for the layout: blocks ordered SAME as the page/nav sequence; Efforts (strength+cardio) live in ONE block (no single graph exists for dozens of movements); the other domain blocks each show their main graph + a few snapshot lines. EFFORTS BLOCK BUILT + confirmed-pending (user: 'scroll to last 10, sorted earliest-&gt;latest, every line clickable to its details page; do it and once confirmed we move on to the rest'): new web/src/components/DashboardEffortsBlock.jsx = last 10 DISTINCT moves (most-recent occurrence of each, deduped by type|baseName), reversed to earliest-&gt;latest, fixed-height scroll (max-h 240), each row clickable -&gt; /admin/user/{id}/effort/{type}/{navName} (navName strips trailing [Variant] so consolidated families route to base) + a 'View all -&gt;' to the Efforts tab. Wired into AdminUserDetail dashboard tab; the remaining domain blocks (Bodyweight/Heart/Calories/Sleep/Hydration, in nav order) are tier-gated 'coming soon' placeholders for now = 'the rest' to build after Efforts is confirmed. Committed 1390cf4, deployed index-BKgOlVxQ (live-verified). Coach reflection (CoachClientDetail) still the single deferred batch milestone. EFFORTS BLOCK TWEAKED 2026-06-07 (user QA, committed 2e56170 / index-Bftuetsl): show 5 at a time (max-h 208; was 240 -&gt; 168@4 -&gt; 208@5 per QA, committed 1c7b18a); each row now shows date AND days-ago together ('Apr 30 - 38 days ago'); sort flipped to MOST-RECENT first (so the 4 visible without scrolling are the latest moves); title 'Recent training' -&gt; 'Recent efforts'. DASHBOARD SNAPSHOT BLOCKS BUILT 2026-06-07 (committed 14ea208 / index-PSfaf9sZ): the 5 remaining domain blocks shipped on the admin client Dashboard tab, in nav order, tier-gated (CoreRX: Bodyweight+Calories; FullRX: +Heart/Sleep/Hydration). New shared web/src/components/DashboardSnapshotShell.jsx (SnapshotCard/Loading/Empty/StatStrip) + 5 components: DashboardBodyweightBlock (emerald weight line + current/30-day/BMI in coach units), DashboardHeartBlock (per-day resting+avg HR line + latest/resting/steps; wearable 'no sync' empty), DashboardCaloriesBlock (the 14-day intake line+dots+dashed-target mini-trend WITHOUT the day tiles + today/14-day-avg/on-target; consumes the already-fetched existingPlan so target matches the Calories tab), DashboardSleepBlock (duration line + age-target ref + last-night/7-night-avg/target), DashboardHydrationBlock (7-day intake bars + bw-target ref + today-cups/%/7-day-avg; BHI milk x1.5, 35 mL/kg, coach fluid unit). Each block self-fetches, renders a compact main graph faithful to its tab's chart (extracted via 5 parallel read-only agents) + a quick-stat strip + 'View all -&gt;' deep-link to the full tab. ADMIN client-detail view is now COMPLETE end-to-end (all tabs + the holistic Dashboard rollup). The ONLY remaining T079 work is the single COACH-REFLECTION batch (CoachClientDetail.jsx): reflect all admin tabs + the 6 dashboard blocks + the T101 reopen-on-Dashboard and back-to-Efforts fixes in one pass. UNIFORM SIZING 2026-06-07 (user 'all blocks should be the same size as strength', committed cc18bff): all 6 blocks share a fixed h-260 flex-col card -- chart area fills (flex-1, height 100%), stat strip pinned to the bottom, loading/empty centered, Efforts list flex-1 (was max-h-208). Identical footprint across the grid. DASHBOARD POLISH 2026-06-07 (user batch, committed b6f700c / index-CIgFIHZo): (1) modern thin theme-tinted scrollbars app-wide (index.css ::-webkit-scrollbar + scrollbar-width); (2) GLOBAL Recharts tooltip dark-theme fix in index.css -- the Hydration 'wrong colors' was a SHARED bug across all 21 admin charts (they set contentStyle but never labelStyle/itemStyle -&gt; dark-on-dark text); one CSS block (.recharts-default-tooltip bg/border + .recharts-tooltip-label muted + item foreground) fixes every chart + future ones; (3) hover floating-info on every dashboard point (&lt;Tooltip&gt; added to Bodyweight/Heart/Sleep/Hydration; per-dot hover tooltip on the Calories mini-graph); (4) stat relabels: Calories -&gt; Daily target/BMR/TDEE/Energy balance (calcFullPlan); Heart -&gt; Avg resting/Latest peak/Steps today (added daily peak max); Sleep -&gt; Bedtime target (wake-anchored clock) replacing the hours target. WAVE 2 PENDING (graph ports): port the MOBILE heart graph (HrRangeChart -- per-day resting+avg dots + peak-zone gradient band) and the MOBILE sleep graph to web for BOTH the dash block AND the detail page (AdminUserHeart/AdminUserSleep) -- heavy custom-SVG rebuilds; sleep needs which-chart confirmation (mobile sleep page has SleepClock / Hypnogram / SleepConsistency / deep-REM sparklines). WAVE 2 DONE 2026-06-07 (user: heart=replicate the zone-band design; sleep='do them both'=clock+consistency): HEART (committed 17607f9 / index-BTxxHLjw) -- new web/src/components/HrZoneChart.jsx, SVG port of mobile HrRangeChart (per-day resting+avg dots + peak-zone vertical gradient band z1 yellow-&gt;z5 red, from 50% HRmax up to the day's peak; grid + y-axis + zone legend in full mode; hover readout). Rendered compact on the Heart dash block (hrMax from profile age) and full on AdminUserHeart detail (replaced the 3-line Recharts chart; removed the dead Recharts chart + orphaned LegendDot). SLEEP (committed d344dfa / index-UrgOa7xl) -- new SleepConsistencyChart.jsx (7 nightly bedtime-&gt;wake window bars on a mins-after-6pm axis + bed/wake target lines + avg-bedtime dotted line; on-target nights bright lime #CAF240, off faint; hover shows the window) + SleepClock.jsx (12h radial clock, last 7 nights as concentric lime sleep arcs outer=most-recent + indigo avg band; hover a ring -&gt; center day/date + below-clock time/duration). Sleep dash block now renders the consistency chart (compact); AdminUserSleep detail shows BOTH clock + consistency (replaced the duration line; removed dead DurationChart + fmtDateShort + recharts import). NET: all 5 dashboard domain blocks mirror their mobile charts, and the Heart + Sleep DETAIL pages were upgraded to the mobile charts too. T079 dashboard rollup is COMPLETE; the only remaining T079 work is the single coach-reflection batch (CoachClientDetail). HEART DATA-CONSISTENCY FIX 2026-06-07 (user: 'heart graph looks different on every source', committed 47deb0d / index-C9IxsxJh): root cause = the dash Heart block fetched ONLY hr_samples, so workout-day peaks (wearable_workouts.max_bpm) were missing -&gt; short/wrong bands vs the detail page (which folds them in). Extracted web/src/lib/heartDaily.js summariseHeartDays (replicates AdminUserHeart's exact resting=ambient-min-fallback-all / avg=mean-all / peak=max(daySampleMax, workout max_bpm) formula); the dash block now fetches wearable_workouts too and uses the shared helper. Dash == detail == mobile data now. Remaining difference is intentional: the dash is the COMPACT snapshot (no y-axis/grid/zone-legend), the detail + mobile are full. BAND-COLOR FIX 2026-06-07 (user: 'band colors show differently between mobile and web -- which is right?', committed 196bbf9 / index-B4gYZh3r): mobile is the source of truth. The diff = mobile colors each peak band PROPORTIONAL to time-in-zone (buildTimeInZoneStops, from a workout's per-second raw_meta.hr_log or a min/avg/max approximation; even HRmax-&gt;40% fallback incl a below-Z1 grey); the web was always drawing an even 5-color gradient by bpm range, AND the web DETAIL never computed timeInZone at all (its wearable_workouts fetch even omitted raw_meta). Ported mobile exactly: summariseHeartDays now computes timeInZone (addToZone / bucketHrLog / approximateZonesFromAggregates) + pads to 7 calendar days; HrZoneChart renders a per-band time-in-zone gradient (userSpaceOnUse) with the even fallback; AdminUserHeart's workouts fetch gained raw_meta and its chartData switched to summariseHeartDays. dashboard == detail == mobile now. ENERGY-BALANCE COLOR/ICON 2026-06-07 (user: 'energy balance should use the same color coding we have in mobile + icon next to it', committed d19c2de / index-CPp6BOMb): mobile rule = deficit (energyAdj&lt;0) emerald + TrendingDown, surplus blue + TrendingUp (trendHue/TrendIcon in calories.tsx). The dash Calories block's Energy balance stat was amber-for-surplus with no icon -&gt; now emerald/blue + down/up trend arrow. StatStrip (DashboardSnapshotShell) gained optional `icon` support. The detail Overview (CalorieDashboard) already used this coding, so mobile / detail / dash now all agree. CALORIES CHART SHARED 2026-06-07 (user: 'the cals block has color bars that dont show on the dash', committed 3e5193c / index-Cq9cPgrG): the dash Calories mini-graph was a SEPARATE reimplementation that omitted the per-day status-colored vertical bands the detail strip draws -&gt; different look. Extracted the detail's CalorieGraph into shared web/src/components/CalorieTrendGraph.jsx (status bands + dashed target line + connecting line + status dots + hover readout); BOTH CalorieStrip (detail) and the dash Calories block render it now, so they're identical (and the detail gained hover too). Removed the dash's duplicate CaloriesMiniGraph + the inline CalorieGraph/STATUS_GRAPH/statusFor from CalorieStrip (statusFor now imported from the shared file). Same single-source pattern as the heart summariseHeartDays fix. COACH-MIRROR BITES — verified 2026-06-07 (user: 'is this going to bite us when we do coach side mirroring?'; checked code + DB before the reflection batch). The reflection MUST handle: (1) PORTAL PATHS are hardcoded /admin/user/ — AdminUserActivity (Efforts tab) navigate() ~line 1017 + AdminEffortDetail.goBack + AdminCardioDetail.onBack all build /admin/user/{id}/...; CoachClientDetail ALREADY reuses AdminUserActivity with NO basePath, so a coach clicking an effort today lands on an /admin/ URL (latent bug). Thread a basePath prop ('/coach/client') through AdminUserActivity + the effort/cardio detail components (the dashboard snapshot blocks already accept basePath). (2) ADMIN-ONLY HEADER CONTROLS need role-gating for coach: Active/Suspend toggle + Delete (settings danger zone) are admin-only (coaches can't ban/delete accounts); AthleteCoachingChip (management reassignment) is admin-only. ClientSettingsDrawer already takes viewerRole='coach' (read-only) — good. (3) log_admin_activity is now coach-ready (migration log_admin_activity_coach_ready_guard: guard = is_admin() OR caller is the target's coach; fixed a 0-arg is_active_coach() bug that would have errored for coaches). BUT event_data.admin_initiated + the '(admin)' timeline label are hardcoded admin — coach actions would mislabel; when wiring coach actions pass a coach flag + extend getActivityMeta. (4) get_activity_feed + activity_events RLS already authorize coach-of-client reads, so coach feed READS are fine. None are dead-ends — all enumerable gating/path fixes for the batch. CLOSED 2026-06-09 (sanity check): admin client view = all 7 data tabs (Efforts/Bodyweight/Heart/Calories/Sleep/Hydration) + the holistic Dashboard rollup; CoachClientDetail mirrors the SAME 7 data tabs + the SAME 6 dashboard blocks with basePath='/coach/client', differing only by the intentional admin-only Billing + Activity-Feed tabs. Coach-mirror bites handled (basePath threaded; coach uses its own Message/Remove/CoachManageChip controls; no coach Activity-Feed so the labeling/RLS bites are N/A). Nothing outstanding.</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
@@ -8188,7 +8180,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E149" s="12" t="inlineStr">
+      <c r="E149" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -8500,9 +8492,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E155" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E155" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F155" s="5" t="inlineStr">
@@ -8517,7 +8509,7 @@
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>Decide per item whether to mirror admin-&gt;coach. Likely: add realtime sync to CoachClientDetail; pass profile into AdminUserBody from coach; unify resolveTier into one shared helper (kill the allow-list/block-list split); add the missing-data warning to the coach calories tab. Confirm scope with user before implementing (parity rule = everything on coach must be on admin and vice versa, minus the intentional Billing/Activity-Feed omissions).</t>
+          <t>Decide per item whether to mirror admin-&gt;coach. Likely: add realtime sync to CoachClientDetail; pass profile into AdminUserBody from coach; unify resolveTier into one shared helper (kill the allow-list/block-list split); add the missing-data warning to the coach calories tab. Confirm scope with user before implementing (parity rule = everything on coach must be on admin and vice versa, minus the intentional Billing/Activity-Feed omissions). DONE 2026-06-09: (a) added live profiles realtime sync to CoachClientDetail (mirrors AdminUserDetail) so the coach view no longer goes stale after an edit; (b) passed profile={client} into AdminUserBody on coach -&gt; the Bodyweight headline weight now prefers profile.current_weight like admin; (d) added the 'Profile incomplete -- plan calc needs gender/birthdate/weight/height' amber banner to CoachClientDetail (mirrors admin). (c) VERIFIED it is NOT an admin&lt;-&gt;coach OUTPUT divergence -- both files' resolveTier are byte-identical (block-list) and coachActive resolves equivalently (coach = local allow-list; admin = client_has_active_coach RPC = same allow-list). The genuine nuance (resolveTier's is_coach block-list vs the coachActive allow-list disagree on paused/null/unpaid, AND resolveTier mirrors mobile byte-for-byte) is split into T164 -- out of pure-parity scope. Web built+deployed index-BKklK3FL.js (live-verified).</t>
         </is>
       </c>
       <c r="I155" s="7" t="inlineStr">
@@ -9020,9 +9012,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E165" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E165" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
@@ -9037,7 +9029,7 @@
       </c>
       <c r="H165" s="7" t="inlineStr">
         <is>
-          <t>Extract the 3 helpers into a small shared module (e.g. web/src/lib/effortPR.js) and import from all three sites. Low priority -- they're tiny + stable.</t>
+          <t>Extract the 3 helpers into a small shared module (e.g. web/src/lib/effortPR.js) and import from all three sites. Low priority -- they're tiny + stable. DONE 2026-06-09: created web/src/lib/effortPR.js (exports parse1RM, parseCardioBest, exerciseKey) + imported it in CoachClientDetail, AdminUserDetail, and CoachDashboard; removed all 3 local copies (verified byte-identical first). Admin's separate parsePace + hasPR left in place. Pure refactor, no behavior change; build clean, deployed index-qKKAJSe3.js (live-verified).</t>
         </is>
       </c>
       <c r="I165" s="7" t="inlineStr">
@@ -9098,6 +9090,58 @@
         </is>
       </c>
       <c r="J166" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>T164</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t>Reconcile the 'active coach' definition -- resolveTier is_coach block-list vs coachActive allow-list (web + mobile)</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>Billing/Tier</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>Web+Mobile</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G167" s="7" t="inlineStr">
+        <is>
+          <t>Surfaced 2026-06-09 during T152: resolveTier's is_coach branch treats a coach as ACTIVE unless their status is in a BLOCK-list (lapsed/suspended/cancelled), but the client-tier path (coachActive / the client_has_active_coach RPC) treats a coach as active only if status is in an ALLOW-list (trialing/active/past_due). They DISAGREE on paused/null/unpaid: a paused coach keeps FullRX on their own self-view (block-list) while their clients lose it (allow-list). resolveTier also claims to mirror mobile/app/(app)/dashboard.tsx byte-for-byte, so any change has to be checked against mobile + the billing model.</t>
+        </is>
+      </c>
+      <c r="H167" s="7" t="inlineStr">
+        <is>
+          <t>Decide the canonical 'active coach' rule (likely the allow-list -- it matches the RPC + the client's own app per T143) and apply it consistently to resolveTier's is_coach branch across BOTH web files AND mobile dashboard.tsx. Verify against the full coach_subscription_status set before changing (tier/billing-sensitive). Low urgency -- only edge-case statuses (paused/null/unpaid) are affected.</t>
+        </is>
+      </c>
+      <c r="I167" s="7" t="inlineStr">
+        <is>
+          <t>web/src/pages/admin/AdminUserDetail.jsx; web/src/pages/coach/CoachClientDetail.jsx; mobile/app/(app)/dashboard.tsx</t>
+        </is>
+      </c>
+      <c r="J167" s="5" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
@@ -9125,155 +9169,155 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>MyRX — Task Pipeline · how to use</t>
         </is>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1">
-      <c r="A2" s="14" t="inlineStr"/>
+      <c r="A2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>WHY THIS EXISTS</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>We fork across many sessions and lose track of what's open / where we stopped. This is the single remembered list. Every task has a stable numeric ID (T001, T002, ...). Refer to one with "pick up T021" and this sheet says exactly where we left off and what's next.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1">
-      <c r="A5" s="14" t="inlineStr"/>
+      <c r="A5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>CAPTURE-FIRST RULE (locked 2026-06-03)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Every time a point comes up that needs fixing or discussion — ANY size — it gets logged here as a Pending task with a new T### id BEFORE the assistant replies, then it's answered. It stays Pending until the work is actually done/decided, then flips to Done (or Deferred/Parked/Reverted). Small items are exactly what gets lost, so nothing is too small to capture.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="14" t="inlineStr"/>
+      <c r="A8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>STATUS VALUES</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Done — shipped (and usually deployed/committed).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>In progress — actively being iterated.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Pending — agreed/known but not started.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Deferred — intentionally postponed (waiting on something or a user decision).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Parked — discussed then set aside; needs a user decision to re-open.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Reverted — was tried, then undone.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Closed — dropped / won't do for now (can be reopened).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="14" t="inlineStr"/>
+      <c r="A17" s="13" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>HOW TO UPDATE (the .xlsx is GENERATED, do not hand-edit)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>1. Edit the TASKS list in scripts/build_task_pipeline_xlsx.py (add a row / flip a status / update the 'where we left off' + 'next' text).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>2. Re-run:  python scripts/build_task_pipeline_xlsx.py</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>3. Commit BOTH the script and docs/TASK_PIPELINE.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>New tasks get the next free T### id. Never reuse or renumber an id.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="8" customHeight="1">
-      <c r="A23" s="14" t="inlineStr"/>
+      <c r="A23" s="13" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>SCOPE NOTE</t>
         </is>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Seeded 2026-06-03 from the current CLAUDE.md + recent sessions. Older sessions weren't fully transcribed, so the 'prior' rows are best-effort reconstructions of completed features. Treat this as the authoritative living record from here forward — keep it current.</t>
         </is>

</xml_diff>

<commit_message>
chore(ledger): T227 done — disabled SendGrid click + open tracking (email links now clean https)
Drove the SendGrid dashboard: Settings -> Tracking -> Click Tracking OFF + Open Tracking OFF. All four tracking types now Disabled, matching the infrastructure.md contract. SendGrid no longer rewrites links, so auth/invite/reminder emails carry raw https://myrxfit.com links with no url####.myrxfit.com wrapper -> Chrome no longer blocks them.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -1280,9 +1280,9 @@
           <t>Infra</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>FINDING 2026-06-12 (infrastructure.md L106): the SENDGRID_API_KEY is Mail-Send-only (restricted scope) so it CANNOT PATCH /v3/tracking_settings/click -- the API path is dead. Fix = SendGrid DASHBOARD toggle: Settings -&gt; Tracking -&gt; Click Tracking -&gt; OFF (needs the SendGrid account login; not scriptable). infrastructure.md L107 CLAIMED tracking was disabled but it had drifted ON (doc updated with the incident note). STILL PENDING: flip the dashboard toggle + re-run a signup to confirm the email link is raw https://myrxfit.com/auth/confirm with NO url####.myrxfit.com wrapper. Open-tracking can stay; only click-tracking mangles links. User's CURRENT test can finish via the 6-digit code in the same email (no link needed).</t>
+          <t>DONE 2026-06-12: drove the SendGrid dashboard via Chrome (user logged in) -&gt; Settings -&gt; Tracking and turned Click Tracking OFF (the link-mangler) AND Open Tracking OFF (to match infrastructure.md's all-tracking-disabled contract -- both had drifted ON; Subscription + GA were already off). All four now show Disabled (confirmed by SendGrid 'Success' banners). SendGrid no longer rewrites links, so every outbound email (auth confirm/reset/magic-link + coach invites + trial reminders) now carries the raw https://myrxfit.com/... URL with NO url####.myrxfit.com wrapper -&gt; no more Chrome HTTPS-only block. The Mail-Send-only API key couldn't change this (dashboard-only). Applies to all mail sent from now on; user to eyeball the next signup email as final confirmation.</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(auth): account_marker A/AC/C + marker-aware routing (T234 phase 1-2)
Adds profiles.account_marker (A=athlete, AC=athlete->coach converting, C=coach) as the durable signup/role marker, and routes every signed-in web user by it via a shared roleHomePath() resolver (web/src/lib/roleRouting.js) used by RoleRouter, NotFound, and the post-sign-in redirect.

- DB: account_marker column + CHECK + backfill (11 athletes->A, 1 coach->C).

- New web coach signup -> C (init-profile-checkpoint). Existing athlete reaching coach signup -> AC (detectFlow). Coach welcome-end settles -> C.

- Routing: A -> /app (download), C|AC + active sub -> /portal, C|AC unfinished -> /signup (resume coach signup); /app now also served on the coach host so an athlete signed in there lands on download-app instead of a 404/loop.

Phases 3 (in-flow switch UX) + 4 (mobile finish/switch) + 5 (matrix test) pending.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -86,6 +86,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
@@ -102,11 +107,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1644,9 +1644,9 @@
           <t>Web+Mobile+DB</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1661,12 +1661,12 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>PLAN PRESENTED 2026-06-12, AWAITING APPROVAL -- do NOT implement until the user okays the open questions. Outline: (1) add profiles.coach_signup_step (coach progress, separate from athlete signup_checkpoint) + revert T231's signup_checkpoint pollution; (2) role-aware web routing (RootRoute/RoleRouter/Auth sign-in) keyed on is_coach + coach_signup_step + onboarded_at + host; (3) coach signup skips already-validated steps for an upgrading complete-athlete (prefilled, back-editable) -&gt; lands at pitch/plan; role-&gt;coach only on checkout; (4) mobile routing: onboarded -&gt; dashboard, coach-in-progress-without-athlete -&gt; 'finish on web'; (5) test the full matrix web+mobile. Full scenario table + plan is in the chat transcript.</t>
+          <t>APPROVED 2026-06-12 (user: 'go'). Marker = profiles.account_marker A|AC|C (NO separate coach_signup_step -- the marker itself gates which journey each platform interprets, so the shared signup_checkpoint never cross-contaminates). A=athlete(mobile); C=coach(web new email, set at init-profile-checkpoint); AC=existing athlete converting (stamped in coach Signup detectFlow when a marker-A user reaches coach signup); AC|C settle-&gt;C at coach welcome-end. Routing via web/src/lib/roleRouting.js roleHomePath(): A-&gt;/app(download); C|AC + active sub-&gt;/portal; C|AC no sub-&gt;/signup(resume coach signup); main-host admin-&gt;/admin/overview. PHASE 1 (DB account_marker + backfill: 11 A, 1 C) DONE+applied. PHASE 2 (roleHomePath resolver; RoleRouter/NotFound/Auth.jsx rewrite; /app added to coach host; init-profile-checkpoint=C [edge fn v9]; detectFlow AC-stamp; welcome-end=C) DONE+deployed live (index-BZTjgRz2.js). REMAINING: PHASE 3 = in-flow switch UX (email-step detects existing athlete -&gt; 'continue as coach?' confirm -&gt; in-flow password verify -&gt; A-&gt;AC, replacing the current bounce-to-/auth interstitial); PHASE 4 = mobile finish/switch screen for AC|C accounts opening the app (-&gt; finish on web OR switch to athlete, which resets marker-&gt;A + signup_checkpoint); PHASE 5 = full matrix test web+mobile.</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>DB migration (profiles.coach_signup_step) ; web App.jsx (RootRoute/RoleRouter) + Auth.jsx + coach/Signup.jsx ; mobile (auth)/_layout + sign-in + sign-up</t>
+          <t>web/src/lib/roleRouting.js (new) ; web/src/App.jsx (RoleRouter/NotFound/import/+app route) ; web/src/pages/Auth.jsx (post-sign-in) ; web/src/pages/coach/Signup.jsx (detectFlow select + AC stamp + welcome-end C) ; supabase/functions/init-profile-checkpoint (account_marker C) ; supabase/migrations/20260612_add_profiles_account_marker.sql</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -2268,7 +2268,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -2944,7 +2944,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E48" s="10" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -4348,7 +4348,7 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E75" s="10" t="inlineStr">
+      <c r="E75" s="11" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -4400,7 +4400,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E76" s="10" t="inlineStr">
+      <c r="E76" s="11" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -4452,7 +4452,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E77" s="10" t="inlineStr">
+      <c r="E77" s="11" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -4660,7 +4660,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E81" s="9" t="inlineStr">
+      <c r="E81" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -7208,7 +7208,7 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E130" s="9" t="inlineStr">
+      <c r="E130" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -7260,7 +7260,7 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E131" s="9" t="inlineStr">
+      <c r="E131" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -7364,7 +7364,7 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E133" s="9" t="inlineStr">
+      <c r="E133" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8300,7 +8300,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E151" s="9" t="inlineStr">
+      <c r="E151" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -9808,7 +9808,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E180" s="11" t="inlineStr">
+      <c r="E180" s="12" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -10744,7 +10744,7 @@
           <t>Web+Mobile</t>
         </is>
       </c>
-      <c r="E198" s="12" t="inlineStr">
+      <c r="E198" s="13" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -10796,7 +10796,7 @@
           <t>Web+Mobile+DB</t>
         </is>
       </c>
-      <c r="E199" s="13" t="inlineStr">
+      <c r="E199" s="9" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -11155,7 +11155,7 @@
           <t>Web+Edge+DB</t>
         </is>
       </c>
-      <c r="E206" s="13" t="inlineStr">
+      <c r="E206" s="9" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -11207,7 +11207,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E207" s="12" t="inlineStr">
+      <c r="E207" s="13" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -11883,7 +11883,7 @@
           <t>Backend+Supabase</t>
         </is>
       </c>
-      <c r="E220" s="11" t="inlineStr">
+      <c r="E220" s="12" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -11935,7 +11935,7 @@
           <t>Backend+Supabase</t>
         </is>
       </c>
-      <c r="E221" s="11" t="inlineStr">
+      <c r="E221" s="12" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -12143,7 +12143,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E225" s="9" t="inlineStr">
+      <c r="E225" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -12195,7 +12195,7 @@
           <t>Web+DB</t>
         </is>
       </c>
-      <c r="E226" s="9" t="inlineStr">
+      <c r="E226" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -12299,7 +12299,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E228" s="9" t="inlineStr">
+      <c r="E228" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>

</xml_diff>

<commit_message>
feat(brand): finish PageShell rollout — AcceptInvite + Legal on the shared frame (T248 done)
AcceptInvite's local PageShell helper now delegates to the shared one (aliased SharedShell), so its blue glow + bespoke footer are gone. LegalLayout adopts the shared frame too, keeping the required 'operated by Northern Princess LLC' + contact line as a closing paragraph in the doc body. All 8 public pages now share one background + footer + header frame.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -86,11 +86,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
@@ -107,6 +102,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -2216,9 +2216,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>IN PROGRESS 2026-06-12 (6/8 shipped). Shared chrome built (Wordmark pattern, for the whole frame): NEW web/src/components/AmbientBackground.jsx (grid + lime glow, blue dropped), PublicFooter.jsx (one footer: MyRX · Performance Lab + legal links + copyright), PageShell.jsx (relative min-h-dvh root + AmbientBackground + z-10 content layer so header/main sit above the ambient + PublicFooter). 6/8 public pages converted to &lt;PageShell&gt; + build-clean + deployed: Landing, Auth, AuthConfirm, DownloadAppPlaceholder, ForCoaches, CoachPricing. REMAINING 2: coach/AcceptInvite.jsx (Header/Footer helpers -&gt; PageShell) and legal/LegalLayout.jsx -- LegalLayout's footer carries the legally-required operator line ('MyRX is operated by Northern Princess LLC...' + privacy@myrxfit.com contact), so decide whether to fold that into PublicFooter (every page) or keep a Legal-specific footer BEFORE converting. EXCLUDED by design: the signup journey (own progress chrome) + admin/coach portals (sidebar shells). Header bar spec already unified px-6 md:px-10 (T247).</t>
+          <t>DONE 2026-06-12. Shared chrome (Wordmark pattern, for the whole frame): NEW web/src/components/AmbientBackground.jsx (grid + lime glow; off-brand blue dropped), PublicFooter.jsx (one footer everywhere: MyRX · Performance Lab + legal links + copyright), PageShell.jsx (relative min-h-dvh root + AmbientBackground + z-10 content layer so header/main sit above the ambient + PublicFooter). ALL 8 public pages converted: Landing, Auth, AuthConfirm, DownloadAppPlaceholder, ForCoaches, CoachPricing (each wraps its own &lt;header&gt;+&lt;main&gt; in &lt;PageShell&gt;); coach/AcceptInvite (its LOCAL PageShell helper now delegates to the shared one imported as SharedShell -- all call sites unchanged); legal/LegalLayout (operator line 'MyRX is operated by Northern Princess LLC... privacy@myrxfit.com' KEPT as a closing &lt;p&gt; in the doc body so legal pages don't lose required info; its FOOTER_LINKS nav dropped in favor of the shared footer). Result: identical background + footer + header-bar frame on every public page; content inside still page-specific. EXCLUDED by design: signup journey (own progress chrome) + admin/coach portals (sidebar shells). Two clean builds; deployed (6-page batch index-bi6iHLXw.js, then the final 2). User verifies visually.</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2996,7 +2996,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -3672,7 +3672,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E62" s="11" t="inlineStr">
+      <c r="E62" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5076,7 +5076,7 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E89" s="11" t="inlineStr">
+      <c r="E89" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5128,7 +5128,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E90" s="11" t="inlineStr">
+      <c r="E90" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5180,7 +5180,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E91" s="11" t="inlineStr">
+      <c r="E91" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5388,7 +5388,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E95" s="10" t="inlineStr">
+      <c r="E95" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -7936,7 +7936,7 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E144" s="10" t="inlineStr">
+      <c r="E144" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -7988,7 +7988,7 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E145" s="10" t="inlineStr">
+      <c r="E145" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8092,7 +8092,7 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E147" s="10" t="inlineStr">
+      <c r="E147" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -9028,7 +9028,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E165" s="10" t="inlineStr">
+      <c r="E165" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -10536,7 +10536,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E194" s="12" t="inlineStr">
+      <c r="E194" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -11472,7 +11472,7 @@
           <t>Web+Mobile</t>
         </is>
       </c>
-      <c r="E212" s="13" t="inlineStr">
+      <c r="E212" s="12" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -11524,7 +11524,7 @@
           <t>Web+Mobile+DB</t>
         </is>
       </c>
-      <c r="E213" s="9" t="inlineStr">
+      <c r="E213" s="13" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -11883,7 +11883,7 @@
           <t>Web+Edge+DB</t>
         </is>
       </c>
-      <c r="E220" s="9" t="inlineStr">
+      <c r="E220" s="13" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -11935,7 +11935,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E221" s="13" t="inlineStr">
+      <c r="E221" s="12" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -12611,7 +12611,7 @@
           <t>Backend+Supabase</t>
         </is>
       </c>
-      <c r="E234" s="12" t="inlineStr">
+      <c r="E234" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -12663,7 +12663,7 @@
           <t>Backend+Supabase</t>
         </is>
       </c>
-      <c r="E235" s="12" t="inlineStr">
+      <c r="E235" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -12871,7 +12871,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E239" s="10" t="inlineStr">
+      <c r="E239" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -12923,7 +12923,7 @@
           <t>Web+DB</t>
         </is>
       </c>
-      <c r="E240" s="10" t="inlineStr">
+      <c r="E240" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -13027,7 +13027,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E242" s="10" t="inlineStr">
+      <c r="E242" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>

</xml_diff>

<commit_message>
feat(brand/mobile): one shared ambient on every auth/onboarding screen (T253 phase 2)
Each auth screen had its own backdrop with different values — welcome/sign-in/forgot-password used a lime + an off-brand SKY-BLUE glow (sign-in bumped), and the signup journey had grid only (no glow); accept-invite + coach-pending had nothing. New mobile/src/components/AmbientBackground.tsx (react-native-svg — matching the existing backdrops; Skia is for charts) is the single source of truth: two LIME glows + a faint grid, identical everywhere, no blue. Applied to welcome, sign-in, forgot-password, sign-up, accept-invite, coach-pending. App tabs/dashboards stay flat (same as web). The old per-screen Backdrop functions are now dead code (cleanup follow-up).
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -86,11 +86,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
@@ -107,6 +102,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -2476,9 +2476,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>DECISIONS 2026-06-12: size = 28px (assistant's call -- user was torn; 28 matches the always-visible app top bar + web). Ambient = YES (user: 'Logo + ambient'). PHASE 1 (wordmark) DONE: NEW mobile/src/components/Wordmark.tsx (Image, 28px, width derived from 1781/390 aspect, dark wordmark; style prop for positioning only). Replaced the Image usages on sign-in (24-&gt;28), accept-invite (24-&gt;28), welcome/carousel (36-&gt;28, kept marginBottom 8), and the app top bar (was already 28, now via the component); removed the now-dead LOGO_DARK const in (app)/_layout. Kept the signup welcome slogan hero (56) + the LoadingScreen animated splash as intentional exceptions. tsc gate, then reload. PHASE 2 (PENDING): Skia ambient (grid + lime glow) behind the mobile AUTH/ONBOARDING screens only (welcome, sign-in, sign-up, accept-invite, forgot-password, coach-pending) -- NOT the app tabs (mirrors the web 'dashboards stay flat' decision). Needs an @shopify/react-native-skia ambient component (verify Skia setup first).</t>
+          <t>DECISIONS 2026-06-12: size = 28px (assistant's call -- user was torn; 28 matches the always-visible app top bar + web). Ambient = YES (user: 'Logo + ambient'). PHASE 1 (wordmark) DONE: NEW mobile/src/components/Wordmark.tsx (Image, 28px, width derived from 1781/390 aspect, dark wordmark; style prop for positioning only). Replaced the Image usages on sign-in (24-&gt;28), accept-invite (24-&gt;28), welcome/carousel (36-&gt;28, kept marginBottom 8), and the app top bar (was already 28, now via the component); removed the now-dead LOGO_DARK const in (app)/_layout. Kept the signup welcome slogan hero (56) + the LoadingScreen animated splash as intentional exceptions. tsc gate, then reload. PHASE 2 DONE 2026-06-12: used react-native-svg, NOT Skia -- the existing per-screen backdrops (welcome/sign-in/forgot-password = lime + off-brand SKY-BLUE + grid; sign-up = grid only) were already SVG-based, so matched that (Skia is for the charts). NEW mobile/src/components/AmbientBackground.tsx: one Svg with two LIME radial glows (TL 0.38 behind the wordmark + TR 0.20 balance; the off-brand blue is GONE) + a 12x24 grid at opacity 0.10, StyleSheet.absoluteFill + pointerEvents none. Applied to ALL 6 auth/onboarding screens: welcome/sign-in/forgot-password swapped &lt;Backdrop/&gt; -&gt; &lt;AmbientBackground/&gt;; sign-up swapped &lt;SignupBackdrop/&gt; (the journey now gets the glow too, per 'exact same everywhere' -- overrides the old 'signup drops the glow' choice); accept-invite + coach-pending got it added to their roots (behind content, first child). App tabs/dashboards stay flat (mirrors the web dashboards-flat call). The old per-screen Backdrop/SignupBackdrop functions are now DEAD CODE -- spawned a cleanup task chip. tsc gate; user reloads on device to verify.</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -3256,7 +3256,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E54" s="10" t="inlineStr">
+      <c r="E54" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -3932,7 +3932,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E67" s="11" t="inlineStr">
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5336,7 +5336,7 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E94" s="11" t="inlineStr">
+      <c r="E94" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5388,7 +5388,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E95" s="11" t="inlineStr">
+      <c r="E95" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5440,7 +5440,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E96" s="11" t="inlineStr">
+      <c r="E96" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5648,7 +5648,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E100" s="10" t="inlineStr">
+      <c r="E100" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8196,7 +8196,7 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E149" s="10" t="inlineStr">
+      <c r="E149" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8248,7 +8248,7 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E150" s="10" t="inlineStr">
+      <c r="E150" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8352,7 +8352,7 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E152" s="10" t="inlineStr">
+      <c r="E152" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -9288,7 +9288,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E170" s="10" t="inlineStr">
+      <c r="E170" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -10796,7 +10796,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E199" s="12" t="inlineStr">
+      <c r="E199" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -11732,7 +11732,7 @@
           <t>Web+Mobile</t>
         </is>
       </c>
-      <c r="E217" s="13" t="inlineStr">
+      <c r="E217" s="12" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -11784,7 +11784,7 @@
           <t>Web+Mobile+DB</t>
         </is>
       </c>
-      <c r="E218" s="9" t="inlineStr">
+      <c r="E218" s="13" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -12143,7 +12143,7 @@
           <t>Web+Edge+DB</t>
         </is>
       </c>
-      <c r="E225" s="9" t="inlineStr">
+      <c r="E225" s="13" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
@@ -12195,7 +12195,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E226" s="13" t="inlineStr">
+      <c r="E226" s="12" t="inlineStr">
         <is>
           <t>Parked</t>
         </is>
@@ -12871,7 +12871,7 @@
           <t>Backend+Supabase</t>
         </is>
       </c>
-      <c r="E239" s="12" t="inlineStr">
+      <c r="E239" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -12923,7 +12923,7 @@
           <t>Backend+Supabase</t>
         </is>
       </c>
-      <c r="E240" s="12" t="inlineStr">
+      <c r="E240" s="11" t="inlineStr">
         <is>
           <t>Reverted</t>
         </is>
@@ -13131,7 +13131,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E244" s="10" t="inlineStr">
+      <c r="E244" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -13183,7 +13183,7 @@
           <t>Web+DB</t>
         </is>
       </c>
-      <c r="E245" s="10" t="inlineStr">
+      <c r="E245" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -13287,7 +13287,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E247" s="10" t="inlineStr">
+      <c r="E247" s="9" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>

</xml_diff>

<commit_message>
docs(pipeline): T214 done (purged 10 orphan auth rows), T199 done (coach subdomain verified live), T194 go-live note
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -81,17 +81,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E5E7EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -747,7 +747,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Investigate 10 auth.users rows with no matching profiles row (21 auth vs 11 profiles)</t>
+          <t>Investigate + purge orphaned auth.users rows with no matching profiles row</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -760,9 +760,9 @@
           <t>DB</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Surfaced during the T213 verification: auth.users=21 but profiles=11 -&gt; 10 auth-only accounts with no profile. Likely incomplete signups (auth row created, profile never completed -&gt; ProtectedLayout blocks them so they're inert) OR residue from a pre-anonymization-era hard delete. Not related to the 3 test accounts (fully purged). Inert but untidy.</t>
+          <t>Surfaced during T213 verification: auth.users &gt;&gt; profiles. At investigation (2026-06-13): 22 auth / 12 profiles / 10 orphaned auth / 0 dangling profiles. Enumerated the 10 -- ALL were the user's own May-30 signup-flow test aliases: jarrah.motaz+{signuptest,invitetest,magictest,resettest,chgfrom}@gmail.com + motaz.jarrah+{same}@hotmail.com. No profile, no logged data, all created the same test day. Inert (the profile-completeness gate blocks profile-less accounts from the app) but untidy. WHY THE ADMIN UI COULDN'T REACH THEM: the client roster lists PROFILES; these have none -- so the user's manual cleanup (which removed 7 profile-having accounts, profiles 12-&gt;5, auth 22-&gt;15) left ALL 10 orphans untouched (orphan count stayed 10).</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Enumerate the 10 (select id,email,created_at,last_sign_in from auth.users where id not in (select id from profiles)); classify incomplete-signup vs orphan; decide keep vs purge. If purge: they have no profile so a plain auth.users delete cascades cleanly. Low priority.</t>
+          <t>DONE 2026-06-13: hard-deleted all 10 orphaned auth.users via SQL (DELETE ... WHERE id NOT IN profiles RETURNING email) -- succeeded with NO FK violation, confirming zero associated rows in any public table. Re-verified: 5 auth = 5 profiles, 0 orphaned auth, 0 orphaned profiles (perfect 1:1). Authorized by the user's explicit 'delete all unnecessary accounts' directive; the 10 were unambiguous self-created test cruft matching the description, so proceeded without a separate confirm. FUTURE PREVENTION (not built): abandoned test signups (signUp that never completes a profile) still leave auth-only rows -- a periodic orphan sweep, or always writing a stub profile at signUp, would stop them accumulating.</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
+      <c r="E59" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -4192,7 +4192,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E72" s="10" t="inlineStr">
+      <c r="E72" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5596,7 +5596,7 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E99" s="10" t="inlineStr">
+      <c r="E99" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5648,7 +5648,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E100" s="10" t="inlineStr">
+      <c r="E100" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5700,7 +5700,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E101" s="10" t="inlineStr">
+      <c r="E101" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -5908,7 +5908,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E105" s="9" t="inlineStr">
+      <c r="E105" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -5960,7 +5960,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E106" s="8" t="inlineStr">
+      <c r="E106" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8456,7 +8456,7 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E154" s="9" t="inlineStr">
+      <c r="E154" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8508,7 +8508,7 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E155" s="9" t="inlineStr">
+      <c r="E155" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -8612,7 +8612,7 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E157" s="9" t="inlineStr">
+      <c r="E157" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -9548,7 +9548,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E175" s="9" t="inlineStr">
+      <c r="E175" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -12148,9 +12148,9 @@
           <t>Web+DNS+Edge</t>
         </is>
       </c>
-      <c r="E225" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E225" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F225" s="5" t="inlineStr">
@@ -12160,7 +12160,7 @@
       </c>
       <c r="G225" s="7" t="inlineStr">
         <is>
-          <t>User 2026-06-11: 'i think i want to make our website very clear on standing, so it should be athlete.myrxfit.com and coach.myrxfit.com, isnt that more modern and helpful?' Asking opinion + proposing the split. ASSESSMENT: the instinct (clear audience separation) is good + modern, BUT asymmetric -- athletes have NO web app (mobile-only per the role rule), so athlete.myrxfit.com would be a marketing/DOWNLOAD funnel, not an athlete web app; coach.myrxfit.com hosts the real web product (portal + signup + coach marketing). REAL COST (touches a lot; several steps are USER-side): (1) DNS CNAMEs for both subdomains; (2) Cloudflare Pages custom domains on the myrx project (or split into 2 projects); (3) app made host-aware (one bundle landing coach.* on the coach surface, athlete.* on the download funnel) OR two builds; (4) auth redirects + Supabase redirect allowlist + mobile emailRedirectTo (currently myrxfit.com/auth/confirm) -- TOUCHY, can break mobile auth confirmation; (5) Android App Links assetlinks.json (.well-known) must live on the athlete deep-link host; (6) Stripe success/cancel URLs (coach-signup SITE_URL) -&gt; coach.myrxfit.com; (7) email templates + external links. RECOMMENDATION: do it as its OWN focused project AFTER the current coach-billing testing -- rushing DNS/auth-redirect changes now would risk the flows being tested. Confirm the athlete.* = download-funnel intent. NOT STARTED (planning only, presented to user 2026-06-11). || UPDATE 2026-06-11 (user revised + approved): myrxfit.com = purely INFORMATIVE landing (NO athlete sign-in/sign-up/pricing -- 'assume it's free until you make an account in the app'); coach.myrxfit.com = full coach side. CODE DONE + DEPLOYED (live-verified): (a) Auth.jsx REWRITTEN to sign-in only (clean; the dead signup steps/handlers/state/unused imports physically removed -- resolves the T198 follow-up); (b) Landing.jsx stripped to pure info -- removed Pricing/Sign-in/Get-started nav + both hero CTAs + the download button (-&gt; 'Coming soon to iOS and Android'); kept the demo card + feature grid + a single 'For Coaches' link; Apple+Google store badges + a QR drop in here at app launch; (c) athlete /pricing route + Pricing.jsx DELETED (old /pricing -&gt; Redirect to /); (d) App.jsx host-aware: isCoachHost() (/^coach\./) -&gt; coach.myrxfit.com root renders ForCoaches (coach landing), myrxfit.com root renders Landing; signed-in users role-route either way; dev/preview hosts (localhost, *.pages.dev) get the main landing. INFRA PENDING (needs USER -- wrangler 4.x has NO 'pages domain' cmd + the CF API token isn't in env, wrangler deploys via cached OAuth): attach coach.myrxfit.com as a Custom Domain on the myrx Pages project (CF auto-creates the proxied CNAME + cert since myrxfit.com is in the same account). DEFERRED phase-2 (touchy, AFTER coach.* verified live): point coach auth/Stripe(SITE_URL)/email redirects + the Landing 'For Coaches' link at coach.myrxfit.com; mobile auth deep-links + assetlinks stay on myrxfit.com.</t>
+          <t>User 2026-06-11: 'i think i want to make our website very clear on standing, so it should be athlete.myrxfit.com and coach.myrxfit.com, isnt that more modern and helpful?' Asking opinion + proposing the split. ASSESSMENT: the instinct (clear audience separation) is good + modern, BUT asymmetric -- athletes have NO web app (mobile-only per the role rule), so athlete.myrxfit.com would be a marketing/DOWNLOAD funnel, not an athlete web app; coach.myrxfit.com hosts the real web product (portal + signup + coach marketing). REAL COST (touches a lot; several steps are USER-side): (1) DNS CNAMEs for both subdomains; (2) Cloudflare Pages custom domains on the myrx project (or split into 2 projects); (3) app made host-aware (one bundle landing coach.* on the coach surface, athlete.* on the download funnel) OR two builds; (4) auth redirects + Supabase redirect allowlist + mobile emailRedirectTo (currently myrxfit.com/auth/confirm) -- TOUCHY, can break mobile auth confirmation; (5) Android App Links assetlinks.json (.well-known) must live on the athlete deep-link host; (6) Stripe success/cancel URLs (coach-signup SITE_URL) -&gt; coach.myrxfit.com; (7) email templates + external links. RECOMMENDATION: do it as its OWN focused project AFTER the current coach-billing testing -- rushing DNS/auth-redirect changes now would risk the flows being tested. Confirm the athlete.* = download-funnel intent. NOT STARTED (planning only, presented to user 2026-06-11). || UPDATE 2026-06-11 (user revised + approved): myrxfit.com = purely INFORMATIVE landing (NO athlete sign-in/sign-up/pricing -- 'assume it's free until you make an account in the app'); coach.myrxfit.com = full coach side. CODE DONE + DEPLOYED (live-verified): (a) Auth.jsx REWRITTEN to sign-in only (clean; the dead signup steps/handlers/state/unused imports physically removed -- resolves the T198 follow-up); (b) Landing.jsx stripped to pure info -- removed Pricing/Sign-in/Get-started nav + both hero CTAs + the download button (-&gt; 'Coming soon to iOS and Android'); kept the demo card + feature grid + a single 'For Coaches' link; Apple+Google store badges + a QR drop in here at app launch; (c) athlete /pricing route + Pricing.jsx DELETED (old /pricing -&gt; Redirect to /); (d) App.jsx host-aware: isCoachHost() (/^coach\./) -&gt; coach.myrxfit.com root renders ForCoaches (coach landing), myrxfit.com root renders Landing; signed-in users role-route either way; dev/preview hosts (localhost, *.pages.dev) get the main landing. INFRA PENDING (needs USER -- wrangler 4.x has NO 'pages domain' cmd + the CF API token isn't in env, wrangler deploys via cached OAuth): attach coach.myrxfit.com as a Custom Domain on the myrx Pages project (CF auto-creates the proxied CNAME + cert since myrxfit.com is in the same account). DEFERRED phase-2 (touchy, AFTER coach.* verified live): point coach auth/Stripe(SITE_URL)/email redirects + the Landing 'For Coaches' link at coach.myrxfit.com; mobile auth deep-links + assetlinks stay on myrxfit.com. || VERIFIED DONE 2026-06-13 (user: '199 is complete, verify'): coach.myrxfit.com is LIVE (HTTP 200, serving the current bundle index-BcLFY8xr.js) -- the Custom Domain is attached on the myrx Pages project + cert issued. myrxfit.com apex also 200 (the informative landing). athlete.myrxfit.com does NOT resolve (HTTP 000) -- CORRECT by design (athletes are mobile-only; the apex is their download/landing, no athlete. subdomain). Host-aware split (isCoachHost) confirmed live. The deferred phase-2 redirects remain OPTIONAL polish, not blockers. SIDE FINDING (separate, minor): www.myrxfit.com returns 522 (no origin/redirect for the www host) -- a www-&gt;apex redirect rule would fix it if desired.</t>
         </is>
       </c>
       <c r="H225" s="7" t="inlineStr">
@@ -12420,7 +12420,7 @@
       </c>
       <c r="H230" s="5" t="inlineStr">
         <is>
-          <t>PROPOSED PLAN (presented to user 2026-06-11, AWAITING approval + decisions). PHASE 1 (core security fix): (1a) coach-signup STOPS granting is_coach=true -- it only creates the Stripe customer + checkout session (user stays 'pending payment'); (1b) the webhook becomes the SOLE granter -- on subscription.created (status trialing) it sets is_coach=true + status + tier + trial-end; (1c) the portal gate switches from 'is_coach===true' to 'is_coach AND status IN (trialing,active,past_due)' (reuse is_active_coach()); past_due kept IN so the Smart-Retries grace window does not lock a coach out mid-fix. PHASE 2 (resume): a user who finished their details but bailed at the Stripe page (is_coach still false, pending checkout) is sent straight back to the payment step on next login -- not locked out, not let in. PHASE 3 (manage/cancel in-app): replace the CoachProfile placeholder with a real 'Manage plan' that opens Stripe's billing portal (update card / cancel / switch tier); mirrors the athlete Manage-plan concept. [CAN DEFER -- not a security hole.] PHASE 4 (must-fix bugs + cleanup): widen coach_subscriptions.tier CHECK to include 'elite' (unblocks Elite -- SEVERE, fix regardless); fix the annual renewal copy to the recurring-17%-off model; reconcile the 3 drifted migration files to live. PHASE 5: wipe+reseed the test DB once everything is secured (the long-standing T165 step). TESTING: real Stripe TEST mode + test cards (4242...) -&gt; full end-to-end coach signup is testable NOW, before flipping to live. OPEN DECISIONS: (D1) hardening depth -- client gate + webhook truth (good), OR ALSO add server-side DB rules (RLS/RPC) so coach data is unreachable without a live sub even via a hand-crafted request (more bulletproof, more work)? (D2) build in-app cancel/manage now (Phase 3) or defer? (D3) confirm annual = recurring 17% off forever (=&gt; fix the UI copy). || CLARIFIED 2026-06-11 (user: 'the coach can only access their coach portal on WEB; on MOBILE they only access their own athlete account'). REFRAME: ALL coach-PORTAL access work is WEB (CoachProtectedLayout + coach signup + Stripe manage). MOBILE has NO coach portal -- a coach on mobile is just an athlete. The one mobile angle: a paying coach gets full athlete features on their OWN mobile account as a PERK (resolveTier is_coach branch); that perk must follow the LIVE coach subscription, so mobile resolveTier should grant it ONLY for live statuses (trialing/active/past_due) -- a lapsed coach reverts to the normal athlete experience (free) on mobile, not full-features-forever. Resolves the T164 is_coach block-list-vs-allow-list divergence (post-Phase-1 a coach never has a null status; the unlock keys on live status). Net: Phase-1 'is_coach only after Stripe' + webhook-truth status drives BOTH the web portal gate AND the mobile athlete perk from one source. || DECISIONS LOCKED 2026-06-11 (user: 'all items are in, nothing after, run it on dependency sequence so it all builds clean'): D1=EXTREME bulletproof -&gt; ADD server-side enforcement (RLS/RPC) so coach data + portal endpoints are unreachable without a LIVE coach sub even via a hand-crafted request, not just the client gate. D2=BUILD manage/cancel now: WEB gets the real Stripe billing portal (update card / cancel / switch tier); MOBILE shows ONLY an informational pointer ('your coach plan was purchased on the web -- manage it at myrxfit.com'), NO in-app buy/manage CTA -- Apple/Google store-rule legality to be verified before wording (user flagged). D3=annual is recurring 17%-off EVERY year (confirmed) -&gt; fix the 'first year then full price' copy. item5: a lapsed coach reverts to FREE athlete on mobile (confirmed). BUILD ORDER (dependency-clean): (1) DB foundation -- widen coach_subscriptions.tier to include 'elite' + reconcile 3 drifted migration files; (2) stripe-webhook becomes the GRANTER (sets is_coach + status on subscription.created/active; clears on cancel/lapse) -- BEFORE step 3 to avoid an access gap; (3) coach-signup STOPS granting (only creates Stripe customer+checkout + a pending marker); (4) web portal gate requires LIVE status; (5) web resume routes an unpaid coach back to checkout; (6) mobile resolveTier perk follows live status; (7) EXTREME server-side RLS/RPC hardening; (8) manage/cancel -- new Stripe customer-portal edge fn + web button + mobile pointer message; (9) annual copy fix; (10) wipe+reseed test DB LAST. Building in this order. || PROGRESS 2026-06-11: STEPS 1-3 DONE + DEPLOYED. (1) migration t194_fix_coach_subscriptions_tier_elite -- migrated legacy 'unlimited' rows to 'elite' + widened the CHECK to starter/pro/elite (Elite signups no longer crash the webhook). (1b) migration t194_profiles_coach_stripe_customer_id -- new pending-coach marker + portal customer ref. (2) stripe-webhook v8 (verify_jwt=false) is now the SOLE granter: added isLiveCoachStatus(trialing/active/past_due) + set is_coach on all 4 profiles-mirror paths (created/updated -&gt; isLiveCoachStatus(status); deleted -&gt; false; invoice.paid -&gt; true; invoice.payment_failed/past_due -&gt; true grace) + sync coach_stripe_customer_id. (3) coach-signup v10 (verify_jwt=true) STOPS granting -- removed the pre-Stripe is_coach/trialing upsert; now only creates/reuses the Stripe customer (stores coach_stripe_customer_id as the pending marker, reuses on retry so no orphan customers), simplified the duplicate-block to is_coach===true, metadata coach_id now = user.id. Both deployed via Supabase MCP (CLI had no token; assistant doesn't handle credentials). The grant flip is LIVE + testable with a Stripe TEST card on a FRESH (non-coach) account: complete checkout -&gt; webhook grants -&gt; portal admits (is_coach now true); abandon checkout -&gt; is_coach stays false -&gt; existing gate bounces to /app. NOTE item 6 (mobile perk) is now largely handled FOR FREE because is_coach is webhook-managed to be true only for live statuses -&gt; resolveTier's is_coach branch already yields the athlete path for a lapsed coach; step 6 just needs to VERIFY/simplify resolveTier. NEXT: step 4 (web gate live-status check via is_active_coach), then 5/6/7/8/9/10. || CLARIFIED 2026-06-11 (user: 'a coach doesnt pay for their athlete account independently, it comes free with their web subscription; they have NO payment wall inside the app whatsoever -- is this a problem?'). ANSWER: NOT a problem, and the deployed code already matches this. A coach gets the full mobile athlete app FREE via their web coach subscription (the is_coach perk -&gt; resolveTier grants full features); they NEVER see an in-app paywall. Store-legal because the SAME athlete premium IS sold via IAP to regular athletes (Apple 3.1.3(b) multiplatform: features 'acquired on your web site' are allowed provided they are 'also available as in-app purchases within the app' -- they are; the coach simply has a comp entitlement = Netflix/Spotify pattern). The coach B2B sub is a WEB/Stripe business purchase for the PORTAL, not mobile digital content, so it does not need IAP. NOTHING in the grant-flip adds a mobile paywall for coaches -- the perk is auto-granted from is_coach. ONE mobile billing-surface nuance for item 8/10: a coach opening the mobile athlete Billing tab must see a REASSURING 'you have full access through your coach plan (manage it at myrxfit.com)' state, NOT an upgrade/paywall prompt -- informational pointer only. A LAPSED coach (is_coach=false) correctly becomes a normal free athlete on mobile and only THEN sees the normal athlete upgrade options (they lost the perk by not paying) -- expected, not a paywall-on-coaches. ADD to step 6/8 scope: confirm the mobile athlete BillingTab renders the coach reassurance state when is_coach=true. || PROGRESS 2026-06-11 cont'd: STEPS 4 + 6 DONE (web staged for end-of-build deploy; mobile tsc clean). (4) web CoachProtectedLayout (App.jsx) now gates on LIVE status not just is_coach: admits is_superuser OR (is_coach AND status IN trialing/active/past_due AND !deactivated_at) -- mirrors is_active_coach() EXACTLY; a lapsed/pending coach (is_coach=true non-live, OR is_coach=false with a coach_stripe_customer_id) routes to /coach/signup to resubscribe (sets up step 5), a plain athlete to /app. (6) flipped resolveTier from BLOCK-list to ALLOW-list in ALL 4 copies (mobile RadialNav.tsx + dashboard.tsx, web AdminUserDetail.jsx + CoachClientDetail.jsx): is_coach=true grants fullrx ONLY for trialing/active/past_due, else drops to the b2c tier -- closes the T164 block-list-vs-allow-list divergence for good. NET: every surface (DB is_active_coach + client_has_active_coach, web portal gate, 4 resolveTier copies, webhook granter, coach-signup) now shares ONE live-status definition [trialing, active, past_due]. Web build+deploy BATCHED for when web steps (5/8/9) are done so the user tests the whole coach flow once at the end (their request: 'ill test in the end'). NEXT: step 5 (web resume -- route an abandoned/lapsed coach back to checkout, reusing their pending Stripe customer), then 7 (server-side RLS/RPC hardening), 8 (manage/cancel + mobile reassurance state), 9 (annual copy), 10 (wipe+reseed). || STEP 5 DONE 2026-06-11 (web, staged): coach Signup.jsx detectFlow now lands a RETURNING coach (has coach_stripe_customer_id OR a past coach_subscription_status) directly on the PLAN screen of the 8-screen RESUME flow (skips welcome/magic/promise) instead of step 0 -- abandoned-checkout or lapsed coach re-subscribes in 2 taps (plan -&gt; stripe). coach-signup reuses their existing Stripe customer (step 3) so no orphans. A brand-new coach (existing athlete upgrading, no coach history) still starts at welcome for the full pitch. Added coach_stripe_customer_id to the detectFlow select. Abandon path verified by construction: Stripe cancel_url=/coach/signup?cancelled=1 -&gt; detectFlow sees the stored customer id -&gt; PLAN; the step-4 gate also routes a lapsed/pending coach to /coach/signup -&gt; PLAN. NEXT: step 7 (server-side RLS/RPC = extreme-bulletproof; audit coach-data policies + add is_active_coach() enforcement), then 8/9/10. || STEP 7 DONE 2026-06-11 (migration t194_coach_rls_require_active_subscription): EXTREME server-side hardening applied + VERIFIED. Audited pg_policies -&gt; 24 policies granted a coach access to client data keyed ONLY on the roster link (coach_id=auth.uid()), NO active-sub check -- a lapsed coach could read/write roster data (profiles, efforts, bodyweight, calorie_logs, calorie_plans x4, food_logs, messages x4, activity_events, hr_samples, sleep_sessions, step_samples, user_integrations, water_logs, wearable_workouts, coach_invites insert+update) via a hand-crafted API call. Prefixed all 24 with public.is_active_coach(auth.uid()) (SECURITY DEFINER -&gt; bypasses RLS internally, no profiles recursion). Verified: only 4 coach-matching policies remain WITHOUT the guard, all intentional -- the 2 calorie_plans 'Users ... own plan when self-managed' (client-self, matched on the macros_managed_by_coach column name), coach_invites SELECT + coach_subscriptions SELECT (a lapsed coach must still SEE their own invites + sub to re-subscribe). Client + server now enforce the IDENTICAL live-coach rule [trialing,active,past_due] across DB RLS, the web portal gate, all 4 resolveTier copies, the webhook, and coach-signup. STEPS 1-7 DONE. NEXT: 8 (manage/cancel: new Stripe customer-portal edge fn + web button + mobile reassurance state), 9 (annual copy), 10 (wipe+reseed -- LAST, destructive, confirm with user). || STEP 8 DONE 2026-06-11 (manage/cancel). (a) NEW edge fn coach-billing-portal (v1, verify_jwt=true): looks up profiles.coach_stripe_customer_id, creates a Stripe Billing Portal session, returns the url; NOT gated on is_active_coach (a lapsed coach must reach the portal to update card / reactivate). (b) web CoachProfile Billing tab: replaced the 'Stripe emails you a link' placeholder with a real 'Manage plan' button -&gt; invokes coach-billing-portal -&gt; redirects to Stripe's hosted portal (update card / switch tier / cancel); changes flow back via the webhook. (c) mobile BillingTab: added a COACH-self branch in CurrentSection (priority 2, after anonymized) -&gt; a coach sees 'Full access through your coach plan ... manage ... on the web at myrxfit.com' (PLAIN TEXT, NO in-app buy/manage CTA -&gt; store-compliant per the 3.1.3(b) research) instead of the athlete free/upgrade state. mobile tsc clean; web staged. USER PREREQUISITE (one-time, assistant CANNOT do -- no Stripe dashboard access / no key handling): enable + configure the Stripe Customer Portal (Dashboard -&gt; Settings -&gt; Billing -&gt; Customer portal), add the coach products so tier-switching + cancellation are allowed. Until that's saved, the portal session call errors. NEXT: step 9 (annual copy -- fix 'first year then full price' -&gt; recurring 17%-off EVERY year across coachPlan.js + Signup.jsx + CoachPricing.jsx + ForCoaches.jsx; D3 confirmed), then 10 (wipe+reseed, destructive, confirm). || STEP 9 DONE + WEB DEPLOYED 2026-06-11. Annual copy fixed to the RECURRING-discount model (D3) across coachPlan.js (removed renewalAnnual export + reworded comment), Signup.jsx (removed local renewalAnnual + 'first year, then $X/yr' -&gt; 'Billed yearly, cancel any time'; badge '2 months free first year' -&gt; '2 months free'; 'Renews at' summary now shows the annual price not monthly*12), CoachPricing.jsx (import + FAQ + caption + price disclosure + a stale layout comment), ForCoaches.jsx (import + '$X/yr (first year), then $Y/yr' -&gt; '$X/yr (billed yearly)'). Verified ZERO dangling renewalAnnual usages (a dangling ref would build clean but crash at runtime). Web built (index-xW5C70HF.js) + deployed via wrangler + LIVE-verified on myrxfit.com (hash match). ALL WEB STEPS (4, 5, 8-button, 9) now LIVE. STEPS 1-9 DONE. ONLY step 10 left: wipe+reseed the test DB -- DESTRUCTIVE, awaiting user confirmation + what to seed. OUTSTANDING USER ACTION: enable the Stripe Customer Portal in the dashboard (Settings -&gt; Billing -&gt; Customer portal) so the web 'Manage plan' button works.</t>
+          <t>PROPOSED PLAN (presented to user 2026-06-11, AWAITING approval + decisions). PHASE 1 (core security fix): (1a) coach-signup STOPS granting is_coach=true -- it only creates the Stripe customer + checkout session (user stays 'pending payment'); (1b) the webhook becomes the SOLE granter -- on subscription.created (status trialing) it sets is_coach=true + status + tier + trial-end; (1c) the portal gate switches from 'is_coach===true' to 'is_coach AND status IN (trialing,active,past_due)' (reuse is_active_coach()); past_due kept IN so the Smart-Retries grace window does not lock a coach out mid-fix. PHASE 2 (resume): a user who finished their details but bailed at the Stripe page (is_coach still false, pending checkout) is sent straight back to the payment step on next login -- not locked out, not let in. PHASE 3 (manage/cancel in-app): replace the CoachProfile placeholder with a real 'Manage plan' that opens Stripe's billing portal (update card / cancel / switch tier); mirrors the athlete Manage-plan concept. [CAN DEFER -- not a security hole.] PHASE 4 (must-fix bugs + cleanup): widen coach_subscriptions.tier CHECK to include 'elite' (unblocks Elite -- SEVERE, fix regardless); fix the annual renewal copy to the recurring-17%-off model; reconcile the 3 drifted migration files to live. PHASE 5: wipe+reseed the test DB once everything is secured (the long-standing T165 step). TESTING: real Stripe TEST mode + test cards (4242...) -&gt; full end-to-end coach signup is testable NOW, before flipping to live. OPEN DECISIONS: (D1) hardening depth -- client gate + webhook truth (good), OR ALSO add server-side DB rules (RLS/RPC) so coach data is unreachable without a live sub even via a hand-crafted request (more bulletproof, more work)? (D2) build in-app cancel/manage now (Phase 3) or defer? (D3) confirm annual = recurring 17% off forever (=&gt; fix the UI copy). || CLARIFIED 2026-06-11 (user: 'the coach can only access their coach portal on WEB; on MOBILE they only access their own athlete account'). REFRAME: ALL coach-PORTAL access work is WEB (CoachProtectedLayout + coach signup + Stripe manage). MOBILE has NO coach portal -- a coach on mobile is just an athlete. The one mobile angle: a paying coach gets full athlete features on their OWN mobile account as a PERK (resolveTier is_coach branch); that perk must follow the LIVE coach subscription, so mobile resolveTier should grant it ONLY for live statuses (trialing/active/past_due) -- a lapsed coach reverts to the normal athlete experience (free) on mobile, not full-features-forever. Resolves the T164 is_coach block-list-vs-allow-list divergence (post-Phase-1 a coach never has a null status; the unlock keys on live status). Net: Phase-1 'is_coach only after Stripe' + webhook-truth status drives BOTH the web portal gate AND the mobile athlete perk from one source. || DECISIONS LOCKED 2026-06-11 (user: 'all items are in, nothing after, run it on dependency sequence so it all builds clean'): D1=EXTREME bulletproof -&gt; ADD server-side enforcement (RLS/RPC) so coach data + portal endpoints are unreachable without a LIVE coach sub even via a hand-crafted request, not just the client gate. D2=BUILD manage/cancel now: WEB gets the real Stripe billing portal (update card / cancel / switch tier); MOBILE shows ONLY an informational pointer ('your coach plan was purchased on the web -- manage it at myrxfit.com'), NO in-app buy/manage CTA -- Apple/Google store-rule legality to be verified before wording (user flagged). D3=annual is recurring 17%-off EVERY year (confirmed) -&gt; fix the 'first year then full price' copy. item5: a lapsed coach reverts to FREE athlete on mobile (confirmed). BUILD ORDER (dependency-clean): (1) DB foundation -- widen coach_subscriptions.tier to include 'elite' + reconcile 3 drifted migration files; (2) stripe-webhook becomes the GRANTER (sets is_coach + status on subscription.created/active; clears on cancel/lapse) -- BEFORE step 3 to avoid an access gap; (3) coach-signup STOPS granting (only creates Stripe customer+checkout + a pending marker); (4) web portal gate requires LIVE status; (5) web resume routes an unpaid coach back to checkout; (6) mobile resolveTier perk follows live status; (7) EXTREME server-side RLS/RPC hardening; (8) manage/cancel -- new Stripe customer-portal edge fn + web button + mobile pointer message; (9) annual copy fix; (10) wipe+reseed test DB LAST. Building in this order. || PROGRESS 2026-06-11: STEPS 1-3 DONE + DEPLOYED. (1) migration t194_fix_coach_subscriptions_tier_elite -- migrated legacy 'unlimited' rows to 'elite' + widened the CHECK to starter/pro/elite (Elite signups no longer crash the webhook). (1b) migration t194_profiles_coach_stripe_customer_id -- new pending-coach marker + portal customer ref. (2) stripe-webhook v8 (verify_jwt=false) is now the SOLE granter: added isLiveCoachStatus(trialing/active/past_due) + set is_coach on all 4 profiles-mirror paths (created/updated -&gt; isLiveCoachStatus(status); deleted -&gt; false; invoice.paid -&gt; true; invoice.payment_failed/past_due -&gt; true grace) + sync coach_stripe_customer_id. (3) coach-signup v10 (verify_jwt=true) STOPS granting -- removed the pre-Stripe is_coach/trialing upsert; now only creates/reuses the Stripe customer (stores coach_stripe_customer_id as the pending marker, reuses on retry so no orphan customers), simplified the duplicate-block to is_coach===true, metadata coach_id now = user.id. Both deployed via Supabase MCP (CLI had no token; assistant doesn't handle credentials). The grant flip is LIVE + testable with a Stripe TEST card on a FRESH (non-coach) account: complete checkout -&gt; webhook grants -&gt; portal admits (is_coach now true); abandon checkout -&gt; is_coach stays false -&gt; existing gate bounces to /app. NOTE item 6 (mobile perk) is now largely handled FOR FREE because is_coach is webhook-managed to be true only for live statuses -&gt; resolveTier's is_coach branch already yields the athlete path for a lapsed coach; step 6 just needs to VERIFY/simplify resolveTier. NEXT: step 4 (web gate live-status check via is_active_coach), then 5/6/7/8/9/10. || CLARIFIED 2026-06-11 (user: 'a coach doesnt pay for their athlete account independently, it comes free with their web subscription; they have NO payment wall inside the app whatsoever -- is this a problem?'). ANSWER: NOT a problem, and the deployed code already matches this. A coach gets the full mobile athlete app FREE via their web coach subscription (the is_coach perk -&gt; resolveTier grants full features); they NEVER see an in-app paywall. Store-legal because the SAME athlete premium IS sold via IAP to regular athletes (Apple 3.1.3(b) multiplatform: features 'acquired on your web site' are allowed provided they are 'also available as in-app purchases within the app' -- they are; the coach simply has a comp entitlement = Netflix/Spotify pattern). The coach B2B sub is a WEB/Stripe business purchase for the PORTAL, not mobile digital content, so it does not need IAP. NOTHING in the grant-flip adds a mobile paywall for coaches -- the perk is auto-granted from is_coach. ONE mobile billing-surface nuance for item 8/10: a coach opening the mobile athlete Billing tab must see a REASSURING 'you have full access through your coach plan (manage it at myrxfit.com)' state, NOT an upgrade/paywall prompt -- informational pointer only. A LAPSED coach (is_coach=false) correctly becomes a normal free athlete on mobile and only THEN sees the normal athlete upgrade options (they lost the perk by not paying) -- expected, not a paywall-on-coaches. ADD to step 6/8 scope: confirm the mobile athlete BillingTab renders the coach reassurance state when is_coach=true. || PROGRESS 2026-06-11 cont'd: STEPS 4 + 6 DONE (web staged for end-of-build deploy; mobile tsc clean). (4) web CoachProtectedLayout (App.jsx) now gates on LIVE status not just is_coach: admits is_superuser OR (is_coach AND status IN trialing/active/past_due AND !deactivated_at) -- mirrors is_active_coach() EXACTLY; a lapsed/pending coach (is_coach=true non-live, OR is_coach=false with a coach_stripe_customer_id) routes to /coach/signup to resubscribe (sets up step 5), a plain athlete to /app. (6) flipped resolveTier from BLOCK-list to ALLOW-list in ALL 4 copies (mobile RadialNav.tsx + dashboard.tsx, web AdminUserDetail.jsx + CoachClientDetail.jsx): is_coach=true grants fullrx ONLY for trialing/active/past_due, else drops to the b2c tier -- closes the T164 block-list-vs-allow-list divergence for good. NET: every surface (DB is_active_coach + client_has_active_coach, web portal gate, 4 resolveTier copies, webhook granter, coach-signup) now shares ONE live-status definition [trialing, active, past_due]. Web build+deploy BATCHED for when web steps (5/8/9) are done so the user tests the whole coach flow once at the end (their request: 'ill test in the end'). NEXT: step 5 (web resume -- route an abandoned/lapsed coach back to checkout, reusing their pending Stripe customer), then 7 (server-side RLS/RPC hardening), 8 (manage/cancel + mobile reassurance state), 9 (annual copy), 10 (wipe+reseed). || STEP 5 DONE 2026-06-11 (web, staged): coach Signup.jsx detectFlow now lands a RETURNING coach (has coach_stripe_customer_id OR a past coach_subscription_status) directly on the PLAN screen of the 8-screen RESUME flow (skips welcome/magic/promise) instead of step 0 -- abandoned-checkout or lapsed coach re-subscribes in 2 taps (plan -&gt; stripe). coach-signup reuses their existing Stripe customer (step 3) so no orphans. A brand-new coach (existing athlete upgrading, no coach history) still starts at welcome for the full pitch. Added coach_stripe_customer_id to the detectFlow select. Abandon path verified by construction: Stripe cancel_url=/coach/signup?cancelled=1 -&gt; detectFlow sees the stored customer id -&gt; PLAN; the step-4 gate also routes a lapsed/pending coach to /coach/signup -&gt; PLAN. NEXT: step 7 (server-side RLS/RPC = extreme-bulletproof; audit coach-data policies + add is_active_coach() enforcement), then 8/9/10. || STEP 7 DONE 2026-06-11 (migration t194_coach_rls_require_active_subscription): EXTREME server-side hardening applied + VERIFIED. Audited pg_policies -&gt; 24 policies granted a coach access to client data keyed ONLY on the roster link (coach_id=auth.uid()), NO active-sub check -- a lapsed coach could read/write roster data (profiles, efforts, bodyweight, calorie_logs, calorie_plans x4, food_logs, messages x4, activity_events, hr_samples, sleep_sessions, step_samples, user_integrations, water_logs, wearable_workouts, coach_invites insert+update) via a hand-crafted API call. Prefixed all 24 with public.is_active_coach(auth.uid()) (SECURITY DEFINER -&gt; bypasses RLS internally, no profiles recursion). Verified: only 4 coach-matching policies remain WITHOUT the guard, all intentional -- the 2 calorie_plans 'Users ... own plan when self-managed' (client-self, matched on the macros_managed_by_coach column name), coach_invites SELECT + coach_subscriptions SELECT (a lapsed coach must still SEE their own invites + sub to re-subscribe). Client + server now enforce the IDENTICAL live-coach rule [trialing,active,past_due] across DB RLS, the web portal gate, all 4 resolveTier copies, the webhook, and coach-signup. STEPS 1-7 DONE. NEXT: 8 (manage/cancel: new Stripe customer-portal edge fn + web button + mobile reassurance state), 9 (annual copy), 10 (wipe+reseed -- LAST, destructive, confirm with user). || STEP 8 DONE 2026-06-11 (manage/cancel). (a) NEW edge fn coach-billing-portal (v1, verify_jwt=true): looks up profiles.coach_stripe_customer_id, creates a Stripe Billing Portal session, returns the url; NOT gated on is_active_coach (a lapsed coach must reach the portal to update card / reactivate). (b) web CoachProfile Billing tab: replaced the 'Stripe emails you a link' placeholder with a real 'Manage plan' button -&gt; invokes coach-billing-portal -&gt; redirects to Stripe's hosted portal (update card / switch tier / cancel); changes flow back via the webhook. (c) mobile BillingTab: added a COACH-self branch in CurrentSection (priority 2, after anonymized) -&gt; a coach sees 'Full access through your coach plan ... manage ... on the web at myrxfit.com' (PLAIN TEXT, NO in-app buy/manage CTA -&gt; store-compliant per the 3.1.3(b) research) instead of the athlete free/upgrade state. mobile tsc clean; web staged. USER PREREQUISITE (one-time, assistant CANNOT do -- no Stripe dashboard access / no key handling): enable + configure the Stripe Customer Portal (Dashboard -&gt; Settings -&gt; Billing -&gt; Customer portal), add the coach products so tier-switching + cancellation are allowed. Until that's saved, the portal session call errors. NEXT: step 9 (annual copy -- fix 'first year then full price' -&gt; recurring 17%-off EVERY year across coachPlan.js + Signup.jsx + CoachPricing.jsx + ForCoaches.jsx; D3 confirmed), then 10 (wipe+reseed, destructive, confirm). || STEP 9 DONE + WEB DEPLOYED 2026-06-11. Annual copy fixed to the RECURRING-discount model (D3) across coachPlan.js (removed renewalAnnual export + reworded comment), Signup.jsx (removed local renewalAnnual + 'first year, then $X/yr' -&gt; 'Billed yearly, cancel any time'; badge '2 months free first year' -&gt; '2 months free'; 'Renews at' summary now shows the annual price not monthly*12), CoachPricing.jsx (import + FAQ + caption + price disclosure + a stale layout comment), ForCoaches.jsx (import + '$X/yr (first year), then $Y/yr' -&gt; '$X/yr (billed yearly)'). Verified ZERO dangling renewalAnnual usages (a dangling ref would build clean but crash at runtime). Web built (index-xW5C70HF.js) + deployed via wrangler + LIVE-verified on myrxfit.com (hash match). ALL WEB STEPS (4, 5, 8-button, 9) now LIVE. STEPS 1-9 DONE. ONLY step 10 left: wipe+reseed the test DB -- DESTRUCTIVE, awaiting user confirmation + what to seed. OUTSTANDING USER ACTION: enable the Stripe Customer Portal in the dashboard (Settings -&gt; Billing -&gt; Customer portal) so the web 'Manage plan' button works. || GO-LIVE STATUS 2026-06-13 (user: 'the coach payment layer is now complete, the only thing left is to turn on the live switch, so keep it open noting this'): the BUILD is complete -- steps 1-9 built/deployed/verified end-to-end in Stripe TEST mode. The ONLY remaining item is flipping Stripe TEST -&gt; LIVE: live API keys (edge-fn secrets), live products/prices by lookup_key coach_&lt;tier&gt;_&lt;interval&gt;, live webhook endpoint + signing secret, and the one-time Customer Portal enable in the LIVE dashboard. Keeping this task OPEN as the go-live tracker; nothing left to build. (Step 10 wipe+reseed-test-DB is moot at go-live -- the live DB starts clean.)</t>
         </is>
       </c>
       <c r="I230" s="5" t="inlineStr">
@@ -13391,7 +13391,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E249" s="9" t="inlineStr">
+      <c r="E249" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -13443,7 +13443,7 @@
           <t>Web+DB</t>
         </is>
       </c>
-      <c r="E250" s="9" t="inlineStr">
+      <c r="E250" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -13547,7 +13547,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E252" s="9" t="inlineStr">
+      <c r="E252" s="8" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -13807,7 +13807,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E257" s="8" t="inlineStr">
+      <c r="E257" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat(brand): roll out 3-tier lime button system across coach web + admin + mobile — cancels→outline, See/Manage plan→soft (T264)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -3048,9 +3048,9 @@
           <t>Web+Mobile</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>ROLLOUT PENDING (big cross-surface sweep; approach proposed to user 2026-06-13). Smart path: many buttons route through SHARED components (coach Signup PrimaryButton/SecondaryButton; mobile button components) -&gt; restyle the shared component to a 3-variant API, then fix ad-hoc inline buttons. Surfaces: athlete web (Landing done / Auth / AuthConfirm / DownloadApp / legal), coach web (ForCoaches / CoachPricing / coach Signup / CoachProfile / AcceptInvite / ReactivationGate), mobile (every screen's primary/save/back/cancel/nav), admin portal = SCOPE TBD (user said athlete+coach+mobile, didn't name admin). Plan: phased + reviewable, one deploy per surface; OR a parallel multi-agent sweep if the user wants speed. Destructive (delete/wipe/sign-out) NOT touched (stays red).</t>
+          <t>ROLLOUT PENDING (big cross-surface sweep; approach proposed to user 2026-06-13). Smart path: many buttons route through SHARED components (coach Signup PrimaryButton/SecondaryButton; mobile button components) -&gt; restyle the shared component to a 3-variant API, then fix ad-hoc inline buttons. Surfaces: athlete web (Landing done / Auth / AuthConfirm / DownloadApp / legal), coach web (ForCoaches / CoachPricing / coach Signup / CoachProfile / AcceptInvite / ReactivationGate), mobile (every screen's primary/save/back/cancel/nav), admin portal = SCOPE TBD (user said athlete+coach+mobile, didn't name admin). Plan: phased + reviewable, one deploy per surface; OR a parallel multi-agent sweep if the user wants speed. Destructive (delete/wipe/sign-out) NOT touched (stays red). || SHIPPED 2026-06-13 (web deployed hash index-jF3ZOvex.js; mobile tsc clean) via 4 parallel sub-editors, one per surface. RESULT -- athlete web: 0 changes (already consistent; backs/forgot/sign-in are text links, CTAs solid). coach web: 3 cancels -&gt; outline (ForCoaches 'See pricing', Welcome 'Refresh', CoachProfile delete-modal 'Cancel') + signup SecondaryButton + For Coaches link done earlier. admin: 9 form/modal cancels + OperationsPanel 'Discard' -&gt; outline (AdminMovements x4, AdminFoodLibrary x2, AdminUserDetail x2, AdminUserBody x1, OperationsPanel x1). mobile: 8 across 7 files -&gt; outline cancels (settings smallBtnSecondary + modalBtnCancel; accept-invite/AcceptInviteModal/coach-pending secondaryBtn; TrialEndedModal 'Stay on Free'; ImageCropper 'Cancel') + BillingTab 'See plans'/'Manage plan' -&gt; soft lime + ArrowRight. CTAs were already solid everywhere. GOTCHA (worth a scars note): subagents default to the session cwd = the STALE .claude worktree; the admin agent edited the worktree (lost) -&gt; re-ran FORCED to the main repo; coach/mobile agents self-detected. FLAGGED for user (left as-is): bare-TEXT cancels with no box (CoachClientDetail RemoveFromRoster 'Cancel'; mobile 'Use a different email'/'Skip'/'Not now') -- box them as outline-lime for consistency? ; ForCoaches non-recommended tier 'Start trial' cards (de-emphasized CTAs); mobile PlanCards downgrade (locked blue tier-compare palette); a few solid CTAs that also navigate (Finish on the web, Open Billing) left solid.</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(pipeline): close T208/T172/T097 (verified), record T260 findings
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -86,12 +86,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0E7FF"/>
+        <fgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
+        <fgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>AWAITING USER GO (irreversible): delete both 'Exposed' MyRX Deploy tokens via the dashboard (... menu -&gt; Delete) or the API (DELETE /user/tokens/{id}). The new 'MyRX infra (Claude Code)' token already covers Pages:Edit so deploys keep working after deletion. NOT touched without explicit user confirmation, per the 'never act beyond the given direction' rule.</t>
+          <t>USER SAID 'fix it' 2026-06-14 + asked: do we lose anything / why exposed / to whom / how to prevent recurrence. ANSWERED: (a) deleting ruins NOTHING -- these are the OLD 'MyRX Deploy' tokens, separate from the current deploy path (wrangler authenticates via its own stored login; the new 'MyRX infra' token covers Pages:Edit), and CF auto-revokes 'Exposed' tokens so they're already dead weight; (b) exposed because deploy tokens were historically committed to tracked files (CLAUDE.md) and pushed to GitHub, where CF's GitHub secret-scanning integration found them; (c) to whom = anyone with repo/GitHub access + CF's scanner (the value sat in git history); (d) prevention NOW in place -- .gitignore blocks .env* (verified), scripts/git-hooks/pre-commit secret-scan hook exists (verified), GitHub push protection is the server-side net (user to confirm enabled), and tokens now live ONLY in env / wrangler-auth, never in files. CANNOT DELETE FROM HERE: $env:CLOUDFLARE_API_TOKEN isn't in the tool shell, managing user API tokens needs the 'User &gt; API Tokens' permission the infra token lacks, and wrangler has no delete-token command -&gt; the deletion is the user's 2-click dashboard action (My Profile -&gt; API Tokens -&gt; each 'MyRX Deploy' ... menu -&gt; Delete). Stays Pending until done.</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
@@ -4212,9 +4212,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Cross-platform parity follow-up flagged during T203: the coach promise-card 'pace'-&gt;'rate' fix (energy-balance rate vs cardio pace) may have a parallel in the MOBILE athlete signup WhatsNextScreen if its client-facing copy carries the same 'goal weight and pace' phrasing. Offered to the user; deferred pending go-ahead.</t>
+          <t>Cross-platform parity follow-up flagged during T203: the coach promise-card 'pace'-&gt;'rate' fix (energy-balance rate vs cardio pace) may have a parallel in the MOBILE athlete signup WhatsNextScreen if its client-facing copy carries the same 'goal weight and pace' phrasing. Offered to the user; deferred pending go-ahead. VERIFIED + CLOSED 2026-06-14: read WhatsNextScreen (sign-up.tsx ~L1430) -- its three T168-locked cards carry NO 'goal weight and pace' phrasing; 'pace' shows up only in the separate cardio-reveal screen (legit cardio pace, not energy-balance rate). No parallel to the coach promise-card fix -&gt; nothing to change.</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
@@ -4888,7 +4888,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E86" s="10" t="inlineStr">
+      <c r="E86" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -6292,7 +6292,7 @@
           <t>Cross</t>
         </is>
       </c>
-      <c r="E113" s="10" t="inlineStr">
+      <c r="E113" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -6344,7 +6344,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E114" s="10" t="inlineStr">
+      <c r="E114" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -6396,7 +6396,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E115" s="10" t="inlineStr">
+      <c r="E115" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -6604,7 +6604,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E119" s="9" t="inlineStr">
+      <c r="E119" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -9152,7 +9152,7 @@
           <t>Web + Stripe + Supabase</t>
         </is>
       </c>
-      <c r="E168" s="9" t="inlineStr">
+      <c r="E168" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -9204,9 +9204,9 @@
           <t>Repo-wide</t>
         </is>
       </c>
-      <c r="E169" s="9" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E169" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F169" s="5" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="H169" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS 2026-06-06: sweep CLAUDE.md first (the contract) -&gt; DB semirx-&gt;corerx CHECK migration -&gt; web display/tier code + legal + marketing. The WORKING coach Stripe plumbing (coach-signup / stripe-webhook / workers) stays untouched except semirx-&gt;corerx naming. NOTE the FUNCTIONAL subscription wiring (individual checkout, Stripe products/prices, the model switch) is the T096 build, not this naming/doc sweep -- but every STATEMENT of tiers/prices gets corrected to the lock now. DOC/LEGAL SWEEP DONE 2026-06-06: (1) CLAUDE.md swept (commit f0fbc47) -- locks 18/19/20 + Stream B + launch-checklist IAP + table descriptions now state ONLY the subscription model ($4.99/$6.99 athlete, $19/$39/$99 coach, recurring 17% annual), semirx + one-time/lifetime + first-year-only all removed. (2) DB verified ALREADY CLEAN via MCP -- b2c_purchases.tier CHECK = ('corerx','fullrx'), no semirx, table empty -&gt; NO migration needed. (3) Legal pages (CoachAgreement/RefundPolicy/TermsOfService/PrivacyPolicy) corrected to subscription + new prices + recurring annual; killed one-time/lifetime + the $228/$468/$1188 year-2 figures (kept legit coach $39 + the coach-pro $389-&gt;$292 pro-rated-refund example). (4) Marketing/brand docs (branding/BRAND.md + docs/marketing/*) corrected. 'semirx' string exists nowhere in live code/docs now (only the immutable historical migration FILE 20260524 + the spent rename-stripe script -- correctly left as history; live DB is corerx). Built+deployed index-BtVET8aQ. REMAINING = the T096 FUNCTIONAL build (not a doc fix): live pricing CODE -- Pricing.jsx ATHLETE_TIERS (still one-time/wrong-split), coachPlan.js annual framing, coach Signup/CoachPricing/ForCoaches first-year copy, CoachClientDetail TIER_RANK (Heart-&gt;FullRX), BillingView/BillingTab/AccountSettings/EditProfile -- all get the new model+prices when Stripe subscriptions + individual checkout are wired (they move together). === DEFERRED 2026-06-07 with T096: the doc/legal/marketing/CLAUDE.md/DB sweep is DONE + shipped; the remaining WEB PRICING-CODE sweep (Pricing.jsx tiers-&gt;subscription, coach pages first-year-&gt;recurring, gating Heart-&gt;FullRX, billing-display copy) rides with the T096 billing build (deferred).</t>
+          <t>IN PROGRESS 2026-06-06: sweep CLAUDE.md first (the contract) -&gt; DB semirx-&gt;corerx CHECK migration -&gt; web display/tier code + legal + marketing. The WORKING coach Stripe plumbing (coach-signup / stripe-webhook / workers) stays untouched except semirx-&gt;corerx naming. NOTE the FUNCTIONAL subscription wiring (individual checkout, Stripe products/prices, the model switch) is the T096 build, not this naming/doc sweep -- but every STATEMENT of tiers/prices gets corrected to the lock now. DOC/LEGAL SWEEP DONE 2026-06-06: (1) CLAUDE.md swept (commit f0fbc47) -- locks 18/19/20 + Stream B + launch-checklist IAP + table descriptions now state ONLY the subscription model ($4.99/$6.99 athlete, $19/$39/$99 coach, recurring 17% annual), semirx + one-time/lifetime + first-year-only all removed. (2) DB verified ALREADY CLEAN via MCP -- b2c_purchases.tier CHECK = ('corerx','fullrx'), no semirx, table empty -&gt; NO migration needed. (3) Legal pages (CoachAgreement/RefundPolicy/TermsOfService/PrivacyPolicy) corrected to subscription + new prices + recurring annual; killed one-time/lifetime + the $228/$468/$1188 year-2 figures (kept legit coach $39 + the coach-pro $389-&gt;$292 pro-rated-refund example). (4) Marketing/brand docs (branding/BRAND.md + docs/marketing/*) corrected. 'semirx' string exists nowhere in live code/docs now (only the immutable historical migration FILE 20260524 + the spent rename-stripe script -- correctly left as history; live DB is corerx). Built+deployed index-BtVET8aQ. REMAINING = the T096 FUNCTIONAL build (not a doc fix): live pricing CODE -- Pricing.jsx ATHLETE_TIERS (still one-time/wrong-split), coachPlan.js annual framing, coach Signup/CoachPricing/ForCoaches first-year copy, CoachClientDetail TIER_RANK (Heart-&gt;FullRX), BillingView/BillingTab/AccountSettings/EditProfile -- all get the new model+prices when Stripe subscriptions + individual checkout are wired (they move together). === DEFERRED 2026-06-07 with T096: the doc/legal/marketing/CLAUDE.md/DB sweep is DONE + shipped; the remaining WEB PRICING-CODE sweep (Pricing.jsx tiers-&gt;subscription, coach pages first-year-&gt;recurring, gating Heart-&gt;FullRX, billing-display copy) rides with the T096 billing build (deferred). VERIFIED + CLOSED 2026-06-14 (the NAMING/COPY sweep -- this task's scope -- is complete): (a) Pricing.jsx is GONE (athlete web retired); (b) CoachClientDetail TIER_RANK gates Heart at FULLRX (corerx=1/fullrx=2; Heart pill + DashboardHeartBlock both &gt;= fullrx) -- the 'Heart wrongly in CoreRX' bug is fixed; (c) coach annual copy is recurring (CoachPricing FAQ answer already said 'recurs every year'; fixed the leftover stale QUESTION title 'first-year discount' -&gt; 'annual discount', commit 2073d74); (d) grep of live web/src for first-year/one-time/lifetime/228/468/1188 finds only legit OTP autoComplete + b2c_purchase billing-event labels, no stale pricing copy. The FUNCTIONAL billing build (individual checkout, IAP wiring, billing-page UI) is tracked by T096, not here.</t>
         </is>
       </c>
       <c r="I169" s="7" t="inlineStr">
@@ -9308,7 +9308,7 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E171" s="9" t="inlineStr">
+      <c r="E171" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -10244,7 +10244,7 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E189" s="9" t="inlineStr">
+      <c r="E189" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -14087,7 +14087,7 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E263" s="9" t="inlineStr">
+      <c r="E263" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -14139,7 +14139,7 @@
           <t>Web+DB</t>
         </is>
       </c>
-      <c r="E264" s="9" t="inlineStr">
+      <c r="E264" s="10" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -14243,9 +14243,9 @@
           <t>Web</t>
         </is>
       </c>
-      <c r="E266" s="9" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E266" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F266" s="5" t="inlineStr">
@@ -14255,7 +14255,7 @@
       </c>
       <c r="G266" s="5" t="inlineStr">
         <is>
-          <t>Surfaced 2026-06-10: after finalizing the athlete paywall tier copy on MOBILE (short benefit bullets, 'Fuel &amp; body' / 'Recovery &amp; vitals' taglines, dropped the 'Dashboard'-as-feature line + 'no ads'), the same copy was briefly synced to web/src/pages/Pricing.jsx then REVERTED on user instruction -- web is the coach-facing surface right now and athlete-web is frozen; the public athlete /pricing page stays on its OLD copy until we deliberately do the athlete-web pass.</t>
+          <t>Surfaced 2026-06-10: after finalizing the athlete paywall tier copy on MOBILE (short benefit bullets, 'Fuel &amp; body' / 'Recovery &amp; vitals' taglines, dropped the 'Dashboard'-as-feature line + 'no ads'), the same copy was briefly synced to web/src/pages/Pricing.jsx then REVERTED on user instruction -- web is the coach-facing surface right now and athlete-web is frozen; the public athlete /pricing page stays on its OLD copy until we deliberately do the athlete-web pass. CLOSED-OBSOLETE 2026-06-14: there is no web athlete /pricing page anymore -- web/src/pages/Pricing.jsx does not exist (athlete web retired May 27 2026; App.jsx routes the athlete-host /pricing -&gt; Redirect to /). No sync target -&gt; nothing to do.</t>
         </is>
       </c>
       <c r="H266" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(billing): archive unused athlete Stripe test products (T099); close T174/T175 (won't-do)
T099: ran a TEST-only archive script (sk_test_ guard, athlete-audience filter) -> CoreRX + FullRX products + their 4 prices archived; coach products untouched. T174 (athlete web billing page) + T175 (region-aware routing) closed as won't-do -- launch is native-for-all, no athlete web funnel.
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -9308,9 +9308,9 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E171" s="10" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E171" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
@@ -9325,7 +9325,7 @@
       </c>
       <c r="H171" s="7" t="inlineStr">
         <is>
-          <t>DEFERRED with T096 (billing resume): archive the 2 athlete Stripe products in TEST mode (active=false) to avoid confusion; easy to revive if a web-athlete option is ever added.</t>
+          <t>DEFERRED with T096 (billing resume): archive the 2 athlete Stripe products in TEST mode (active=false) to avoid confusion; easy to revive if a web-athlete option is ever added. DONE 2026-06-14: wrote + ran scripts/archive-stripe-athlete-products.mjs (TEST mode, sk_test_ guard, targets ONLY metadata myrx_audience=athlete) -- archived products CoreRX (prod_UeqnSTO3oR6Lm7) + FullRX (prod_UeqnvBeFTrOHOT) and their 4 prices (corerx/fullrx monthly+annual). 0 active athlete products remain; 3 coach products untouched. Reversible by re-running setup-stripe-sandbox-prices.mjs.</t>
         </is>
       </c>
       <c r="I171" s="7" t="inlineStr">
@@ -14087,9 +14087,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E263" s="10" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E263" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F263" s="5" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="H263" s="7" t="inlineStr">
         <is>
-          <t>Branch on storefront: US -&gt; show 'Subscribe on the web' external link (commission-free); EU storefronts -&gt; external link (entitlement + ~13-20% fee); all other storefronts incl. India + UK -&gt; native IAP purchase + OS-level subscription management. Needs the native billing integration present (to READ the storefront AND run IAP for RoW -- this is the deferred real-IAP module; region detection rides on top). DECIDE: does RoW get native IAP (eats 15-30% on those buyers) or stay email-only (fee-free, no in-app buy)? Manage-surface also differs: web-bought -&gt; our web page; IAP-bought -&gt; Apple/Google native subscription settings (app can deep-link there).</t>
+          <t>Branch on storefront: US -&gt; show 'Subscribe on the web' external link (commission-free); EU storefronts -&gt; external link (entitlement + ~13-20% fee); all other storefronts incl. India + UK -&gt; native IAP purchase + OS-level subscription management. Needs the native billing integration present (to READ the storefront AND run IAP for RoW -- this is the deferred real-IAP module; region detection rides on top). DECIDE: does RoW get native IAP (eats 15-30% on those buyers) or stay email-only (fee-free, no in-app buy)? Manage-surface also differs: web-bought -&gt; our web page; IAP-bought -&gt; Apple/Google native subscription settings (app can deep-link there). CLOSED 2026-06-14 (user: not needed anymore) -- WON'T DO: with launch native-for-all (everyone gets the native store) and the athlete web funnel (T174) dropped, there's no in-app web link to region-gate, so there's nothing to route.</t>
         </is>
       </c>
       <c r="I263" s="7" t="inlineStr">
@@ -14139,9 +14139,9 @@
           <t>Web+DB</t>
         </is>
       </c>
-      <c r="E264" s="10" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E264" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
@@ -14156,7 +14156,7 @@
       </c>
       <c r="H264" s="5" t="inlineStr">
         <is>
-          <t>DECISIONS CONFIRMED 2026-06-10: (1) surface = a /billing route on the existing web app (NOT a subdomain); (2) login = Supabase magic-link primary (+ password fallback); (3) B2C Stripe products + stripe-webhook extension dependency acknowledged. GATED on T176 (launch-rail revenue research) -- BUILD only if that research favors the web funnel; else this stays parked and we keep native-for-all at launch. Remaining scope when greenlit: header 'Signed in as &lt;name&gt; &lt;email&gt;' + avatar + plan state ('FullRX trial -- N days left'); CoreRX/FullRX cards (mirror mobile PlanCards copy) w/ monthly|annual toggle; Stripe Checkout (NEW B2C products corerx_/fullrx_ monthly+annual) -&gt; stripe-webhook writes profiles.b2c_subscription_tier (the same column the app gates on) -&gt; app unlocks; Stripe customer portal for manage/cancel; coach/superuser guard -&gt; redirect to /coach.</t>
+          <t>DECISIONS CONFIRMED 2026-06-10: (1) surface = a /billing route on the existing web app (NOT a subdomain); (2) login = Supabase magic-link primary (+ password fallback); (3) B2C Stripe products + stripe-webhook extension dependency acknowledged. GATED on T176 (launch-rail revenue research) -- BUILD only if that research favors the web funnel; else this stays parked and we keep native-for-all at launch. Remaining scope when greenlit: header 'Signed in as &lt;name&gt; &lt;email&gt;' + avatar + plan state ('FullRX trial -- N days left'); CoreRX/FullRX cards (mirror mobile PlanCards copy) w/ monthly|annual toggle; Stripe Checkout (NEW B2C products corerx_/fullrx_ monthly+annual) -&gt; stripe-webhook writes profiles.b2c_subscription_tier (the same column the app gates on) -&gt; app unlocks; Stripe customer portal for manage/cancel; coach/superuser guard -&gt; redirect to /coach. CLOSED 2026-06-14 (user: not needed anymore) -- WON'T DO: the athlete web billing page is not being built. Launch is native-for-all (athletes subscribe via Apple/Google IAP), so there's no web checkout/funnel to host. Revive only if a web funnel is ever justified.</t>
         </is>
       </c>
       <c r="I264" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(pipeline): close T260 (user deleted the exposed Cloudflare tokens)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -2840,9 +2840,9 @@
           <t>Cloudflare</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>USER SAID 'fix it' 2026-06-14 + asked: do we lose anything / why exposed / to whom / how to prevent recurrence. ANSWERED: (a) deleting ruins NOTHING -- these are the OLD 'MyRX Deploy' tokens, separate from the current deploy path (wrangler authenticates via its own stored login; the new 'MyRX infra' token covers Pages:Edit), and CF auto-revokes 'Exposed' tokens so they're already dead weight; (b) exposed because deploy tokens were historically committed to tracked files (CLAUDE.md) and pushed to GitHub, where CF's GitHub secret-scanning integration found them; (c) to whom = anyone with repo/GitHub access + CF's scanner (the value sat in git history); (d) prevention NOW in place -- .gitignore blocks .env* (verified), scripts/git-hooks/pre-commit secret-scan hook exists (verified), GitHub push protection is the server-side net (user to confirm enabled), and tokens now live ONLY in env / wrangler-auth, never in files. CANNOT DELETE FROM HERE: $env:CLOUDFLARE_API_TOKEN isn't in the tool shell, managing user API tokens needs the 'User &gt; API Tokens' permission the infra token lacks, and wrangler has no delete-token command -&gt; the deletion is the user's 2-click dashboard action (My Profile -&gt; API Tokens -&gt; each 'MyRX Deploy' ... menu -&gt; Delete). Stays Pending until done.</t>
+          <t>USER SAID 'fix it' 2026-06-14 + asked: do we lose anything / why exposed / to whom / how to prevent recurrence. ANSWERED: (a) deleting ruins NOTHING -- these are the OLD 'MyRX Deploy' tokens, separate from the current deploy path (wrangler authenticates via its own stored login; the new 'MyRX infra' token covers Pages:Edit), and CF auto-revokes 'Exposed' tokens so they're already dead weight; (b) exposed because deploy tokens were historically committed to tracked files (CLAUDE.md) and pushed to GitHub, where CF's GitHub secret-scanning integration found them; (c) to whom = anyone with repo/GitHub access + CF's scanner (the value sat in git history); (d) prevention NOW in place -- .gitignore blocks .env* (verified), scripts/git-hooks/pre-commit secret-scan hook exists (verified), GitHub push protection is the server-side net (user to confirm enabled), and tokens now live ONLY in env / wrangler-auth, never in files. CANNOT DELETE FROM HERE: $env:CLOUDFLARE_API_TOKEN isn't in the tool shell, managing user API tokens needs the 'User &gt; API Tokens' permission the infra token lacks, and wrangler has no delete-token command -&gt; the deletion is the user's 2-click dashboard action (My Profile -&gt; API Tokens -&gt; each 'MyRX Deploy' ... menu -&gt; Delete). DONE 2026-06-14: user confirmed both 'Exposed' MyRX Deploy tokens deleted in the CF dashboard. Deploys unaffected (wrangler's own stored auth + the 'MyRX infra' token cover Pages:Edit). Prevention layers (gitignore .env*, pre-commit secret hook) remain in place.</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(pipeline): T166 -> In progress (system studied, proposal recorded)
</commit_message>
<xml_diff>
--- a/docs/TASK_PIPELINE.xlsx
+++ b/docs/TASK_PIPELINE.xlsx
@@ -14556,9 +14556,9 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="E272" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="E272" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
@@ -14568,7 +14568,7 @@
       </c>
       <c r="G272" s="5" t="inlineStr">
         <is>
-          <t>Surfaced 2026-06-09 during T165 reverse-trial design. The athlete trial reminders (7-days-left, 2-days-left, day-30-ended) and future event nudges need a real delivery channel. DECISION: build a proper push + in-app notification system LATER as its own task; for NOW (T165), trial reminders ship via EMAIL only. Likely Expo push notifications + an in-app inbox; backend trigger via a scheduled Supabase function / cron reading trial_ends_at. UPDATE 2026-06-10: the EMAIL channel is now SHELVED (user dropped email sending -- see T165; pg_cron job paused, edge fn + template kept only for reference), so trial reminders currently have NO delivery channel until this system ships. Linking them here is therefore a hard requirement of THIS build, not a 'later migration'.</t>
+          <t>Surfaced 2026-06-09 during T165 reverse-trial design. The athlete trial reminders (7-days-left, 2-days-left, day-30-ended) and future event nudges need a real delivery channel. DECISION: build a proper push + in-app notification system LATER as its own task; for NOW (T165), trial reminders ship via EMAIL only. Likely Expo push notifications + an in-app inbox; backend trigger via a scheduled Supabase function / cron reading trial_ends_at. UPDATE 2026-06-10: the EMAIL channel is now SHELVED (user dropped email sending -- see T165; pg_cron job paused, edge fn + template kept only for reference), so trial reminders currently have NO delivery channel until this system ships. Linking them here is therefore a hard requirement of THIS build, not a 'later migration'. STUDY + PROPOSAL 2026-06-14 (-&gt; In progress): mapped the whole system (3 explore passes). CURRENT STATE: expo-notifications installed + permission already asked at signup, but NO push-token capture/storage, NO runtime handlers, NO notifications/token tables, NO prefs columns; Supabase realtime already powers chat-unread + admin badges; the (shelved) trial-reminders edge fn + pg_cron-nonce rail is the proven dispatcher template. PROPOSED ARCH: one notifications table that drives BOTH an in-app bell+feed AND device push; push-token capture on login; an Expo-push dispatcher edge fn mirroring trial-reminders; event-driven writes (coach msg/suggestion, plan update, PR, invite-accepted) + scheduled nudges (log/streak/hydration/bedtime/next-step + trial 7d/2d/day-30) on the existing hourly cron; a Settings 'Notifications' section (master + per-type toggles + quiet hours); deep-link tap routing. SCOPE SPLIT: athlete=mobile (Expo push + in-app) is the core; coach=web keeps its live unread badges (web/browser push = optional later phase). GATING: in-app feed + table + prefs + dispatcher logic + token capture are ALL buildable NOW; Android push delivery needs a FREE Firebase/FCM project (doable now); iOS push needs paid Apple/APNs (deferred with iOS, same gate as T261). PHASES: 1) in-app center + table + prefs + top event writes + trial reminders re-pointed off the shelved email; 2) Android FCM push live; 3) scheduled nudges; 4) iOS APNs when enrolled; 5) optional coach web push. AWAITING USER decisions (scope split / bell+feed vs badges-only / v1 event set / nudge aggressiveness / Firebase-now vs defer-all-delivery) before building.</t>
         </is>
       </c>
       <c r="H272" s="5" t="inlineStr">

</xml_diff>